<commit_message>
debugging: possible worksheet protection issue
</commit_message>
<xml_diff>
--- a/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
+++ b/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1a2ae81d67634e6/Desktop/Michanikos Artifex Enterprises/MAE Custom Digital Solutions/Workshop Inventory System and Dashboard/GITHUB_MAE_Workshop Inventory App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="8_{EF717C5C-A94F-4A9F-962B-1D35F2984CA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D72D3722-99EF-4559-A18B-5ECB6588E0DC}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="8_{EF717C5C-A94F-4A9F-962B-1D35F2984CA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{016B787D-1E55-48D2-9E34-AFB43FDC6BA6}"/>
   <bookViews>
-    <workbookView xWindow="5268" yWindow="240" windowWidth="16428" windowHeight="11904" firstSheet="6" activeTab="7" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
+    <workbookView xWindow="3804" yWindow="348" windowWidth="16428" windowHeight="11904" firstSheet="6" activeTab="7" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
   </bookViews>
   <sheets>
     <sheet name="Master Dashboard" sheetId="1" r:id="rId1"/>
@@ -1506,7 +1506,6 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G1000" xr:uid="{5CDD912B-3197-4C62-9DE2-F15AE0580881}">
       <formula1>"YES, NO"</formula1>

</xml_diff>

<commit_message>
added two test worksheets to .xlsx
</commit_message>
<xml_diff>
--- a/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
+++ b/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
@@ -5,23 +5,25 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1a2ae81d67634e6/Desktop/Michanikos Artifex Enterprises/MAE Custom Digital Solutions/Workshop Inventory System and Dashboard/GITHUB_MAE_Workshop Inventory App/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MWEAK\OneDrive\Desktop\Michanikos Artifex Enterprises\MAE Custom Digital Solutions\MAE Workshop Inventory Management System\GITHUB_MAE_Workshop Inventory App\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="8_{EF717C5C-A94F-4A9F-962B-1D35F2984CA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E9532D93-E9B6-4C63-954B-A8B5037E0768}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CE4ED70-7C3C-4CCA-B9CD-0FFB5498A43E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6996" yWindow="432" windowWidth="14832" windowHeight="11904" firstSheet="7" activeTab="8" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
+    <workbookView xWindow="5088" yWindow="0" windowWidth="18048" windowHeight="12336" activeTab="1" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
   </bookViews>
   <sheets>
-    <sheet name="Master Dashboard" sheetId="1" r:id="rId1"/>
-    <sheet name="Resell Inventory" sheetId="2" r:id="rId2"/>
-    <sheet name="Shop Machinery" sheetId="3" r:id="rId3"/>
-    <sheet name="Maintenance Log" sheetId="4" r:id="rId4"/>
-    <sheet name="Shop Power Tools" sheetId="5" r:id="rId5"/>
-    <sheet name="Shop Hand Tools" sheetId="6" r:id="rId6"/>
-    <sheet name="Shop Consumables" sheetId="7" r:id="rId7"/>
-    <sheet name="Shop Overhead" sheetId="8" r:id="rId8"/>
-    <sheet name="Supplier Contacts" sheetId="9" r:id="rId9"/>
+    <sheet name="TEST Inventory" sheetId="10" r:id="rId1"/>
+    <sheet name="TEST Dashboard" sheetId="11" r:id="rId2"/>
+    <sheet name="Master Dashboard" sheetId="1" r:id="rId3"/>
+    <sheet name="Resell Inventory" sheetId="2" r:id="rId4"/>
+    <sheet name="Shop Machinery" sheetId="3" r:id="rId5"/>
+    <sheet name="Maintenance Log" sheetId="4" r:id="rId6"/>
+    <sheet name="Shop Power Tools" sheetId="5" r:id="rId7"/>
+    <sheet name="Shop Hand Tools" sheetId="6" r:id="rId8"/>
+    <sheet name="Shop Consumables" sheetId="7" r:id="rId9"/>
+    <sheet name="Shop Overhead" sheetId="8" r:id="rId10"/>
+    <sheet name="Supplier Contacts" sheetId="9" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -44,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="66">
   <si>
     <t>mae_id</t>
   </si>
@@ -203,6 +205,45 @@
   </si>
   <si>
     <t>Website Link</t>
+  </si>
+  <si>
+    <t>TEST String</t>
+  </si>
+  <si>
+    <t>TEST Integer</t>
+  </si>
+  <si>
+    <t>TEST Currency</t>
+  </si>
+  <si>
+    <t>TEST Formula</t>
+  </si>
+  <si>
+    <t>TEST Dropdown</t>
+  </si>
+  <si>
+    <t>TEST calc from other table</t>
+  </si>
+  <si>
+    <t>TEST Number Calc from other table</t>
+  </si>
+  <si>
+    <t>testing</t>
+  </si>
+  <si>
+    <t>Red</t>
+  </si>
+  <si>
+    <t>hot</t>
+  </si>
+  <si>
+    <t>White</t>
+  </si>
+  <si>
+    <t>cold</t>
+  </si>
+  <si>
+    <t>Blue</t>
   </si>
 </sst>
 </file>
@@ -270,7 +311,29 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="88">
+  <dxfs count="95">
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="0"/>
@@ -612,156 +675,186 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:F2" totalsRowShown="0" headerRowDxfId="87" dataDxfId="86">
-  <autoFilter ref="A1:F2" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}" name="TEST_Inventory" displayName="TEST_Inventory" ref="A1:F4" totalsRowShown="0">
+  <autoFilter ref="A1:F4" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="85"/>
-    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Inventory Value" dataDxfId="84"/>
-    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Low Stock Alerts" dataDxfId="83"/>
-    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Upcoming Maintenance" dataDxfId="82"/>
-    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Monthly Overhead Total" dataDxfId="81"/>
-    <tableColumn id="6" xr3:uid="{86A5DBCB-1064-4926-8405-405B453A4546}" name="Supplier Performance" dataDxfId="80"/>
+    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="0">
+      <calculatedColumnFormula>TEST_Inventory[[#This Row],[TEST Integer]]*TEST_Inventory[[#This Row],[TEST Currency]]</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="6" xr3:uid="{AB3A5F3C-FCF0-4466-90FD-8ABB6E18DF5C}" name="TEST Dropdown"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:L2" totalsRowShown="0" headerRowDxfId="79" dataDxfId="78">
-  <autoFilter ref="A1:L2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}"/>
-  <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="77"/>
-    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="76"/>
-    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="75"/>
-    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="74"/>
-    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="73"/>
-    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="72"/>
-    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="71"/>
-    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="70"/>
-    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="69"/>
-    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="68"/>
-    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="67"/>
-    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location" dataDxfId="66"/>
+<file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:G2" totalsRowShown="0" headerRowDxfId="26" dataDxfId="25">
+  <autoFilter ref="A1:G2" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="24"/>
+    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="23"/>
+    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="22"/>
+    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="21"/>
+    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="20"/>
+    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="19"/>
+    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="18"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:J2" insertRow="1" totalsRowShown="0" headerRowDxfId="65" dataDxfId="64">
-  <autoFilter ref="A1:J2" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}"/>
-  <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="63"/>
-    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="62"/>
-    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Model" dataDxfId="61"/>
-    <tableColumn id="4" xr3:uid="{217066CA-63B7-4030-A7FC-54062BE2122E}" name="Manufacturer/Brand" dataDxfId="60"/>
-    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="59"/>
-    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="58"/>
-    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="57"/>
-    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="56"/>
-    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Status" dataDxfId="55"/>
-    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link" dataDxfId="54"/>
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:I2" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16">
+  <autoFilter ref="A1:I2" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}"/>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Supplier Contact Name" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{F7DF2706-439F-40D6-BF96-93ED9838637D}" name="Category" dataDxfId="13"/>
+    <tableColumn id="4" xr3:uid="{63FEC657-4243-4948-9860-735C45290A9E}" name="Account Number" dataDxfId="12"/>
+    <tableColumn id="5" xr3:uid="{2DC90AB0-B9FF-46C3-BC3D-46A6FED781D0}" name="Primary Contact" dataDxfId="11"/>
+    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="10"/>
+    <tableColumn id="7" xr3:uid="{0377D2F7-FA15-4632-BBB9-90166C714228}" name="Phone" dataDxfId="9"/>
+    <tableColumn id="8" xr3:uid="{E2101DCF-5000-49E7-A91F-E543538927B7}" name="Lead Time" dataDxfId="8"/>
+    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Website Link" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:H2" totalsRowShown="0" headerRowDxfId="53" dataDxfId="52">
-  <autoFilter ref="A1:H2" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}"/>
-  <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="51"/>
-    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="50"/>
-    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="49"/>
-    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="48"/>
-    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="47"/>
-    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="46"/>
-    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="45"/>
-    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="44"/>
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}" name="TEST_Dashboard" displayName="TEST_Dashboard" ref="A1:B2" totalsRowShown="0">
+  <autoFilter ref="A1:B2" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="2">
+      <calculatedColumnFormula>SUM(TEST_Inventory[TEST Currency])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="1">
+      <calculatedColumnFormula>SUM(TEST_Inventory[TEST Integer])</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:E2" totalsRowShown="0" headerRowDxfId="43" dataDxfId="42">
-  <autoFilter ref="A1:E2" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}"/>
-  <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="41"/>
-    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Tool ID" dataDxfId="40"/>
-    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Model" dataDxfId="39"/>
-    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Category" dataDxfId="38"/>
-    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="37"/>
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:F2" totalsRowShown="0" headerRowDxfId="94" dataDxfId="93">
+  <autoFilter ref="A1:F2" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="92"/>
+    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Inventory Value" dataDxfId="91"/>
+    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Low Stock Alerts" dataDxfId="90"/>
+    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Upcoming Maintenance" dataDxfId="89"/>
+    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Monthly Overhead Total" dataDxfId="88"/>
+    <tableColumn id="6" xr3:uid="{86A5DBCB-1064-4926-8405-405B453A4546}" name="Supplier Performance" dataDxfId="87"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:E2" totalsRowShown="0" headerRowDxfId="36" dataDxfId="35">
-  <autoFilter ref="A1:E2" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}"/>
-  <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="34"/>
-    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Tool ID" dataDxfId="33"/>
-    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Model" dataDxfId="32"/>
-    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="31"/>
-    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="30"/>
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:L2" totalsRowShown="0" headerRowDxfId="86" dataDxfId="85">
+  <autoFilter ref="A1:L2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}"/>
+  <tableColumns count="12">
+    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="84"/>
+    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="83"/>
+    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="82"/>
+    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="81"/>
+    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="80"/>
+    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="79"/>
+    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="78"/>
+    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="77">
+      <calculatedColumnFormula>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="76"/>
+    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="75"/>
+    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="74"/>
+    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location" dataDxfId="73"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
-<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:H2" insertRow="1" totalsRowShown="0" headerRowDxfId="29" dataDxfId="28">
-  <autoFilter ref="A1:H2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
-  <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="27"/>
-    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="26"/>
-    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="SKU/Item ID" dataDxfId="25"/>
-    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="24"/>
-    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="23"/>
-    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="22"/>
-    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="21"/>
-    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Preferred Supplier" dataDxfId="20"/>
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:J2" insertRow="1" totalsRowShown="0" headerRowDxfId="72" dataDxfId="71">
+  <autoFilter ref="A1:J2" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}"/>
+  <tableColumns count="10">
+    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="70"/>
+    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="69"/>
+    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Model" dataDxfId="68"/>
+    <tableColumn id="4" xr3:uid="{217066CA-63B7-4030-A7FC-54062BE2122E}" name="Manufacturer/Brand" dataDxfId="67"/>
+    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="66"/>
+    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="65"/>
+    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="64"/>
+    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="63"/>
+    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Status" dataDxfId="62"/>
+    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link" dataDxfId="61"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
-<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:G2" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
-  <autoFilter ref="A1:G2" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}"/>
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="15"/>
-    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="14"/>
-    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="13"/>
-    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="12"/>
-    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="11"/>
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:H2" totalsRowShown="0" headerRowDxfId="60" dataDxfId="59">
+  <autoFilter ref="A1:H2" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="58"/>
+    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="57"/>
+    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="56"/>
+    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="55"/>
+    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="54"/>
+    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="53"/>
+    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="52"/>
+    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="51"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:E2" totalsRowShown="0" headerRowDxfId="50" dataDxfId="49">
+  <autoFilter ref="A1:E2" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="48"/>
+    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Tool ID" dataDxfId="47"/>
+    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Model" dataDxfId="46"/>
+    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Category" dataDxfId="45"/>
+    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="44"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:E2" totalsRowShown="0" headerRowDxfId="43" dataDxfId="42">
+  <autoFilter ref="A1:E2" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="41"/>
+    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Tool ID" dataDxfId="40"/>
+    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Model" dataDxfId="39"/>
+    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="38"/>
+    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="37"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:I2" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
-  <autoFilter ref="A1:I2" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}"/>
-  <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Supplier Contact Name" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{F7DF2706-439F-40D6-BF96-93ED9838637D}" name="Category" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{63FEC657-4243-4948-9860-735C45290A9E}" name="Account Number" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{2DC90AB0-B9FF-46C3-BC3D-46A6FED781D0}" name="Primary Contact" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{0377D2F7-FA15-4632-BBB9-90166C714228}" name="Phone" dataDxfId="2"/>
-    <tableColumn id="8" xr3:uid="{E2101DCF-5000-49E7-A91F-E543538927B7}" name="Lead Time" dataDxfId="1"/>
-    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Website Link" dataDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:H2" insertRow="1" totalsRowShown="0" headerRowDxfId="36" dataDxfId="35">
+  <autoFilter ref="A1:H2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="34"/>
+    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="33"/>
+    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="SKU/Item ID" dataDxfId="32"/>
+    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="31"/>
+    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="30"/>
+    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="29"/>
+    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="28"/>
+    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Preferred Supplier" dataDxfId="27"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1083,6 +1176,251 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19832549-C5E9-4018-9E8B-E2F74EABCB4B}">
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="9" style="1" customWidth="1"/>
+    <col min="2" max="2" width="12" style="4" customWidth="1"/>
+    <col min="3" max="3" width="12.88671875" style="10" customWidth="1"/>
+    <col min="4" max="4" width="14.5546875" style="5" customWidth="1"/>
+    <col min="5" max="5" width="14" style="5" customWidth="1"/>
+    <col min="6" max="6" width="15.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="F1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B2" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C2" s="10">
+        <v>3</v>
+      </c>
+      <c r="D2" s="5">
+        <v>100</v>
+      </c>
+      <c r="E2" s="5">
+        <f>TEST_Inventory[[#This Row],[TEST Integer]]*TEST_Inventory[[#This Row],[TEST Currency]]</f>
+        <v>300</v>
+      </c>
+      <c r="F2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B3" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="C3" s="10">
+        <v>4</v>
+      </c>
+      <c r="D3" s="5">
+        <v>10</v>
+      </c>
+      <c r="E3" s="5">
+        <f>TEST_Inventory[[#This Row],[TEST Integer]]*TEST_Inventory[[#This Row],[TEST Currency]]</f>
+        <v>40</v>
+      </c>
+      <c r="F3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B4" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C4" s="10">
+        <v>5</v>
+      </c>
+      <c r="D4" s="5">
+        <v>20</v>
+      </c>
+      <c r="E4" s="5">
+        <f>TEST_Inventory[[#This Row],[TEST Integer]]*TEST_Inventory[[#This Row],[TEST Currency]]</f>
+        <v>100</v>
+      </c>
+      <c r="F4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F1:F1048576" xr:uid="{B24FB432-D812-4DA7-AD2F-DE8035FBCC42}">
+      <formula1>"Red, White, Blue"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3185D484-1AEA-488F-ADB2-C66611F8B5C9}">
+  <sheetPr codeName="Sheet8"/>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="9" style="1" customWidth="1"/>
+    <col min="2" max="2" width="28.88671875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="60.6640625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="19.33203125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="10.33203125" style="7" customWidth="1"/>
+    <col min="6" max="6" width="9.33203125" style="3" customWidth="1"/>
+    <col min="7" max="7" width="11.33203125" style="2" customWidth="1"/>
+    <col min="8" max="16384" width="8.88671875" style="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>45</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G1000" xr:uid="{5CDD912B-3197-4C62-9DE2-F15AE0580881}">
+      <formula1>"YES, NO"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B1000" xr:uid="{AA2AF827-8A0A-4B34-A36E-624457B5758A}">
+      <formula1>"Rent/Mortgage, Utilities, Insurance, Other"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6150BED1-88FC-488E-B7E1-4C6CBEB9589C}">
+  <sheetPr codeName="Sheet9"/>
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="9" style="1" customWidth="1"/>
+    <col min="2" max="2" width="30.5546875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="26.33203125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="17" style="2" customWidth="1"/>
+    <col min="5" max="5" width="21" style="2" customWidth="1"/>
+    <col min="6" max="6" width="20.6640625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="12.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.109375" style="2" customWidth="1"/>
+    <col min="9" max="9" width="32.33203125" style="2" customWidth="1"/>
+    <col min="10" max="16384" width="8.88671875" style="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{849BF9A6-CD45-4FD2-AD73-886C99848EAC}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="24.21875" style="5" customWidth="1"/>
+    <col min="2" max="2" width="31.5546875" style="10" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="5">
+        <f>SUM(TEST_Inventory[TEST Currency])</f>
+        <v>130</v>
+      </c>
+      <c r="B2" s="10">
+        <f>SUM(TEST_Inventory[TEST Integer])</f>
+        <v>12</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2834D935-E140-4D64-A4CD-4A9FB8899FE0}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:F1"/>
@@ -1126,10 +1464,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDE7BF89-A2E7-4A6F-B822-317739E206EC}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
@@ -1185,8 +1523,20 @@
         <v>16</v>
       </c>
     </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="F2" s="3">
+        <v>5</v>
+      </c>
+      <c r="G2" s="3">
+        <v>5</v>
+      </c>
+      <c r="H2" s="5">
+        <f>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</f>
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
-  <dataValidations count="2">
+  <dataValidations disablePrompts="1" count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I1000" xr:uid="{F45414DD-76C8-4DC4-96E2-15B89FDB5B51}">
       <formula1>"work not started, restoration in progress, for sale, sold"</formula1>
     </dataValidation>
@@ -1202,7 +1552,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B027EC69-551F-4051-8A71-8B106D207C6D}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:J1"/>
@@ -1266,7 +1616,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB7AACC4-9DA2-4A53-AD77-8C5E0C1BF474}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:H1"/>
@@ -1325,7 +1675,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEDDDAA7-75C3-4AA5-ABFD-D5FB4C627E4C}">
   <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:E1"/>
@@ -1372,7 +1722,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F39ADDA6-CD5F-4655-A9C0-9676DDAC362E}">
   <sheetPr codeName="Sheet6"/>
   <dimension ref="A1:E1"/>
@@ -1416,7 +1766,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E1902F1-C59B-4A1A-9D95-2C39AEF944E5}">
   <sheetPr codeName="Sheet7"/>
   <dimension ref="A1:H1"/>
@@ -1465,114 +1815,4 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3185D484-1AEA-488F-ADB2-C66611F8B5C9}">
-  <sheetPr codeName="Sheet8"/>
-  <dimension ref="A1:G1"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="9" style="1" customWidth="1"/>
-    <col min="2" max="2" width="28.88671875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="60.6640625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="19.33203125" style="2" customWidth="1"/>
-    <col min="5" max="5" width="10.33203125" style="7" customWidth="1"/>
-    <col min="6" max="6" width="9.33203125" style="3" customWidth="1"/>
-    <col min="7" max="7" width="11.33203125" style="2" customWidth="1"/>
-    <col min="8" max="16384" width="8.88671875" style="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>45</v>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G1000" xr:uid="{5CDD912B-3197-4C62-9DE2-F15AE0580881}">
-      <formula1>"YES, NO"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B1000" xr:uid="{AA2AF827-8A0A-4B34-A36E-624457B5758A}">
-      <formula1>"Rent/Mortgage, Utilities, Insurance, Other"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6150BED1-88FC-488E-B7E1-4C6CBEB9589C}">
-  <sheetPr codeName="Sheet9"/>
-  <dimension ref="A1:I1"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="9" style="1" customWidth="1"/>
-    <col min="2" max="2" width="30.5546875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="26.33203125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="17" style="2" customWidth="1"/>
-    <col min="5" max="5" width="21" style="2" customWidth="1"/>
-    <col min="6" max="6" width="20.6640625" style="2" customWidth="1"/>
-    <col min="7" max="7" width="12.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.109375" style="2" customWidth="1"/>
-    <col min="9" max="9" width="32.33203125" style="2" customWidth="1"/>
-    <col min="10" max="16384" width="8.88671875" style="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>52</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
updated master Excel spreadsheet
</commit_message>
<xml_diff>
--- a/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
+++ b/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MWEAK\OneDrive\Desktop\Michanikos Artifex Enterprises\MAE Custom Digital Solutions\MAE Workshop Inventory Management System\GITHUB_MAE_Workshop Inventory App\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1a2ae81d67634e6/Desktop/Michanikos Artifex Enterprises/MAE Custom Digital Solutions/MAE Workshop Inventory Management System/GITHUB_MAE_Workshop Inventory App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CE4ED70-7C3C-4CCA-B9CD-0FFB5498A43E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="45" documentId="13_ncr:1_{8CE4ED70-7C3C-4CCA-B9CD-0FFB5498A43E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C37D2403-5298-468D-9B1D-AEA9CE38C7EF}"/>
   <bookViews>
-    <workbookView xWindow="2184" yWindow="336" windowWidth="20856" windowHeight="11904" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
+    <workbookView xWindow="-180" yWindow="0" windowWidth="16728" windowHeight="11904" firstSheet="8" activeTab="10" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
   </bookViews>
   <sheets>
     <sheet name="TEST Inventory" sheetId="10" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="70">
   <si>
     <t>mae_id</t>
   </si>
@@ -117,9 +117,6 @@
     <t>Status</t>
   </si>
   <si>
-    <t>Manual Link</t>
-  </si>
-  <si>
     <t>Log ID</t>
   </si>
   <si>
@@ -186,27 +183,12 @@
     <t>Auto-Pay?</t>
   </si>
   <si>
-    <t>Supplier Contact Name</t>
-  </si>
-  <si>
-    <t>Account Number</t>
-  </si>
-  <si>
-    <t>Primary Contact</t>
-  </si>
-  <si>
     <t>Email</t>
   </si>
   <si>
     <t>Phone</t>
   </si>
   <si>
-    <t>Lead Time</t>
-  </si>
-  <si>
-    <t>Website Link</t>
-  </si>
-  <si>
     <t>TEST String</t>
   </si>
   <si>
@@ -244,6 +226,36 @@
   </si>
   <si>
     <t>Blue</t>
+  </si>
+  <si>
+    <t>Website</t>
+  </si>
+  <si>
+    <t>Supplier Name</t>
+  </si>
+  <si>
+    <t>Contact Person</t>
+  </si>
+  <si>
+    <t>Notes/Other Info</t>
+  </si>
+  <si>
+    <t>Manual Link/Other Info</t>
+  </si>
+  <si>
+    <t>Asset Description</t>
+  </si>
+  <si>
+    <t>Functional Category</t>
+  </si>
+  <si>
+    <t>Operational Category</t>
+  </si>
+  <si>
+    <t>Power Source</t>
+  </si>
+  <si>
+    <t>Current Inventory Value</t>
   </si>
 </sst>
 </file>
@@ -254,10 +266,16 @@
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="mm/dd/yyyy"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -311,22 +329,32 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="95">
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
+  <dxfs count="98">
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -679,11 +707,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}" name="TEST_Inventory" displayName="TEST_Inventory" ref="A1:F4" totalsRowShown="0">
   <autoFilter ref="A1:F4" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="94"/>
-    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="93"/>
-    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="92"/>
-    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="91"/>
-    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="90">
+    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="97"/>
+    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="96"/>
+    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="95"/>
+    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="94"/>
+    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="93">
       <calculatedColumnFormula>TEST_Inventory[[#This Row],[TEST Integer]]*TEST_Inventory[[#This Row],[TEST Currency]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{AB3A5F3C-FCF0-4466-90FD-8ABB6E18DF5C}" name="TEST Dropdown"/>
@@ -693,34 +721,32 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:G2" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:G2" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
   <autoFilter ref="A1:G2" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="15"/>
-    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="14"/>
-    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="13"/>
-    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="12"/>
-    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="11"/>
+    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="18"/>
+    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="17"/>
+    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="16"/>
+    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="15"/>
+    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:I2" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
-  <autoFilter ref="A1:I2" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}"/>
-  <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Supplier Contact Name" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{F7DF2706-439F-40D6-BF96-93ED9838637D}" name="Category" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{63FEC657-4243-4948-9860-735C45290A9E}" name="Account Number" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{2DC90AB0-B9FF-46C3-BC3D-46A6FED781D0}" name="Primary Contact" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{0377D2F7-FA15-4632-BBB9-90166C714228}" name="Phone" dataDxfId="2"/>
-    <tableColumn id="8" xr3:uid="{E2101DCF-5000-49E7-A91F-E543538927B7}" name="Lead Time" dataDxfId="1"/>
-    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Website Link" dataDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+  <autoFilter ref="A1:G2" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="11"/>
+    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="10"/>
+    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="9"/>
+    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="5"/>
+    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -730,10 +756,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}" name="TEST_Dashboard" displayName="TEST_Dashboard" ref="A1:B2" totalsRowShown="0">
   <autoFilter ref="A1:B2" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="89">
+    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="92">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Currency])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="88">
+    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="91">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Integer])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -742,119 +768,124 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:F2" totalsRowShown="0" headerRowDxfId="87" dataDxfId="86">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:F2" totalsRowShown="0" headerRowDxfId="90" dataDxfId="89">
   <autoFilter ref="A1:F2" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="85"/>
-    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Inventory Value" dataDxfId="84"/>
-    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Low Stock Alerts" dataDxfId="83"/>
-    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Upcoming Maintenance" dataDxfId="82"/>
-    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Monthly Overhead Total" dataDxfId="81"/>
-    <tableColumn id="6" xr3:uid="{86A5DBCB-1064-4926-8405-405B453A4546}" name="Supplier Performance" dataDxfId="80"/>
+    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="88"/>
+    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Inventory Value" dataDxfId="87"/>
+    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Low Stock Alerts" dataDxfId="86"/>
+    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Upcoming Maintenance" dataDxfId="85"/>
+    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Monthly Overhead Total" dataDxfId="84"/>
+    <tableColumn id="6" xr3:uid="{86A5DBCB-1064-4926-8405-405B453A4546}" name="Supplier Performance" dataDxfId="83"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:L2" totalsRowShown="0" headerRowDxfId="79" dataDxfId="78">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:L2" totalsRowShown="0" headerRowDxfId="82" dataDxfId="81">
   <autoFilter ref="A1:L2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="77"/>
-    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="76"/>
-    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="75"/>
-    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="74"/>
-    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="73"/>
-    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="72"/>
-    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="71"/>
-    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="70">
+    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="80"/>
+    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="79"/>
+    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="78"/>
+    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="77"/>
+    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="76"/>
+    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="75"/>
+    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="74"/>
+    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="73">
       <calculatedColumnFormula>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="69"/>
-    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="68"/>
-    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="67"/>
-    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location" dataDxfId="66"/>
+    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="72"/>
+    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="71"/>
+    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="70"/>
+    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location" dataDxfId="69"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:J2" insertRow="1" totalsRowShown="0" headerRowDxfId="65" dataDxfId="64">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:J2" insertRow="1" totalsRowShown="0" headerRowDxfId="68" dataDxfId="67">
   <autoFilter ref="A1:J2" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="63"/>
-    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="62"/>
-    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Model" dataDxfId="61"/>
-    <tableColumn id="4" xr3:uid="{217066CA-63B7-4030-A7FC-54062BE2122E}" name="Manufacturer/Brand" dataDxfId="60"/>
-    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="59"/>
-    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="58"/>
-    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="57"/>
-    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="56"/>
-    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Status" dataDxfId="55"/>
-    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link" dataDxfId="54"/>
+    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="66"/>
+    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="65"/>
+    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Model" dataDxfId="64"/>
+    <tableColumn id="4" xr3:uid="{217066CA-63B7-4030-A7FC-54062BE2122E}" name="Manufacturer/Brand" dataDxfId="63"/>
+    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="62"/>
+    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="61"/>
+    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="60"/>
+    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="59"/>
+    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Status" dataDxfId="58"/>
+    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="57"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:H2" totalsRowShown="0" headerRowDxfId="53" dataDxfId="52">
-  <autoFilter ref="A1:H2" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}"/>
-  <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="51"/>
-    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="50"/>
-    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="49"/>
-    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="48"/>
-    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="47"/>
-    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="46"/>
-    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="45"/>
-    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="44"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:I2" totalsRowShown="0" headerRowDxfId="56" dataDxfId="55">
+  <autoFilter ref="A1:I2" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}"/>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="54"/>
+    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="53"/>
+    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="52"/>
+    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset Description" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="51"/>
+    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="50"/>
+    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="49"/>
+    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="48"/>
+    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="47"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:E2" totalsRowShown="0" headerRowDxfId="43" dataDxfId="42">
-  <autoFilter ref="A1:E2" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}"/>
-  <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="41"/>
-    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Tool ID" dataDxfId="40"/>
-    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Model" dataDxfId="39"/>
-    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Category" dataDxfId="38"/>
-    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="37"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:G2" totalsRowShown="0" headerRowDxfId="46" dataDxfId="45">
+  <autoFilter ref="A1:G2" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="44"/>
+    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Tool ID" dataDxfId="43"/>
+    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Model" dataDxfId="42"/>
+    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="41"/>
+    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="40"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:E2" totalsRowShown="0" headerRowDxfId="36" dataDxfId="35">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:E2" totalsRowShown="0" headerRowDxfId="39" dataDxfId="38">
   <autoFilter ref="A1:E2" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="34"/>
-    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Tool ID" dataDxfId="33"/>
-    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Model" dataDxfId="32"/>
-    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="31"/>
-    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="30"/>
+    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="37"/>
+    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Tool ID" dataDxfId="36"/>
+    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Model" dataDxfId="35"/>
+    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="34"/>
+    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="33"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:H2" insertRow="1" totalsRowShown="0" headerRowDxfId="29" dataDxfId="28">
-  <autoFilter ref="A1:H2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
-  <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="27"/>
-    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="26"/>
-    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="SKU/Item ID" dataDxfId="25"/>
-    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="24"/>
-    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="23"/>
-    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="22"/>
-    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="21"/>
-    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Preferred Supplier" dataDxfId="20"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:J2" insertRow="1" totalsRowShown="0" headerRowDxfId="32" dataDxfId="31">
+  <autoFilter ref="A1:J2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
+  <tableColumns count="10">
+    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="30"/>
+    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="29"/>
+    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="SKU/Item ID" dataDxfId="28"/>
+    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="27"/>
+    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="26"/>
+    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="25"/>
+    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="24"/>
+    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="0"/>
+    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Preferred Supplier" dataDxfId="23"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1193,24 +1224,24 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="F1" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B2" s="4" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="C2" s="10">
         <v>3</v>
@@ -1223,12 +1254,12 @@
         <v>300</v>
       </c>
       <c r="F2" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B3" s="4" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="C3" s="10">
         <v>4</v>
@@ -1241,12 +1272,12 @@
         <v>40</v>
       </c>
       <c r="F3" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B4" s="4" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="C4" s="10">
         <v>5</v>
@@ -1259,7 +1290,7 @@
         <v>100</v>
       </c>
       <c r="F4" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -1296,22 +1327,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="F1" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="4" t="s">
         <v>44</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -1333,48 +1364,39 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6150BED1-88FC-488E-B7E1-4C6CBEB9589C}">
   <sheetPr codeName="Sheet9"/>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
-    <col min="2" max="2" width="30.5546875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="26.33203125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="17" style="2" customWidth="1"/>
-    <col min="5" max="5" width="21" style="2" customWidth="1"/>
-    <col min="6" max="6" width="20.6640625" style="2" customWidth="1"/>
-    <col min="7" max="7" width="12.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.109375" style="2" customWidth="1"/>
-    <col min="9" max="9" width="32.33203125" style="2" customWidth="1"/>
-    <col min="10" max="16384" width="8.88671875" style="6"/>
+    <col min="2" max="2" width="25.109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="30.5546875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="21" style="2" customWidth="1"/>
+    <col min="5" max="6" width="20.6640625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="32.33203125" style="2" customWidth="1"/>
+    <col min="8" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="C1" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>47</v>
-      </c>
       <c r="E1" s="4" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -1396,10 +1418,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -1536,7 +1558,7 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations disablePrompts="1" count="2">
+  <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I1000" xr:uid="{F45414DD-76C8-4DC4-96E2-15B89FDB5B51}">
       <formula1>"work not started, restoration in progress, for sale, sold"</formula1>
     </dataValidation>
@@ -1600,7 +1622,7 @@
         <v>22</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>23</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -1619,52 +1641,56 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB7AACC4-9DA2-4A53-AD77-8C5E0C1BF474}">
   <sheetPr codeName="Sheet4"/>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9" style="1" customWidth="1"/>
-    <col min="2" max="2" width="7.6640625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="9.5546875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="13.33203125" style="7" customWidth="1"/>
-    <col min="5" max="5" width="13.33203125" style="6" customWidth="1"/>
-    <col min="6" max="6" width="15.88671875" style="6" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.6640625" style="3" customWidth="1"/>
-    <col min="8" max="8" width="17.5546875" style="7" customWidth="1"/>
-    <col min="9" max="16384" width="8.88671875" style="6"/>
+    <col min="1" max="1" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.6640625" style="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.6640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.33203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18" style="7" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="F1" t="s">
         <v>25</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>26</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="I1" s="8" t="s">
         <v>28</v>
-      </c>
-      <c r="H1" s="8" t="s">
-        <v>29</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E1000" xr:uid="{E5FFE733-A9D3-430E-8950-CAD58FEAE2C9}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F1000" xr:uid="{E5FFE733-A9D3-430E-8950-CAD58FEAE2C9}">
       <formula1>"Preventive, Repair"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F1000" xr:uid="{8BC162F1-575A-44E2-AA38-454BF93A8AFF}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G1000" xr:uid="{8BC162F1-575A-44E2-AA38-454BF93A8AFF}">
       <formula1>"Self in Shop, Contractor in Shop, Out of Shop"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1678,40 +1704,49 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEDDDAA7-75C3-4AA5-ABFD-D5FB4C627E4C}">
   <sheetPr codeName="Sheet5"/>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
     <col min="2" max="2" width="8.6640625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="72.5546875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="13.109375" style="6" customWidth="1"/>
-    <col min="5" max="5" width="13.5546875" style="6" customWidth="1"/>
-    <col min="6" max="16384" width="8.88671875" style="6"/>
+    <col min="3" max="3" width="50.44140625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="19.88671875" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.88671875" style="6" customWidth="1"/>
+    <col min="6" max="6" width="14.44140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.5546875" style="6" customWidth="1"/>
+    <col min="8" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E1" t="s">
+        <v>67</v>
+      </c>
+      <c r="F1" t="s">
+        <v>68</v>
+      </c>
+      <c r="G1" t="s">
         <v>31</v>
-      </c>
-      <c r="D1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E1" t="s">
-        <v>32</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D1000" xr:uid="{FF61F80C-5E23-45D6-B39D-7C5635258115}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:F1000" xr:uid="{FF61F80C-5E23-45D6-B39D-7C5635258115}">
       <formula1>"Circular Saw, Drill, Sander, Grinder, Other"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E1000" xr:uid="{DB752B4D-0E75-42D1-B907-2DBC5792F422}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G1000" xr:uid="{DB752B4D-0E75-42D1-B907-2DBC5792F422}">
       <formula1>"New, Operational, Needs Repair, Broken"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1741,16 +1776,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>30</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>31</v>
       </c>
       <c r="D1" t="s">
         <v>8</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -1769,21 +1804,22 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E1902F1-C59B-4A1A-9D95-2C39AEF944E5}">
   <sheetPr codeName="Sheet7"/>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
     <col min="2" max="2" width="41.6640625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="18.44140625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="15.5546875" style="2" customWidth="1"/>
-    <col min="5" max="5" width="14.33203125" style="9" customWidth="1"/>
-    <col min="6" max="6" width="14.109375" style="9" customWidth="1"/>
-    <col min="7" max="7" width="10.44140625" style="3" customWidth="1"/>
-    <col min="8" max="8" width="46.6640625" style="2" customWidth="1"/>
-    <col min="9" max="16384" width="8.88671875" style="6"/>
+    <col min="3" max="4" width="18.44140625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="15.5546875" style="2" customWidth="1"/>
+    <col min="6" max="6" width="14.33203125" style="9" customWidth="1"/>
+    <col min="7" max="7" width="14.109375" style="9" customWidth="1"/>
+    <col min="8" max="8" width="10.44140625" style="3" customWidth="1"/>
+    <col min="9" max="9" width="22.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="46.6640625" style="2" customWidth="1"/>
+    <col min="11" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1791,22 +1827,28 @@
         <v>7</v>
       </c>
       <c r="C1" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="F1" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="G1" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="H1" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="I1" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="J1" s="4" t="s">
         <v>38</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added formulas to excel spreadsheet and updated formatting for dates and currency
</commit_message>
<xml_diff>
--- a/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
+++ b/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1a2ae81d67634e6/Desktop/Michanikos Artifex Enterprises/MAE Custom Digital Solutions/MAE Workshop Inventory Management System/GITHUB_MAE_Workshop Inventory App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="45" documentId="13_ncr:1_{8CE4ED70-7C3C-4CCA-B9CD-0FFB5498A43E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C37D2403-5298-468D-9B1D-AEA9CE38C7EF}"/>
+  <xr:revisionPtr revIDLastSave="68" documentId="13_ncr:1_{8CE4ED70-7C3C-4CCA-B9CD-0FFB5498A43E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0F0FF794-C0F8-4640-A91F-B46240745C39}"/>
   <bookViews>
-    <workbookView xWindow="-180" yWindow="0" windowWidth="16728" windowHeight="11904" firstSheet="8" activeTab="10" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="6" activeTab="10" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
   </bookViews>
   <sheets>
     <sheet name="TEST Inventory" sheetId="10" r:id="rId1"/>
@@ -262,9 +262,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    <numFmt numFmtId="165" formatCode="mm/dd/yyyy"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -317,14 +316,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -335,55 +334,7 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -391,36 +342,6 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="mm/dd/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
       <protection locked="0" hidden="0"/>
     </dxf>
@@ -433,78 +354,11 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="mm/dd/yyyy"/>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -512,42 +366,7 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="mm/dd/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -555,37 +374,7 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="mm/dd/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -597,7 +386,15 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -605,30 +402,228 @@
       <protection locked="1" hidden="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="mm/dd/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="1" hidden="1"/>
     </dxf>
@@ -639,56 +634,60 @@
       <protection locked="1" hidden="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
+      <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -703,15 +702,19 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}" name="TEST_Inventory" displayName="TEST_Inventory" ref="A1:F4" totalsRowShown="0">
   <autoFilter ref="A1:F4" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="97"/>
-    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="96"/>
-    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="95"/>
-    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="94"/>
-    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="93">
+    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="88"/>
+    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="87"/>
+    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="86"/>
+    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="85"/>
+    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="84">
       <calculatedColumnFormula>TEST_Inventory[[#This Row],[TEST Integer]]*TEST_Inventory[[#This Row],[TEST Currency]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{AB3A5F3C-FCF0-4466-90FD-8ABB6E18DF5C}" name="TEST Dropdown"/>
@@ -721,32 +724,32 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:G2" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:G2" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23">
   <autoFilter ref="A1:G2" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="20"/>
-    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="19"/>
-    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="18"/>
-    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="17"/>
-    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="16"/>
-    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="15"/>
-    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="14"/>
+    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="22"/>
+    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="20"/>
+    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="0"/>
+    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="18"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="97" dataDxfId="96">
   <autoFilter ref="A1:G2" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="11"/>
-    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="10"/>
-    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="9"/>
-    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="5"/>
-    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="95"/>
+    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="94"/>
+    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="93"/>
+    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="92"/>
+    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="91"/>
+    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="90"/>
+    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="89"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -756,10 +759,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}" name="TEST_Dashboard" displayName="TEST_Dashboard" ref="A1:B2" totalsRowShown="0">
   <autoFilter ref="A1:B2" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="92">
+    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="83">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Currency])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="91">
+    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="82">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Integer])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -768,124 +771,126 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:F2" totalsRowShown="0" headerRowDxfId="90" dataDxfId="89">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:F2" totalsRowShown="0" headerRowDxfId="81" dataDxfId="80">
   <autoFilter ref="A1:F2" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="88"/>
-    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Inventory Value" dataDxfId="87"/>
-    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Low Stock Alerts" dataDxfId="86"/>
-    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Upcoming Maintenance" dataDxfId="85"/>
-    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Monthly Overhead Total" dataDxfId="84"/>
-    <tableColumn id="6" xr3:uid="{86A5DBCB-1064-4926-8405-405B453A4546}" name="Supplier Performance" dataDxfId="83"/>
+    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="79"/>
+    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Inventory Value" dataDxfId="78"/>
+    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Low Stock Alerts" dataDxfId="77"/>
+    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Upcoming Maintenance" dataDxfId="76"/>
+    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Monthly Overhead Total" dataDxfId="75"/>
+    <tableColumn id="6" xr3:uid="{86A5DBCB-1064-4926-8405-405B453A4546}" name="Supplier Performance" dataDxfId="74"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:L2" totalsRowShown="0" headerRowDxfId="82" dataDxfId="81">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:L2" totalsRowShown="0" headerRowDxfId="73" dataDxfId="72">
   <autoFilter ref="A1:L2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="80"/>
-    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="79"/>
-    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="78"/>
-    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="77"/>
-    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="76"/>
-    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="75"/>
-    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="74"/>
-    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="73">
+    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="71"/>
+    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="70"/>
+    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="69"/>
+    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="68"/>
+    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="14"/>
+    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="15"/>
+    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="16"/>
+    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="17">
       <calculatedColumnFormula>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="72"/>
-    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="71"/>
-    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="70"/>
-    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location" dataDxfId="69"/>
+    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="67"/>
+    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="12"/>
+    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="13"/>
+    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location" dataDxfId="66"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:J2" insertRow="1" totalsRowShown="0" headerRowDxfId="68" dataDxfId="67">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:J2" insertRow="1" totalsRowShown="0" headerRowDxfId="65" dataDxfId="64">
   <autoFilter ref="A1:J2" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="66"/>
-    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="65"/>
-    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Model" dataDxfId="64"/>
-    <tableColumn id="4" xr3:uid="{217066CA-63B7-4030-A7FC-54062BE2122E}" name="Manufacturer/Brand" dataDxfId="63"/>
-    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="62"/>
-    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="61"/>
-    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="60"/>
-    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="59"/>
-    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Status" dataDxfId="58"/>
-    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="57"/>
+    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="63"/>
+    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="62"/>
+    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Model" dataDxfId="61"/>
+    <tableColumn id="4" xr3:uid="{217066CA-63B7-4030-A7FC-54062BE2122E}" name="Manufacturer/Brand" dataDxfId="60"/>
+    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="59"/>
+    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="11"/>
+    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="10"/>
+    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="58"/>
+    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Status" dataDxfId="57"/>
+    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="56"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:I2" totalsRowShown="0" headerRowDxfId="56" dataDxfId="55">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:I2" totalsRowShown="0" headerRowDxfId="55" dataDxfId="54">
   <autoFilter ref="A1:I2" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="54"/>
-    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="53"/>
-    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="52"/>
-    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset Description" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="51"/>
-    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="50"/>
-    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="49"/>
-    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="48"/>
-    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="47"/>
+    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="53"/>
+    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="52"/>
+    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="51"/>
+    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset Description" dataDxfId="50"/>
+    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="49"/>
+    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="48"/>
+    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="8"/>
+    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:G2" totalsRowShown="0" headerRowDxfId="46" dataDxfId="45">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:G2" totalsRowShown="0" headerRowDxfId="47" dataDxfId="46">
   <autoFilter ref="A1:G2" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="44"/>
-    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Tool ID" dataDxfId="43"/>
-    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Model" dataDxfId="42"/>
-    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="41"/>
-    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="3"/>
-    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="40"/>
+    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="45"/>
+    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Tool ID" dataDxfId="44"/>
+    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Model" dataDxfId="43"/>
+    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="42"/>
+    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="41"/>
+    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="40"/>
+    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="39"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:E2" totalsRowShown="0" headerRowDxfId="39" dataDxfId="38">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:E2" totalsRowShown="0" headerRowDxfId="38" dataDxfId="37">
   <autoFilter ref="A1:E2" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="37"/>
-    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Tool ID" dataDxfId="36"/>
-    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Model" dataDxfId="35"/>
-    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="34"/>
-    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="33"/>
+    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="36"/>
+    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Tool ID" dataDxfId="35"/>
+    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Model" dataDxfId="34"/>
+    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="33"/>
+    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:J2" insertRow="1" totalsRowShown="0" headerRowDxfId="32" dataDxfId="31">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:J2" totalsRowShown="0" headerRowDxfId="32" dataDxfId="31">
   <autoFilter ref="A1:J2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="30"/>
     <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="29"/>
     <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="SKU/Item ID" dataDxfId="28"/>
-    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="1"/>
-    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="27"/>
-    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="26"/>
-    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="25"/>
-    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="24"/>
-    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="0"/>
-    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Preferred Supplier" dataDxfId="23"/>
+    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="27"/>
+    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="26"/>
+    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="4"/>
+    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="3"/>
+    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="2">
+      <calculatedColumnFormula>Shop_Consumables[[#This Row],[Current Stock]]*Shop_Consumables[[#This Row],[Unit Cost]]</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Preferred Supplier" dataDxfId="25"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1213,7 +1218,7 @@
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
     <col min="2" max="2" width="12" style="4" customWidth="1"/>
-    <col min="3" max="3" width="12.88671875" style="10" customWidth="1"/>
+    <col min="3" max="3" width="12.88671875" style="8" customWidth="1"/>
     <col min="4" max="4" width="14.5546875" style="5" customWidth="1"/>
     <col min="5" max="5" width="14" style="5" customWidth="1"/>
     <col min="6" max="6" width="15.5546875" customWidth="1"/>
@@ -1226,7 +1231,7 @@
       <c r="B1" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="8" t="s">
         <v>48</v>
       </c>
       <c r="D1" s="5" t="s">
@@ -1243,7 +1248,7 @@
       <c r="B2" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="C2" s="10">
+      <c r="C2" s="8">
         <v>3</v>
       </c>
       <c r="D2" s="5">
@@ -1261,7 +1266,7 @@
       <c r="B3" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="8">
         <v>4</v>
       </c>
       <c r="D3" s="5">
@@ -1279,7 +1284,7 @@
       <c r="B4" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="8">
         <v>5</v>
       </c>
       <c r="D4" s="5">
@@ -1316,7 +1321,7 @@
     <col min="2" max="2" width="28.88671875" style="2" customWidth="1"/>
     <col min="3" max="3" width="60.6640625" style="2" customWidth="1"/>
     <col min="4" max="4" width="19.33203125" style="2" customWidth="1"/>
-    <col min="5" max="5" width="10.33203125" style="7" customWidth="1"/>
+    <col min="5" max="5" width="10.33203125" style="10" customWidth="1"/>
     <col min="6" max="6" width="9.33203125" style="3" customWidth="1"/>
     <col min="7" max="7" width="11.33203125" style="2" customWidth="1"/>
     <col min="8" max="16384" width="8.88671875" style="6"/>
@@ -1335,7 +1340,7 @@
       <c r="D1" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="9" t="s">
         <v>42</v>
       </c>
       <c r="F1" s="5" t="s">
@@ -1413,14 +1418,14 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.21875" style="5" customWidth="1"/>
-    <col min="2" max="2" width="31.5546875" style="10" customWidth="1"/>
+    <col min="2" max="2" width="31.5546875" style="8" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="8" t="s">
         <v>53</v>
       </c>
     </row>
@@ -1429,7 +1434,7 @@
         <f>SUM(TEST_Inventory[TEST Currency])</f>
         <v>130</v>
       </c>
-      <c r="B2" s="10">
+      <c r="B2" s="8">
         <f>SUM(TEST_Inventory[TEST Integer])</f>
         <v>12</v>
       </c>
@@ -1496,7 +1501,7 @@
     <col min="2" max="2" width="9.5546875" style="2" customWidth="1"/>
     <col min="3" max="3" width="31.44140625" style="2" customWidth="1"/>
     <col min="4" max="4" width="10.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17" style="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17" style="10" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.33203125" style="3" customWidth="1"/>
     <col min="7" max="7" width="16.5546875" style="3" customWidth="1"/>
     <col min="8" max="8" width="16.6640625" style="5" customWidth="1"/>
@@ -1520,7 +1525,7 @@
       <c r="D1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="9" t="s">
         <v>9</v>
       </c>
       <c r="F1" s="5" t="s">
@@ -1585,7 +1590,7 @@
     <col min="3" max="3" width="28.6640625" style="2" customWidth="1"/>
     <col min="4" max="4" width="26.33203125" style="2" customWidth="1"/>
     <col min="5" max="5" width="14.88671875" style="2" customWidth="1"/>
-    <col min="6" max="6" width="14.6640625" style="7" customWidth="1"/>
+    <col min="6" max="6" width="14.6640625" style="10" customWidth="1"/>
     <col min="7" max="7" width="14.6640625" style="3" customWidth="1"/>
     <col min="8" max="8" width="12.33203125" style="2" customWidth="1"/>
     <col min="9" max="9" width="11.44140625" style="6" customWidth="1"/>
@@ -1609,7 +1614,7 @@
       <c r="E1" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="F1" s="9" t="s">
         <v>20</v>
       </c>
       <c r="G1" s="5" t="s">
@@ -1648,11 +1653,11 @@
     <col min="2" max="2" width="8.109375" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.88671875" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="17.88671875" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.6640625" style="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.6640625" style="10" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.6640625" style="6" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14.33203125" style="6" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="7" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18" style="7" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18" style="10" bestFit="1" customWidth="1"/>
     <col min="10" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
@@ -1669,7 +1674,7 @@
       <c r="D1" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="9" t="s">
         <v>24</v>
       </c>
       <c r="F1" t="s">
@@ -1681,7 +1686,7 @@
       <c r="H1" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="I1" s="9" t="s">
         <v>28</v>
       </c>
     </row>
@@ -1767,7 +1772,7 @@
     <col min="2" max="2" width="8.6640625" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="54.6640625" style="2" customWidth="1"/>
     <col min="4" max="4" width="10.5546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.33203125" style="9" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.33203125" style="7" bestFit="1" customWidth="1"/>
     <col min="6" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
@@ -1784,7 +1789,7 @@
       <c r="D1" t="s">
         <v>8</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="8" t="s">
         <v>32</v>
       </c>
     </row>
@@ -1804,15 +1809,15 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E1902F1-C59B-4A1A-9D95-2C39AEF944E5}">
   <sheetPr codeName="Sheet7"/>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
     <col min="2" max="2" width="41.6640625" style="2" customWidth="1"/>
     <col min="3" max="4" width="18.44140625" style="2" customWidth="1"/>
     <col min="5" max="5" width="15.5546875" style="2" customWidth="1"/>
-    <col min="6" max="6" width="14.33203125" style="9" customWidth="1"/>
-    <col min="7" max="7" width="14.109375" style="9" customWidth="1"/>
+    <col min="6" max="6" width="14.33203125" style="7" customWidth="1"/>
+    <col min="7" max="7" width="14.109375" style="7" customWidth="1"/>
     <col min="8" max="8" width="10.44140625" style="3" customWidth="1"/>
     <col min="9" max="9" width="22.6640625" style="3" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="46.6640625" style="2" customWidth="1"/>
@@ -1835,10 +1840,10 @@
       <c r="E1" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="F1" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="G1" s="10" t="s">
+      <c r="G1" s="8" t="s">
         <v>36</v>
       </c>
       <c r="H1" s="5" t="s">
@@ -1849,6 +1854,12 @@
       </c>
       <c r="J1" s="4" t="s">
         <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="I2" s="3">
+        <f>Shop_Consumables[[#This Row],[Current Stock]]*Shop_Consumables[[#This Row],[Unit Cost]]</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
adjusted Excel and Config to set up for adding scannable label function
</commit_message>
<xml_diff>
--- a/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
+++ b/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1a2ae81d67634e6/Desktop/Michanikos Artifex Enterprises/MAE Custom Digital Solutions/MAE Workshop Inventory Management System/GITHUB_MAE_Workshop Inventory App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="72" documentId="13_ncr:1_{8CE4ED70-7C3C-4CCA-B9CD-0FFB5498A43E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DE8518B2-23EF-47F3-97B4-D169D46D5DAD}"/>
+  <xr:revisionPtr revIDLastSave="158" documentId="13_ncr:1_{8CE4ED70-7C3C-4CCA-B9CD-0FFB5498A43E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ABB9F3C2-348F-4DA3-81FE-138FD69AE7EB}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
+    <workbookView xWindow="144" yWindow="0" windowWidth="11532" windowHeight="11904" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
   </bookViews>
   <sheets>
     <sheet name="TEST Inventory" sheetId="10" r:id="rId1"/>
@@ -24,6 +24,7 @@
     <sheet name="Shop Consumables" sheetId="7" r:id="rId9"/>
     <sheet name="Shop Overhead" sheetId="8" r:id="rId10"/>
     <sheet name="Supplier Contacts" sheetId="9" r:id="rId11"/>
+    <sheet name="Location" sheetId="12" r:id="rId12"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -46,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="73">
   <si>
     <t>mae_id</t>
   </si>
@@ -114,9 +115,6 @@
     <t>Purchase Cost</t>
   </si>
   <si>
-    <t>Status</t>
-  </si>
-  <si>
     <t>Log ID</t>
   </si>
   <si>
@@ -135,9 +133,6 @@
     <t>Next Service Date</t>
   </si>
   <si>
-    <t>Tool ID</t>
-  </si>
-  <si>
     <t>Tool Name/Model</t>
   </si>
   <si>
@@ -147,9 +142,6 @@
     <t>Quantity</t>
   </si>
   <si>
-    <t>SKU/Item ID</t>
-  </si>
-  <si>
     <t>Unit of Measure</t>
   </si>
   <si>
@@ -243,9 +235,6 @@
     <t>Manual Link/Other Info</t>
   </si>
   <si>
-    <t>Asset Description</t>
-  </si>
-  <si>
     <t>Functional Category</t>
   </si>
   <si>
@@ -256,6 +245,27 @@
   </si>
   <si>
     <t>Current Inventory Value</t>
+  </si>
+  <si>
+    <t>Location_ID</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Parent_Location</t>
+  </si>
+  <si>
+    <t>Asset and Service Description</t>
+  </si>
+  <si>
+    <t>Asset_ID</t>
+  </si>
+  <si>
+    <t>hidden test</t>
   </si>
 </sst>
 </file>
@@ -328,27 +338,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="98">
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
+  <dxfs count="111">
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="1" hidden="1"/>
@@ -358,6 +348,118 @@
       <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -388,158 +490,216 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
@@ -580,108 +740,6 @@
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
       <protection locked="0" hidden="0"/>
@@ -707,14 +765,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}" name="TEST_Inventory" displayName="TEST_Inventory" ref="A1:F4" totalsRowShown="0">
-  <autoFilter ref="A1:F4" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}" name="TEST_Inventory" displayName="TEST_Inventory" ref="A1:F5" totalsRowShown="0">
+  <autoFilter ref="A1:F5" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="85"/>
-    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="84"/>
-    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="83"/>
-    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="82"/>
-    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="81">
+    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="98"/>
+    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="97"/>
+    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="96"/>
+    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="95"/>
+    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="94">
       <calculatedColumnFormula>TEST_Inventory[[#This Row],[TEST Integer]]*TEST_Inventory[[#This Row],[TEST Currency]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{AB3A5F3C-FCF0-4466-90FD-8ABB6E18DF5C}" name="TEST Dropdown"/>
@@ -724,32 +782,46 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:G2" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:G2" totalsRowShown="0" headerRowDxfId="40" dataDxfId="39">
   <autoFilter ref="A1:G2" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="15"/>
-    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="14"/>
-    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="13"/>
-    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="12"/>
-    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="11"/>
-    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="10"/>
-    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="9"/>
+    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="38"/>
+    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="37"/>
+    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="36"/>
+    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="35"/>
+    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="34"/>
+    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="33"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="32" dataDxfId="31">
   <autoFilter ref="A1:G2" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="6"/>
-    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="4"/>
-    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="3"/>
-    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="2"/>
-    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="1"/>
-    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="1"/>
+    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="30"/>
+    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="29"/>
+    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="28"/>
+    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="27"/>
+    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="26"/>
+    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="25"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}" name="Location" displayName="Location" ref="A1:E2" insertRow="1" totalsRowShown="0">
+  <autoFilter ref="A1:E2" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="24"/>
+    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Name" dataDxfId="23"/>
+    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="22"/>
+    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="21"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -759,10 +831,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}" name="TEST_Dashboard" displayName="TEST_Dashboard" ref="A1:B2" totalsRowShown="0">
   <autoFilter ref="A1:B2" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="80">
+    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="93">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Currency])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="79">
+    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="92">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Integer])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -771,126 +843,134 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:F2" totalsRowShown="0" headerRowDxfId="78" dataDxfId="77">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:F2" totalsRowShown="0" headerRowDxfId="91" dataDxfId="90">
   <autoFilter ref="A1:F2" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="76"/>
-    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Inventory Value" dataDxfId="75"/>
-    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Low Stock Alerts" dataDxfId="74"/>
-    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Upcoming Maintenance" dataDxfId="73"/>
-    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Monthly Overhead Total" dataDxfId="72"/>
-    <tableColumn id="6" xr3:uid="{86A5DBCB-1064-4926-8405-405B453A4546}" name="Supplier Performance" dataDxfId="71"/>
+    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Inventory Value" dataDxfId="89"/>
+    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Low Stock Alerts" dataDxfId="88"/>
+    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Upcoming Maintenance" dataDxfId="87"/>
+    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Monthly Overhead Total" dataDxfId="86"/>
+    <tableColumn id="6" xr3:uid="{86A5DBCB-1064-4926-8405-405B453A4546}" name="Supplier Performance" dataDxfId="85"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:L2" totalsRowShown="0" headerRowDxfId="70" dataDxfId="69">
-  <autoFilter ref="A1:L2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}"/>
-  <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="68"/>
-    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="67"/>
-    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="66"/>
-    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="65"/>
-    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="64"/>
-    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="63"/>
-    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="62"/>
-    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="61">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:M2" totalsRowShown="0" headerRowDxfId="110" dataDxfId="109">
+  <autoFilter ref="A1:M2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}"/>
+  <tableColumns count="13">
+    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="108"/>
+    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="107"/>
+    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="106"/>
+    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="105"/>
+    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="104"/>
+    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="103"/>
+    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="102">
       <calculatedColumnFormula>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="60"/>
-    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="59"/>
-    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="58"/>
-    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location" dataDxfId="57"/>
+    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="101"/>
+    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="100"/>
+    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="99"/>
+    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="20"/>
+    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="19"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:J2" insertRow="1" totalsRowShown="0" headerRowDxfId="56" dataDxfId="55">
-  <autoFilter ref="A1:J2" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}"/>
-  <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="54"/>
-    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="53"/>
-    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Model" dataDxfId="52"/>
-    <tableColumn id="4" xr3:uid="{217066CA-63B7-4030-A7FC-54062BE2122E}" name="Manufacturer/Brand" dataDxfId="51"/>
-    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="50"/>
-    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="49"/>
-    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="48"/>
-    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="47"/>
-    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Status" dataDxfId="46"/>
-    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="45"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="84" dataDxfId="83">
+  <autoFilter ref="A1:K2" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="82"/>
+    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Model" dataDxfId="81"/>
+    <tableColumn id="4" xr3:uid="{217066CA-63B7-4030-A7FC-54062BE2122E}" name="Manufacturer/Brand" dataDxfId="80"/>
+    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="79"/>
+    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="78"/>
+    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="77"/>
+    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="76"/>
+    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="18"/>
+    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="75"/>
+    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="74"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:I2" totalsRowShown="0" headerRowDxfId="44" dataDxfId="43">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:I2" totalsRowShown="0" headerRowDxfId="73" dataDxfId="72">
   <autoFilter ref="A1:I2" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="42"/>
-    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="41"/>
-    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="40"/>
-    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset Description" dataDxfId="39"/>
-    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="38"/>
-    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="37"/>
-    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="36"/>
-    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="35"/>
-    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="34"/>
+    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="71"/>
+    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="70"/>
+    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="69"/>
+    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="68"/>
+    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="67"/>
+    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="66"/>
+    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="65"/>
+    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="64"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:G2" totalsRowShown="0" headerRowDxfId="33" dataDxfId="32">
-  <autoFilter ref="A1:G2" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}"/>
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="31"/>
-    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Tool ID" dataDxfId="30"/>
-    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Model" dataDxfId="29"/>
-    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="28"/>
-    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="27"/>
-    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="26"/>
-    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="25"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:I2" totalsRowShown="0" headerRowDxfId="63" dataDxfId="62">
+  <autoFilter ref="A1:I2" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}"/>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="61"/>
+    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Model" dataDxfId="60"/>
+    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="16"/>
+    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="17"/>
+    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="59"/>
+    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="58"/>
+    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="57"/>
+    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="56"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:E2" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23">
-  <autoFilter ref="A1:E2" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}"/>
-  <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="22"/>
-    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Tool ID" dataDxfId="21"/>
-    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Model" dataDxfId="20"/>
-    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="19"/>
-    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="18"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:H2" totalsRowShown="0" headerRowDxfId="55" dataDxfId="54">
+  <autoFilter ref="A1:H2" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="53"/>
+    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Model" dataDxfId="52"/>
+    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="15"/>
+    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="51"/>
+    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="14"/>
+    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="50"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:J2" totalsRowShown="0" headerRowDxfId="97" dataDxfId="96">
-  <autoFilter ref="A1:J2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
-  <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="95"/>
-    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="94"/>
-    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="SKU/Item ID" dataDxfId="93"/>
-    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="92"/>
-    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="91"/>
-    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="90"/>
-    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="89"/>
-    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="88"/>
-    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="87">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:K2" totalsRowShown="0" headerRowDxfId="49" dataDxfId="48">
+  <autoFilter ref="A1:K2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="47"/>
+    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="46"/>
+    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="45"/>
+    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="44"/>
+    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="43"/>
+    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="10"/>
+    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="11"/>
+    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="42">
       <calculatedColumnFormula>Shop_Consumables[[#This Row],[Current Stock]]*Shop_Consumables[[#This Row],[Unit Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Preferred Supplier" dataDxfId="86"/>
+    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="12"/>
+    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Preferred Supplier" dataDxfId="41"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1213,7 +1293,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19832549-C5E9-4018-9E8B-E2F74EABCB4B}">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
@@ -1229,24 +1309,24 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="F1" t="s">
         <v>48</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="F1" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B2" s="4" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C2" s="8">
         <v>3</v>
@@ -1259,12 +1339,12 @@
         <v>300</v>
       </c>
       <c r="F2" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B3" s="4" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C3" s="8">
         <v>4</v>
@@ -1277,12 +1357,12 @@
         <v>40</v>
       </c>
       <c r="F3" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B4" s="4" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C4" s="8">
         <v>5</v>
@@ -1295,7 +1375,22 @@
         <v>100</v>
       </c>
       <c r="F4" t="s">
-        <v>59</v>
+        <v>56</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B5" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5" s="8">
+        <v>1000</v>
+      </c>
+      <c r="D5" s="5">
+        <v>1000</v>
+      </c>
+      <c r="E5" s="5">
+        <f>TEST_Inventory[[#This Row],[TEST Integer]]*TEST_Inventory[[#This Row],[TEST Currency]]</f>
+        <v>1000000</v>
       </c>
     </row>
   </sheetData>
@@ -1332,22 +1427,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="E1" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>41</v>
-      </c>
-      <c r="E1" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -1386,22 +1481,59 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="F1" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="G1" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="G1" s="4" t="s">
-        <v>63</v>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6A08BCD-5A8C-45EE-A940-2FEFA1E5B102}">
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="9" style="1" customWidth="1"/>
+    <col min="2" max="2" width="15.6640625" style="4" customWidth="1"/>
+    <col min="3" max="3" width="27.44140625" style="4" customWidth="1"/>
+    <col min="4" max="4" width="21.6640625" style="4" customWidth="1"/>
+    <col min="5" max="5" width="30" style="4" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -1423,20 +1555,20 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="5">
         <f>SUM(TEST_Inventory[TEST Currency])</f>
-        <v>130</v>
+        <v>1130</v>
       </c>
       <c r="B2" s="8">
         <f>SUM(TEST_Inventory[TEST Integer])</f>
-        <v>12</v>
+        <v>1012</v>
       </c>
     </row>
   </sheetData>
@@ -1494,7 +1626,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDE7BF89-A2E7-4A6F-B822-317739E206EC}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
@@ -1508,11 +1640,12 @@
     <col min="9" max="9" width="19.109375" style="2" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="16.6640625" style="3" customWidth="1"/>
     <col min="11" max="11" width="16.88671875" style="3" customWidth="1"/>
-    <col min="12" max="12" width="22.33203125" style="2" customWidth="1"/>
-    <col min="13" max="16384" width="8.88671875" style="6"/>
+    <col min="12" max="12" width="16.88671875" style="2" customWidth="1"/>
+    <col min="13" max="13" width="22.33203125" style="2" customWidth="1"/>
+    <col min="14" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1549,20 +1682,26 @@
       <c r="L1" s="4" t="s">
         <v>16</v>
       </c>
+      <c r="M1" s="4" t="s">
+        <v>66</v>
+      </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="H2" s="5">
         <f>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</f>
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I1000" xr:uid="{F45414DD-76C8-4DC4-96E2-15B89FDB5B51}">
+  <dataValidations count="3">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I3:I1000" xr:uid="{F45414DD-76C8-4DC4-96E2-15B89FDB5B51}">
       <formula1>"work not started, restoration in progress, for sale, sold"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2" xr:uid="{C1AA0387-29B3-4797-A152-88A8C024D825}">
       <formula1>"Machinery, Furniture, Electronics, Craft, Other"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2" xr:uid="{3C9AD8AD-AB10-403F-A04B-87B1D7C9B98E}">
+      <formula1>"Not Started, In-Progress, Complete, For Sale, Sold"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1576,7 +1715,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B027EC69-551F-4051-8A71-8B106D207C6D}">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
@@ -1586,13 +1725,13 @@
     <col min="5" max="5" width="14.88671875" style="2" customWidth="1"/>
     <col min="6" max="6" width="14.6640625" style="10" customWidth="1"/>
     <col min="7" max="7" width="14.6640625" style="3" customWidth="1"/>
-    <col min="8" max="8" width="12.33203125" style="2" customWidth="1"/>
-    <col min="9" max="9" width="11.44140625" style="6" customWidth="1"/>
-    <col min="10" max="10" width="32.6640625" style="2" customWidth="1"/>
-    <col min="11" max="16384" width="8.88671875" style="6"/>
+    <col min="8" max="9" width="12.33203125" style="2" customWidth="1"/>
+    <col min="10" max="10" width="11.44140625" style="6" customWidth="1"/>
+    <col min="11" max="11" width="32.6640625" style="2" customWidth="1"/>
+    <col min="12" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1617,17 +1756,23 @@
       <c r="H1" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="I1" t="s">
-        <v>22</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>64</v>
+      <c r="I1" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="J1" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>61</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I1000" xr:uid="{D25ACF8B-D3DC-4EFD-9C68-FC99372E0DCF}">
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J3:J1000" xr:uid="{D25ACF8B-D3DC-4EFD-9C68-FC99372E0DCF}">
       <formula1>"Operational, Needs Repair, Unusable"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2" xr:uid="{4B2064CB-79C2-427D-B2C2-7CE85187D094}">
+      <formula1>"Operational, Needs Repair, Repair In-Progress, Unusable/Junk"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1646,7 +1791,7 @@
     <col min="1" max="1" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.109375" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.88671875" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="28.21875" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.6640625" style="10" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.6640625" style="6" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14.33203125" style="6" bestFit="1" customWidth="1"/>
@@ -1660,28 +1805,28 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="E1" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="F1" t="s">
         <v>24</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>25</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="I1" s="9" t="s">
         <v>27</v>
-      </c>
-      <c r="I1" s="9" t="s">
-        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -1703,50 +1848,70 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEDDDAA7-75C3-4AA5-ABFD-D5FB4C627E4C}">
   <sheetPr codeName="Sheet5"/>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
     <col min="2" max="2" width="8.6640625" style="2" customWidth="1"/>
     <col min="3" max="3" width="50.44140625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="19.88671875" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.88671875" style="6" customWidth="1"/>
-    <col min="6" max="6" width="14.44140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.5546875" style="6" customWidth="1"/>
-    <col min="8" max="16384" width="8.88671875" style="6"/>
+    <col min="4" max="4" width="15.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.88671875" style="6" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.88671875" style="6" customWidth="1"/>
+    <col min="8" max="8" width="14.44140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5546875" style="6" customWidth="1"/>
+    <col min="10" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="F1" t="s">
+        <v>62</v>
+      </c>
+      <c r="G1" t="s">
+        <v>63</v>
+      </c>
+      <c r="H1" t="s">
+        <v>64</v>
+      </c>
+      <c r="I1" t="s">
         <v>29</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="D1" t="s">
-        <v>66</v>
-      </c>
-      <c r="E1" t="s">
-        <v>67</v>
-      </c>
-      <c r="F1" t="s">
-        <v>68</v>
-      </c>
-      <c r="G1" t="s">
-        <v>31</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:F1000" xr:uid="{FF61F80C-5E23-45D6-B39D-7C5635258115}">
+  <dataValidations count="6">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F3:F1000 G3:G1000 H3:H1000" xr:uid="{FF61F80C-5E23-45D6-B39D-7C5635258115}">
       <formula1>"Circular Saw, Drill, Sander, Grinder, Other"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G1000" xr:uid="{DB752B4D-0E75-42D1-B907-2DBC5792F422}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I3:I1000" xr:uid="{DB752B4D-0E75-42D1-B907-2DBC5792F422}">
       <formula1>"New, Operational, Needs Repair, Broken"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2" xr:uid="{05EFC744-2B0C-453D-A1B6-F8391608434D}">
+      <formula1>"Drilling, Cutting, Grinding, Sanding, Fastening, Shaping/Routing, Other"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2" xr:uid="{194EFB2B-690A-4D50-8AF6-E8ED45FE2FCA}">
+      <formula1>"Portable/Handheld, Stationary/Bench Top, Outdoor Power Equipment, "</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2" xr:uid="{47F6EF9A-B127-4EB7-A5E8-0075055489DC}">
+      <formula1>"Corded(A/C), Cordless/Battery, Pneumatic/Air, Fuel-Powered"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2" xr:uid="{980AB122-9104-490B-993D-4F2FEF3A4EE6}">
+      <formula1>"Operational, Needs Repair, Repair In-Progress, Unusable/Junk"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1759,37 +1924,49 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F39ADDA6-CD5F-4655-A9C0-9676DDAC362E}">
   <sheetPr codeName="Sheet6"/>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.6640625" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="54.6640625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="10.5546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.33203125" style="7" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="8.88671875" style="6"/>
+    <col min="4" max="4" width="15.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.5546875" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.88671875" style="2" customWidth="1"/>
+    <col min="8" max="8" width="10.33203125" style="7" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="G1" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="H1" s="8" t="s">
         <v>30</v>
-      </c>
-      <c r="D1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>32</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D1000" xr:uid="{B6CB3C84-EE01-4878-B558-650FC19D8248}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:G1000" xr:uid="{B6CB3C84-EE01-4878-B558-650FC19D8248}">
       <formula1>"Saw, Hammer, Screwdriver, Wrench, Sockets, Pliers, Measuring, Files, Other"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1803,7 +1980,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E1902F1-C59B-4A1A-9D95-2C39AEF944E5}">
   <sheetPr codeName="Sheet7"/>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
@@ -1814,11 +1991,12 @@
     <col min="7" max="7" width="14.109375" style="7" customWidth="1"/>
     <col min="8" max="8" width="10.44140625" style="3" customWidth="1"/>
     <col min="9" max="9" width="22.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="46.6640625" style="2" customWidth="1"/>
-    <col min="11" max="16384" width="8.88671875" style="6"/>
+    <col min="10" max="10" width="22.6640625" style="2" customWidth="1"/>
+    <col min="11" max="11" width="46.6640625" style="2" customWidth="1"/>
+    <col min="12" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1826,37 +2004,45 @@
         <v>7</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>33</v>
+        <v>71</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>8</v>
       </c>
       <c r="E1" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="H1" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="I1" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="K1" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="G1" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>38</v>
-      </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="I2" s="3">
         <f>Shop_Consumables[[#This Row],[Current Stock]]*Shop_Consumables[[#This Row],[Unit Cost]]</f>
         <v>0</v>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2" xr:uid="{D2C605E8-D02B-4558-82DE-3169088704E8}">
+      <formula1>"Fasteners/Hardware,Abrasives/Cutting,Fluids/Lubricants/Chemicals,Primer/Paint,Safety/PPE,Shop/Janitorial,Welding,Electrical,Other"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>

<commit_message>
changes to .xlsx and config.js
</commit_message>
<xml_diff>
--- a/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
+++ b/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1a2ae81d67634e6/Desktop/Michanikos Artifex Enterprises/MAE Custom Digital Solutions/MAE Workshop Inventory Management System/GITHUB_MAE_Workshop Inventory App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="158" documentId="13_ncr:1_{8CE4ED70-7C3C-4CCA-B9CD-0FFB5498A43E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ABB9F3C2-348F-4DA3-81FE-138FD69AE7EB}"/>
+  <xr:revisionPtr revIDLastSave="168" documentId="13_ncr:1_{8CE4ED70-7C3C-4CCA-B9CD-0FFB5498A43E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E789E0F7-216E-4E2A-ADA1-9CBE7F355456}"/>
   <bookViews>
-    <workbookView xWindow="144" yWindow="0" windowWidth="11532" windowHeight="11904" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
+    <workbookView xWindow="36" yWindow="0" windowWidth="11532" windowHeight="11904" firstSheet="9" activeTab="9" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
   </bookViews>
   <sheets>
     <sheet name="TEST Inventory" sheetId="10" r:id="rId1"/>
@@ -341,10 +341,50 @@
   <dxfs count="111">
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
@@ -352,114 +392,197 @@
       <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -470,236 +593,8 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
@@ -740,6 +635,111 @@
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
       <protection locked="0" hidden="0"/>
@@ -768,11 +768,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}" name="TEST_Inventory" displayName="TEST_Inventory" ref="A1:F5" totalsRowShown="0">
   <autoFilter ref="A1:F5" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="98"/>
-    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="97"/>
-    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="96"/>
-    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="95"/>
-    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="94">
+    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="97"/>
+    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="96"/>
+    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="95"/>
+    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="94"/>
+    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="93">
       <calculatedColumnFormula>TEST_Inventory[[#This Row],[TEST Integer]]*TEST_Inventory[[#This Row],[TEST Currency]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{AB3A5F3C-FCF0-4466-90FD-8ABB6E18DF5C}" name="TEST Dropdown"/>
@@ -782,32 +782,32 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:G2" totalsRowShown="0" headerRowDxfId="40" dataDxfId="39">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:G2" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
   <autoFilter ref="A1:G2" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="38"/>
-    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="37"/>
-    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="36"/>
-    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="35"/>
-    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="34"/>
-    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="33"/>
+    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="20"/>
+    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="19"/>
+    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="0"/>
+    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="18"/>
+    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="17"/>
+    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="32" dataDxfId="31">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
   <autoFilter ref="A1:G2" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="1"/>
-    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="30"/>
-    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="29"/>
-    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="28"/>
-    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="27"/>
-    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="26"/>
-    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="25"/>
+    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="13"/>
+    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="11"/>
+    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="9"/>
+    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="8"/>
+    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -817,11 +817,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}" name="Location" displayName="Location" ref="A1:E2" insertRow="1" totalsRowShown="0">
   <autoFilter ref="A1:E2" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="0"/>
-    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="24"/>
-    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Name" dataDxfId="23"/>
-    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="22"/>
-    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="21"/>
+    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Name" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -831,10 +831,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}" name="TEST_Dashboard" displayName="TEST_Dashboard" ref="A1:B2" totalsRowShown="0">
   <autoFilter ref="A1:B2" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="93">
+    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="92">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Currency])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="92">
+    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="91">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Integer])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -843,134 +843,134 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:F2" totalsRowShown="0" headerRowDxfId="91" dataDxfId="90">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:F2" totalsRowShown="0" headerRowDxfId="90" dataDxfId="89">
   <autoFilter ref="A1:F2" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Inventory Value" dataDxfId="89"/>
-    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Low Stock Alerts" dataDxfId="88"/>
-    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Upcoming Maintenance" dataDxfId="87"/>
-    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Monthly Overhead Total" dataDxfId="86"/>
-    <tableColumn id="6" xr3:uid="{86A5DBCB-1064-4926-8405-405B453A4546}" name="Supplier Performance" dataDxfId="85"/>
+    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="88"/>
+    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Inventory Value" dataDxfId="87"/>
+    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Low Stock Alerts" dataDxfId="86"/>
+    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Upcoming Maintenance" dataDxfId="85"/>
+    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Monthly Overhead Total" dataDxfId="84"/>
+    <tableColumn id="6" xr3:uid="{86A5DBCB-1064-4926-8405-405B453A4546}" name="Supplier Performance" dataDxfId="83"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:M2" totalsRowShown="0" headerRowDxfId="110" dataDxfId="109">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:M2" totalsRowShown="0" headerRowDxfId="82" dataDxfId="81">
   <autoFilter ref="A1:M2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="108"/>
-    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="107"/>
-    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="106"/>
-    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="105"/>
-    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="104"/>
-    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="103"/>
-    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="102">
+    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="80"/>
+    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="79"/>
+    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="78"/>
+    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="77"/>
+    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="76"/>
+    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="75"/>
+    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="74"/>
+    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="73">
       <calculatedColumnFormula>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="101"/>
-    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="100"/>
-    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="99"/>
-    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="20"/>
-    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="19"/>
+    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="72"/>
+    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="71"/>
+    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="70"/>
+    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="69"/>
+    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="68"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="84" dataDxfId="83">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="110" dataDxfId="109">
   <autoFilter ref="A1:K2" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="82"/>
-    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Model" dataDxfId="81"/>
-    <tableColumn id="4" xr3:uid="{217066CA-63B7-4030-A7FC-54062BE2122E}" name="Manufacturer/Brand" dataDxfId="80"/>
-    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="79"/>
-    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="78"/>
-    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="77"/>
-    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="76"/>
-    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="18"/>
-    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="75"/>
-    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="74"/>
+    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="108"/>
+    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="107"/>
+    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Model" dataDxfId="106"/>
+    <tableColumn id="4" xr3:uid="{217066CA-63B7-4030-A7FC-54062BE2122E}" name="Manufacturer/Brand" dataDxfId="105"/>
+    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="104"/>
+    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="103"/>
+    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="102"/>
+    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="101"/>
+    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="100"/>
+    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="99"/>
+    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="98"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:I2" totalsRowShown="0" headerRowDxfId="73" dataDxfId="72">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:I2" totalsRowShown="0" headerRowDxfId="67" dataDxfId="66">
   <autoFilter ref="A1:I2" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="71"/>
-    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="70"/>
-    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="69"/>
-    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="68"/>
-    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="67"/>
-    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="66"/>
-    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="65"/>
-    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="64"/>
+    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="65"/>
+    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="64"/>
+    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="63"/>
+    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="62"/>
+    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="61"/>
+    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="60"/>
+    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="59"/>
+    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="58"/>
+    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="57"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:I2" totalsRowShown="0" headerRowDxfId="63" dataDxfId="62">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:I2" totalsRowShown="0" headerRowDxfId="56" dataDxfId="55">
   <autoFilter ref="A1:I2" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="61"/>
-    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Model" dataDxfId="60"/>
-    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="16"/>
-    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="17"/>
-    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="59"/>
-    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="58"/>
-    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="57"/>
-    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="56"/>
+    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="54"/>
+    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="53"/>
+    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Model" dataDxfId="52"/>
+    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="51"/>
+    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="50"/>
+    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="49"/>
+    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="48"/>
+    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="47"/>
+    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="46"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:H2" totalsRowShown="0" headerRowDxfId="55" dataDxfId="54">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:H2" totalsRowShown="0" headerRowDxfId="45" dataDxfId="44">
   <autoFilter ref="A1:H2" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="53"/>
-    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Model" dataDxfId="52"/>
-    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="15"/>
-    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="51"/>
-    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="14"/>
-    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="13"/>
-    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="50"/>
+    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="43"/>
+    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="42"/>
+    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Model" dataDxfId="41"/>
+    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="40"/>
+    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="39"/>
+    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="1"/>
+    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="38"/>
+    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="37"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:K2" totalsRowShown="0" headerRowDxfId="49" dataDxfId="48">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:K2" totalsRowShown="0" headerRowDxfId="36" dataDxfId="35">
   <autoFilter ref="A1:K2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="3"/>
-    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="47"/>
-    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="46"/>
-    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="45"/>
-    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="44"/>
-    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="43"/>
-    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="10"/>
-    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="11"/>
-    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="42">
+    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="34"/>
+    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="33"/>
+    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="32"/>
+    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="31"/>
+    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="30"/>
+    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="29"/>
+    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="28"/>
+    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="27"/>
+    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="26">
       <calculatedColumnFormula>Shop_Consumables[[#This Row],[Current Stock]]*Shop_Consumables[[#This Row],[Unit Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="12"/>
-    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Preferred Supplier" dataDxfId="41"/>
+    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="25"/>
+    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Preferred Supplier" dataDxfId="24"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1446,12 +1446,18 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G1000" xr:uid="{5CDD912B-3197-4C62-9DE2-F15AE0580881}">
+  <dataValidations count="4">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3:B1000" xr:uid="{AA2AF827-8A0A-4B34-A36E-624457B5758A}">
+      <formula1>"Rent/Mortgage, Utilities, Insurance, Other"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2" xr:uid="{63C2185A-207B-4EF1-BB04-3B86B2517042}">
+      <formula1>"Facility Costs/Rent/Mortgage,Insurance,Debt/Leases on Equipment/Business Loans,Subscriptions,Salaries,Utilities,Maintnance/Repair,Marketing/Advertising,Professional Fees,Travel/Vehicles,Depreciations,Other/Miscellaneous"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G3:G1000 G2" xr:uid="{5CDD912B-3197-4C62-9DE2-F15AE0580881}">
       <formula1>"YES, NO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B1000" xr:uid="{AA2AF827-8A0A-4B34-A36E-624457B5758A}">
-      <formula1>"Rent/Mortgage, Utilities, Insurance, Other"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2" xr:uid="{D24BB2FF-F2D7-4CAB-A302-F301339BCAE8}">
+      <formula1>"Upon Receipt,Monthly,Weekly,Quarterly,Semi-Annually,Yearly,Other"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1698,7 +1704,7 @@
       <formula1>"work not started, restoration in progress, for sale, sold"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2" xr:uid="{C1AA0387-29B3-4797-A152-88A8C024D825}">
-      <formula1>"Machinery, Furniture, Electronics, Craft, Other"</formula1>
+      <formula1>"Machinery, Furniture, Electronics, Craft, Auto Related, Other"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2" xr:uid="{3C9AD8AD-AB10-403F-A04B-87B1D7C9B98E}">
       <formula1>"Not Started, In-Progress, Complete, For Sale, Sold"</formula1>
@@ -1830,12 +1836,15 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F1000" xr:uid="{E5FFE733-A9D3-430E-8950-CAD58FEAE2C9}">
       <formula1>"Preventive, Repair"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G1000" xr:uid="{8BC162F1-575A-44E2-AA38-454BF93A8AFF}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G3:G1000" xr:uid="{8BC162F1-575A-44E2-AA38-454BF93A8AFF}">
       <formula1>"Self in Shop, Contractor in Shop, Out of Shop"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2" xr:uid="{D78DF6AB-EB66-4EBB-ABC5-55445DBB08E9}">
+      <formula1>"Self in Shop, Contractor in Shop, Outside Facility"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1965,9 +1974,15 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:G1000" xr:uid="{B6CB3C84-EE01-4878-B558-650FC19D8248}">
+  <dataValidations count="3">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E3:E1000 F3:F1000 G3:G1000" xr:uid="{B6CB3C84-EE01-4878-B558-650FC19D8248}">
       <formula1>"Saw, Hammer, Screwdriver, Wrench, Sockets, Pliers, Measuring, Files, Other"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2" xr:uid="{ACB7A40B-F0EE-4387-88E4-5140AB68313F}">
+      <formula1>"Fastening/Turning,Measuring/Layout,Striking/Hammering,Gripping/Holding,Cutting/Shaping,Other"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2" xr:uid="{2E543736-2E6D-4F90-9169-21BA7CCD7676}">
+      <formula1>"Operational,Needs Repair,Repair In-Progress,Unusable/Junk"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix typo in excel
</commit_message>
<xml_diff>
--- a/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
+++ b/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1a2ae81d67634e6/Desktop/Michanikos Artifex Enterprises/MAE Custom Digital Solutions/MAE Workshop Inventory Management System/GITHUB_MAE_Workshop Inventory App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="168" documentId="13_ncr:1_{8CE4ED70-7C3C-4CCA-B9CD-0FFB5498A43E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E789E0F7-216E-4E2A-ADA1-9CBE7F355456}"/>
+  <xr:revisionPtr revIDLastSave="169" documentId="13_ncr:1_{8CE4ED70-7C3C-4CCA-B9CD-0FFB5498A43E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A0D98F39-3C9B-480F-9D1D-D5B9BCB7A188}"/>
   <bookViews>
-    <workbookView xWindow="36" yWindow="0" windowWidth="11532" windowHeight="11904" firstSheet="9" activeTab="9" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
+    <workbookView xWindow="1920" yWindow="1056" windowWidth="11532" windowHeight="11904" firstSheet="9" activeTab="9" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
   </bookViews>
   <sheets>
     <sheet name="TEST Inventory" sheetId="10" r:id="rId1"/>
@@ -341,14 +341,6 @@
   <dxfs count="111">
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -402,14 +394,149 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="0"/>
     </dxf>
@@ -432,6 +559,13 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="0"/>
     </dxf>
@@ -440,130 +574,11 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -703,26 +718,11 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -768,11 +768,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}" name="TEST_Inventory" displayName="TEST_Inventory" ref="A1:F5" totalsRowShown="0">
   <autoFilter ref="A1:F5" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="97"/>
-    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="96"/>
-    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="95"/>
-    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="94"/>
-    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="93">
+    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="101"/>
+    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="100"/>
+    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="99"/>
+    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="98"/>
+    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="97">
       <calculatedColumnFormula>TEST_Inventory[[#This Row],[TEST Integer]]*TEST_Inventory[[#This Row],[TEST Currency]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{AB3A5F3C-FCF0-4466-90FD-8ABB6E18DF5C}" name="TEST Dropdown"/>
@@ -782,32 +782,32 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:G2" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:G2" totalsRowShown="0" headerRowDxfId="110" dataDxfId="109">
   <autoFilter ref="A1:G2" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="20"/>
-    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="0"/>
-    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="18"/>
-    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="17"/>
-    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="16"/>
+    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="108"/>
+    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="107"/>
+    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="106"/>
+    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="105"/>
+    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="104"/>
+    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="103"/>
+    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="102"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
   <autoFilter ref="A1:G2" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="13"/>
-    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="11"/>
-    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="10"/>
-    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="9"/>
-    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="8"/>
-    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="7"/>
+    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="11"/>
+    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="9"/>
+    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="7"/>
+    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="6"/>
+    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -817,11 +817,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}" name="Location" displayName="Location" ref="A1:E2" insertRow="1" totalsRowShown="0">
   <autoFilter ref="A1:E2" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Name" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Name" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -831,10 +831,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}" name="TEST_Dashboard" displayName="TEST_Dashboard" ref="A1:B2" totalsRowShown="0">
   <autoFilter ref="A1:B2" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="92">
+    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="96">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Currency])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="91">
+    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="95">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Integer])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -843,134 +843,134 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:F2" totalsRowShown="0" headerRowDxfId="90" dataDxfId="89">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:F2" totalsRowShown="0" headerRowDxfId="94" dataDxfId="93">
   <autoFilter ref="A1:F2" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="88"/>
-    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Inventory Value" dataDxfId="87"/>
-    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Low Stock Alerts" dataDxfId="86"/>
-    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Upcoming Maintenance" dataDxfId="85"/>
-    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Monthly Overhead Total" dataDxfId="84"/>
-    <tableColumn id="6" xr3:uid="{86A5DBCB-1064-4926-8405-405B453A4546}" name="Supplier Performance" dataDxfId="83"/>
+    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="92"/>
+    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Inventory Value" dataDxfId="91"/>
+    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Low Stock Alerts" dataDxfId="90"/>
+    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Upcoming Maintenance" dataDxfId="89"/>
+    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Monthly Overhead Total" dataDxfId="88"/>
+    <tableColumn id="6" xr3:uid="{86A5DBCB-1064-4926-8405-405B453A4546}" name="Supplier Performance" dataDxfId="87"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:M2" totalsRowShown="0" headerRowDxfId="82" dataDxfId="81">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:M2" totalsRowShown="0" headerRowDxfId="86" dataDxfId="85">
   <autoFilter ref="A1:M2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="80"/>
-    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="79"/>
-    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="78"/>
-    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="77"/>
-    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="76"/>
-    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="75"/>
-    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="74"/>
-    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="73">
+    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="84"/>
+    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="83"/>
+    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="82"/>
+    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="81"/>
+    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="80"/>
+    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="79"/>
+    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="78"/>
+    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="77">
       <calculatedColumnFormula>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="72"/>
-    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="71"/>
-    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="70"/>
-    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="69"/>
-    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="68"/>
+    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="76"/>
+    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="75"/>
+    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="74"/>
+    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="73"/>
+    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="72"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="110" dataDxfId="109">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="71" dataDxfId="70">
   <autoFilter ref="A1:K2" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="108"/>
-    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="107"/>
-    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Model" dataDxfId="106"/>
-    <tableColumn id="4" xr3:uid="{217066CA-63B7-4030-A7FC-54062BE2122E}" name="Manufacturer/Brand" dataDxfId="105"/>
-    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="104"/>
-    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="103"/>
-    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="102"/>
-    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="101"/>
-    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="100"/>
-    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="99"/>
-    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="98"/>
+    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="69"/>
+    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="68"/>
+    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Model" dataDxfId="67"/>
+    <tableColumn id="4" xr3:uid="{217066CA-63B7-4030-A7FC-54062BE2122E}" name="Manufacturer/Brand" dataDxfId="66"/>
+    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="65"/>
+    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="64"/>
+    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="63"/>
+    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="62"/>
+    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="61"/>
+    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="60"/>
+    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="59"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:I2" totalsRowShown="0" headerRowDxfId="67" dataDxfId="66">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:I2" totalsRowShown="0" headerRowDxfId="58" dataDxfId="57">
   <autoFilter ref="A1:I2" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="65"/>
-    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="64"/>
-    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="63"/>
-    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="62"/>
-    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="61"/>
-    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="60"/>
-    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="59"/>
-    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="58"/>
-    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="57"/>
+    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="56"/>
+    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="55"/>
+    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="54"/>
+    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="53"/>
+    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="52"/>
+    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="51"/>
+    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="50"/>
+    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="49"/>
+    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="48"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:I2" totalsRowShown="0" headerRowDxfId="56" dataDxfId="55">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:I2" totalsRowShown="0" headerRowDxfId="47" dataDxfId="46">
   <autoFilter ref="A1:I2" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="54"/>
-    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="53"/>
-    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Model" dataDxfId="52"/>
-    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="51"/>
-    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="50"/>
-    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="49"/>
-    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="48"/>
-    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="47"/>
-    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="46"/>
+    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="45"/>
+    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="44"/>
+    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Model" dataDxfId="43"/>
+    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="42"/>
+    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="41"/>
+    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="40"/>
+    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="39"/>
+    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="38"/>
+    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="37"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:H2" totalsRowShown="0" headerRowDxfId="45" dataDxfId="44">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:H2" totalsRowShown="0" headerRowDxfId="36" dataDxfId="35">
   <autoFilter ref="A1:H2" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="43"/>
-    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="42"/>
-    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Model" dataDxfId="41"/>
-    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="40"/>
-    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="39"/>
-    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="1"/>
-    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="38"/>
-    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="37"/>
+    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="34"/>
+    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="33"/>
+    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Model" dataDxfId="32"/>
+    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="31"/>
+    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="30"/>
+    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="29"/>
+    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="28"/>
+    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="27"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:K2" totalsRowShown="0" headerRowDxfId="36" dataDxfId="35">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:K2" totalsRowShown="0" headerRowDxfId="26" dataDxfId="25">
   <autoFilter ref="A1:K2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="34"/>
-    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="33"/>
-    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="32"/>
-    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="31"/>
-    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="30"/>
-    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="29"/>
-    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="28"/>
-    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="27"/>
-    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="26">
+    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="24"/>
+    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="23"/>
+    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="22"/>
+    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="21"/>
+    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="20"/>
+    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="19"/>
+    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="18"/>
+    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="17"/>
+    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="16">
       <calculatedColumnFormula>Shop_Consumables[[#This Row],[Current Stock]]*Shop_Consumables[[#This Row],[Unit Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="25"/>
-    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Preferred Supplier" dataDxfId="24"/>
+    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="15"/>
+    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Preferred Supplier" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1451,7 +1451,7 @@
       <formula1>"Rent/Mortgage, Utilities, Insurance, Other"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2" xr:uid="{63C2185A-207B-4EF1-BB04-3B86B2517042}">
-      <formula1>"Facility Costs/Rent/Mortgage,Insurance,Debt/Leases on Equipment/Business Loans,Subscriptions,Salaries,Utilities,Maintnance/Repair,Marketing/Advertising,Professional Fees,Travel/Vehicles,Depreciations,Other/Miscellaneous"</formula1>
+      <formula1>"Facility Costs/Rent/Mortgage,Insurance,Debt/Leases on Equipment/Business Loans,Subscriptions,Salaries,Utilities,Maintnance/Repair,Marketing/Advertising,Professional Fees,Travel/Vehicles,Depreciation,Other/Miscellaneous"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G3:G1000 G2" xr:uid="{5CDD912B-3197-4C62-9DE2-F15AE0580881}">
       <formula1>"YES, NO"</formula1>

</xml_diff>

<commit_message>
changed Master Dashboard in config.js and the master .xslx
</commit_message>
<xml_diff>
--- a/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
+++ b/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1a2ae81d67634e6/Desktop/Michanikos Artifex Enterprises/MAE Custom Digital Solutions/MAE Workshop Inventory Management System/GITHUB_MAE_Workshop Inventory App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="169" documentId="13_ncr:1_{8CE4ED70-7C3C-4CCA-B9CD-0FFB5498A43E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A0D98F39-3C9B-480F-9D1D-D5B9BCB7A188}"/>
+  <xr:revisionPtr revIDLastSave="201" documentId="13_ncr:1_{8CE4ED70-7C3C-4CCA-B9CD-0FFB5498A43E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{01356BB7-B8FE-4F8F-9695-A7A2451B0C5D}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="3" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
+    <workbookView xWindow="492" yWindow="456" windowWidth="17448" windowHeight="11904" firstSheet="2" activeTab="2" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
   </bookViews>
   <sheets>
     <sheet name="TEST Inventory" sheetId="10" r:id="rId1"/>
@@ -46,27 +46,34 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="74">
   <si>
     <t>mae_id</t>
   </si>
   <si>
-    <t>Total Inventory Value</t>
-  </si>
-  <si>
-    <t>Low Stock Alerts</t>
-  </si>
-  <si>
-    <t>Upcoming Maintenance</t>
-  </si>
-  <si>
-    <t>Monthly Overhead Total</t>
-  </si>
-  <si>
-    <t>Supplier Performance</t>
-  </si>
-  <si>
     <t>Asset ID</t>
   </si>
   <si>
@@ -266,6 +273,24 @@
   </si>
   <si>
     <t>hidden test</t>
+  </si>
+  <si>
+    <t>Total Resell Investment</t>
+  </si>
+  <si>
+    <t>Total Actual Sales</t>
+  </si>
+  <si>
+    <t>Total Shop Asset Value</t>
+  </si>
+  <si>
+    <t>Low Stock Items Count</t>
+  </si>
+  <si>
+    <t>Total Monthly Overhead</t>
+  </si>
+  <si>
+    <t>Equipment Needing Repair</t>
   </si>
 </sst>
 </file>
@@ -310,7 +335,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
       <protection hidden="1"/>
@@ -334,11 +359,39 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="111">
+  <dxfs count="112">
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
@@ -587,6 +640,87 @@
     </dxf>
     <dxf>
       <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -622,107 +756,6 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -768,11 +801,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}" name="TEST_Inventory" displayName="TEST_Inventory" ref="A1:F5" totalsRowShown="0">
   <autoFilter ref="A1:F5" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="97"/>
-    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="96"/>
-    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="95"/>
-    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="94"/>
-    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="93">
+    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="96"/>
+    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="95"/>
+    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="94"/>
+    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="93"/>
+    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="92">
       <calculatedColumnFormula>TEST_Inventory[[#This Row],[TEST Integer]]*TEST_Inventory[[#This Row],[TEST Currency]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{AB3A5F3C-FCF0-4466-90FD-8ABB6E18DF5C}" name="TEST Dropdown"/>
@@ -782,32 +815,32 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:G2" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:G2" totalsRowShown="0" headerRowDxfId="28" dataDxfId="27">
   <autoFilter ref="A1:G2" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="20"/>
-    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="19"/>
-    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="18"/>
-    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="17"/>
-    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="16"/>
-    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="15"/>
-    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="14"/>
+    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="26"/>
+    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="25"/>
+    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="24"/>
+    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="23"/>
+    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="22"/>
+    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="21"/>
+    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
   <autoFilter ref="A1:G2" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="11"/>
-    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="9"/>
-    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="7"/>
-    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="6"/>
-    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="17"/>
+    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="15"/>
+    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="14"/>
+    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="13"/>
+    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="12"/>
+    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="11"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -817,11 +850,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}" name="Location" displayName="Location" ref="A1:E2" insertRow="1" totalsRowShown="0">
   <autoFilter ref="A1:E2" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Name" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Name" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -831,10 +864,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}" name="TEST_Dashboard" displayName="TEST_Dashboard" ref="A1:B2" totalsRowShown="0">
   <autoFilter ref="A1:B2" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="92">
+    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="91">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Currency])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="91">
+    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="90">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Integer])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -843,134 +876,147 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:F2" totalsRowShown="0" headerRowDxfId="90" dataDxfId="89">
-  <autoFilter ref="A1:F2" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}"/>
-  <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="88"/>
-    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Inventory Value" dataDxfId="87"/>
-    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Low Stock Alerts" dataDxfId="86"/>
-    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Upcoming Maintenance" dataDxfId="85"/>
-    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Monthly Overhead Total" dataDxfId="84"/>
-    <tableColumn id="6" xr3:uid="{86A5DBCB-1064-4926-8405-405B453A4546}" name="Supplier Performance" dataDxfId="83"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:G2" totalsRowShown="0" headerRowDxfId="89" dataDxfId="88">
+  <autoFilter ref="A1:G2" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="87"/>
+    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="5">
+      <calculatedColumnFormula>SUM(Resell_Inventory[Total Investment])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="4">
+      <calculatedColumnFormula>SUM(Resell_Inventory[Actual Sale Price])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="3">
+      <calculatedColumnFormula>SUM(Shop_Machinery[Purchase Cost],Shop_Power_Tools[Purchase Price],Shop_Hand_Tools[Purchase Price],Shop_Consumables[Current Inventory Value])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="2">
+      <calculatedColumnFormula array="1">SUMPRODUCT(--(Shop_Consumables[Current Stock]&lt;=Shop_Consumables[Reorder Point]))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Monthly Overhead" dataDxfId="1">
+      <calculatedColumnFormula>SUM(Shop_Overhead[Amount])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="6" xr3:uid="{86A5DBCB-1064-4926-8405-405B453A4546}" name="Equipment Needing Repair" dataDxfId="0">
+      <calculatedColumnFormula>COUNTIFS(Shop_Machinery[Condition], "Needs Repair") + COUNTIFS(Shop_Power_Tools[Condition], "Needs Repair") + COUNTIFS(Shop_Hand_Tools[Condition], "Needs Repair")</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:M2" totalsRowShown="0" headerRowDxfId="82" dataDxfId="81">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:M2" totalsRowShown="0" headerRowDxfId="111" dataDxfId="110">
   <autoFilter ref="A1:M2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="80"/>
-    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="79"/>
-    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="78"/>
-    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="77"/>
-    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="76"/>
-    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="75"/>
-    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="74"/>
-    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="73">
+    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="109"/>
+    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="108"/>
+    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="107"/>
+    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="106"/>
+    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="105"/>
+    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="104"/>
+    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="103"/>
+    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="102">
       <calculatedColumnFormula>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="72"/>
-    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="71"/>
-    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="70"/>
-    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="69"/>
-    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="68"/>
+    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="101"/>
+    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="100"/>
+    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="99"/>
+    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="98"/>
+    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="97"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="110" dataDxfId="109">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="86" dataDxfId="85">
   <autoFilter ref="A1:K2" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="108"/>
-    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="107"/>
-    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Model" dataDxfId="106"/>
-    <tableColumn id="4" xr3:uid="{217066CA-63B7-4030-A7FC-54062BE2122E}" name="Manufacturer/Brand" dataDxfId="105"/>
-    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="104"/>
-    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="103"/>
-    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="102"/>
-    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="101"/>
-    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="100"/>
-    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="99"/>
-    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="98"/>
+    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="84"/>
+    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="83"/>
+    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Model" dataDxfId="82"/>
+    <tableColumn id="4" xr3:uid="{217066CA-63B7-4030-A7FC-54062BE2122E}" name="Manufacturer/Brand" dataDxfId="81"/>
+    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="80"/>
+    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="79"/>
+    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="78"/>
+    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="77"/>
+    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="76"/>
+    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="75"/>
+    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="74"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:I2" totalsRowShown="0" headerRowDxfId="67" dataDxfId="66">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:I2" totalsRowShown="0" headerRowDxfId="73" dataDxfId="72">
   <autoFilter ref="A1:I2" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="65"/>
-    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="64"/>
-    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="63"/>
-    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="62"/>
-    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="61"/>
-    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="60"/>
-    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="59"/>
-    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="58"/>
-    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="57"/>
+    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="71"/>
+    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="70"/>
+    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="69"/>
+    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="68"/>
+    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="67"/>
+    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="66"/>
+    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="65"/>
+    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="64"/>
+    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="63"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:I2" totalsRowShown="0" headerRowDxfId="56" dataDxfId="55">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:I2" totalsRowShown="0" headerRowDxfId="62" dataDxfId="61">
   <autoFilter ref="A1:I2" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="54"/>
-    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="53"/>
-    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Model" dataDxfId="52"/>
-    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="51"/>
-    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="50"/>
-    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="49"/>
-    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="48"/>
-    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="47"/>
-    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="46"/>
+    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="60"/>
+    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="59"/>
+    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Model" dataDxfId="58"/>
+    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="57"/>
+    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="56"/>
+    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="55"/>
+    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="54"/>
+    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="53"/>
+    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="52"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:H2" totalsRowShown="0" headerRowDxfId="45" dataDxfId="44">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:H2" totalsRowShown="0" headerRowDxfId="51" dataDxfId="50">
   <autoFilter ref="A1:H2" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="43"/>
-    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="42"/>
-    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Model" dataDxfId="41"/>
-    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="40"/>
-    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="39"/>
-    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="38"/>
-    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="37"/>
-    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="36"/>
+    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="49"/>
+    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="48"/>
+    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Model" dataDxfId="47"/>
+    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="46"/>
+    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="45"/>
+    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="44"/>
+    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="43"/>
+    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="42"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:K2" totalsRowShown="0" headerRowDxfId="35" dataDxfId="34">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:K2" totalsRowShown="0" headerRowDxfId="41" dataDxfId="40">
   <autoFilter ref="A1:K2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="33"/>
-    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="32"/>
-    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="31"/>
-    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="30"/>
-    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="29"/>
-    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="28"/>
-    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="27"/>
-    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="26"/>
-    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="25">
+    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="39"/>
+    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="38"/>
+    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="37"/>
+    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="36"/>
+    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="35"/>
+    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="34"/>
+    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="33"/>
+    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="32"/>
+    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="31">
       <calculatedColumnFormula>Shop_Consumables[[#This Row],[Current Stock]]*Shop_Consumables[[#This Row],[Unit Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="24"/>
-    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Preferred Supplier" dataDxfId="23"/>
+    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="30"/>
+    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Preferred Supplier" dataDxfId="29"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1309,24 +1355,24 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="F1" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B2" s="4" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="C2" s="8">
         <v>3</v>
@@ -1339,12 +1385,12 @@
         <v>300</v>
       </c>
       <c r="F2" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B3" s="4" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="C3" s="8">
         <v>4</v>
@@ -1357,12 +1403,12 @@
         <v>40</v>
       </c>
       <c r="F3" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B4" s="4" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="C4" s="8">
         <v>5</v>
@@ -1375,12 +1421,12 @@
         <v>100</v>
       </c>
       <c r="F4" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B5" s="4" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C5" s="8">
         <v>1000</v>
@@ -1427,22 +1473,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G1" s="4" t="s">
         <v>36</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="E1" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -1487,22 +1533,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -1530,16 +1576,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -1561,10 +1607,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -1588,36 +1634,66 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2834D935-E140-4D64-A4CD-4A9FB8899FE0}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9" style="1" customWidth="1"/>
-    <col min="2" max="2" width="20" style="3" customWidth="1"/>
-    <col min="3" max="3" width="16.44140625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="22.33203125" style="2" customWidth="1"/>
-    <col min="5" max="5" width="22.33203125" style="3" customWidth="1"/>
-    <col min="6" max="6" width="21" style="2" customWidth="1"/>
-    <col min="7" max="16384" width="8.88671875" style="6"/>
+    <col min="1" max="1" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.109375" style="3" customWidth="1"/>
+    <col min="3" max="3" width="18" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.109375" style="12" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.77734375" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.6640625" style="7" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="E1" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B2" s="3">
+        <f>SUM(Resell_Inventory[Total Investment])</f>
+        <v>0</v>
+      </c>
+      <c r="C2" s="3">
+        <f>SUM(Resell_Inventory[Actual Sale Price])</f>
+        <v>0</v>
+      </c>
+      <c r="D2" s="3">
+        <f>SUM(Shop_Machinery[Purchase Cost],Shop_Power_Tools[Purchase Price],Shop_Hand_Tools[Purchase Price],Shop_Consumables[Current Inventory Value])</f>
+        <v>0</v>
+      </c>
+      <c r="E2" s="12" cm="1">
+        <f t="array" ref="E2">SUMPRODUCT(--(Shop_Consumables[Current Stock]&lt;=Shop_Consumables[Reorder Point]))</f>
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>5</v>
+      <c r="F2" s="3">
+        <f>SUM(Shop_Overhead[Amount])</f>
+        <v>0</v>
+      </c>
+      <c r="G2" s="7">
+        <f>COUNTIFS(Shop_Machinery[Condition], "Needs Repair") + COUNTIFS(Shop_Power_Tools[Condition], "Needs Repair") + COUNTIFS(Shop_Hand_Tools[Condition], "Needs Repair")</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1656,40 +1732,40 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="H1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="J1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="L1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="H1" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="K1" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="L1" s="4" t="s">
-        <v>16</v>
-      </c>
       <c r="M1" s="4" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
@@ -1742,34 +1818,34 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="J1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -1811,28 +1887,28 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="I1" s="9" t="s">
         <v>22</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="E1" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="F1" t="s">
-        <v>24</v>
-      </c>
-      <c r="G1" t="s">
-        <v>25</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="I1" s="9" t="s">
-        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -1877,28 +1953,28 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="F1" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="G1" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="H1" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="I1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -1952,25 +2028,25 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E1" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="H1" s="8" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -2016,34 +2092,34 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
changed an item in config.js (locked: true) for a formula cell in Shop_Consumables; added sheetConfig to deleteExcelRow in app.js; apparently accidentally deleted.
</commit_message>
<xml_diff>
--- a/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
+++ b/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1a2ae81d67634e6/Desktop/Michanikos Artifex Enterprises/MAE Custom Digital Solutions/MAE Workshop Inventory Management System/GITHUB_MAE_Workshop Inventory App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="201" documentId="13_ncr:1_{8CE4ED70-7C3C-4CCA-B9CD-0FFB5498A43E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{01356BB7-B8FE-4F8F-9695-A7A2451B0C5D}"/>
+  <xr:revisionPtr revIDLastSave="203" documentId="13_ncr:1_{8CE4ED70-7C3C-4CCA-B9CD-0FFB5498A43E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B8B87146-5498-47F5-8A05-588FF53502A7}"/>
   <bookViews>
-    <workbookView xWindow="492" yWindow="456" windowWidth="17448" windowHeight="11904" firstSheet="2" activeTab="2" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
   </bookViews>
   <sheets>
     <sheet name="TEST Inventory" sheetId="10" r:id="rId1"/>
@@ -369,15 +369,190 @@
   </cellStyles>
   <dxfs count="112">
     <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -385,342 +560,111 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -768,6 +712,62 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -801,11 +801,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}" name="TEST_Inventory" displayName="TEST_Inventory" ref="A1:F5" totalsRowShown="0">
   <autoFilter ref="A1:F5" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="96"/>
-    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="95"/>
-    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="94"/>
-    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="93"/>
-    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="92">
+    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="102"/>
+    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="101"/>
+    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="100"/>
+    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="99"/>
+    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="98">
       <calculatedColumnFormula>TEST_Inventory[[#This Row],[TEST Integer]]*TEST_Inventory[[#This Row],[TEST Currency]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{AB3A5F3C-FCF0-4466-90FD-8ABB6E18DF5C}" name="TEST Dropdown"/>
@@ -815,32 +815,32 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:G2" totalsRowShown="0" headerRowDxfId="28" dataDxfId="27">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:G2" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
   <autoFilter ref="A1:G2" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="26"/>
-    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="25"/>
-    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="24"/>
-    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="23"/>
-    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="22"/>
-    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="21"/>
-    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="20"/>
+    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="18"/>
+    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="17"/>
+    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="16"/>
+    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="15"/>
+    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
   <autoFilter ref="A1:G2" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="17"/>
-    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="16"/>
-    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="15"/>
-    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="14"/>
-    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="13"/>
-    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="12"/>
-    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="11"/>
+    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="11"/>
+    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="9"/>
+    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="7"/>
+    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="6"/>
+    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -850,11 +850,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}" name="Location" displayName="Location" ref="A1:E2" insertRow="1" totalsRowShown="0">
   <autoFilter ref="A1:E2" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Name" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Name" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -864,10 +864,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}" name="TEST_Dashboard" displayName="TEST_Dashboard" ref="A1:B2" totalsRowShown="0">
   <autoFilter ref="A1:B2" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="91">
+    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="97">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Currency])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="90">
+    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="96">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Integer])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -876,26 +876,26 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:G2" totalsRowShown="0" headerRowDxfId="89" dataDxfId="88">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:G2" totalsRowShown="0" headerRowDxfId="111" dataDxfId="110">
   <autoFilter ref="A1:G2" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="87"/>
-    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="5">
+    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="109"/>
+    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="108">
       <calculatedColumnFormula>SUM(Resell_Inventory[Total Investment])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="4">
+    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="107">
       <calculatedColumnFormula>SUM(Resell_Inventory[Actual Sale Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="3">
+    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="106">
       <calculatedColumnFormula>SUM(Shop_Machinery[Purchase Cost],Shop_Power_Tools[Purchase Price],Shop_Hand_Tools[Purchase Price],Shop_Consumables[Current Inventory Value])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="2">
+    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="105">
       <calculatedColumnFormula array="1">SUMPRODUCT(--(Shop_Consumables[Current Stock]&lt;=Shop_Consumables[Reorder Point]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Monthly Overhead" dataDxfId="1">
+    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Monthly Overhead" dataDxfId="104">
       <calculatedColumnFormula>SUM(Shop_Overhead[Amount])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{86A5DBCB-1064-4926-8405-405B453A4546}" name="Equipment Needing Repair" dataDxfId="0">
+    <tableColumn id="6" xr3:uid="{86A5DBCB-1064-4926-8405-405B453A4546}" name="Equipment Needing Repair" dataDxfId="103">
       <calculatedColumnFormula>COUNTIFS(Shop_Machinery[Condition], "Needs Repair") + COUNTIFS(Shop_Power_Tools[Condition], "Needs Repair") + COUNTIFS(Shop_Hand_Tools[Condition], "Needs Repair")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -904,119 +904,119 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:M2" totalsRowShown="0" headerRowDxfId="111" dataDxfId="110">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:M2" totalsRowShown="0" headerRowDxfId="95" dataDxfId="94">
   <autoFilter ref="A1:M2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="109"/>
-    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="108"/>
-    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="107"/>
-    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="106"/>
-    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="105"/>
-    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="104"/>
-    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="103"/>
-    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="102">
+    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="93"/>
+    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="92"/>
+    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="91"/>
+    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="90"/>
+    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="89"/>
+    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="88"/>
+    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="87"/>
+    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="86">
       <calculatedColumnFormula>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="101"/>
-    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="100"/>
-    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="99"/>
-    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="98"/>
-    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="97"/>
+    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="85"/>
+    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="84"/>
+    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="83"/>
+    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="82"/>
+    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="81"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="86" dataDxfId="85">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="80" dataDxfId="79">
   <autoFilter ref="A1:K2" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="84"/>
-    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="83"/>
-    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Model" dataDxfId="82"/>
-    <tableColumn id="4" xr3:uid="{217066CA-63B7-4030-A7FC-54062BE2122E}" name="Manufacturer/Brand" dataDxfId="81"/>
-    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="80"/>
-    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="79"/>
-    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="78"/>
-    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="77"/>
-    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="76"/>
-    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="75"/>
-    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="74"/>
+    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="78"/>
+    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="77"/>
+    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Model" dataDxfId="76"/>
+    <tableColumn id="4" xr3:uid="{217066CA-63B7-4030-A7FC-54062BE2122E}" name="Manufacturer/Brand" dataDxfId="75"/>
+    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="74"/>
+    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="73"/>
+    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="72"/>
+    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="71"/>
+    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="70"/>
+    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="69"/>
+    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="68"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:I2" totalsRowShown="0" headerRowDxfId="73" dataDxfId="72">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:I2" totalsRowShown="0" headerRowDxfId="67" dataDxfId="66">
   <autoFilter ref="A1:I2" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="71"/>
-    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="70"/>
-    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="69"/>
-    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="68"/>
-    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="67"/>
-    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="66"/>
-    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="65"/>
-    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="64"/>
-    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="63"/>
+    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="65"/>
+    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="64"/>
+    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="63"/>
+    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="62"/>
+    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="61"/>
+    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="60"/>
+    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="59"/>
+    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="58"/>
+    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="57"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:I2" totalsRowShown="0" headerRowDxfId="62" dataDxfId="61">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:I2" totalsRowShown="0" headerRowDxfId="56" dataDxfId="55">
   <autoFilter ref="A1:I2" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="60"/>
-    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="59"/>
-    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Model" dataDxfId="58"/>
-    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="57"/>
-    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="56"/>
-    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="55"/>
-    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="54"/>
-    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="53"/>
-    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="52"/>
+    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="54"/>
+    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="53"/>
+    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Model" dataDxfId="52"/>
+    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="51"/>
+    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="50"/>
+    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="49"/>
+    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="48"/>
+    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="47"/>
+    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="46"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:H2" totalsRowShown="0" headerRowDxfId="51" dataDxfId="50">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:H2" totalsRowShown="0" headerRowDxfId="45" dataDxfId="44">
   <autoFilter ref="A1:H2" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="49"/>
-    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="48"/>
-    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Model" dataDxfId="47"/>
-    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="46"/>
-    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="45"/>
-    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="44"/>
-    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="43"/>
-    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="42"/>
+    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="43"/>
+    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="42"/>
+    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Model" dataDxfId="41"/>
+    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="40"/>
+    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="39"/>
+    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="38"/>
+    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="37"/>
+    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="36"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:K2" totalsRowShown="0" headerRowDxfId="41" dataDxfId="40">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:K2" totalsRowShown="0" headerRowDxfId="35" dataDxfId="34">
   <autoFilter ref="A1:K2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="39"/>
-    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="38"/>
-    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="37"/>
-    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="36"/>
-    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="35"/>
-    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="34"/>
-    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="33"/>
-    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="32"/>
-    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="31">
+    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="33"/>
+    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="32"/>
+    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="31"/>
+    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="30"/>
+    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="29"/>
+    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="28"/>
+    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="27"/>
+    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="26"/>
+    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="25">
       <calculatedColumnFormula>Shop_Consumables[[#This Row],[Current Stock]]*Shop_Consumables[[#This Row],[Unit Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="30"/>
-    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Preferred Supplier" dataDxfId="29"/>
+    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="24"/>
+    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Preferred Supplier" dataDxfId="23"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>

</xml_diff>

<commit_message>
redid config.js and excel to add columns for chart.js
</commit_message>
<xml_diff>
--- a/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
+++ b/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1a2ae81d67634e6/Desktop/Michanikos Artifex Enterprises/MAE Custom Digital Solutions/MAE Workshop Inventory Management System/GITHUB_MAE_Workshop Inventory App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="203" documentId="13_ncr:1_{8CE4ED70-7C3C-4CCA-B9CD-0FFB5498A43E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B8B87146-5498-47F5-8A05-588FF53502A7}"/>
+  <xr:revisionPtr revIDLastSave="244" documentId="13_ncr:1_{8CE4ED70-7C3C-4CCA-B9CD-0FFB5498A43E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F30B6345-D464-467A-9681-0001AF1B6C51}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="9180" activeTab="2" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
   </bookViews>
   <sheets>
     <sheet name="TEST Inventory" sheetId="10" r:id="rId1"/>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="78">
   <si>
     <t>mae_id</t>
   </si>
@@ -291,6 +291,18 @@
   </si>
   <si>
     <t>Equipment Needing Repair</t>
+  </si>
+  <si>
+    <t>Total Machinery Value</t>
+  </si>
+  <si>
+    <t>Total Power Tool Value</t>
+  </si>
+  <si>
+    <t>Total Consumables Value</t>
+  </si>
+  <si>
+    <t>Total Hand Tool Value</t>
   </si>
 </sst>
 </file>
@@ -300,7 +312,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -313,6 +325,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -335,7 +353,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
       <protection hidden="1"/>
@@ -363,11 +381,47 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="112">
+  <dxfs count="116">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
@@ -665,6 +719,58 @@
     </dxf>
     <dxf>
       <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -712,62 +818,6 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -793,19 +843,15 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}" name="TEST_Inventory" displayName="TEST_Inventory" ref="A1:F5" totalsRowShown="0">
   <autoFilter ref="A1:F5" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="102"/>
-    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="101"/>
-    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="100"/>
-    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="99"/>
-    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="98">
+    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="100"/>
+    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="99"/>
+    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="98"/>
+    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="97"/>
+    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="96">
       <calculatedColumnFormula>TEST_Inventory[[#This Row],[TEST Integer]]*TEST_Inventory[[#This Row],[TEST Currency]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{AB3A5F3C-FCF0-4466-90FD-8ABB6E18DF5C}" name="TEST Dropdown"/>
@@ -815,32 +861,32 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:G2" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:G2" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26">
   <autoFilter ref="A1:G2" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="20"/>
-    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="19"/>
-    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="18"/>
-    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="17"/>
-    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="16"/>
-    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="15"/>
-    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="14"/>
+    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="25"/>
+    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="24"/>
+    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="23"/>
+    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="22"/>
+    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="21"/>
+    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="20"/>
+    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="19"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
   <autoFilter ref="A1:G2" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="11"/>
-    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="9"/>
-    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="7"/>
-    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="6"/>
-    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="16"/>
+    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="14"/>
+    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="13"/>
+    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="12"/>
+    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="11"/>
+    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -850,11 +896,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}" name="Location" displayName="Location" ref="A1:E2" insertRow="1" totalsRowShown="0">
   <autoFilter ref="A1:E2" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Name" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Name" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -864,10 +910,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}" name="TEST_Dashboard" displayName="TEST_Dashboard" ref="A1:B2" totalsRowShown="0">
   <autoFilter ref="A1:B2" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="97">
+    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="95">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Currency])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="96">
+    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="94">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Integer])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -876,26 +922,38 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:G2" totalsRowShown="0" headerRowDxfId="111" dataDxfId="110">
-  <autoFilter ref="A1:G2" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}"/>
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="109"/>
-    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="108">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:K2" totalsRowShown="0" headerRowDxfId="93" dataDxfId="92">
+  <autoFilter ref="A1:K2" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="91"/>
+    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="90">
       <calculatedColumnFormula>SUM(Resell_Inventory[Total Investment])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="107">
+    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="89">
       <calculatedColumnFormula>SUM(Resell_Inventory[Actual Sale Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="106">
-      <calculatedColumnFormula>SUM(Shop_Machinery[Purchase Cost],Shop_Power_Tools[Purchase Price],Shop_Hand_Tools[Purchase Price],Shop_Consumables[Current Inventory Value])</calculatedColumnFormula>
+    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="4">
+      <calculatedColumnFormula>SUM(Shop_Machinery[Purchase Cost])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="105">
+    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="3">
+      <calculatedColumnFormula>SUM(Shop_Power_Tools[Purchase Price])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="2">
+      <calculatedColumnFormula>SUM(Shop_Hand_Tools[Purchase Price])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="1">
+      <calculatedColumnFormula>SUM(Shop_Consumables[Current Inventory Value])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="0">
+      <calculatedColumnFormula>SUM(D2,E2,F2,G2)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="88">
       <calculatedColumnFormula array="1">SUMPRODUCT(--(Shop_Consumables[Current Stock]&lt;=Shop_Consumables[Reorder Point]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Monthly Overhead" dataDxfId="104">
+    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Monthly Overhead" dataDxfId="87">
       <calculatedColumnFormula>SUM(Shop_Overhead[Amount])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{86A5DBCB-1064-4926-8405-405B453A4546}" name="Equipment Needing Repair" dataDxfId="103">
+    <tableColumn id="6" xr3:uid="{86A5DBCB-1064-4926-8405-405B453A4546}" name="Equipment Needing Repair" dataDxfId="86">
       <calculatedColumnFormula>COUNTIFS(Shop_Machinery[Condition], "Needs Repair") + COUNTIFS(Shop_Power_Tools[Condition], "Needs Repair") + COUNTIFS(Shop_Hand_Tools[Condition], "Needs Repair")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -904,119 +962,119 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:M2" totalsRowShown="0" headerRowDxfId="95" dataDxfId="94">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:M2" totalsRowShown="0" headerRowDxfId="115" dataDxfId="114">
   <autoFilter ref="A1:M2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="93"/>
-    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="92"/>
-    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="91"/>
-    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="90"/>
-    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="89"/>
-    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="88"/>
-    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="87"/>
-    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="86">
+    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="113"/>
+    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="112"/>
+    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="111"/>
+    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="110"/>
+    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="109"/>
+    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="108"/>
+    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="107"/>
+    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="106">
       <calculatedColumnFormula>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="85"/>
-    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="84"/>
-    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="83"/>
-    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="82"/>
-    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="81"/>
+    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="105"/>
+    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="104"/>
+    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="103"/>
+    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="102"/>
+    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="101"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="80" dataDxfId="79">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="85" dataDxfId="84">
   <autoFilter ref="A1:K2" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="78"/>
-    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="77"/>
-    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Model" dataDxfId="76"/>
-    <tableColumn id="4" xr3:uid="{217066CA-63B7-4030-A7FC-54062BE2122E}" name="Manufacturer/Brand" dataDxfId="75"/>
-    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="74"/>
-    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="73"/>
-    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="72"/>
-    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="71"/>
-    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="70"/>
-    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="69"/>
-    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="68"/>
+    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="83"/>
+    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="82"/>
+    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Model" dataDxfId="81"/>
+    <tableColumn id="4" xr3:uid="{217066CA-63B7-4030-A7FC-54062BE2122E}" name="Manufacturer/Brand" dataDxfId="80"/>
+    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="79"/>
+    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="78"/>
+    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="77"/>
+    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="76"/>
+    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="75"/>
+    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="74"/>
+    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="73"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:I2" totalsRowShown="0" headerRowDxfId="67" dataDxfId="66">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:I2" totalsRowShown="0" headerRowDxfId="72" dataDxfId="71">
   <autoFilter ref="A1:I2" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="65"/>
-    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="64"/>
-    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="63"/>
-    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="62"/>
-    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="61"/>
-    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="60"/>
-    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="59"/>
-    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="58"/>
-    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="57"/>
+    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="70"/>
+    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="69"/>
+    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="68"/>
+    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="67"/>
+    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="66"/>
+    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="65"/>
+    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="64"/>
+    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="63"/>
+    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="62"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:I2" totalsRowShown="0" headerRowDxfId="56" dataDxfId="55">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:I2" totalsRowShown="0" headerRowDxfId="61" dataDxfId="60">
   <autoFilter ref="A1:I2" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="54"/>
-    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="53"/>
-    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Model" dataDxfId="52"/>
-    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="51"/>
-    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="50"/>
-    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="49"/>
-    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="48"/>
-    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="47"/>
-    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="46"/>
+    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="59"/>
+    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="58"/>
+    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Model" dataDxfId="57"/>
+    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="56"/>
+    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="55"/>
+    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="54"/>
+    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="53"/>
+    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="52"/>
+    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="51"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:H2" totalsRowShown="0" headerRowDxfId="45" dataDxfId="44">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:H2" totalsRowShown="0" headerRowDxfId="50" dataDxfId="49">
   <autoFilter ref="A1:H2" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="43"/>
-    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="42"/>
-    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Model" dataDxfId="41"/>
-    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="40"/>
-    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="39"/>
-    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="38"/>
-    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="37"/>
-    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="36"/>
+    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="48"/>
+    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="47"/>
+    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Model" dataDxfId="46"/>
+    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="45"/>
+    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="44"/>
+    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="43"/>
+    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="42"/>
+    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="41"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:K2" totalsRowShown="0" headerRowDxfId="35" dataDxfId="34">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:K2" totalsRowShown="0" headerRowDxfId="40" dataDxfId="39">
   <autoFilter ref="A1:K2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="33"/>
-    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="32"/>
-    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="31"/>
-    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="30"/>
-    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="29"/>
-    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="28"/>
-    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="27"/>
-    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="26"/>
-    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="25">
+    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="38"/>
+    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="37"/>
+    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="36"/>
+    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="35"/>
+    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="34"/>
+    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="33"/>
+    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="32"/>
+    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="31"/>
+    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="30">
       <calculatedColumnFormula>Shop_Consumables[[#This Row],[Current Stock]]*Shop_Consumables[[#This Row],[Unit Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="24"/>
-    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Preferred Supplier" dataDxfId="23"/>
+    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="29"/>
+    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Preferred Supplier" dataDxfId="28"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1634,20 +1692,24 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2834D935-E140-4D64-A4CD-4A9FB8899FE0}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="29.109375" style="3" customWidth="1"/>
     <col min="3" max="3" width="18" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="22" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.109375" style="12" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.77734375" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25.6640625" style="7" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.88671875" style="6"/>
+    <col min="4" max="4" width="21.44140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.77734375" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.44140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.109375" style="12" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22.77734375" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="25.6640625" style="7" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1658,19 +1720,31 @@
         <v>69</v>
       </c>
       <c r="D1" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="H1" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="I1" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="G1" s="8" t="s">
+      <c r="K1" s="8" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B2" s="3">
         <f>SUM(Resell_Inventory[Total Investment])</f>
         <v>0</v>
@@ -1680,23 +1754,40 @@
         <v>0</v>
       </c>
       <c r="D2" s="3">
-        <f>SUM(Shop_Machinery[Purchase Cost],Shop_Power_Tools[Purchase Price],Shop_Hand_Tools[Purchase Price],Shop_Consumables[Current Inventory Value])</f>
+        <f>SUM(Shop_Machinery[Purchase Cost])</f>
         <v>0</v>
       </c>
-      <c r="E2" s="12" cm="1">
-        <f t="array" ref="E2">SUMPRODUCT(--(Shop_Consumables[Current Stock]&lt;=Shop_Consumables[Reorder Point]))</f>
+      <c r="E2" s="3">
+        <f>SUM(Shop_Power_Tools[Purchase Price])</f>
+        <v>0</v>
+      </c>
+      <c r="F2" s="3">
+        <f>SUM(Shop_Hand_Tools[Purchase Price])</f>
+        <v>0</v>
+      </c>
+      <c r="G2" s="3">
+        <f>SUM(Shop_Consumables[Current Inventory Value])</f>
+        <v>0</v>
+      </c>
+      <c r="H2" s="13">
+        <f>SUM(D2,E2,F2,G2)</f>
+        <v>0</v>
+      </c>
+      <c r="I2" s="12" cm="1">
+        <f t="array" ref="I2">SUMPRODUCT(--(Shop_Consumables[Current Stock]&lt;=Shop_Consumables[Reorder Point]))</f>
         <v>1</v>
       </c>
-      <c r="F2" s="3">
+      <c r="J2" s="3">
         <f>SUM(Shop_Overhead[Amount])</f>
         <v>0</v>
       </c>
-      <c r="G2" s="7">
+      <c r="K2" s="7">
         <f>COUNTIFS(Shop_Machinery[Condition], "Needs Repair") + COUNTIFS(Shop_Power_Tools[Condition], "Needs Repair") + COUNTIFS(Shop_Hand_Tools[Condition], "Needs Repair")</f>
         <v>0</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
changed conifg.js and Master Excel file for Overhead  Snapshot in Master Dashboard file to "Total Amount Due Next 30 Days" and updated formula
</commit_message>
<xml_diff>
--- a/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
+++ b/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1a2ae81d67634e6/Desktop/Michanikos Artifex Enterprises/MAE Custom Digital Solutions/MAE Workshop Inventory Management System/GITHUB_MAE_Workshop Inventory App/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MWEAK\OneDrive\Desktop\Michanikos Artifex Enterprises\MAE Custom Digital Solutions\MAE Workshop Inventory Management System\GITHUB_MAE_Workshop Inventory App\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="244" documentId="13_ncr:1_{8CE4ED70-7C3C-4CCA-B9CD-0FFB5498A43E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F30B6345-D464-467A-9681-0001AF1B6C51}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="9180" activeTab="2" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
+    <workbookView xWindow="5580" yWindow="2064" windowWidth="19560" windowHeight="11904" activeTab="2" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
   </bookViews>
   <sheets>
     <sheet name="TEST Inventory" sheetId="10" r:id="rId1"/>
@@ -287,9 +287,6 @@
     <t>Low Stock Items Count</t>
   </si>
   <si>
-    <t>Total Monthly Overhead</t>
-  </si>
-  <si>
     <t>Equipment Needing Repair</t>
   </si>
   <si>
@@ -303,6 +300,9 @@
   </si>
   <si>
     <t>Total Hand Tool Value</t>
+  </si>
+  <si>
+    <t>Total Amount Due Next 30 Days</t>
   </si>
 </sst>
 </file>
@@ -390,6 +390,396 @@
   </cellStyles>
   <dxfs count="116">
     <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -423,401 +813,11 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -847,11 +847,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}" name="TEST_Inventory" displayName="TEST_Inventory" ref="A1:F5" totalsRowShown="0">
   <autoFilter ref="A1:F5" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="100"/>
-    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="99"/>
-    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="98"/>
-    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="97"/>
-    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="96">
+    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="102"/>
+    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="101"/>
+    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="100"/>
+    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="99"/>
+    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="98">
       <calculatedColumnFormula>TEST_Inventory[[#This Row],[TEST Integer]]*TEST_Inventory[[#This Row],[TEST Currency]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{AB3A5F3C-FCF0-4466-90FD-8ABB6E18DF5C}" name="TEST Dropdown"/>
@@ -861,32 +861,32 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:G2" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:G2" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
   <autoFilter ref="A1:G2" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="25"/>
-    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="24"/>
-    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="23"/>
-    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="22"/>
-    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="21"/>
-    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="20"/>
-    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="19"/>
+    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="18"/>
+    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="17"/>
+    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="16"/>
+    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="15"/>
+    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
   <autoFilter ref="A1:G2" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="16"/>
-    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="15"/>
-    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="14"/>
-    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="13"/>
-    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="12"/>
-    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="11"/>
-    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="10"/>
+    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="11"/>
+    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="9"/>
+    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="7"/>
+    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="6"/>
+    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -896,11 +896,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}" name="Location" displayName="Location" ref="A1:E2" insertRow="1" totalsRowShown="0">
   <autoFilter ref="A1:E2" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Name" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Name" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -910,10 +910,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}" name="TEST_Dashboard" displayName="TEST_Dashboard" ref="A1:B2" totalsRowShown="0">
   <autoFilter ref="A1:B2" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="95">
+    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="97">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Currency])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="94">
+    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="96">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Integer])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -922,38 +922,38 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:K2" totalsRowShown="0" headerRowDxfId="93" dataDxfId="92">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:K2" totalsRowShown="0" headerRowDxfId="115" dataDxfId="114">
   <autoFilter ref="A1:K2" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="91"/>
-    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="90">
+    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="113"/>
+    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="112">
       <calculatedColumnFormula>SUM(Resell_Inventory[Total Investment])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="89">
+    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="111">
       <calculatedColumnFormula>SUM(Resell_Inventory[Actual Sale Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="4">
+    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="110">
       <calculatedColumnFormula>SUM(Shop_Machinery[Purchase Cost])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="3">
+    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="109">
       <calculatedColumnFormula>SUM(Shop_Power_Tools[Purchase Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="2">
+    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="108">
       <calculatedColumnFormula>SUM(Shop_Hand_Tools[Purchase Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="1">
+    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="107">
       <calculatedColumnFormula>SUM(Shop_Consumables[Current Inventory Value])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="0">
+    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="106">
       <calculatedColumnFormula>SUM(D2,E2,F2,G2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="88">
+    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="105">
       <calculatedColumnFormula array="1">SUMPRODUCT(--(Shop_Consumables[Current Stock]&lt;=Shop_Consumables[Reorder Point]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Monthly Overhead" dataDxfId="87">
-      <calculatedColumnFormula>SUM(Shop_Overhead[Amount])</calculatedColumnFormula>
+    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="104">
+      <calculatedColumnFormula>SUMIFS(Shop_Overhead[Amount], Shop_Overhead[Due Date], "&lt;="&amp;TODAY()+30, Shop_Overhead[Due Date], "&gt;="&amp;TODAY())</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{86A5DBCB-1064-4926-8405-405B453A4546}" name="Equipment Needing Repair" dataDxfId="86">
+    <tableColumn id="6" xr3:uid="{86A5DBCB-1064-4926-8405-405B453A4546}" name="Equipment Needing Repair" dataDxfId="103">
       <calculatedColumnFormula>COUNTIFS(Shop_Machinery[Condition], "Needs Repair") + COUNTIFS(Shop_Power_Tools[Condition], "Needs Repair") + COUNTIFS(Shop_Hand_Tools[Condition], "Needs Repair")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -962,119 +962,119 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:M2" totalsRowShown="0" headerRowDxfId="115" dataDxfId="114">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:M2" totalsRowShown="0" headerRowDxfId="95" dataDxfId="94">
   <autoFilter ref="A1:M2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="113"/>
-    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="112"/>
-    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="111"/>
-    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="110"/>
-    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="109"/>
-    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="108"/>
-    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="107"/>
-    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="106">
+    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="93"/>
+    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="92"/>
+    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="91"/>
+    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="90"/>
+    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="89"/>
+    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="88"/>
+    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="87"/>
+    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="86">
       <calculatedColumnFormula>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="105"/>
-    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="104"/>
-    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="103"/>
-    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="102"/>
-    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="101"/>
+    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="85"/>
+    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="84"/>
+    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="83"/>
+    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="82"/>
+    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="81"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="85" dataDxfId="84">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="80" dataDxfId="79">
   <autoFilter ref="A1:K2" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="83"/>
-    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="82"/>
-    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Model" dataDxfId="81"/>
-    <tableColumn id="4" xr3:uid="{217066CA-63B7-4030-A7FC-54062BE2122E}" name="Manufacturer/Brand" dataDxfId="80"/>
-    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="79"/>
-    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="78"/>
-    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="77"/>
-    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="76"/>
-    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="75"/>
-    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="74"/>
-    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="73"/>
+    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="78"/>
+    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="77"/>
+    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Model" dataDxfId="76"/>
+    <tableColumn id="4" xr3:uid="{217066CA-63B7-4030-A7FC-54062BE2122E}" name="Manufacturer/Brand" dataDxfId="75"/>
+    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="74"/>
+    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="73"/>
+    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="72"/>
+    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="71"/>
+    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="70"/>
+    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="69"/>
+    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="68"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:I2" totalsRowShown="0" headerRowDxfId="72" dataDxfId="71">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:I2" totalsRowShown="0" headerRowDxfId="67" dataDxfId="66">
   <autoFilter ref="A1:I2" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="70"/>
-    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="69"/>
-    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="68"/>
-    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="67"/>
-    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="66"/>
-    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="65"/>
-    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="64"/>
-    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="63"/>
-    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="62"/>
+    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="65"/>
+    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="64"/>
+    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="63"/>
+    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="62"/>
+    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="61"/>
+    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="60"/>
+    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="59"/>
+    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="58"/>
+    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="57"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:I2" totalsRowShown="0" headerRowDxfId="61" dataDxfId="60">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:I2" totalsRowShown="0" headerRowDxfId="56" dataDxfId="55">
   <autoFilter ref="A1:I2" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="59"/>
-    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="58"/>
-    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Model" dataDxfId="57"/>
-    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="56"/>
-    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="55"/>
-    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="54"/>
-    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="53"/>
-    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="52"/>
-    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="51"/>
+    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="54"/>
+    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="53"/>
+    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Model" dataDxfId="52"/>
+    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="51"/>
+    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="50"/>
+    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="49"/>
+    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="48"/>
+    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="47"/>
+    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="46"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:H2" totalsRowShown="0" headerRowDxfId="50" dataDxfId="49">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:H2" totalsRowShown="0" headerRowDxfId="45" dataDxfId="44">
   <autoFilter ref="A1:H2" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="48"/>
-    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="47"/>
-    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Model" dataDxfId="46"/>
-    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="45"/>
-    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="44"/>
-    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="43"/>
-    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="42"/>
-    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="41"/>
+    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="43"/>
+    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="42"/>
+    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Model" dataDxfId="41"/>
+    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="40"/>
+    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="39"/>
+    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="38"/>
+    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="37"/>
+    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="36"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:K2" totalsRowShown="0" headerRowDxfId="40" dataDxfId="39">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:K2" totalsRowShown="0" headerRowDxfId="35" dataDxfId="34">
   <autoFilter ref="A1:K2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="38"/>
-    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="37"/>
-    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="36"/>
-    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="35"/>
-    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="34"/>
-    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="33"/>
-    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="32"/>
-    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="31"/>
-    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="30">
+    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="33"/>
+    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="32"/>
+    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="31"/>
+    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="30"/>
+    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="29"/>
+    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="28"/>
+    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="27"/>
+    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="26"/>
+    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="25">
       <calculatedColumnFormula>Shop_Consumables[[#This Row],[Current Stock]]*Shop_Consumables[[#This Row],[Unit Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="29"/>
-    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Preferred Supplier" dataDxfId="28"/>
+    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="24"/>
+    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Preferred Supplier" dataDxfId="23"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1704,7 +1704,7 @@
     <col min="7" max="7" width="24.33203125" style="3" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="22" style="3" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="22.109375" style="12" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="22.77734375" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="29" style="3" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="25.6640625" style="7" bestFit="1" customWidth="1"/>
     <col min="12" max="16384" width="8.88671875" style="6"/>
   </cols>
@@ -1720,16 +1720,16 @@
         <v>69</v>
       </c>
       <c r="D1" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="G1" s="5" t="s">
         <v>75</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>76</v>
       </c>
       <c r="H1" s="5" t="s">
         <v>70</v>
@@ -1738,10 +1738,10 @@
         <v>71</v>
       </c>
       <c r="J1" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="K1" s="8" t="s">
         <v>72</v>
-      </c>
-      <c r="K1" s="8" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
@@ -1778,7 +1778,7 @@
         <v>1</v>
       </c>
       <c r="J2" s="3">
-        <f>SUM(Shop_Overhead[Amount])</f>
+        <f ca="1">SUMIFS(Shop_Overhead[Amount], Shop_Overhead[Due Date], "&lt;="&amp;TODAY()+30, Shop_Overhead[Due Date], "&gt;="&amp;TODAY())</f>
         <v>0</v>
       </c>
       <c r="K2" s="7">

</xml_diff>

<commit_message>
added new worksheet/table to config.js and Excel to support Master Dashboard Overhead functionality
</commit_message>
<xml_diff>
--- a/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
+++ b/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
@@ -5,26 +5,27 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MWEAK\OneDrive\Desktop\Michanikos Artifex Enterprises\MAE Custom Digital Solutions\MAE Workshop Inventory Management System\GITHUB_MAE_Workshop Inventory App\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1a2ae81d67634e6/Desktop/Michanikos Artifex Enterprises/MAE Custom Digital Solutions/MAE Workshop Inventory Management System/GITHUB_MAE_Workshop Inventory App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD064C17-0AAC-40F7-A2B6-B50A57BE904F}"/>
   <bookViews>
-    <workbookView xWindow="5580" yWindow="2064" windowWidth="19560" windowHeight="11904" activeTab="2" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="10740" firstSheet="2" activeTab="3" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
   </bookViews>
   <sheets>
     <sheet name="TEST Inventory" sheetId="10" r:id="rId1"/>
     <sheet name="TEST Dashboard" sheetId="11" r:id="rId2"/>
     <sheet name="Master Dashboard" sheetId="1" r:id="rId3"/>
-    <sheet name="Resell Inventory" sheetId="2" r:id="rId4"/>
-    <sheet name="Shop Machinery" sheetId="3" r:id="rId5"/>
-    <sheet name="Maintenance Log" sheetId="4" r:id="rId6"/>
-    <sheet name="Shop Power Tools" sheetId="5" r:id="rId7"/>
-    <sheet name="Shop Hand Tools" sheetId="6" r:id="rId8"/>
-    <sheet name="Shop Consumables" sheetId="7" r:id="rId9"/>
-    <sheet name="Shop Overhead" sheetId="8" r:id="rId10"/>
-    <sheet name="Supplier Contacts" sheetId="9" r:id="rId11"/>
-    <sheet name="Location" sheetId="12" r:id="rId12"/>
+    <sheet name="Overhead Summary" sheetId="13" r:id="rId4"/>
+    <sheet name="Resell Inventory" sheetId="2" r:id="rId5"/>
+    <sheet name="Shop Machinery" sheetId="3" r:id="rId6"/>
+    <sheet name="Maintenance Log" sheetId="4" r:id="rId7"/>
+    <sheet name="Shop Power Tools" sheetId="5" r:id="rId8"/>
+    <sheet name="Shop Hand Tools" sheetId="6" r:id="rId9"/>
+    <sheet name="Shop Consumables" sheetId="7" r:id="rId10"/>
+    <sheet name="Shop Overhead" sheetId="8" r:id="rId11"/>
+    <sheet name="Supplier Contacts" sheetId="9" r:id="rId12"/>
+    <sheet name="Location" sheetId="12" r:id="rId13"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -69,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="79">
   <si>
     <t>mae_id</t>
   </si>
@@ -303,6 +304,9 @@
   </si>
   <si>
     <t>Total Amount Due Next 30 Days</t>
+  </si>
+  <si>
+    <t>Annual Total</t>
   </si>
 </sst>
 </file>
@@ -388,7 +392,13 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="116">
+  <dxfs count="118">
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
@@ -847,11 +857,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}" name="TEST_Inventory" displayName="TEST_Inventory" ref="A1:F5" totalsRowShown="0">
   <autoFilter ref="A1:F5" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="102"/>
-    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="101"/>
-    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="100"/>
-    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="99"/>
-    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="98">
+    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="104"/>
+    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="103"/>
+    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="102"/>
+    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="101"/>
+    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="100">
       <calculatedColumnFormula>TEST_Inventory[[#This Row],[TEST Integer]]*TEST_Inventory[[#This Row],[TEST Currency]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{AB3A5F3C-FCF0-4466-90FD-8ABB6E18DF5C}" name="TEST Dropdown"/>
@@ -861,46 +871,68 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:G2" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
-  <autoFilter ref="A1:G2" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}"/>
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="20"/>
-    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="19"/>
-    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="18"/>
-    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="17"/>
-    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="16"/>
-    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="15"/>
-    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="14"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:K2" totalsRowShown="0" headerRowDxfId="37" dataDxfId="36">
+  <autoFilter ref="A1:K2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="35"/>
+    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="34"/>
+    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="33"/>
+    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="32"/>
+    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="31"/>
+    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="30"/>
+    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="29"/>
+    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="28"/>
+    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="27">
+      <calculatedColumnFormula>Shop_Consumables[[#This Row],[Current Stock]]*Shop_Consumables[[#This Row],[Unit Cost]]</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="26"/>
+    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Preferred Supplier" dataDxfId="25"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
-  <autoFilter ref="A1:G2" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:G2" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23">
+  <autoFilter ref="A1:G2" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="11"/>
-    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="9"/>
-    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="7"/>
-    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="6"/>
-    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="22"/>
+    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="20"/>
+    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="18"/>
+    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="17"/>
+    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
+  <autoFilter ref="A1:G2" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="13"/>
+    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="11"/>
+    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="9"/>
+    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="8"/>
+    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="7"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}" name="Location" displayName="Location" ref="A1:E2" insertRow="1" totalsRowShown="0">
   <autoFilter ref="A1:E2" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Name" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Name" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -910,10 +942,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}" name="TEST_Dashboard" displayName="TEST_Dashboard" ref="A1:B2" totalsRowShown="0">
   <autoFilter ref="A1:B2" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="97">
+    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="99">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Currency])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="96">
+    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="98">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Integer])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -922,38 +954,38 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:K2" totalsRowShown="0" headerRowDxfId="115" dataDxfId="114">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:K2" totalsRowShown="0" headerRowDxfId="117" dataDxfId="116">
   <autoFilter ref="A1:K2" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="113"/>
-    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="112">
+    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="115"/>
+    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="114">
       <calculatedColumnFormula>SUM(Resell_Inventory[Total Investment])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="111">
+    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="113">
       <calculatedColumnFormula>SUM(Resell_Inventory[Actual Sale Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="110">
+    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="112">
       <calculatedColumnFormula>SUM(Shop_Machinery[Purchase Cost])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="109">
+    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="111">
       <calculatedColumnFormula>SUM(Shop_Power_Tools[Purchase Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="108">
+    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="110">
       <calculatedColumnFormula>SUM(Shop_Hand_Tools[Purchase Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="107">
+    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="109">
       <calculatedColumnFormula>SUM(Shop_Consumables[Current Inventory Value])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="106">
+    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="108">
       <calculatedColumnFormula>SUM(D2,E2,F2,G2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="105">
+    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="107">
       <calculatedColumnFormula array="1">SUMPRODUCT(--(Shop_Consumables[Current Stock]&lt;=Shop_Consumables[Reorder Point]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="104">
+    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="106">
       <calculatedColumnFormula>SUMIFS(Shop_Overhead[Amount], Shop_Overhead[Due Date], "&lt;="&amp;TODAY()+30, Shop_Overhead[Due Date], "&gt;="&amp;TODAY())</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{86A5DBCB-1064-4926-8405-405B453A4546}" name="Equipment Needing Repair" dataDxfId="103">
+    <tableColumn id="6" xr3:uid="{86A5DBCB-1064-4926-8405-405B453A4546}" name="Equipment Needing Repair" dataDxfId="105">
       <calculatedColumnFormula>COUNTIFS(Shop_Machinery[Condition], "Needs Repair") + COUNTIFS(Shop_Power_Tools[Condition], "Needs Repair") + COUNTIFS(Shop_Hand_Tools[Condition], "Needs Repair")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -962,119 +994,110 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:M2" totalsRowShown="0" headerRowDxfId="95" dataDxfId="94">
-  <autoFilter ref="A1:M2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}"/>
-  <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="93"/>
-    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="92"/>
-    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="91"/>
-    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="90"/>
-    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="89"/>
-    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="88"/>
-    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="87"/>
-    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="86">
-      <calculatedColumnFormula>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</calculatedColumnFormula>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{F579DA07-7AD6-49DA-9B44-D5B1132EDAC6}" name="Overhead_Summary" displayName="Overhead_Summary" ref="A9:B10" totalsRowShown="0">
+  <autoFilter ref="A9:B10" xr:uid="{F579DA07-7AD6-49DA-9B44-D5B1132EDAC6}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{7CA4839C-9603-479D-BD1C-8377DFA9603C}" name="Expense Category" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{FE0F7616-EAF3-443D-AC69-DE6541DC10E5}" name="Annual Total" dataDxfId="0">
+      <calculatedColumnFormula>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="85"/>
-    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="84"/>
-    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="83"/>
-    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="82"/>
-    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="81"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="80" dataDxfId="79">
-  <autoFilter ref="A1:K2" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}"/>
-  <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="78"/>
-    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="77"/>
-    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Model" dataDxfId="76"/>
-    <tableColumn id="4" xr3:uid="{217066CA-63B7-4030-A7FC-54062BE2122E}" name="Manufacturer/Brand" dataDxfId="75"/>
-    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="74"/>
-    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="73"/>
-    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="72"/>
-    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="71"/>
-    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="70"/>
-    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="69"/>
-    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="68"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:M2" totalsRowShown="0" headerRowDxfId="97" dataDxfId="96">
+  <autoFilter ref="A1:M2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}"/>
+  <tableColumns count="13">
+    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="95"/>
+    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="94"/>
+    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="93"/>
+    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="92"/>
+    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="91"/>
+    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="90"/>
+    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="89"/>
+    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="88">
+      <calculatedColumnFormula>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="87"/>
+    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="86"/>
+    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="85"/>
+    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="84"/>
+    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="83"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:I2" totalsRowShown="0" headerRowDxfId="67" dataDxfId="66">
-  <autoFilter ref="A1:I2" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}"/>
-  <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="65"/>
-    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="64"/>
-    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="63"/>
-    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="62"/>
-    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="61"/>
-    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="60"/>
-    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="59"/>
-    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="58"/>
-    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="57"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="82" dataDxfId="81">
+  <autoFilter ref="A1:K2" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="80"/>
+    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="79"/>
+    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Model" dataDxfId="78"/>
+    <tableColumn id="4" xr3:uid="{217066CA-63B7-4030-A7FC-54062BE2122E}" name="Manufacturer/Brand" dataDxfId="77"/>
+    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="76"/>
+    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="75"/>
+    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="74"/>
+    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="73"/>
+    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="72"/>
+    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="71"/>
+    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="70"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:I2" totalsRowShown="0" headerRowDxfId="56" dataDxfId="55">
-  <autoFilter ref="A1:I2" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:I2" totalsRowShown="0" headerRowDxfId="69" dataDxfId="68">
+  <autoFilter ref="A1:I2" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="54"/>
-    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="53"/>
-    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Model" dataDxfId="52"/>
-    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="51"/>
-    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="50"/>
-    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="49"/>
-    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="48"/>
-    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="47"/>
-    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="46"/>
+    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="67"/>
+    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="66"/>
+    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="65"/>
+    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="64"/>
+    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="63"/>
+    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="62"/>
+    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="61"/>
+    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="60"/>
+    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="59"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:H2" totalsRowShown="0" headerRowDxfId="45" dataDxfId="44">
-  <autoFilter ref="A1:H2" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}"/>
-  <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="43"/>
-    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="42"/>
-    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Model" dataDxfId="41"/>
-    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="40"/>
-    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="39"/>
-    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="38"/>
-    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="37"/>
-    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="36"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:I2" totalsRowShown="0" headerRowDxfId="58" dataDxfId="57">
+  <autoFilter ref="A1:I2" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}"/>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="56"/>
+    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="55"/>
+    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Model" dataDxfId="54"/>
+    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="53"/>
+    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="52"/>
+    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="51"/>
+    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="50"/>
+    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="49"/>
+    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="48"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:K2" totalsRowShown="0" headerRowDxfId="35" dataDxfId="34">
-  <autoFilter ref="A1:K2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
-  <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="33"/>
-    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="32"/>
-    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="31"/>
-    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="30"/>
-    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="29"/>
-    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="28"/>
-    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="27"/>
-    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="26"/>
-    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="25">
-      <calculatedColumnFormula>Shop_Consumables[[#This Row],[Current Stock]]*Shop_Consumables[[#This Row],[Unit Cost]]</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="24"/>
-    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Preferred Supplier" dataDxfId="23"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:H2" totalsRowShown="0" headerRowDxfId="47" dataDxfId="46">
+  <autoFilter ref="A1:H2" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="45"/>
+    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="44"/>
+    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Model" dataDxfId="43"/>
+    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="42"/>
+    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="41"/>
+    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="40"/>
+    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="39"/>
+    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="38"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1511,6 +1534,79 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E1902F1-C59B-4A1A-9D95-2C39AEF944E5}">
+  <sheetPr codeName="Sheet7"/>
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="9" style="1" customWidth="1"/>
+    <col min="2" max="2" width="41.6640625" style="2" customWidth="1"/>
+    <col min="3" max="4" width="18.44140625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="15.5546875" style="2" customWidth="1"/>
+    <col min="6" max="6" width="14.33203125" style="7" customWidth="1"/>
+    <col min="7" max="7" width="14.109375" style="7" customWidth="1"/>
+    <col min="8" max="8" width="10.44140625" style="3" customWidth="1"/>
+    <col min="9" max="9" width="22.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22.6640625" style="2" customWidth="1"/>
+    <col min="11" max="11" width="46.6640625" style="2" customWidth="1"/>
+    <col min="12" max="16384" width="8.88671875" style="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="I2" s="3">
+        <f>Shop_Consumables[[#This Row],[Current Stock]]*Shop_Consumables[[#This Row],[Unit Cost]]</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2" xr:uid="{D2C605E8-D02B-4558-82DE-3169088704E8}">
+      <formula1>"Fasteners/Hardware,Abrasives/Cutting,Fluids/Lubricants/Chemicals,Primer/Paint,Safety/PPE,Shop/Janitorial,Welding,Electrical,Other"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3185D484-1AEA-488F-ADB2-C66611F8B5C9}">
   <sheetPr codeName="Sheet8"/>
   <dimension ref="A1:G1"/>
@@ -1571,7 +1667,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6150BED1-88FC-488E-B7E1-4C6CBEB9589C}">
   <sheetPr codeName="Sheet9"/>
   <dimension ref="A1:G1"/>
@@ -1617,7 +1713,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6A08BCD-5A8C-45EE-A940-2FEFA1E5B102}">
   <dimension ref="A1:E1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1797,6 +1893,37 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E53ED58-AF1A-4384-BD5D-DFB0D7D062C9}">
+  <dimension ref="A9:B10"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="17.44140625" style="4" customWidth="1"/>
+    <col min="2" max="2" width="13" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B10" s="5">
+        <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDE7BF89-A2E7-4A6F-B822-317739E206EC}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:M2"/>
@@ -1885,7 +2012,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B027EC69-551F-4051-8A71-8B106D207C6D}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:K1"/>
@@ -1955,7 +2082,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB7AACC4-9DA2-4A53-AD77-8C5E0C1BF474}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:I1"/>
@@ -2021,7 +2148,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEDDDAA7-75C3-4AA5-ABFD-D5FB4C627E4C}">
   <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:I1"/>
@@ -2097,7 +2224,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F39ADDA6-CD5F-4655-A9C0-9676DDAC362E}">
   <sheetPr codeName="Sheet6"/>
   <dimension ref="A1:H1"/>
@@ -2157,77 +2284,4 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E1902F1-C59B-4A1A-9D95-2C39AEF944E5}">
-  <sheetPr codeName="Sheet7"/>
-  <dimension ref="A1:K2"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="9" style="1" customWidth="1"/>
-    <col min="2" max="2" width="41.6640625" style="2" customWidth="1"/>
-    <col min="3" max="4" width="18.44140625" style="2" customWidth="1"/>
-    <col min="5" max="5" width="15.5546875" style="2" customWidth="1"/>
-    <col min="6" max="6" width="14.33203125" style="7" customWidth="1"/>
-    <col min="7" max="7" width="14.109375" style="7" customWidth="1"/>
-    <col min="8" max="8" width="10.44140625" style="3" customWidth="1"/>
-    <col min="9" max="9" width="22.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="22.6640625" style="2" customWidth="1"/>
-    <col min="11" max="11" width="46.6640625" style="2" customWidth="1"/>
-    <col min="12" max="16384" width="8.88671875" style="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="I2" s="3">
-        <f>Shop_Consumables[[#This Row],[Current Stock]]*Shop_Consumables[[#This Row],[Unit Cost]]</f>
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2" xr:uid="{D2C605E8-D02B-4558-82DE-3169088704E8}">
-      <formula1>"Fasteners/Hardware,Abrasives/Cutting,Fluids/Lubricants/Chemicals,Primer/Paint,Safety/PPE,Shop/Janitorial,Welding,Electrical,Other"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
in Excel added rows to table  Overhead_Summary, header: Expense Category to pre-populate the rows for the dropdown items to support creating a bar chart
</commit_message>
<xml_diff>
--- a/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
+++ b/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1a2ae81d67634e6/Desktop/Michanikos Artifex Enterprises/MAE Custom Digital Solutions/MAE Workshop Inventory Management System/GITHUB_MAE_Workshop Inventory App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD064C17-0AAC-40F7-A2B6-B50A57BE904F}"/>
+  <xr:revisionPtr revIDLastSave="39" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8DDDCEF0-EDD9-474C-93D2-3E6F966A0FB5}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="10740" firstSheet="2" activeTab="3" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="3" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
   </bookViews>
   <sheets>
     <sheet name="TEST Inventory" sheetId="10" r:id="rId1"/>
@@ -70,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="91">
   <si>
     <t>mae_id</t>
   </si>
@@ -307,6 +307,42 @@
   </si>
   <si>
     <t>Annual Total</t>
+  </si>
+  <si>
+    <t>Facility Costs/Rent/Mortgage</t>
+  </si>
+  <si>
+    <t>Insurance</t>
+  </si>
+  <si>
+    <t>Debt/Leases on Equipment/Business Loans</t>
+  </si>
+  <si>
+    <t>Subscriptions</t>
+  </si>
+  <si>
+    <t>Salaries</t>
+  </si>
+  <si>
+    <t>Utilities</t>
+  </si>
+  <si>
+    <t>Maintnance/Repair</t>
+  </si>
+  <si>
+    <t>Marketing/Advertising</t>
+  </si>
+  <si>
+    <t>Professional Fees</t>
+  </si>
+  <si>
+    <t>Travel/Vehicles</t>
+  </si>
+  <si>
+    <t>Depreciation</t>
+  </si>
+  <si>
+    <t>Other/Miscellaneous</t>
   </si>
 </sst>
 </file>
@@ -394,12 +430,6 @@
   </cellStyles>
   <dxfs count="118">
     <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
@@ -754,28 +784,6 @@
     </dxf>
     <dxf>
       <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
@@ -840,6 +848,34 @@
     <dxf>
       <protection locked="1" hidden="0"/>
     </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -853,15 +889,19 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}" name="TEST_Inventory" displayName="TEST_Inventory" ref="A1:F5" totalsRowShown="0">
   <autoFilter ref="A1:F5" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="104"/>
-    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="103"/>
-    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="102"/>
-    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="101"/>
-    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="100">
+    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="115"/>
+    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="114"/>
+    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="113"/>
+    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="112"/>
+    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="111">
       <calculatedColumnFormula>TEST_Inventory[[#This Row],[TEST Integer]]*TEST_Inventory[[#This Row],[TEST Currency]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{AB3A5F3C-FCF0-4466-90FD-8ABB6E18DF5C}" name="TEST Dropdown"/>
@@ -871,54 +911,54 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:K2" totalsRowShown="0" headerRowDxfId="37" dataDxfId="36">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:K2" totalsRowShown="0" headerRowDxfId="35" dataDxfId="34">
   <autoFilter ref="A1:K2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="35"/>
-    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="34"/>
-    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="33"/>
-    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="32"/>
-    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="31"/>
-    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="30"/>
-    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="29"/>
-    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="28"/>
-    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="27">
+    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="33"/>
+    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="32"/>
+    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="31"/>
+    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="30"/>
+    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="29"/>
+    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="28"/>
+    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="27"/>
+    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="26"/>
+    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="25">
       <calculatedColumnFormula>Shop_Consumables[[#This Row],[Current Stock]]*Shop_Consumables[[#This Row],[Unit Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="26"/>
-    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Preferred Supplier" dataDxfId="25"/>
+    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="24"/>
+    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Preferred Supplier" dataDxfId="23"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:G2" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:G2" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
   <autoFilter ref="A1:G2" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="22"/>
-    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="21"/>
-    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="20"/>
-    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="19"/>
-    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="18"/>
-    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="17"/>
-    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="16"/>
+    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="18"/>
+    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="17"/>
+    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="16"/>
+    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="15"/>
+    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
   <autoFilter ref="A1:G2" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="13"/>
-    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="11"/>
-    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="10"/>
-    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="9"/>
-    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="8"/>
-    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="7"/>
+    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="11"/>
+    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="9"/>
+    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="7"/>
+    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="6"/>
+    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -928,11 +968,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}" name="Location" displayName="Location" ref="A1:E2" insertRow="1" totalsRowShown="0">
   <autoFilter ref="A1:E2" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Name" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Name" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -942,10 +982,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}" name="TEST_Dashboard" displayName="TEST_Dashboard" ref="A1:B2" totalsRowShown="0">
   <autoFilter ref="A1:B2" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="99">
+    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="110">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Currency])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="98">
+    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="109">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Integer])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -954,38 +994,38 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:K2" totalsRowShown="0" headerRowDxfId="117" dataDxfId="116">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:K2" totalsRowShown="0" headerRowDxfId="108" dataDxfId="107">
   <autoFilter ref="A1:K2" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="115"/>
-    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="114">
+    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="106"/>
+    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="105">
       <calculatedColumnFormula>SUM(Resell_Inventory[Total Investment])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="113">
+    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="104">
       <calculatedColumnFormula>SUM(Resell_Inventory[Actual Sale Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="112">
+    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="103">
       <calculatedColumnFormula>SUM(Shop_Machinery[Purchase Cost])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="111">
+    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="102">
       <calculatedColumnFormula>SUM(Shop_Power_Tools[Purchase Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="110">
+    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="101">
       <calculatedColumnFormula>SUM(Shop_Hand_Tools[Purchase Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="109">
+    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="100">
       <calculatedColumnFormula>SUM(Shop_Consumables[Current Inventory Value])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="108">
+    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="99">
       <calculatedColumnFormula>SUM(D2,E2,F2,G2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="107">
+    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="98">
       <calculatedColumnFormula array="1">SUMPRODUCT(--(Shop_Consumables[Current Stock]&lt;=Shop_Consumables[Reorder Point]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="106">
+    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="97">
       <calculatedColumnFormula>SUMIFS(Shop_Overhead[Amount], Shop_Overhead[Due Date], "&lt;="&amp;TODAY()+30, Shop_Overhead[Due Date], "&gt;="&amp;TODAY())</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{86A5DBCB-1064-4926-8405-405B453A4546}" name="Equipment Needing Repair" dataDxfId="105">
+    <tableColumn id="6" xr3:uid="{86A5DBCB-1064-4926-8405-405B453A4546}" name="Equipment Needing Repair" dataDxfId="96">
       <calculatedColumnFormula>COUNTIFS(Shop_Machinery[Condition], "Needs Repair") + COUNTIFS(Shop_Power_Tools[Condition], "Needs Repair") + COUNTIFS(Shop_Hand_Tools[Condition], "Needs Repair")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -994,11 +1034,11 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{F579DA07-7AD6-49DA-9B44-D5B1132EDAC6}" name="Overhead_Summary" displayName="Overhead_Summary" ref="A9:B10" totalsRowShown="0">
-  <autoFilter ref="A9:B10" xr:uid="{F579DA07-7AD6-49DA-9B44-D5B1132EDAC6}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{F579DA07-7AD6-49DA-9B44-D5B1132EDAC6}" name="Overhead_Summary" displayName="Overhead_Summary" ref="A9:B21" totalsRowShown="0">
+  <autoFilter ref="A9:B21" xr:uid="{F579DA07-7AD6-49DA-9B44-D5B1132EDAC6}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{7CA4839C-9603-479D-BD1C-8377DFA9603C}" name="Expense Category" dataDxfId="1"/>
-    <tableColumn id="2" xr3:uid="{FE0F7616-EAF3-443D-AC69-DE6541DC10E5}" name="Annual Total" dataDxfId="0">
+    <tableColumn id="1" xr3:uid="{7CA4839C-9603-479D-BD1C-8377DFA9603C}" name="Expense Category" dataDxfId="117"/>
+    <tableColumn id="2" xr3:uid="{FE0F7616-EAF3-443D-AC69-DE6541DC10E5}" name="Annual Total" dataDxfId="116">
       <calculatedColumnFormula>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1007,97 +1047,97 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:M2" totalsRowShown="0" headerRowDxfId="97" dataDxfId="96">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:M2" totalsRowShown="0" headerRowDxfId="95" dataDxfId="94">
   <autoFilter ref="A1:M2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="95"/>
-    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="94"/>
-    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="93"/>
-    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="92"/>
-    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="91"/>
-    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="90"/>
-    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="89"/>
-    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="88">
+    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="93"/>
+    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="92"/>
+    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="91"/>
+    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="90"/>
+    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="89"/>
+    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="88"/>
+    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="87"/>
+    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="86">
       <calculatedColumnFormula>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="87"/>
-    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="86"/>
-    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="85"/>
-    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="84"/>
-    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="83"/>
+    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="85"/>
+    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="84"/>
+    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="83"/>
+    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="82"/>
+    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="81"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="82" dataDxfId="81">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="80" dataDxfId="79">
   <autoFilter ref="A1:K2" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="80"/>
-    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="79"/>
-    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Model" dataDxfId="78"/>
-    <tableColumn id="4" xr3:uid="{217066CA-63B7-4030-A7FC-54062BE2122E}" name="Manufacturer/Brand" dataDxfId="77"/>
-    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="76"/>
-    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="75"/>
-    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="74"/>
-    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="73"/>
-    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="72"/>
-    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="71"/>
-    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="70"/>
+    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="78"/>
+    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="77"/>
+    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Model" dataDxfId="76"/>
+    <tableColumn id="4" xr3:uid="{217066CA-63B7-4030-A7FC-54062BE2122E}" name="Manufacturer/Brand" dataDxfId="75"/>
+    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="74"/>
+    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="73"/>
+    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="72"/>
+    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="71"/>
+    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="70"/>
+    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="69"/>
+    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="68"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:I2" totalsRowShown="0" headerRowDxfId="69" dataDxfId="68">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:I2" totalsRowShown="0" headerRowDxfId="67" dataDxfId="66">
   <autoFilter ref="A1:I2" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="67"/>
-    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="66"/>
-    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="65"/>
-    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="64"/>
-    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="63"/>
-    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="62"/>
-    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="61"/>
-    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="60"/>
-    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="59"/>
+    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="65"/>
+    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="64"/>
+    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="63"/>
+    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="62"/>
+    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="61"/>
+    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="60"/>
+    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="59"/>
+    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="58"/>
+    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="57"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:I2" totalsRowShown="0" headerRowDxfId="58" dataDxfId="57">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:I2" totalsRowShown="0" headerRowDxfId="56" dataDxfId="55">
   <autoFilter ref="A1:I2" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="56"/>
-    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="55"/>
-    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Model" dataDxfId="54"/>
-    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="53"/>
-    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="52"/>
-    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="51"/>
-    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="50"/>
-    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="49"/>
-    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="48"/>
+    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="54"/>
+    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="53"/>
+    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Model" dataDxfId="52"/>
+    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="51"/>
+    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="50"/>
+    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="49"/>
+    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="48"/>
+    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="47"/>
+    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="46"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:H2" totalsRowShown="0" headerRowDxfId="47" dataDxfId="46">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:H2" totalsRowShown="0" headerRowDxfId="45" dataDxfId="44">
   <autoFilter ref="A1:H2" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="45"/>
-    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="44"/>
-    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Model" dataDxfId="43"/>
-    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="42"/>
-    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="41"/>
-    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="40"/>
-    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="39"/>
-    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="38"/>
+    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="43"/>
+    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="42"/>
+    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Model" dataDxfId="41"/>
+    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="40"/>
+    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="39"/>
+    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="38"/>
+    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="37"/>
+    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="36"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1894,11 +1934,11 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E53ED58-AF1A-4384-BD5D-DFB0D7D062C9}">
-  <dimension ref="A9:B10"/>
+  <dimension ref="A9:B21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.44140625" style="4" customWidth="1"/>
-    <col min="2" max="2" width="13" style="5" customWidth="1"/>
+    <col min="1" max="1" width="42.21875" style="4" customWidth="1"/>
+    <col min="2" max="2" width="17.5546875" style="5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
@@ -1910,12 +1950,119 @@
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>79</v>
+      </c>
       <c r="B10" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
         <v>0</v>
       </c>
     </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B11" s="5">
+        <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B12" s="5">
+        <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B13" s="5">
+        <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B14" s="5">
+        <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B15" s="5">
+        <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B16" s="5">
+        <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B17" s="5">
+        <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B18" s="5">
+        <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B19" s="5">
+        <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B20" s="5">
+        <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B21" s="5">
+        <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A10:A21" xr:uid="{5D203998-8919-42E9-9815-48F6851487A8}">
+      <formula1>"Facility Costs/Rent/Mortgage,Insurance,Debt/Leases on Equipment/Business Loans,Subscriptions,Salaries,Utilities,Maintnance/Repair,Marketing/Advertising,Professional Fees,Travel/Vehicles,Depreciation,Other/Miscellaneous"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>

<commit_message>
adjusted config.js and Excel files to modify REPAIRS NEEDED card, changed header in Master Dashboard table and modified formula
</commit_message>
<xml_diff>
--- a/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
+++ b/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1a2ae81d67634e6/Desktop/Michanikos Artifex Enterprises/MAE Custom Digital Solutions/MAE Workshop Inventory Management System/GITHUB_MAE_Workshop Inventory App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="39" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8DDDCEF0-EDD9-474C-93D2-3E6F966A0FB5}"/>
+  <xr:revisionPtr revIDLastSave="43" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BEABFFD0-A58D-4212-9E38-85E81197F3AD}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="3" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
+    <workbookView xWindow="336" yWindow="492" windowWidth="19560" windowHeight="11904" firstSheet="2" activeTab="2" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
   </bookViews>
   <sheets>
     <sheet name="TEST Inventory" sheetId="10" r:id="rId1"/>
@@ -288,9 +288,6 @@
     <t>Low Stock Items Count</t>
   </si>
   <si>
-    <t>Equipment Needing Repair</t>
-  </si>
-  <si>
     <t>Total Machinery Value</t>
   </si>
   <si>
@@ -343,6 +340,9 @@
   </si>
   <si>
     <t>Other/Miscellaneous</t>
+  </si>
+  <si>
+    <t>Equipment With Operational Issues</t>
   </si>
 </sst>
 </file>
@@ -1025,8 +1025,12 @@
     <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="97">
       <calculatedColumnFormula>SUMIFS(Shop_Overhead[Amount], Shop_Overhead[Due Date], "&lt;="&amp;TODAY()+30, Shop_Overhead[Due Date], "&gt;="&amp;TODAY())</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{86A5DBCB-1064-4926-8405-405B453A4546}" name="Equipment Needing Repair" dataDxfId="96">
-      <calculatedColumnFormula>COUNTIFS(Shop_Machinery[Condition], "Needs Repair") + COUNTIFS(Shop_Power_Tools[Condition], "Needs Repair") + COUNTIFS(Shop_Hand_Tools[Condition], "Needs Repair")</calculatedColumnFormula>
+    <tableColumn id="6" xr3:uid="{86A5DBCB-1064-4926-8405-405B453A4546}" name="Equipment With Operational Issues" dataDxfId="96">
+      <calculatedColumnFormula array="1">SUM(
+  COUNTIFS(Shop_Machinery[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"}),
+  COUNTIFS(Shop_Power_Tools[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"}),
+  COUNTIFS(Shop_Hand_Tools[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"})
+)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1841,7 +1845,7 @@
     <col min="8" max="8" width="22" style="3" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="22.109375" style="12" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="29" style="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="25.6640625" style="7" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="32.88671875" style="7" bestFit="1" customWidth="1"/>
     <col min="12" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
@@ -1856,16 +1860,16 @@
         <v>69</v>
       </c>
       <c r="D1" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="G1" s="5" t="s">
         <v>74</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>75</v>
       </c>
       <c r="H1" s="5" t="s">
         <v>70</v>
@@ -1874,10 +1878,10 @@
         <v>71</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="K1" s="8" t="s">
-        <v>72</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
@@ -1917,8 +1921,12 @@
         <f ca="1">SUMIFS(Shop_Overhead[Amount], Shop_Overhead[Due Date], "&lt;="&amp;TODAY()+30, Shop_Overhead[Due Date], "&gt;="&amp;TODAY())</f>
         <v>0</v>
       </c>
-      <c r="K2" s="7">
-        <f>COUNTIFS(Shop_Machinery[Condition], "Needs Repair") + COUNTIFS(Shop_Power_Tools[Condition], "Needs Repair") + COUNTIFS(Shop_Hand_Tools[Condition], "Needs Repair")</f>
+      <c r="K2" s="7" cm="1">
+        <f t="array" ref="K2">SUM(
+  COUNTIFS(Shop_Machinery[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"}),
+  COUNTIFS(Shop_Power_Tools[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"}),
+  COUNTIFS(Shop_Hand_Tools[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"})
+)</f>
         <v>0</v>
       </c>
     </row>
@@ -1946,12 +1954,12 @@
         <v>31</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B10" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -1960,7 +1968,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B11" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -1969,7 +1977,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B12" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -1978,7 +1986,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B13" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -1987,7 +1995,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B14" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -1996,7 +2004,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B15" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2005,7 +2013,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B16" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2014,7 +2022,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B17" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2023,7 +2031,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B18" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2032,7 +2040,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B19" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2041,7 +2049,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B20" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2050,7 +2058,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B21" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>

</xml_diff>

<commit_message>
added header to Master Dashboard for Shop Maintenance card (config and Excel)
</commit_message>
<xml_diff>
--- a/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
+++ b/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1a2ae81d67634e6/Desktop/Michanikos Artifex Enterprises/MAE Custom Digital Solutions/MAE Workshop Inventory Management System/GITHUB_MAE_Workshop Inventory App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="44" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9905A512-ACB8-47C8-9AD8-3BB2AAD9C911}"/>
+  <xr:revisionPtr revIDLastSave="50" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{500E71F6-AF5A-46F6-8554-36A5F3630222}"/>
   <bookViews>
-    <workbookView xWindow="3540" yWindow="1788" windowWidth="19560" windowHeight="11904" firstSheet="2" activeTab="2" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
+    <workbookView xWindow="11256" yWindow="108" windowWidth="11844" windowHeight="11904" firstSheet="2" activeTab="2" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
   </bookViews>
   <sheets>
     <sheet name="TEST Inventory" sheetId="10" r:id="rId1"/>
@@ -70,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="92">
   <si>
     <t>mae_id</t>
   </si>
@@ -343,6 +343,9 @@
   </si>
   <si>
     <t>Equipment With Operational Issues</t>
+  </si>
+  <si>
+    <t>Maintenance Items Due in Next 30 Days</t>
   </si>
 </sst>
 </file>
@@ -393,7 +396,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
       <protection hidden="1"/>
@@ -424,11 +427,20 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="118">
+  <dxfs count="119">
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
@@ -786,8 +798,32 @@
       <protection locked="1" hidden="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
@@ -848,34 +884,6 @@
     <dxf>
       <protection locked="1" hidden="0"/>
     </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -889,19 +897,15 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}" name="TEST_Inventory" displayName="TEST_Inventory" ref="A1:F5" totalsRowShown="0">
   <autoFilter ref="A1:F5" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="115"/>
-    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="114"/>
-    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="113"/>
-    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="112"/>
-    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="111">
+    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="106"/>
+    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="105"/>
+    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="104"/>
+    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="103"/>
+    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="102">
       <calculatedColumnFormula>TEST_Inventory[[#This Row],[TEST Integer]]*TEST_Inventory[[#This Row],[TEST Currency]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{AB3A5F3C-FCF0-4466-90FD-8ABB6E18DF5C}" name="TEST Dropdown"/>
@@ -911,54 +915,54 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:K2" totalsRowShown="0" headerRowDxfId="35" dataDxfId="34">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:K2" totalsRowShown="0" headerRowDxfId="37" dataDxfId="36">
   <autoFilter ref="A1:K2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="33"/>
-    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="32"/>
-    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="31"/>
-    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="30"/>
-    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="29"/>
-    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="28"/>
-    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="27"/>
-    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="26"/>
-    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="25">
+    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="35"/>
+    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="34"/>
+    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="33"/>
+    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="32"/>
+    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="31"/>
+    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="30"/>
+    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="29"/>
+    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="28"/>
+    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="27">
       <calculatedColumnFormula>Shop_Consumables[[#This Row],[Current Stock]]*Shop_Consumables[[#This Row],[Unit Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="24"/>
-    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Preferred Supplier" dataDxfId="23"/>
+    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="26"/>
+    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Preferred Supplier" dataDxfId="25"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:G2" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:G2" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23">
   <autoFilter ref="A1:G2" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="20"/>
-    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="19"/>
-    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="18"/>
-    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="17"/>
-    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="16"/>
-    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="15"/>
-    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="14"/>
+    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="22"/>
+    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="20"/>
+    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="18"/>
+    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="17"/>
+    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
   <autoFilter ref="A1:G2" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="11"/>
-    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="9"/>
-    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="7"/>
-    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="6"/>
-    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="13"/>
+    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="11"/>
+    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="9"/>
+    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="8"/>
+    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -968,11 +972,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}" name="Location" displayName="Location" ref="A1:E2" insertRow="1" totalsRowShown="0">
   <autoFilter ref="A1:E2" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Name" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Name" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -982,10 +986,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}" name="TEST_Dashboard" displayName="TEST_Dashboard" ref="A1:B2" totalsRowShown="0">
   <autoFilter ref="A1:B2" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="110">
+    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="101">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Currency])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="109">
+    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="100">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Integer])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -994,44 +998,49 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:K2" totalsRowShown="0" headerRowDxfId="108" dataDxfId="107">
-  <autoFilter ref="A1:K2" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}"/>
-  <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="106"/>
-    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="105">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:L2" totalsRowShown="0" headerRowDxfId="118" dataDxfId="117">
+  <autoFilter ref="A1:L2" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}"/>
+  <tableColumns count="12">
+    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="116"/>
+    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="115">
       <calculatedColumnFormula>SUM(Resell_Inventory[Total Investment])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="104">
+    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="114">
       <calculatedColumnFormula>SUM(Resell_Inventory[Actual Sale Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="103">
+    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="113">
       <calculatedColumnFormula>SUM(Shop_Machinery[Purchase Cost])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="102">
+    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="112">
       <calculatedColumnFormula>SUM(Shop_Power_Tools[Purchase Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="101">
+    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="111">
       <calculatedColumnFormula>SUM(Shop_Hand_Tools[Purchase Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="100">
+    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="110">
       <calculatedColumnFormula>SUM(Shop_Consumables[Current Inventory Value])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="99">
+    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="109">
       <calculatedColumnFormula>SUM(D2,E2,F2,G2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="98">
+    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="108">
       <calculatedColumnFormula array="1">SUMPRODUCT(--(Shop_Consumables[Current Stock]&lt;=Shop_Consumables[Reorder Point]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="97">
+    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="107">
       <calculatedColumnFormula>SUMIFS(Shop_Overhead[Amount], Shop_Overhead[Due Date], "&lt;="&amp;TODAY()+30, Shop_Overhead[Due Date], "&gt;="&amp;TODAY())</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{86A5DBCB-1064-4926-8405-405B453A4546}" name="Equipment With Operational Issues" dataDxfId="96">
+    <tableColumn id="12" xr3:uid="{E4065760-B1B1-4564-936B-3405D3B80297}" name="Equipment With Operational Issues" dataDxfId="0">
       <calculatedColumnFormula array="1">SUM(
   COUNTIFS(Shop_Machinery[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"}),
   COUNTIFS(Shop_Power_Tools[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"}),
   COUNTIFS(Shop_Hand_Tools[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"})
 )</calculatedColumnFormula>
     </tableColumn>
+    <tableColumn id="6" xr3:uid="{86A5DBCB-1064-4926-8405-405B453A4546}" name="Maintenance Items Due in Next 30 Days" dataDxfId="1">
+      <calculatedColumnFormula>SUM(
+            COUNTIFS(Maintenance_Log[Next Service Date], "&lt;="&amp;TODAY()+30, Maintenance_Log[Next Service Date], "&gt;="&amp;TODAY())
+        )</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1041,8 +1050,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{F579DA07-7AD6-49DA-9B44-D5B1132EDAC6}" name="Overhead_Summary" displayName="Overhead_Summary" ref="A9:B21" totalsRowShown="0">
   <autoFilter ref="A9:B21" xr:uid="{F579DA07-7AD6-49DA-9B44-D5B1132EDAC6}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{7CA4839C-9603-479D-BD1C-8377DFA9603C}" name="Expense Category" dataDxfId="117"/>
-    <tableColumn id="2" xr3:uid="{FE0F7616-EAF3-443D-AC69-DE6541DC10E5}" name="Annual Total" dataDxfId="116">
+    <tableColumn id="1" xr3:uid="{7CA4839C-9603-479D-BD1C-8377DFA9603C}" name="Expense Category" dataDxfId="99"/>
+    <tableColumn id="2" xr3:uid="{FE0F7616-EAF3-443D-AC69-DE6541DC10E5}" name="Annual Total" dataDxfId="98">
       <calculatedColumnFormula>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1051,97 +1060,97 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:M2" totalsRowShown="0" headerRowDxfId="95" dataDxfId="94">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:M2" totalsRowShown="0" headerRowDxfId="97" dataDxfId="96">
   <autoFilter ref="A1:M2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="93"/>
-    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="92"/>
-    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="91"/>
-    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="90"/>
-    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="89"/>
-    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="88"/>
-    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="87"/>
-    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="86">
+    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="95"/>
+    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="94"/>
+    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="93"/>
+    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="92"/>
+    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="91"/>
+    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="90"/>
+    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="89"/>
+    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="88">
       <calculatedColumnFormula>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="85"/>
-    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="84"/>
-    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="83"/>
-    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="82"/>
-    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="81"/>
+    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="87"/>
+    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="86"/>
+    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="85"/>
+    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="84"/>
+    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="83"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="80" dataDxfId="79">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="82" dataDxfId="81">
   <autoFilter ref="A1:K2" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="78"/>
-    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="77"/>
-    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Model" dataDxfId="76"/>
-    <tableColumn id="4" xr3:uid="{217066CA-63B7-4030-A7FC-54062BE2122E}" name="Manufacturer/Brand" dataDxfId="75"/>
-    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="74"/>
-    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="73"/>
-    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="72"/>
-    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="71"/>
-    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="70"/>
-    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="69"/>
-    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="68"/>
+    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="80"/>
+    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="79"/>
+    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Model" dataDxfId="78"/>
+    <tableColumn id="4" xr3:uid="{217066CA-63B7-4030-A7FC-54062BE2122E}" name="Manufacturer/Brand" dataDxfId="77"/>
+    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="76"/>
+    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="75"/>
+    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="74"/>
+    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="73"/>
+    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="72"/>
+    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="71"/>
+    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="70"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:I2" totalsRowShown="0" headerRowDxfId="67" dataDxfId="66">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:I2" totalsRowShown="0" headerRowDxfId="69" dataDxfId="68">
   <autoFilter ref="A1:I2" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="65"/>
-    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="64"/>
-    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="63"/>
-    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="62"/>
-    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="61"/>
-    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="60"/>
-    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="59"/>
-    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="58"/>
-    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="57"/>
+    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="67"/>
+    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="66"/>
+    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="65"/>
+    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="64"/>
+    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="63"/>
+    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="62"/>
+    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="61"/>
+    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="60"/>
+    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="59"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:I2" totalsRowShown="0" headerRowDxfId="56" dataDxfId="55">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:I2" totalsRowShown="0" headerRowDxfId="58" dataDxfId="57">
   <autoFilter ref="A1:I2" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="54"/>
-    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="53"/>
-    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Model" dataDxfId="52"/>
-    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="51"/>
-    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="50"/>
-    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="49"/>
-    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="48"/>
-    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="47"/>
-    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="46"/>
+    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="56"/>
+    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="55"/>
+    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Model" dataDxfId="54"/>
+    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="53"/>
+    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="52"/>
+    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="51"/>
+    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="50"/>
+    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="49"/>
+    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="48"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:H2" totalsRowShown="0" headerRowDxfId="45" dataDxfId="44">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:H2" totalsRowShown="0" headerRowDxfId="47" dataDxfId="46">
   <autoFilter ref="A1:H2" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="43"/>
-    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="42"/>
-    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Model" dataDxfId="41"/>
-    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="40"/>
-    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="39"/>
-    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="38"/>
-    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="37"/>
-    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="36"/>
+    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="45"/>
+    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="44"/>
+    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Model" dataDxfId="43"/>
+    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="42"/>
+    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="41"/>
+    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="40"/>
+    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="39"/>
+    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="38"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1832,7 +1841,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2834D935-E140-4D64-A4CD-4A9FB8899FE0}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
@@ -1845,11 +1854,12 @@
     <col min="8" max="8" width="22" style="3" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="22.109375" style="12" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="29" style="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="32.88671875" style="7" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="8.88671875" style="6"/>
+    <col min="11" max="11" width="32.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="32.88671875" style="7" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1883,8 +1893,11 @@
       <c r="K1" s="8" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L1" s="14" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B2" s="3">
         <f>SUM(Resell_Inventory[Total Investment])</f>
         <v>0</v>
@@ -1927,6 +1940,12 @@
   COUNTIFS(Shop_Power_Tools[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"}),
   COUNTIFS(Shop_Hand_Tools[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"})
 )</f>
+        <v>0</v>
+      </c>
+      <c r="L2" s="7">
+        <f ca="1">SUM(
+            COUNTIFS(Maintenance_Log[Next Service Date], "&lt;="&amp;TODAY()+30, Maintenance_Log[Next Service Date], "&gt;="&amp;TODAY())
+        )</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
updated to config file V 1.5 and excel
</commit_message>
<xml_diff>
--- a/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
+++ b/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1a2ae81d67634e6/Desktop/Michanikos Artifex Enterprises/MAE Custom Digital Solutions/MAE Workshop Inventory Management System/GITHUB_MAE_Workshop Inventory App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="50" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{500E71F6-AF5A-46F6-8554-36A5F3630222}"/>
+  <xr:revisionPtr revIDLastSave="106" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D50FE1C8-7BFF-4F9F-9762-07638FF6C09D}"/>
   <bookViews>
-    <workbookView xWindow="11256" yWindow="108" windowWidth="11844" windowHeight="11904" firstSheet="2" activeTab="2" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
+    <workbookView xWindow="11136" yWindow="132" windowWidth="11844" windowHeight="11904" firstSheet="9" activeTab="10" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
   </bookViews>
   <sheets>
     <sheet name="TEST Inventory" sheetId="10" r:id="rId1"/>
@@ -70,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="95">
   <si>
     <t>mae_id</t>
   </si>
@@ -108,12 +108,6 @@
     <t>Location</t>
   </si>
   <si>
-    <t>Machine Name/Model</t>
-  </si>
-  <si>
-    <t>Manufacturer/Brand</t>
-  </si>
-  <si>
     <t>Serial Number</t>
   </si>
   <si>
@@ -141,9 +135,6 @@
     <t>Next Service Date</t>
   </si>
   <si>
-    <t>Tool Name/Model</t>
-  </si>
-  <si>
     <t>Condition</t>
   </si>
   <si>
@@ -162,9 +153,6 @@
     <t>Unit Cost</t>
   </si>
   <si>
-    <t>Preferred Supplier</t>
-  </si>
-  <si>
     <t>Expense Category</t>
   </si>
   <si>
@@ -346,6 +334,27 @@
   </si>
   <si>
     <t>Maintenance Items Due in Next 30 Days</t>
+  </si>
+  <si>
+    <t>Sold</t>
+  </si>
+  <si>
+    <t>Machine Name/Brand/Model</t>
+  </si>
+  <si>
+    <t>Complete</t>
+  </si>
+  <si>
+    <t>Remarks</t>
+  </si>
+  <si>
+    <t>Tool Name/Brand/Model</t>
+  </si>
+  <si>
+    <t>Tool Name/Brand/Model/Description</t>
+  </si>
+  <si>
+    <t>Supplier/Remarks</t>
   </si>
 </sst>
 </file>
@@ -396,7 +405,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
       <protection hidden="1"/>
@@ -427,12 +436,201 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
+      <protection locked="0"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
+      <protection locked="0"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="119">
+  <dxfs count="124">
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
       <protection locked="0" hidden="0"/>
@@ -443,34 +641,43 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -482,6 +689,36 @@
       <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="1" hidden="1"/>
     </dxf>
@@ -492,7 +729,7 @@
       <protection locked="1" hidden="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -500,6 +737,12 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
       <protection locked="0" hidden="0"/>
     </dxf>
@@ -509,14 +752,6 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
@@ -530,6 +765,13 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="0"/>
     </dxf>
@@ -538,23 +780,7 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -574,174 +800,6 @@
     </dxf>
     <dxf>
       <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -785,10 +843,6 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
@@ -824,6 +878,14 @@
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
@@ -897,15 +959,41 @@
 </styleSheet>
 </file>
 
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<FeaturePropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <bag type="Checkbox"/>
+  <bag type="XFControls">
+    <bagId k="CellControl">0</bagId>
+  </bag>
+  <bag type="XFComplement">
+    <bagId k="XFControls">1</bagId>
+  </bag>
+  <bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <a k="MappedFeaturePropertyBags">
+      <bagId>2</bagId>
+    </a>
+  </bag>
+  <bag type="DXFComplements" extRef="DXFComplementsMapperExtRef">
+    <a k="MappedFeaturePropertyBags">
+      <bagId>2</bagId>
+    </a>
+  </bag>
+</FeaturePropertyBags>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}" name="TEST_Inventory" displayName="TEST_Inventory" ref="A1:F5" totalsRowShown="0">
   <autoFilter ref="A1:F5" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="106"/>
-    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="105"/>
-    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="104"/>
-    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="103"/>
-    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="102">
+    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="109"/>
+    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="108"/>
+    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="107"/>
+    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="106"/>
+    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="105">
       <calculatedColumnFormula>TEST_Inventory[[#This Row],[TEST Integer]]*TEST_Inventory[[#This Row],[TEST Currency]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{AB3A5F3C-FCF0-4466-90FD-8ABB6E18DF5C}" name="TEST Dropdown"/>
@@ -915,54 +1003,55 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:K2" totalsRowShown="0" headerRowDxfId="37" dataDxfId="36">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:K2" totalsRowShown="0" headerRowDxfId="48" dataDxfId="47">
   <autoFilter ref="A1:K2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="35"/>
-    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="34"/>
-    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="33"/>
-    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="32"/>
-    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="31"/>
-    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="30"/>
-    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="29"/>
-    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="28"/>
-    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="27">
+    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="46"/>
+    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="45"/>
+    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="1"/>
+    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="44"/>
+    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="43"/>
+    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="42"/>
+    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="41"/>
+    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="40"/>
+    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="39">
       <calculatedColumnFormula>Shop_Consumables[[#This Row],[Current Stock]]*Shop_Consumables[[#This Row],[Unit Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="26"/>
-    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Preferred Supplier" dataDxfId="25"/>
+    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="38"/>
+    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Supplier/Remarks" dataDxfId="37"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:G2" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23">
-  <autoFilter ref="A1:G2" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}"/>
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="22"/>
-    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="21"/>
-    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="20"/>
-    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="19"/>
-    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="18"/>
-    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="17"/>
-    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="16"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:H2" totalsRowShown="0" headerRowDxfId="36" dataDxfId="35">
+  <autoFilter ref="A1:H2" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="34"/>
+    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="33"/>
+    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="32"/>
+    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="31"/>
+    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="30"/>
+    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="29"/>
+    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="28"/>
+    <tableColumn id="8" xr3:uid="{9140C4E8-CB9E-40BF-ABD9-13A971322B09}" name="Remarks" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26">
   <autoFilter ref="A1:G2" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="13"/>
-    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="11"/>
-    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="10"/>
-    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="9"/>
-    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="8"/>
-    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="7"/>
+    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="25"/>
+    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="24"/>
+    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="23"/>
+    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="22"/>
+    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="21"/>
+    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="20"/>
+    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="19"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -972,11 +1061,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}" name="Location" displayName="Location" ref="A1:E2" insertRow="1" totalsRowShown="0">
   <autoFilter ref="A1:E2" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Name" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="18"/>
+    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="17"/>
+    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Name" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -986,10 +1075,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}" name="TEST_Dashboard" displayName="TEST_Dashboard" ref="A1:B2" totalsRowShown="0">
   <autoFilter ref="A1:B2" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="101">
+    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="104">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Currency])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="100">
+    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="103">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Integer])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -998,45 +1087,45 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:L2" totalsRowShown="0" headerRowDxfId="118" dataDxfId="117">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:L2" totalsRowShown="0" headerRowDxfId="123" dataDxfId="122">
   <autoFilter ref="A1:L2" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="116"/>
-    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="115">
+    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="121"/>
+    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="120">
       <calculatedColumnFormula>SUM(Resell_Inventory[Total Investment])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="114">
+    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="119">
       <calculatedColumnFormula>SUM(Resell_Inventory[Actual Sale Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="113">
+    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="118">
       <calculatedColumnFormula>SUM(Shop_Machinery[Purchase Cost])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="112">
+    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="117">
       <calculatedColumnFormula>SUM(Shop_Power_Tools[Purchase Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="111">
+    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="116">
       <calculatedColumnFormula>SUM(Shop_Hand_Tools[Purchase Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="110">
+    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="115">
       <calculatedColumnFormula>SUM(Shop_Consumables[Current Inventory Value])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="109">
+    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="114">
       <calculatedColumnFormula>SUM(D2,E2,F2,G2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="108">
+    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="113">
       <calculatedColumnFormula array="1">SUMPRODUCT(--(Shop_Consumables[Current Stock]&lt;=Shop_Consumables[Reorder Point]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="107">
+    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="112">
       <calculatedColumnFormula>SUMIFS(Shop_Overhead[Amount], Shop_Overhead[Due Date], "&lt;="&amp;TODAY()+30, Shop_Overhead[Due Date], "&gt;="&amp;TODAY())</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{E4065760-B1B1-4564-936B-3405D3B80297}" name="Equipment With Operational Issues" dataDxfId="0">
+    <tableColumn id="12" xr3:uid="{E4065760-B1B1-4564-936B-3405D3B80297}" name="Equipment With Operational Issues" dataDxfId="111">
       <calculatedColumnFormula array="1">SUM(
   COUNTIFS(Shop_Machinery[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"}),
   COUNTIFS(Shop_Power_Tools[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"}),
   COUNTIFS(Shop_Hand_Tools[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"})
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{86A5DBCB-1064-4926-8405-405B453A4546}" name="Maintenance Items Due in Next 30 Days" dataDxfId="1">
+    <tableColumn id="6" xr3:uid="{86A5DBCB-1064-4926-8405-405B453A4546}" name="Maintenance Items Due in Next 30 Days" dataDxfId="110">
       <calculatedColumnFormula>SUM(
             COUNTIFS(Maintenance_Log[Next Service Date], "&lt;="&amp;TODAY()+30, Maintenance_Log[Next Service Date], "&gt;="&amp;TODAY())
         )</calculatedColumnFormula>
@@ -1050,8 +1139,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{F579DA07-7AD6-49DA-9B44-D5B1132EDAC6}" name="Overhead_Summary" displayName="Overhead_Summary" ref="A9:B21" totalsRowShown="0">
   <autoFilter ref="A9:B21" xr:uid="{F579DA07-7AD6-49DA-9B44-D5B1132EDAC6}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{7CA4839C-9603-479D-BD1C-8377DFA9603C}" name="Expense Category" dataDxfId="99"/>
-    <tableColumn id="2" xr3:uid="{FE0F7616-EAF3-443D-AC69-DE6541DC10E5}" name="Annual Total" dataDxfId="98">
+    <tableColumn id="1" xr3:uid="{7CA4839C-9603-479D-BD1C-8377DFA9603C}" name="Expense Category" dataDxfId="102"/>
+    <tableColumn id="2" xr3:uid="{FE0F7616-EAF3-443D-AC69-DE6541DC10E5}" name="Annual Total" dataDxfId="101">
       <calculatedColumnFormula>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1060,97 +1149,101 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:M2" totalsRowShown="0" headerRowDxfId="97" dataDxfId="96">
-  <autoFilter ref="A1:M2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}"/>
-  <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="95"/>
-    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="94"/>
-    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="93"/>
-    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="92"/>
-    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="91"/>
-    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="90"/>
-    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="89"/>
-    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="88">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:N2" totalsRowShown="0" headerRowDxfId="100" dataDxfId="99">
+  <autoFilter ref="A1:N2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}"/>
+  <tableColumns count="14">
+    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="98"/>
+    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="97"/>
+    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="96"/>
+    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="95"/>
+    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="94"/>
+    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="93"/>
+    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="92">
       <calculatedColumnFormula>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="87"/>
-    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="86"/>
-    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="85"/>
-    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="84"/>
-    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="83"/>
+    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="91"/>
+    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="90"/>
+    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="89"/>
+    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="11"/>
+    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="88"/>
+    <tableColumn id="13" xr3:uid="{885B08CA-5BC3-4FAA-B661-BE5CCBF87448}" name="Sold" dataDxfId="12"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="82" dataDxfId="81">
-  <autoFilter ref="A1:K2" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}"/>
-  <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="80"/>
-    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="79"/>
-    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Model" dataDxfId="78"/>
-    <tableColumn id="4" xr3:uid="{217066CA-63B7-4030-A7FC-54062BE2122E}" name="Manufacturer/Brand" dataDxfId="77"/>
-    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="76"/>
-    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="75"/>
-    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="74"/>
-    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="73"/>
-    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="72"/>
-    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="71"/>
-    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="70"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:J2" insertRow="1" totalsRowShown="0" headerRowDxfId="87" dataDxfId="86">
+  <autoFilter ref="A1:J2" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}"/>
+  <tableColumns count="10">
+    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="85"/>
+    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Brand/Model" dataDxfId="84"/>
+    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="83"/>
+    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="82"/>
+    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="81"/>
+    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="80"/>
+    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="79"/>
+    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="78"/>
+    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="77"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:I2" totalsRowShown="0" headerRowDxfId="69" dataDxfId="68">
-  <autoFilter ref="A1:I2" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}"/>
-  <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="67"/>
-    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="66"/>
-    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="65"/>
-    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="64"/>
-    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="63"/>
-    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="62"/>
-    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="61"/>
-    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="60"/>
-    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="59"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:K2" totalsRowShown="0" headerRowDxfId="76" dataDxfId="75">
+  <autoFilter ref="A1:K2" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="74"/>
+    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="8"/>
+    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="73"/>
+    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="72"/>
+    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="71"/>
+    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="70"/>
+    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="69"/>
+    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="68"/>
+    <tableColumn id="9" xr3:uid="{C040B253-9925-4664-88EB-44A0F3B09681}" name="Complete" dataDxfId="7"/>
+    <tableColumn id="12" xr3:uid="{920CB592-D743-4B33-A796-C7F3DB32211C}" name="Remarks" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:I2" totalsRowShown="0" headerRowDxfId="58" dataDxfId="57">
-  <autoFilter ref="A1:I2" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}"/>
-  <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="56"/>
-    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="55"/>
-    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Model" dataDxfId="54"/>
-    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="53"/>
-    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="52"/>
-    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="51"/>
-    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="50"/>
-    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="49"/>
-    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="48"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:J2" totalsRowShown="0" headerRowDxfId="67" dataDxfId="66">
+  <autoFilter ref="A1:J2" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}"/>
+  <tableColumns count="10">
+    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="65"/>
+    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Brand/Model" dataDxfId="64"/>
+    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="63"/>
+    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="62"/>
+    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="61"/>
+    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="60"/>
+    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="59"/>
+    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="58"/>
+    <tableColumn id="10" xr3:uid="{26197E01-2936-4F5F-8081-3AA351C1CD38}" name="Remarks" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:H2" totalsRowShown="0" headerRowDxfId="47" dataDxfId="46">
-  <autoFilter ref="A1:H2" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}"/>
-  <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="45"/>
-    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="44"/>
-    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Model" dataDxfId="43"/>
-    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="42"/>
-    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="41"/>
-    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="40"/>
-    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="39"/>
-    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="38"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:I2" totalsRowShown="0" headerRowDxfId="57" dataDxfId="56">
+  <autoFilter ref="A1:I2" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}"/>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="55"/>
+    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Brand/Model/Description" dataDxfId="54"/>
+    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="53"/>
+    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="52"/>
+    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="51"/>
+    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="50"/>
+    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="49"/>
+    <tableColumn id="9" xr3:uid="{2B57F5E6-66C5-4DBA-8949-836DE0F0791C}" name="Remarks" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1489,24 +1582,24 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="F1" t="s">
         <v>39</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="F1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B2" s="4" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C2" s="8">
         <v>3</v>
@@ -1519,12 +1612,12 @@
         <v>300</v>
       </c>
       <c r="F2" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B3" s="4" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C3" s="8">
         <v>4</v>
@@ -1537,12 +1630,12 @@
         <v>40</v>
       </c>
       <c r="F3" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B4" s="4" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="C4" s="8">
         <v>5</v>
@@ -1555,12 +1648,12 @@
         <v>100</v>
       </c>
       <c r="F4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B5" s="4" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C5" s="8">
         <v>1000</v>
@@ -1594,7 +1687,8 @@
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
     <col min="2" max="2" width="41.6640625" style="2" customWidth="1"/>
-    <col min="3" max="4" width="18.44140625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="18.44140625" style="14" customWidth="1"/>
+    <col min="4" max="4" width="18.44140625" style="2" customWidth="1"/>
     <col min="5" max="5" width="15.5546875" style="2" customWidth="1"/>
     <col min="6" max="6" width="14.33203125" style="7" customWidth="1"/>
     <col min="7" max="7" width="14.109375" style="7" customWidth="1"/>
@@ -1612,32 +1706,32 @@
       <c r="B1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="4" t="s">
-        <v>66</v>
+      <c r="C1" s="1" t="s">
+        <v>62</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="H1" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="F1" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="G1" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>29</v>
-      </c>
       <c r="I1" s="5" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>30</v>
+        <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
@@ -1662,7 +1756,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3185D484-1AEA-488F-ADB2-C66611F8B5C9}">
   <sheetPr codeName="Sheet8"/>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
@@ -1671,32 +1765,41 @@
     <col min="4" max="4" width="19.33203125" style="2" customWidth="1"/>
     <col min="5" max="5" width="10.33203125" style="10" customWidth="1"/>
     <col min="6" max="6" width="9.33203125" style="3" customWidth="1"/>
-    <col min="7" max="7" width="11.33203125" style="2" customWidth="1"/>
-    <col min="8" max="16384" width="8.88671875" style="6"/>
+    <col min="8" max="8" width="14.33203125" style="2" customWidth="1"/>
+    <col min="9" max="9" width="9.33203125" style="2" customWidth="1"/>
+    <col min="10" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D1" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="E1" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>36</v>
-      </c>
+      <c r="H1" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="I1" s="6"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="G2" s="2"/>
+      <c r="I2" s="6"/>
     </row>
   </sheetData>
   <dataValidations count="4">
@@ -1706,7 +1809,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2" xr:uid="{63C2185A-207B-4EF1-BB04-3B86B2517042}">
       <formula1>"Facility Costs/Rent/Mortgage,Insurance,Debt/Leases on Equipment/Business Loans,Subscriptions,Salaries,Utilities,Maintnance/Repair,Marketing/Advertising,Professional Fees,Travel/Vehicles,Depreciation,Other/Miscellaneous"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G3:G1000 G2" xr:uid="{5CDD912B-3197-4C62-9DE2-F15AE0580881}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H3:I1000 G2:H2" xr:uid="{5CDD912B-3197-4C62-9DE2-F15AE0580881}">
       <formula1>"YES, NO"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2" xr:uid="{D24BB2FF-F2D7-4CAB-A302-F301339BCAE8}">
@@ -1740,22 +1843,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1783,16 +1886,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -1814,10 +1917,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -1864,37 +1967,37 @@
         <v>0</v>
       </c>
       <c r="B1" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="F1" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="I1" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="J1" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="E1" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="I1" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>76</v>
-      </c>
       <c r="K1" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="L1" s="14" t="s">
-        <v>91</v>
+        <v>86</v>
+      </c>
+      <c r="L1" s="8" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
@@ -1970,15 +2073,15 @@
   <sheetData>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B10" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -1987,7 +2090,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B11" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -1996,7 +2099,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B12" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2005,7 +2108,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="B13" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2014,7 +2117,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="B14" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2023,7 +2126,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="B15" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2032,7 +2135,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="B16" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2041,7 +2144,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B17" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2050,7 +2153,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B18" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2059,7 +2162,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B19" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2068,7 +2171,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="B20" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2077,7 +2180,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B21" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2100,11 +2203,11 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDE7BF89-A2E7-4A6F-B822-317739E206EC}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
-    <col min="2" max="2" width="9.5546875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="9.5546875" style="14" customWidth="1"/>
     <col min="3" max="3" width="31.44140625" style="2" customWidth="1"/>
     <col min="4" max="4" width="10.5546875" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17" style="10" bestFit="1" customWidth="1"/>
@@ -2114,16 +2217,18 @@
     <col min="9" max="9" width="19.109375" style="2" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="16.6640625" style="3" customWidth="1"/>
     <col min="11" max="11" width="16.88671875" style="3" customWidth="1"/>
-    <col min="12" max="12" width="16.88671875" style="2" customWidth="1"/>
-    <col min="13" max="13" width="22.33203125" style="2" customWidth="1"/>
-    <col min="14" max="16384" width="8.88671875" style="6"/>
+    <col min="12" max="12" width="16.88671875" style="14" customWidth="1"/>
+    <col min="13" max="13" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="7" style="2" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="16.88671875" style="2" customWidth="1"/>
+    <col min="16" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
@@ -2153,18 +2258,27 @@
       <c r="K1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+        <v>57</v>
+      </c>
+      <c r="N1" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="O1" s="6"/>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="H2" s="5">
         <f>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</f>
         <v>0</v>
       </c>
+      <c r="M2" s="2"/>
+      <c r="N2" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="O2" s="6"/>
     </row>
   </sheetData>
   <dataValidations count="3">
@@ -2189,63 +2303,59 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B027EC69-551F-4051-8A71-8B106D207C6D}">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
-    <col min="2" max="2" width="9.5546875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="9.5546875" style="14" customWidth="1"/>
     <col min="3" max="3" width="28.6640625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="26.33203125" style="2" customWidth="1"/>
-    <col min="5" max="5" width="14.88671875" style="2" customWidth="1"/>
-    <col min="6" max="6" width="14.6640625" style="10" customWidth="1"/>
-    <col min="7" max="7" width="14.6640625" style="3" customWidth="1"/>
-    <col min="8" max="9" width="12.33203125" style="2" customWidth="1"/>
-    <col min="10" max="10" width="11.44140625" style="6" customWidth="1"/>
-    <col min="11" max="11" width="32.6640625" style="2" customWidth="1"/>
-    <col min="12" max="16384" width="8.88671875" style="6"/>
+    <col min="4" max="4" width="14.88671875" style="2" customWidth="1"/>
+    <col min="5" max="5" width="14.6640625" style="10" customWidth="1"/>
+    <col min="6" max="6" width="14.6640625" style="3" customWidth="1"/>
+    <col min="7" max="8" width="12.33203125" style="2" customWidth="1"/>
+    <col min="9" max="9" width="11.44140625" style="6" customWidth="1"/>
+    <col min="10" max="10" width="32.6640625" style="2" customWidth="1"/>
+    <col min="11" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="D1" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>16</v>
+      <c r="G1" s="4" t="s">
+        <v>11</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="J1" t="s">
-        <v>24</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
+      </c>
+      <c r="I1" t="s">
+        <v>21</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>52</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J3:J1000" xr:uid="{D25ACF8B-D3DC-4EFD-9C68-FC99372E0DCF}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I3:I1000" xr:uid="{D25ACF8B-D3DC-4EFD-9C68-FC99372E0DCF}">
       <formula1>"Operational, Needs Repair, Unusable"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2" xr:uid="{4B2064CB-79C2-427D-B2C2-7CE85187D094}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2" xr:uid="{4B2064CB-79C2-427D-B2C2-7CE85187D094}">
       <formula1>"Operational, Needs Repair, Repair In-Progress, Unusable/Junk"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2259,49 +2369,69 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB7AACC4-9DA2-4A53-AD77-8C5E0C1BF474}">
   <sheetPr codeName="Sheet4"/>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.109375" style="14" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.88671875" style="14" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="28.21875" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.6640625" style="10" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.6640625" style="6" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14.33203125" style="6" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="7" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18" style="10" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="8.88671875" style="6"/>
+    <col min="9" max="10" width="18" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18" style="10" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.44140625" style="2" customWidth="1"/>
+    <col min="13" max="13" width="9.88671875" style="3" customWidth="1"/>
+    <col min="14" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="E1" s="9" t="s">
+      <c r="G1" t="s">
         <v>18</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="H1" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="I1" s="9" t="s">
-        <v>22</v>
-      </c>
+      <c r="J1" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="L1" s="6"/>
+      <c r="M1" s="6"/>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="I2" s="10"/>
+      <c r="J2" s="16" t="b">
+        <v>0</v>
+      </c>
+      <c r="K2" s="2"/>
+      <c r="L2" s="6"/>
+      <c r="M2" s="6"/>
     </row>
   </sheetData>
   <dataValidations count="3">
@@ -2325,57 +2455,68 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEDDDAA7-75C3-4AA5-ABFD-D5FB4C627E4C}">
   <sheetPr codeName="Sheet5"/>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
-    <col min="2" max="2" width="8.6640625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="8.6640625" style="14" customWidth="1"/>
     <col min="3" max="3" width="50.44140625" style="2" customWidth="1"/>
     <col min="4" max="4" width="15.6640625" style="3" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12.88671875" style="2" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="19.88671875" style="6" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="19.88671875" style="6" customWidth="1"/>
     <col min="8" max="8" width="14.44140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5546875" style="6" customWidth="1"/>
-    <col min="10" max="16384" width="8.88671875" style="6"/>
+    <col min="9" max="9" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.5546875" style="6" customWidth="1"/>
+    <col min="11" max="11" width="14.44140625" style="2" customWidth="1"/>
+    <col min="12" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>66</v>
+      <c r="B1" s="1" t="s">
+        <v>62</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>23</v>
+        <v>92</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>5</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="F1" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G1" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="H1" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="I1" t="s">
-        <v>24</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="K1" s="6"/>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="I2" s="6"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="6"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <dataValidations count="6">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F3:F1000 G3:G1000 H3:H1000" xr:uid="{FF61F80C-5E23-45D6-B39D-7C5635258115}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K3:K1000 F3:H1000" xr:uid="{FF61F80C-5E23-45D6-B39D-7C5635258115}">
       <formula1>"Circular Saw, Drill, Sander, Grinder, Other"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I3:I1000" xr:uid="{DB752B4D-0E75-42D1-B907-2DBC5792F422}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J3:K1000" xr:uid="{DB752B4D-0E75-42D1-B907-2DBC5792F422}">
       <formula1>"New, Operational, Needs Repair, Broken"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2" xr:uid="{05EFC744-2B0C-453D-A1B6-F8391608434D}">
@@ -2384,11 +2525,11 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2" xr:uid="{194EFB2B-690A-4D50-8AF6-E8ED45FE2FCA}">
       <formula1>"Portable/Handheld, Stationary/Bench Top, Outdoor Power Equipment, "</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2" xr:uid="{47F6EF9A-B127-4EB7-A5E8-0075055489DC}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:J2" xr:uid="{980AB122-9104-490B-993D-4F2FEF3A4EE6}">
+      <formula1>"Operational, Needs Repair, Repair In-Progress, Unusable/Junk"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2 J2" xr:uid="{47F6EF9A-B127-4EB7-A5E8-0075055489DC}">
       <formula1>"Corded(A/C), Cordless/Battery, Pneumatic/Air, Fuel-Powered"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2" xr:uid="{980AB122-9104-490B-993D-4F2FEF3A4EE6}">
-      <formula1>"Operational, Needs Repair, Repair In-Progress, Unusable/Junk"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2401,29 +2542,31 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F39ADDA6-CD5F-4655-A9C0-9676DDAC362E}">
   <sheetPr codeName="Sheet6"/>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.6640625" style="14" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="54.6640625" style="2" customWidth="1"/>
     <col min="4" max="4" width="15.6640625" style="3" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.5546875" style="6" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.88671875" style="2" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.88671875" style="2" customWidth="1"/>
-    <col min="8" max="8" width="10.33203125" style="7" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="8.88671875" style="6"/>
+    <col min="8" max="8" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.33203125" style="7" customWidth="1"/>
+    <col min="10" max="10" width="12.88671875" style="2" customWidth="1"/>
+    <col min="11" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>66</v>
+      <c r="B1" s="1" t="s">
+        <v>62</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>23</v>
+        <v>93</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>5</v>
@@ -2432,24 +2575,33 @@
         <v>3</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="H1" s="8" t="s">
-        <v>25</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="J1" s="6"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H2" s="7"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="6"/>
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E3:E1000 F3:F1000 G3:G1000" xr:uid="{B6CB3C84-EE01-4878-B558-650FC19D8248}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J3:J1000 E3:G1000" xr:uid="{B6CB3C84-EE01-4878-B558-650FC19D8248}">
       <formula1>"Saw, Hammer, Screwdriver, Wrench, Sockets, Pliers, Measuring, Files, Other"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2" xr:uid="{ACB7A40B-F0EE-4387-88E4-5140AB68313F}">
       <formula1>"Fastening/Turning,Measuring/Layout,Striking/Hammering,Gripping/Holding,Cutting/Shaping,Other"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2" xr:uid="{2E543736-2E6D-4F90-9169-21BA7CCD7676}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2 I2" xr:uid="{2E543736-2E6D-4F90-9169-21BA7CCD7676}">
       <formula1>"Operational,Needs Repair,Repair In-Progress,Unusable/Junk"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
changed Excel Shop Machinery, Location: hidden: true
</commit_message>
<xml_diff>
--- a/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
+++ b/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1a2ae81d67634e6/Desktop/Michanikos Artifex Enterprises/MAE Custom Digital Solutions/MAE Workshop Inventory Management System/GITHUB_MAE_Workshop Inventory App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="106" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D50FE1C8-7BFF-4F9F-9762-07638FF6C09D}"/>
+  <xr:revisionPtr revIDLastSave="107" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B5C7C730-4C69-4B8F-B004-8F57EEF1A83F}"/>
   <bookViews>
-    <workbookView xWindow="11136" yWindow="132" windowWidth="11844" windowHeight="11904" firstSheet="9" activeTab="10" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
+    <workbookView xWindow="11136" yWindow="132" windowWidth="11844" windowHeight="11904" firstSheet="4" activeTab="5" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
   </bookViews>
   <sheets>
     <sheet name="TEST Inventory" sheetId="10" r:id="rId1"/>
@@ -462,14 +462,88 @@
   <dxfs count="124">
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="1"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -482,7 +556,96 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -503,6 +666,28 @@
       </extLst>
     </dxf>
     <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="1"/>
     </dxf>
@@ -512,11 +697,54 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="1"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="1"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -529,281 +757,11 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
@@ -843,6 +801,10 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
@@ -856,28 +818,6 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
@@ -934,6 +874,66 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -989,11 +989,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}" name="TEST_Inventory" displayName="TEST_Inventory" ref="A1:F5" totalsRowShown="0">
   <autoFilter ref="A1:F5" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="109"/>
-    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="108"/>
-    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="107"/>
-    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="106"/>
-    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="105">
+    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="113"/>
+    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="112"/>
+    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="111"/>
+    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="110"/>
+    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="109">
       <calculatedColumnFormula>TEST_Inventory[[#This Row],[TEST Integer]]*TEST_Inventory[[#This Row],[TEST Currency]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{AB3A5F3C-FCF0-4466-90FD-8ABB6E18DF5C}" name="TEST Dropdown"/>
@@ -1003,55 +1003,55 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:K2" totalsRowShown="0" headerRowDxfId="48" dataDxfId="47">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:K2" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26">
   <autoFilter ref="A1:K2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="46"/>
-    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="45"/>
-    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="1"/>
-    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="44"/>
-    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="43"/>
-    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="42"/>
-    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="41"/>
-    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="40"/>
-    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="39">
+    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="25"/>
+    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="24"/>
+    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="23"/>
+    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="22"/>
+    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="21"/>
+    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="20"/>
+    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="19"/>
+    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="18"/>
+    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="17">
       <calculatedColumnFormula>Shop_Consumables[[#This Row],[Current Stock]]*Shop_Consumables[[#This Row],[Unit Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="38"/>
-    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Supplier/Remarks" dataDxfId="37"/>
+    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="16"/>
+    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Supplier/Remarks" dataDxfId="15"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:H2" totalsRowShown="0" headerRowDxfId="36" dataDxfId="35">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:H2" totalsRowShown="0" headerRowDxfId="123" dataDxfId="122">
   <autoFilter ref="A1:H2" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="34"/>
-    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="33"/>
-    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="32"/>
-    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="31"/>
-    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="30"/>
-    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="29"/>
-    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="28"/>
-    <tableColumn id="8" xr3:uid="{9140C4E8-CB9E-40BF-ABD9-13A971322B09}" name="Remarks" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="121"/>
+    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="120"/>
+    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="119"/>
+    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="118"/>
+    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="117"/>
+    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="116"/>
+    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="115"/>
+    <tableColumn id="8" xr3:uid="{9140C4E8-CB9E-40BF-ABD9-13A971322B09}" name="Remarks" dataDxfId="114"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13">
   <autoFilter ref="A1:G2" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="25"/>
-    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="24"/>
-    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="23"/>
-    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="22"/>
-    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="21"/>
-    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="20"/>
-    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="19"/>
+    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="12"/>
+    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="10"/>
+    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="9"/>
+    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="8"/>
+    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="7"/>
+    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1061,11 +1061,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}" name="Location" displayName="Location" ref="A1:E2" insertRow="1" totalsRowShown="0">
   <autoFilter ref="A1:E2" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="18"/>
-    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Name" dataDxfId="16"/>
-    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="15"/>
-    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="14"/>
+    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Name" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1075,10 +1075,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}" name="TEST_Dashboard" displayName="TEST_Dashboard" ref="A1:B2" totalsRowShown="0">
   <autoFilter ref="A1:B2" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="104">
+    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="108">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Currency])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="103">
+    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="107">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Integer])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1087,45 +1087,45 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:L2" totalsRowShown="0" headerRowDxfId="123" dataDxfId="122">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:L2" totalsRowShown="0" headerRowDxfId="106" dataDxfId="105">
   <autoFilter ref="A1:L2" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="121"/>
-    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="120">
+    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="104"/>
+    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="103">
       <calculatedColumnFormula>SUM(Resell_Inventory[Total Investment])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="119">
+    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="102">
       <calculatedColumnFormula>SUM(Resell_Inventory[Actual Sale Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="118">
+    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="101">
       <calculatedColumnFormula>SUM(Shop_Machinery[Purchase Cost])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="117">
+    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="100">
       <calculatedColumnFormula>SUM(Shop_Power_Tools[Purchase Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="116">
+    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="99">
       <calculatedColumnFormula>SUM(Shop_Hand_Tools[Purchase Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="115">
+    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="98">
       <calculatedColumnFormula>SUM(Shop_Consumables[Current Inventory Value])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="114">
+    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="97">
       <calculatedColumnFormula>SUM(D2,E2,F2,G2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="113">
+    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="96">
       <calculatedColumnFormula array="1">SUMPRODUCT(--(Shop_Consumables[Current Stock]&lt;=Shop_Consumables[Reorder Point]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="112">
+    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="95">
       <calculatedColumnFormula>SUMIFS(Shop_Overhead[Amount], Shop_Overhead[Due Date], "&lt;="&amp;TODAY()+30, Shop_Overhead[Due Date], "&gt;="&amp;TODAY())</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{E4065760-B1B1-4564-936B-3405D3B80297}" name="Equipment With Operational Issues" dataDxfId="111">
+    <tableColumn id="12" xr3:uid="{E4065760-B1B1-4564-936B-3405D3B80297}" name="Equipment With Operational Issues" dataDxfId="94">
       <calculatedColumnFormula array="1">SUM(
   COUNTIFS(Shop_Machinery[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"}),
   COUNTIFS(Shop_Power_Tools[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"}),
   COUNTIFS(Shop_Hand_Tools[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"})
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{86A5DBCB-1064-4926-8405-405B453A4546}" name="Maintenance Items Due in Next 30 Days" dataDxfId="110">
+    <tableColumn id="6" xr3:uid="{86A5DBCB-1064-4926-8405-405B453A4546}" name="Maintenance Items Due in Next 30 Days" dataDxfId="93">
       <calculatedColumnFormula>SUM(
             COUNTIFS(Maintenance_Log[Next Service Date], "&lt;="&amp;TODAY()+30, Maintenance_Log[Next Service Date], "&gt;="&amp;TODAY())
         )</calculatedColumnFormula>
@@ -1139,8 +1139,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{F579DA07-7AD6-49DA-9B44-D5B1132EDAC6}" name="Overhead_Summary" displayName="Overhead_Summary" ref="A9:B21" totalsRowShown="0">
   <autoFilter ref="A9:B21" xr:uid="{F579DA07-7AD6-49DA-9B44-D5B1132EDAC6}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{7CA4839C-9603-479D-BD1C-8377DFA9603C}" name="Expense Category" dataDxfId="102"/>
-    <tableColumn id="2" xr3:uid="{FE0F7616-EAF3-443D-AC69-DE6541DC10E5}" name="Annual Total" dataDxfId="101">
+    <tableColumn id="1" xr3:uid="{7CA4839C-9603-479D-BD1C-8377DFA9603C}" name="Expense Category" dataDxfId="92"/>
+    <tableColumn id="2" xr3:uid="{FE0F7616-EAF3-443D-AC69-DE6541DC10E5}" name="Annual Total" dataDxfId="91">
       <calculatedColumnFormula>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1149,101 +1149,101 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:N2" totalsRowShown="0" headerRowDxfId="100" dataDxfId="99">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:N2" totalsRowShown="0" headerRowDxfId="90" dataDxfId="89">
   <autoFilter ref="A1:N2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}"/>
   <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="98"/>
-    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="97"/>
-    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="96"/>
-    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="95"/>
-    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="94"/>
-    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="93"/>
-    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="92">
+    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="88"/>
+    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="87"/>
+    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="86"/>
+    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="85"/>
+    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="84"/>
+    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="83"/>
+    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="82"/>
+    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="81">
       <calculatedColumnFormula>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="91"/>
-    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="90"/>
-    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="89"/>
-    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="11"/>
-    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="88"/>
-    <tableColumn id="13" xr3:uid="{885B08CA-5BC3-4FAA-B661-BE5CCBF87448}" name="Sold" dataDxfId="12"/>
+    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="80"/>
+    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="79"/>
+    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="78"/>
+    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="77"/>
+    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="76"/>
+    <tableColumn id="13" xr3:uid="{885B08CA-5BC3-4FAA-B661-BE5CCBF87448}" name="Sold" dataDxfId="75"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:J2" insertRow="1" totalsRowShown="0" headerRowDxfId="87" dataDxfId="86">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:J2" insertRow="1" totalsRowShown="0" headerRowDxfId="74" dataDxfId="73">
   <autoFilter ref="A1:J2" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="85"/>
-    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Brand/Model" dataDxfId="84"/>
-    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="83"/>
-    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="82"/>
-    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="81"/>
-    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="80"/>
-    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="79"/>
-    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="78"/>
-    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="77"/>
+    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="72"/>
+    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="71"/>
+    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Brand/Model" dataDxfId="70"/>
+    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="69"/>
+    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="68"/>
+    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="67"/>
+    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="0"/>
+    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="66"/>
+    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="65"/>
+    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="64"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:K2" totalsRowShown="0" headerRowDxfId="76" dataDxfId="75">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:K2" totalsRowShown="0" headerRowDxfId="63" dataDxfId="62">
   <autoFilter ref="A1:K2" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="74"/>
-    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="8"/>
-    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="73"/>
-    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="72"/>
-    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="71"/>
-    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="70"/>
-    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="69"/>
-    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="68"/>
-    <tableColumn id="9" xr3:uid="{C040B253-9925-4664-88EB-44A0F3B09681}" name="Complete" dataDxfId="7"/>
-    <tableColumn id="12" xr3:uid="{920CB592-D743-4B33-A796-C7F3DB32211C}" name="Remarks" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="61"/>
+    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="60"/>
+    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="59"/>
+    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="58"/>
+    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="57"/>
+    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="56"/>
+    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="55"/>
+    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="54"/>
+    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="53"/>
+    <tableColumn id="9" xr3:uid="{C040B253-9925-4664-88EB-44A0F3B09681}" name="Complete" dataDxfId="52"/>
+    <tableColumn id="12" xr3:uid="{920CB592-D743-4B33-A796-C7F3DB32211C}" name="Remarks" dataDxfId="51"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:J2" totalsRowShown="0" headerRowDxfId="67" dataDxfId="66">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:J2" totalsRowShown="0" headerRowDxfId="50" dataDxfId="49">
   <autoFilter ref="A1:J2" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="65"/>
-    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Brand/Model" dataDxfId="64"/>
-    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="63"/>
-    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="62"/>
-    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="61"/>
-    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="60"/>
-    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="59"/>
-    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="58"/>
-    <tableColumn id="10" xr3:uid="{26197E01-2936-4F5F-8081-3AA351C1CD38}" name="Remarks" dataDxfId="4"/>
+    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="48"/>
+    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="47"/>
+    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Brand/Model" dataDxfId="46"/>
+    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="45"/>
+    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="44"/>
+    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="43"/>
+    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="42"/>
+    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="41"/>
+    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="40"/>
+    <tableColumn id="10" xr3:uid="{26197E01-2936-4F5F-8081-3AA351C1CD38}" name="Remarks" dataDxfId="39"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:I2" totalsRowShown="0" headerRowDxfId="57" dataDxfId="56">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:I2" totalsRowShown="0" headerRowDxfId="38" dataDxfId="37">
   <autoFilter ref="A1:I2" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="55"/>
-    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Brand/Model/Description" dataDxfId="54"/>
-    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="53"/>
-    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="52"/>
-    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="51"/>
-    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="50"/>
-    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="49"/>
-    <tableColumn id="9" xr3:uid="{2B57F5E6-66C5-4DBA-8949-836DE0F0791C}" name="Remarks" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="36"/>
+    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="35"/>
+    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Brand/Model/Description" dataDxfId="34"/>
+    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="33"/>
+    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="32"/>
+    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="31"/>
+    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="30"/>
+    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="29"/>
+    <tableColumn id="9" xr3:uid="{2B57F5E6-66C5-4DBA-8949-836DE0F0791C}" name="Remarks" dataDxfId="28"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2312,7 +2312,8 @@
     <col min="4" max="4" width="14.88671875" style="2" customWidth="1"/>
     <col min="5" max="5" width="14.6640625" style="10" customWidth="1"/>
     <col min="6" max="6" width="14.6640625" style="3" customWidth="1"/>
-    <col min="7" max="8" width="12.33203125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="12.33203125" style="14" customWidth="1"/>
+    <col min="8" max="8" width="12.33203125" style="2" customWidth="1"/>
     <col min="9" max="9" width="11.44140625" style="6" customWidth="1"/>
     <col min="10" max="10" width="32.6640625" style="2" customWidth="1"/>
     <col min="11" max="16384" width="8.88671875" style="6"/>
@@ -2337,7 +2338,7 @@
       <c r="F1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="1" t="s">
         <v>11</v>
       </c>
       <c r="H1" s="4" t="s">

</xml_diff>

<commit_message>
updated config and excel : master dashboard table; maint due in next 30 days hero number formula to include past due and complete NOT checked
</commit_message>
<xml_diff>
--- a/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
+++ b/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1a2ae81d67634e6/Desktop/Michanikos Artifex Enterprises/MAE Custom Digital Solutions/MAE Workshop Inventory Management System/GITHUB_MAE_Workshop Inventory App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="115" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6797F7D7-94CD-45FC-BAA3-D7D495BAC92C}"/>
+  <xr:revisionPtr revIDLastSave="116" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{65F8B0D1-D541-4351-B86F-D14417B70B86}"/>
   <bookViews>
-    <workbookView xWindow="11136" yWindow="132" windowWidth="11844" windowHeight="11904" firstSheet="4" activeTab="4" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="2" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
   </bookViews>
   <sheets>
     <sheet name="TEST Inventory" sheetId="10" r:id="rId1"/>
@@ -453,8 +453,225 @@
   </cellStyles>
   <dxfs count="124">
     <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
       <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -468,14 +685,6 @@
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -487,59 +696,36 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -550,65 +736,6 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -618,155 +745,6 @@
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
@@ -896,9 +874,11 @@
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -907,6 +887,26 @@
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
@@ -981,11 +981,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}" name="TEST_Inventory" displayName="TEST_Inventory" ref="A1:F5" totalsRowShown="0">
   <autoFilter ref="A1:F5" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="111"/>
-    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="110"/>
-    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="109"/>
-    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="108"/>
-    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="107">
+    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="107"/>
+    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="106"/>
+    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="105"/>
+    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="104"/>
+    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="103">
       <calculatedColumnFormula>TEST_Inventory[[#This Row],[TEST Integer]]*TEST_Inventory[[#This Row],[TEST Currency]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{AB3A5F3C-FCF0-4466-90FD-8ABB6E18DF5C}" name="TEST Dropdown"/>
@@ -995,55 +995,55 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:K2" totalsRowShown="0" headerRowDxfId="43" dataDxfId="42">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:K2" totalsRowShown="0" headerRowDxfId="36" dataDxfId="35">
   <autoFilter ref="A1:K2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="41"/>
-    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="40"/>
-    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="39"/>
-    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="38"/>
-    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="37"/>
-    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="36"/>
-    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="35"/>
-    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="34"/>
-    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="33">
+    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="34"/>
+    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="33"/>
+    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="32"/>
+    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="31"/>
+    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="30"/>
+    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="29"/>
+    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="28"/>
+    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="27"/>
+    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="26">
       <calculatedColumnFormula>Shop_Consumables[[#This Row],[Current Stock]]*Shop_Consumables[[#This Row],[Unit Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="32"/>
-    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Supplier/Remarks" dataDxfId="31"/>
+    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="25"/>
+    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Supplier/Remarks" dataDxfId="24"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:H2" totalsRowShown="0" headerRowDxfId="30" dataDxfId="29">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:H2" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
   <autoFilter ref="A1:H2" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="28"/>
-    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="27"/>
-    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="26"/>
-    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="25"/>
-    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="24"/>
-    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="23"/>
-    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="22"/>
-    <tableColumn id="8" xr3:uid="{9140C4E8-CB9E-40BF-ABD9-13A971322B09}" name="Remarks" dataDxfId="21"/>
+    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="20"/>
+    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="19"/>
+    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="18"/>
+    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="17"/>
+    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="16"/>
+    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="15"/>
+    <tableColumn id="8" xr3:uid="{9140C4E8-CB9E-40BF-ABD9-13A971322B09}" name="Remarks" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
   <autoFilter ref="A1:G2" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="18"/>
-    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="16"/>
-    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="15"/>
-    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="14"/>
-    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="13"/>
-    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="12"/>
+    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="11"/>
+    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="9"/>
+    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="7"/>
+    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="6"/>
+    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1053,11 +1053,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}" name="Location" displayName="Location" ref="A1:E2" insertRow="1" totalsRowShown="0">
   <autoFilter ref="A1:E2" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Name" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="7"/>
+    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Name" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1067,10 +1067,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}" name="TEST_Dashboard" displayName="TEST_Dashboard" ref="A1:B2" totalsRowShown="0">
   <autoFilter ref="A1:B2" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="106">
+    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="102">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Currency])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="105">
+    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="101">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Integer])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1079,48 +1079,46 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:L2" totalsRowShown="0" headerRowDxfId="104" dataDxfId="103">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:L2" totalsRowShown="0" headerRowDxfId="100" dataDxfId="99">
   <autoFilter ref="A1:L2" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="102"/>
-    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="101">
+    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="98"/>
+    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="97">
       <calculatedColumnFormula>SUM(Resell_Inventory[Total Investment])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="100">
+    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="96">
       <calculatedColumnFormula>SUM(Resell_Inventory[Actual Sale Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="99">
+    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="95">
       <calculatedColumnFormula>SUM(Shop_Machinery[Purchase Cost])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="98">
+    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="94">
       <calculatedColumnFormula>SUM(Shop_Power_Tools[Purchase Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="97">
+    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="93">
       <calculatedColumnFormula>SUM(Shop_Hand_Tools[Purchase Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="96">
+    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="92">
       <calculatedColumnFormula>SUM(Shop_Consumables[Current Inventory Value])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="95">
+    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="91">
       <calculatedColumnFormula>SUM(D2,E2,F2,G2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="94">
+    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="90">
       <calculatedColumnFormula array="1">SUMPRODUCT(--(Shop_Consumables[Current Stock]&lt;=Shop_Consumables[Reorder Point]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="93">
+    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="89">
       <calculatedColumnFormula>SUMIFS(Shop_Overhead[Amount], Shop_Overhead[Due Date], "&lt;="&amp;TODAY()+30, Shop_Overhead[Due Date], "&gt;="&amp;TODAY())</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{E4065760-B1B1-4564-936B-3405D3B80297}" name="Equipment With Operational Issues" dataDxfId="92">
+    <tableColumn id="12" xr3:uid="{E4065760-B1B1-4564-936B-3405D3B80297}" name="Equipment With Operational Issues" dataDxfId="88">
       <calculatedColumnFormula array="1">SUM(
   COUNTIFS(Shop_Machinery[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"}),
   COUNTIFS(Shop_Power_Tools[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"}),
   COUNTIFS(Shop_Hand_Tools[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"})
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{86A5DBCB-1064-4926-8405-405B453A4546}" name="Maintenance Items Due in Next 30 Days" dataDxfId="91">
-      <calculatedColumnFormula>SUM(
-            COUNTIFS(Maintenance_Log[Next Service Date], "&lt;="&amp;TODAY()+30, Maintenance_Log[Next Service Date], "&gt;="&amp;TODAY())
-        )</calculatedColumnFormula>
+    <tableColumn id="6" xr3:uid="{86A5DBCB-1064-4926-8405-405B453A4546}" name="Maintenance Items Due in Next 30 Days" dataDxfId="87">
+      <calculatedColumnFormula>COUNTIFS(Maintenance_Log[Next Service Date], "&lt;="&amp;TODAY()+30, Maintenance_Log[Complete], "FALSE")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1131,8 +1129,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{F579DA07-7AD6-49DA-9B44-D5B1132EDAC6}" name="Overhead_Summary" displayName="Overhead_Summary" ref="A9:B21" totalsRowShown="0">
   <autoFilter ref="A9:B21" xr:uid="{F579DA07-7AD6-49DA-9B44-D5B1132EDAC6}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{7CA4839C-9603-479D-BD1C-8377DFA9603C}" name="Expense Category" dataDxfId="90"/>
-    <tableColumn id="2" xr3:uid="{FE0F7616-EAF3-443D-AC69-DE6541DC10E5}" name="Annual Total" dataDxfId="89">
+    <tableColumn id="1" xr3:uid="{7CA4839C-9603-479D-BD1C-8377DFA9603C}" name="Expense Category" dataDxfId="86"/>
+    <tableColumn id="2" xr3:uid="{FE0F7616-EAF3-443D-AC69-DE6541DC10E5}" name="Annual Total" dataDxfId="85">
       <calculatedColumnFormula>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1141,101 +1139,101 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:N2" totalsRowShown="0" headerRowDxfId="88" dataDxfId="87">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:N2" totalsRowShown="0" headerRowDxfId="123" dataDxfId="122">
   <autoFilter ref="A1:N2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}"/>
   <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="86"/>
-    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="85"/>
-    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="84"/>
-    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="83"/>
-    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="82"/>
-    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="81"/>
-    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="80"/>
-    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="79">
+    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="121"/>
+    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="120"/>
+    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="119"/>
+    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="118"/>
+    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="117"/>
+    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="116"/>
+    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="115"/>
+    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="114">
       <calculatedColumnFormula>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="78"/>
-    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="77"/>
-    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="0"/>
-    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="3"/>
-    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="2"/>
-    <tableColumn id="13" xr3:uid="{885B08CA-5BC3-4FAA-B661-BE5CCBF87448}" name="Sold" dataDxfId="1"/>
+    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="113"/>
+    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="112"/>
+    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="111"/>
+    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="110"/>
+    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="109"/>
+    <tableColumn id="13" xr3:uid="{885B08CA-5BC3-4FAA-B661-BE5CCBF87448}" name="Sold" dataDxfId="108"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:J2" insertRow="1" totalsRowShown="0" headerRowDxfId="123" dataDxfId="122">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:J2" insertRow="1" totalsRowShown="0" headerRowDxfId="84" dataDxfId="83">
   <autoFilter ref="A1:J2" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="121"/>
-    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="120"/>
-    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Brand/Model" dataDxfId="119"/>
-    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="118"/>
-    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="117"/>
-    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="116"/>
-    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="115"/>
-    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="114"/>
-    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="113"/>
-    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="112"/>
+    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="82"/>
+    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="81"/>
+    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Brand/Model" dataDxfId="80"/>
+    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="79"/>
+    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="78"/>
+    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="77"/>
+    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="76"/>
+    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="75"/>
+    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="74"/>
+    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="73"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:K2" totalsRowShown="0" headerRowDxfId="76" dataDxfId="75">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:K2" totalsRowShown="0" headerRowDxfId="72" dataDxfId="71">
   <autoFilter ref="A1:K2" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="74"/>
-    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="73"/>
-    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="72"/>
-    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="71"/>
-    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="70"/>
-    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="69"/>
-    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="68"/>
-    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="67"/>
-    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="5"/>
-    <tableColumn id="9" xr3:uid="{C040B253-9925-4664-88EB-44A0F3B09681}" name="Complete" dataDxfId="4"/>
-    <tableColumn id="12" xr3:uid="{920CB592-D743-4B33-A796-C7F3DB32211C}" name="Remarks" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="70"/>
+    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="69"/>
+    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="68"/>
+    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="67"/>
+    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="66"/>
+    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="65"/>
+    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="64"/>
+    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="63"/>
+    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="62"/>
+    <tableColumn id="9" xr3:uid="{C040B253-9925-4664-88EB-44A0F3B09681}" name="Complete" dataDxfId="61"/>
+    <tableColumn id="12" xr3:uid="{920CB592-D743-4B33-A796-C7F3DB32211C}" name="Remarks" dataDxfId="60"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:J2" totalsRowShown="0" headerRowDxfId="66" dataDxfId="65">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:J2" totalsRowShown="0" headerRowDxfId="59" dataDxfId="58">
   <autoFilter ref="A1:J2" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="64"/>
-    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="63"/>
-    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Brand/Model" dataDxfId="62"/>
-    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="61"/>
-    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="60"/>
-    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="59"/>
-    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="58"/>
-    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="57"/>
-    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="56"/>
-    <tableColumn id="10" xr3:uid="{26197E01-2936-4F5F-8081-3AA351C1CD38}" name="Remarks" dataDxfId="55"/>
+    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="57"/>
+    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="56"/>
+    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Brand/Model" dataDxfId="55"/>
+    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="54"/>
+    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="53"/>
+    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="52"/>
+    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="51"/>
+    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="50"/>
+    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="49"/>
+    <tableColumn id="10" xr3:uid="{26197E01-2936-4F5F-8081-3AA351C1CD38}" name="Remarks" dataDxfId="48"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:I2" totalsRowShown="0" headerRowDxfId="54" dataDxfId="53">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:I2" totalsRowShown="0" headerRowDxfId="47" dataDxfId="46">
   <autoFilter ref="A1:I2" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="52"/>
-    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="51"/>
-    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Brand/Model/Description" dataDxfId="50"/>
-    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="49"/>
-    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="48"/>
-    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="47"/>
-    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="46"/>
-    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="45"/>
-    <tableColumn id="9" xr3:uid="{2B57F5E6-66C5-4DBA-8949-836DE0F0791C}" name="Remarks" dataDxfId="44"/>
+    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="45"/>
+    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="44"/>
+    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Brand/Model/Description" dataDxfId="43"/>
+    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="42"/>
+    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="41"/>
+    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="40"/>
+    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="39"/>
+    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="38"/>
+    <tableColumn id="9" xr3:uid="{2B57F5E6-66C5-4DBA-8949-836DE0F0791C}" name="Remarks" dataDxfId="37"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2038,9 +2036,7 @@
         <v>0</v>
       </c>
       <c r="L2" s="7">
-        <f ca="1">SUM(
-            COUNTIFS(Maintenance_Log[Next Service Date], "&lt;="&amp;TODAY()+30, Maintenance_Log[Next Service Date], "&gt;="&amp;TODAY())
-        )</f>
+        <f ca="1">COUNTIFS(Maintenance_Log[Next Service Date], "&lt;="&amp;TODAY()+30, Maintenance_Log[Complete], "FALSE")</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added new file: architecture.md; updated Excel and config to prepare for inventory system
</commit_message>
<xml_diff>
--- a/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
+++ b/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1a2ae81d67634e6/Desktop/Michanikos Artifex Enterprises/MAE Custom Digital Solutions/MAE Workshop Inventory Management System/GITHUB_MAE_Workshop Inventory App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="117" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A9962B81-088E-49E9-8BE9-93B51D31B7BC}"/>
+  <xr:revisionPtr revIDLastSave="183" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4B633391-06E1-4FCF-962D-CCDA56611818}"/>
   <bookViews>
-    <workbookView xWindow="11136" yWindow="132" windowWidth="11844" windowHeight="11904" firstSheet="2" activeTab="2" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
+    <workbookView xWindow="2052" yWindow="648" windowWidth="11844" windowHeight="11904" firstSheet="11" activeTab="12" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
   </bookViews>
   <sheets>
     <sheet name="TEST Inventory" sheetId="10" r:id="rId1"/>
@@ -70,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="100">
   <si>
     <t>mae_id</t>
   </si>
@@ -246,9 +246,6 @@
     <t>Location_ID</t>
   </si>
   <si>
-    <t>Name</t>
-  </si>
-  <si>
     <t>Type</t>
   </si>
   <si>
@@ -355,6 +352,24 @@
   </si>
   <si>
     <t>Supplier/Remarks</t>
+  </si>
+  <si>
+    <t>Tag_ID</t>
+  </si>
+  <si>
+    <t>TBD</t>
+  </si>
+  <si>
+    <t>To Be Determined</t>
+  </si>
+  <si>
+    <t>[Placeholder]</t>
+  </si>
+  <si>
+    <t>[To Be Determined]</t>
+  </si>
+  <si>
+    <t>TBD001</t>
   </si>
 </sst>
 </file>
@@ -405,7 +420,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
       <protection hidden="1"/>
@@ -439,27 +454,22 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
       <protection locked="0" hidden="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
       <protection locked="0"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement i="0"/>
-        </ext>
-      </extLst>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="124">
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
+  <dxfs count="129">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -469,209 +479,7 @@
       <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -683,33 +491,265 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="0"/>
     </dxf>
@@ -740,10 +780,6 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="1"/>
     </dxf>
     <dxf>
@@ -775,19 +811,6 @@
     </dxf>
     <dxf>
       <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -960,11 +983,6 @@
   <bag type="XFComplement">
     <bagId k="XFControls">1</bagId>
   </bag>
-  <bag type="XFComplements" extRef="XFComplementsMapperExtRef">
-    <a k="MappedFeaturePropertyBags">
-      <bagId>2</bagId>
-    </a>
-  </bag>
   <bag type="DXFComplements" extRef="DXFComplementsMapperExtRef">
     <a k="MappedFeaturePropertyBags">
       <bagId>2</bagId>
@@ -973,19 +991,15 @@
 </FeaturePropertyBags>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}" name="TEST_Inventory" displayName="TEST_Inventory" ref="A1:F5" totalsRowShown="0">
   <autoFilter ref="A1:F5" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="109"/>
-    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="108"/>
-    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="107"/>
-    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="106"/>
-    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="105">
+    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="114"/>
+    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="113"/>
+    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="112"/>
+    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="111"/>
+    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="110">
       <calculatedColumnFormula>TEST_Inventory[[#This Row],[TEST Integer]]*TEST_Inventory[[#This Row],[TEST Currency]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{AB3A5F3C-FCF0-4466-90FD-8ABB6E18DF5C}" name="TEST Dropdown"/>
@@ -995,67 +1009,68 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:K2" totalsRowShown="0" headerRowDxfId="36" dataDxfId="35">
-  <autoFilter ref="A1:K2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
-  <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="34"/>
-    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="33"/>
-    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="32"/>
-    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="31"/>
-    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="30"/>
-    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="29"/>
-    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="28"/>
-    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="27"/>
-    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:L2" totalsRowShown="0" headerRowDxfId="55" dataDxfId="54">
+  <autoFilter ref="A1:L2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
+  <tableColumns count="12">
+    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="53"/>
+    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="22"/>
+    <tableColumn id="12" xr3:uid="{8F0FD29C-682B-41B4-82F2-913D40801887}" name="Tag_ID" dataDxfId="8"/>
+    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="52"/>
+    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="51"/>
+    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="50"/>
+    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="49"/>
+    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="48"/>
+    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="47"/>
+    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="46">
       <calculatedColumnFormula>Shop_Consumables[[#This Row],[Current Stock]]*Shop_Consumables[[#This Row],[Unit Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="25"/>
-    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Supplier/Remarks" dataDxfId="24"/>
+    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Supplier/Remarks" dataDxfId="45"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:H2" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:H2" totalsRowShown="0" headerRowDxfId="44" dataDxfId="43">
   <autoFilter ref="A1:H2" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="20"/>
-    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="16"/>
-    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="15"/>
-    <tableColumn id="8" xr3:uid="{9140C4E8-CB9E-40BF-ABD9-13A971322B09}" name="Remarks" dataDxfId="14"/>
+    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="42"/>
+    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="41"/>
+    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="40"/>
+    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="39"/>
+    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="38"/>
+    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="37"/>
+    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="36"/>
+    <tableColumn id="8" xr3:uid="{9140C4E8-CB9E-40BF-ABD9-13A971322B09}" name="Remarks" dataDxfId="35"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="34" dataDxfId="33">
   <autoFilter ref="A1:G2" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="11"/>
-    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="9"/>
-    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="7"/>
-    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="6"/>
-    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="32"/>
+    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="31"/>
+    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="30"/>
+    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="29"/>
+    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="28"/>
+    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="27"/>
+    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="26"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}" name="Location" displayName="Location" ref="A1:E2" insertRow="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}" name="Location" displayName="Location" ref="A1:E2" totalsRowShown="0">
   <autoFilter ref="A1:E2" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Name" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Description" dataDxfId="2"/>
     <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="1"/>
     <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="0"/>
   </tableColumns>
@@ -1067,10 +1082,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}" name="TEST_Dashboard" displayName="TEST_Dashboard" ref="A1:B2" totalsRowShown="0">
   <autoFilter ref="A1:B2" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="104">
+    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="109">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Currency])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="103">
+    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="108">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Integer])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1079,46 +1094,46 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:L2" totalsRowShown="0" headerRowDxfId="123" dataDxfId="122">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:L2" totalsRowShown="0" headerRowDxfId="128" dataDxfId="127">
   <autoFilter ref="A1:L2" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="121"/>
-    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="120">
+    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="126"/>
+    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="125">
       <calculatedColumnFormula>SUM(Resell_Inventory[Total Investment])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="119">
+    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="124">
       <calculatedColumnFormula>SUM(Resell_Inventory[Actual Sale Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="118">
+    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="123">
       <calculatedColumnFormula>SUM(Shop_Machinery[Purchase Cost])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="117">
+    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="122">
       <calculatedColumnFormula>SUM(Shop_Power_Tools[Purchase Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="116">
+    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="121">
       <calculatedColumnFormula>SUM(Shop_Hand_Tools[Purchase Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="115">
+    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="120">
       <calculatedColumnFormula>SUM(Shop_Consumables[Current Inventory Value])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="114">
+    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="119">
       <calculatedColumnFormula>SUM(D2,E2,F2,G2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="113">
+    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="118">
       <calculatedColumnFormula array="1">SUMPRODUCT(--(Shop_Consumables[Current Stock]&lt;=Shop_Consumables[Reorder Point]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="112">
+    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="117">
       <calculatedColumnFormula>SUMIFS(Shop_Overhead[Amount], Shop_Overhead[Due Date], "&lt;="&amp;TODAY()+30, Shop_Overhead[Due Date], "&gt;="&amp;TODAY())</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{E4065760-B1B1-4564-936B-3405D3B80297}" name="Equipment With Operational Issues" dataDxfId="111">
+    <tableColumn id="12" xr3:uid="{E4065760-B1B1-4564-936B-3405D3B80297}" name="Equipment With Operational Issues" dataDxfId="116">
       <calculatedColumnFormula array="1">SUM(
   COUNTIFS(Shop_Machinery[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"}),
   COUNTIFS(Shop_Power_Tools[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"}),
   COUNTIFS(Shop_Hand_Tools[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"})
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{86A5DBCB-1064-4926-8405-405B453A4546}" name="Maintenance Items Due in Next 30 Days" dataDxfId="110">
-      <calculatedColumnFormula>COUNTIFS(Maintenance_Log[Next Service Date], "&lt;="&amp;TODAY()+30, Maintenance_Log[Complete], FALSE)</calculatedColumnFormula>
+    <tableColumn id="6" xr3:uid="{86A5DBCB-1064-4926-8405-405B453A4546}" name="Maintenance Items Due in Next 30 Days" dataDxfId="115">
+      <calculatedColumnFormula>COUNTIFS(Maintenance_Log[Next Service Date], "&lt;="&amp;TODAY()+30, #REF!, FALSE)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1129,8 +1144,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{F579DA07-7AD6-49DA-9B44-D5B1132EDAC6}" name="Overhead_Summary" displayName="Overhead_Summary" ref="A9:B21" totalsRowShown="0">
   <autoFilter ref="A9:B21" xr:uid="{F579DA07-7AD6-49DA-9B44-D5B1132EDAC6}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{7CA4839C-9603-479D-BD1C-8377DFA9603C}" name="Expense Category" dataDxfId="102"/>
-    <tableColumn id="2" xr3:uid="{FE0F7616-EAF3-443D-AC69-DE6541DC10E5}" name="Annual Total" dataDxfId="101">
+    <tableColumn id="1" xr3:uid="{7CA4839C-9603-479D-BD1C-8377DFA9603C}" name="Expense Category" dataDxfId="107"/>
+    <tableColumn id="2" xr3:uid="{FE0F7616-EAF3-443D-AC69-DE6541DC10E5}" name="Annual Total" dataDxfId="106">
       <calculatedColumnFormula>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1139,101 +1154,105 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:N2" totalsRowShown="0" headerRowDxfId="100" dataDxfId="99">
-  <autoFilter ref="A1:N2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}"/>
-  <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="98"/>
-    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="97"/>
-    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="96"/>
-    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="95"/>
-    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="94"/>
-    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="93"/>
-    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="92"/>
-    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="91">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:O2" totalsRowShown="0" headerRowDxfId="105" dataDxfId="104">
+  <autoFilter ref="A1:O2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}"/>
+  <tableColumns count="15">
+    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="103"/>
+    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="102"/>
+    <tableColumn id="15" xr3:uid="{D25A390C-69B5-4326-A0D4-10EB45DDE5E5}" name="Tag_ID" dataDxfId="25"/>
+    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="101"/>
+    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="100"/>
+    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="99"/>
+    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="98"/>
+    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="97"/>
+    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="96">
       <calculatedColumnFormula>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="90"/>
-    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="89"/>
-    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="88"/>
-    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="87"/>
-    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="86"/>
-    <tableColumn id="13" xr3:uid="{885B08CA-5BC3-4FAA-B661-BE5CCBF87448}" name="Sold" dataDxfId="85"/>
+    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="95"/>
+    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="94"/>
+    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="93"/>
+    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="92"/>
+    <tableColumn id="16" xr3:uid="{CA8F9851-44B9-4614-9963-24D4EC145034}" name="Sold" dataDxfId="21"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:J2" insertRow="1" totalsRowShown="0" headerRowDxfId="84" dataDxfId="83">
-  <autoFilter ref="A1:J2" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}"/>
-  <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="82"/>
-    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="81"/>
-    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Brand/Model" dataDxfId="80"/>
-    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="79"/>
-    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="78"/>
-    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="77"/>
-    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="76"/>
-    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="75"/>
-    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="74"/>
-    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="73"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="91" dataDxfId="90">
+  <autoFilter ref="A1:K2" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="89"/>
+    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="88"/>
+    <tableColumn id="4" xr3:uid="{17EB0B09-11B3-4E08-9442-E3C9AB87A157}" name="Tag_ID" dataDxfId="24"/>
+    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="20"/>
+    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Brand/Model" dataDxfId="87"/>
+    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="86"/>
+    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="85"/>
+    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="84"/>
+    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="83"/>
+    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="82"/>
+    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="81"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:K2" totalsRowShown="0" headerRowDxfId="72" dataDxfId="71">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:K2" totalsRowShown="0" headerRowDxfId="80" dataDxfId="79">
   <autoFilter ref="A1:K2" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="70"/>
-    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="69"/>
-    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="68"/>
-    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="67"/>
-    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="66"/>
-    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="65"/>
-    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="64"/>
-    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="63"/>
-    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="62"/>
-    <tableColumn id="9" xr3:uid="{C040B253-9925-4664-88EB-44A0F3B09681}" name="Complete" dataDxfId="61"/>
-    <tableColumn id="12" xr3:uid="{920CB592-D743-4B33-A796-C7F3DB32211C}" name="Remarks" dataDxfId="60"/>
+    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="78"/>
+    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="77"/>
+    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="76"/>
+    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="75"/>
+    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="74"/>
+    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="73"/>
+    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="72"/>
+    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="71"/>
+    <tableColumn id="11" xr3:uid="{4809319D-ABCA-43DA-A400-5DC91167D78B}" name="Complete" dataDxfId="7"/>
+    <tableColumn id="12" xr3:uid="{920CB592-D743-4B33-A796-C7F3DB32211C}" name="Remarks" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:J2" totalsRowShown="0" headerRowDxfId="59" dataDxfId="58">
-  <autoFilter ref="A1:J2" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}"/>
-  <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="57"/>
-    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="56"/>
-    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Brand/Model" dataDxfId="55"/>
-    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="54"/>
-    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="53"/>
-    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="52"/>
-    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="51"/>
-    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="50"/>
-    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="49"/>
-    <tableColumn id="10" xr3:uid="{26197E01-2936-4F5F-8081-3AA351C1CD38}" name="Remarks" dataDxfId="48"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:K2" totalsRowShown="0" headerRowDxfId="70" dataDxfId="69">
+  <autoFilter ref="A1:K2" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="68"/>
+    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="67"/>
+    <tableColumn id="11" xr3:uid="{21951C81-00A4-4344-9E81-B1B1DB06ADEF}" name="Tag_ID" dataDxfId="23"/>
+    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Brand/Model" dataDxfId="66"/>
+    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="65"/>
+    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="64"/>
+    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="63"/>
+    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="62"/>
+    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="61"/>
+    <tableColumn id="10" xr3:uid="{26197E01-2936-4F5F-8081-3AA351C1CD38}" name="Remarks" dataDxfId="60"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:I2" totalsRowShown="0" headerRowDxfId="47" dataDxfId="46">
-  <autoFilter ref="A1:I2" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}"/>
-  <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="45"/>
-    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="44"/>
-    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Brand/Model/Description" dataDxfId="43"/>
-    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="42"/>
-    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="41"/>
-    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="40"/>
-    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="39"/>
-    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="38"/>
-    <tableColumn id="9" xr3:uid="{2B57F5E6-66C5-4DBA-8949-836DE0F0791C}" name="Remarks" dataDxfId="37"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:J2" totalsRowShown="0" headerRowDxfId="59" dataDxfId="58">
+  <autoFilter ref="A1:J2" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}"/>
+  <tableColumns count="10">
+    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="57"/>
+    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="56"/>
+    <tableColumn id="10" xr3:uid="{C8BD69AA-9023-4777-9C96-39A81F1E4BE0}" name="Tag_ID" dataDxfId="10"/>
+    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Brand/Model/Description" dataDxfId="12"/>
+    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="13"/>
+    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="14"/>
+    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="17"/>
+    <tableColumn id="9" xr3:uid="{2B57F5E6-66C5-4DBA-8949-836DE0F0791C}" name="Remarks" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1643,7 +1662,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B5" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C5" s="8">
         <v>1000</v>
@@ -1672,67 +1691,79 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E1902F1-C59B-4A1A-9D95-2C39AEF944E5}">
   <sheetPr codeName="Sheet7"/>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
-    <col min="2" max="2" width="41.6640625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="18.44140625" style="14" customWidth="1"/>
-    <col min="4" max="4" width="18.44140625" style="2" customWidth="1"/>
-    <col min="5" max="5" width="15.5546875" style="2" customWidth="1"/>
-    <col min="6" max="6" width="14.33203125" style="7" customWidth="1"/>
-    <col min="7" max="7" width="14.109375" style="7" customWidth="1"/>
-    <col min="8" max="8" width="10.44140625" style="3" customWidth="1"/>
-    <col min="9" max="9" width="22.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="22.6640625" style="2" customWidth="1"/>
-    <col min="11" max="11" width="46.6640625" style="2" customWidth="1"/>
-    <col min="12" max="16384" width="8.88671875" style="6"/>
+    <col min="2" max="2" width="10.33203125" style="14" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.33203125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="22.6640625" style="17" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="41.6640625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="18.44140625" style="2" customWidth="1"/>
+    <col min="8" max="8" width="15.5546875" style="2" customWidth="1"/>
+    <col min="9" max="9" width="14.33203125" style="7" customWidth="1"/>
+    <col min="10" max="10" width="14.109375" style="7" customWidth="1"/>
+    <col min="11" max="11" width="10.44140625" style="3" customWidth="1"/>
+    <col min="13" max="13" width="22.6640625" style="2" customWidth="1"/>
+    <col min="14" max="14" width="46.6640625" style="2" customWidth="1"/>
+    <col min="15" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C1" s="15" t="s">
+        <v>94</v>
+      </c>
+      <c r="D1" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="E1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="D1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="H1" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="G1" s="8" t="s">
+      <c r="I1" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="J1" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="I2" s="3">
+      <c r="L1" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="M1" s="6"/>
+      <c r="N1" s="6"/>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="F2" s="2"/>
+      <c r="H2" s="7"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3">
         <f>Shop_Consumables[[#This Row],[Current Stock]]*Shop_Consumables[[#This Row],[Unit Cost]]</f>
         <v>0</v>
       </c>
+      <c r="L2" s="2"/>
+      <c r="M2" s="6"/>
+      <c r="N2" s="6"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2" xr:uid="{D2C605E8-D02B-4558-82DE-3169088704E8}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2" xr:uid="{D2C605E8-D02B-4558-82DE-3169088704E8}">
       <formula1>"Fasteners/Hardware,Abrasives/Cutting,Fluids/Lubricants/Chemicals,Primer/Paint,Safety/PPE,Shop/Janitorial,Welding,Electrical,Other"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1783,7 +1814,7 @@
         <v>32</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I1" s="6"/>
     </row>
@@ -1861,31 +1892,48 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6A08BCD-5A8C-45EE-A940-2FEFA1E5B102}">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
-    <col min="2" max="2" width="15.6640625" style="4" customWidth="1"/>
+    <col min="2" max="2" width="15.6640625" style="16" customWidth="1"/>
     <col min="3" max="3" width="27.44140625" style="4" customWidth="1"/>
-    <col min="4" max="4" width="21.6640625" style="4" customWidth="1"/>
-    <col min="5" max="5" width="30" style="4" customWidth="1"/>
+    <col min="4" max="4" width="21.6640625" style="16" customWidth="1"/>
+    <col min="5" max="5" width="30" style="16" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="16" t="s">
         <v>57</v>
       </c>
       <c r="C1" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="E1" s="4" t="s">
-        <v>60</v>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B2" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D2" s="16" t="s">
+        <v>97</v>
+      </c>
+      <c r="E2" s="16" t="s">
+        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -1957,37 +2005,37 @@
         <v>0</v>
       </c>
       <c r="B1" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="D1" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="H1" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="D1" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="F1" s="5" t="s">
+      <c r="I1" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="J1" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="G1" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="I1" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>72</v>
-      </c>
       <c r="K1" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="L1" s="8" t="s">
         <v>86</v>
-      </c>
-      <c r="L1" s="8" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
@@ -2035,9 +2083,9 @@
 )</f>
         <v>0</v>
       </c>
-      <c r="L2" s="7">
-        <f ca="1">COUNTIFS(Maintenance_Log[Next Service Date], "&lt;="&amp;TODAY()+30, Maintenance_Log[Complete], FALSE)</f>
-        <v>0</v>
+      <c r="L2" s="7" t="e">
+        <f ca="1">COUNTIFS(Maintenance_Log[Next Service Date], "&lt;="&amp;TODAY()+30, #REF!, FALSE)</f>
+        <v>#REF!</v>
       </c>
     </row>
   </sheetData>
@@ -2064,12 +2112,12 @@
         <v>27</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B10" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2078,7 +2126,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B11" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2087,7 +2135,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B12" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2096,7 +2144,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B13" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2105,7 +2153,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B14" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2114,7 +2162,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B15" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2123,7 +2171,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B16" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2132,7 +2180,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B17" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2141,7 +2189,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B18" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2150,7 +2198,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B19" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2159,7 +2207,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B20" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2168,7 +2216,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B21" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2191,92 +2239,99 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDE7BF89-A2E7-4A6F-B822-317739E206EC}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:R2"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
     <col min="2" max="2" width="9.5546875" style="14" customWidth="1"/>
-    <col min="3" max="3" width="31.44140625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="10.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17" style="10" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.33203125" style="3" customWidth="1"/>
-    <col min="7" max="7" width="16.5546875" style="3" customWidth="1"/>
-    <col min="8" max="8" width="16.6640625" style="5" customWidth="1"/>
-    <col min="9" max="9" width="19.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.6640625" style="3" customWidth="1"/>
-    <col min="11" max="11" width="16.88671875" style="3" customWidth="1"/>
-    <col min="12" max="12" width="16.88671875" style="14" customWidth="1"/>
-    <col min="13" max="13" width="12.88671875" style="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="7" style="2" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="16.88671875" style="2" customWidth="1"/>
-    <col min="16" max="16384" width="8.88671875" style="6"/>
+    <col min="3" max="3" width="9.5546875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="12.88671875" style="16" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="31.44140625" style="2" customWidth="1"/>
+    <col min="6" max="6" width="10.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17" style="10" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.33203125" style="3" customWidth="1"/>
+    <col min="9" max="9" width="16.5546875" style="3" customWidth="1"/>
+    <col min="10" max="10" width="16.6640625" style="5" customWidth="1"/>
+    <col min="11" max="11" width="19.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.6640625" style="3" customWidth="1"/>
+    <col min="13" max="13" width="16.88671875" style="3" customWidth="1"/>
+    <col min="14" max="14" width="16.88671875" style="14" customWidth="1"/>
+    <col min="16" max="16" width="12.88671875" style="16" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.88671875" style="17" customWidth="1"/>
+    <col min="18" max="18" width="16.88671875" style="2" customWidth="1"/>
+    <col min="19" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="15" t="s">
+        <v>94</v>
+      </c>
+      <c r="D1" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="E1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="G1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="K1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="L1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="M1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="N1" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="O1" s="6"/>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="H2" s="5">
+      <c r="O1" s="18" t="s">
+        <v>87</v>
+      </c>
+      <c r="P1" s="6"/>
+      <c r="Q1" s="6"/>
+      <c r="R1" s="6"/>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="D2" s="17"/>
+      <c r="J2" s="5">
         <f>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</f>
         <v>0</v>
       </c>
-      <c r="M2" s="2"/>
-      <c r="N2" s="15" t="b">
-        <v>0</v>
-      </c>
-      <c r="O2" s="6"/>
+      <c r="O2" s="17"/>
+      <c r="P2" s="6"/>
+      <c r="Q2" s="6"/>
+      <c r="R2" s="6"/>
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I3:I1000" xr:uid="{F45414DD-76C8-4DC4-96E2-15B89FDB5B51}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K3:K1000" xr:uid="{F45414DD-76C8-4DC4-96E2-15B89FDB5B51}">
       <formula1>"work not started, restoration in progress, for sale, sold"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2" xr:uid="{C1AA0387-29B3-4797-A152-88A8C024D825}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2" xr:uid="{C1AA0387-29B3-4797-A152-88A8C024D825}">
       <formula1>"Machinery, Furniture, Electronics, Craft, Auto Related, Other"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2" xr:uid="{3C9AD8AD-AB10-403F-A04B-87B1D7C9B98E}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2" xr:uid="{3C9AD8AD-AB10-403F-A04B-87B1D7C9B98E}">
       <formula1>"Not Started, In-Progress, Complete, For Sale, Sold"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2291,60 +2346,70 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B027EC69-551F-4051-8A71-8B106D207C6D}">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
     <col min="2" max="2" width="9.5546875" style="14" customWidth="1"/>
-    <col min="3" max="3" width="28.6640625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="14.88671875" style="2" customWidth="1"/>
-    <col min="5" max="5" width="14.6640625" style="10" customWidth="1"/>
-    <col min="6" max="6" width="14.6640625" style="3" customWidth="1"/>
-    <col min="7" max="7" width="12.33203125" style="14" customWidth="1"/>
-    <col min="8" max="8" width="12.33203125" style="2" customWidth="1"/>
-    <col min="9" max="9" width="11.44140625" style="6" customWidth="1"/>
-    <col min="10" max="10" width="32.6640625" style="2" customWidth="1"/>
-    <col min="11" max="16384" width="8.88671875" style="6"/>
+    <col min="3" max="3" width="9.5546875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="12.33203125" style="17" customWidth="1"/>
+    <col min="5" max="5" width="28.6640625" style="2" customWidth="1"/>
+    <col min="6" max="6" width="14.88671875" style="2" customWidth="1"/>
+    <col min="7" max="7" width="14.6640625" style="10" customWidth="1"/>
+    <col min="8" max="8" width="14.6640625" style="3" customWidth="1"/>
+    <col min="9" max="9" width="12.33203125" style="14" customWidth="1"/>
+    <col min="11" max="11" width="11.44140625" style="6" customWidth="1"/>
+    <col min="12" max="12" width="32.6640625" style="2" customWidth="1"/>
+    <col min="13" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="D1" s="4" t="s">
+      <c r="C1" s="15" t="s">
+        <v>94</v>
+      </c>
+      <c r="D1" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="G1" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="H1" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>21</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="K1" s="4" t="s">
         <v>52</v>
       </c>
+      <c r="L1" s="6"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="J2" s="6"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="6"/>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I3:I1000" xr:uid="{D25ACF8B-D3DC-4EFD-9C68-FC99372E0DCF}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K3:K1000" xr:uid="{D25ACF8B-D3DC-4EFD-9C68-FC99372E0DCF}">
       <formula1>"Operational, Needs Repair, Unusable"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2" xr:uid="{4B2064CB-79C2-427D-B2C2-7CE85187D094}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2" xr:uid="{4B2064CB-79C2-427D-B2C2-7CE85187D094}">
       <formula1>"Operational, Needs Repair, Repair In-Progress, Unusable/Junk"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2370,7 +2435,7 @@
     <col min="7" max="7" width="14.33203125" style="6" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="7" style="3" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="18" style="9" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18" style="4" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.44140625" style="16" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="18" style="2" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="13.44140625" style="2" customWidth="1"/>
     <col min="13" max="13" width="9.88671875" style="3" customWidth="1"/>
@@ -2388,7 +2453,7 @@
         <v>1</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E1" s="9" t="s">
         <v>16</v>
@@ -2405,20 +2470,18 @@
       <c r="I1" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="K1" s="4" t="s">
         <v>90</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>91</v>
       </c>
       <c r="L1" s="6"/>
       <c r="M1" s="6"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="I2" s="10"/>
-      <c r="J2" s="15" t="b">
-        <v>0</v>
-      </c>
+      <c r="J2" s="17"/>
       <c r="L2" s="6"/>
       <c r="M2" s="6"/>
     </row>
@@ -2444,80 +2507,84 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEDDDAA7-75C3-4AA5-ABFD-D5FB4C627E4C}">
   <sheetPr codeName="Sheet5"/>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
     <col min="2" max="2" width="8.6640625" style="14" customWidth="1"/>
-    <col min="3" max="3" width="50.44140625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="15.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.88671875" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.88671875" style="6" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.88671875" style="6" customWidth="1"/>
-    <col min="8" max="8" width="14.44140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.5546875" style="6" customWidth="1"/>
-    <col min="11" max="11" width="14.44140625" style="2" customWidth="1"/>
-    <col min="12" max="16384" width="8.88671875" style="6"/>
+    <col min="3" max="3" width="8.6640625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="12.88671875" style="17" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="50.44140625" style="2" customWidth="1"/>
+    <col min="6" max="6" width="15.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.88671875" style="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.88671875" style="6" customWidth="1"/>
+    <col min="10" max="10" width="14.44140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.5546875" style="6" customWidth="1"/>
+    <col min="13" max="13" width="14.44140625" style="2" customWidth="1"/>
+    <col min="14" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="D1" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C1" s="15" t="s">
+        <v>94</v>
+      </c>
+      <c r="D1" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>53</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>54</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>55</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>21</v>
       </c>
-      <c r="J1" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="K1" s="6"/>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="I2" s="6"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="6"/>
+      <c r="K1" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="M1" s="6"/>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="G2" s="6"/>
+      <c r="K2" s="2"/>
+      <c r="M2" s="6"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <dataValidations count="6">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K3:K1000 F3:H1000" xr:uid="{FF61F80C-5E23-45D6-B39D-7C5635258115}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M3:M1000 H3:J1000" xr:uid="{FF61F80C-5E23-45D6-B39D-7C5635258115}">
       <formula1>"Circular Saw, Drill, Sander, Grinder, Other"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J3:K1000" xr:uid="{DB752B4D-0E75-42D1-B907-2DBC5792F422}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L3:M1000" xr:uid="{DB752B4D-0E75-42D1-B907-2DBC5792F422}">
       <formula1>"New, Operational, Needs Repair, Broken"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2" xr:uid="{05EFC744-2B0C-453D-A1B6-F8391608434D}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2" xr:uid="{05EFC744-2B0C-453D-A1B6-F8391608434D}">
       <formula1>"Drilling, Cutting, Grinding, Sanding, Fastening, Shaping/Routing, Other"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2" xr:uid="{194EFB2B-690A-4D50-8AF6-E8ED45FE2FCA}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2" xr:uid="{194EFB2B-690A-4D50-8AF6-E8ED45FE2FCA}">
       <formula1>"Portable/Handheld, Stationary/Bench Top, Outdoor Power Equipment, "</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:J2" xr:uid="{980AB122-9104-490B-993D-4F2FEF3A4EE6}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:K2" xr:uid="{980AB122-9104-490B-993D-4F2FEF3A4EE6}">
       <formula1>"Operational, Needs Repair, Repair In-Progress, Unusable/Junk"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2 J2" xr:uid="{47F6EF9A-B127-4EB7-A5E8-0075055489DC}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2 K2" xr:uid="{47F6EF9A-B127-4EB7-A5E8-0075055489DC}">
       <formula1>"Corded(A/C), Cordless/Battery, Pneumatic/Air, Fuel-Powered"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2531,66 +2598,73 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F39ADDA6-CD5F-4655-A9C0-9676DDAC362E}">
   <sheetPr codeName="Sheet6"/>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.6640625" style="14" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="54.6640625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="15.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.5546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.88671875" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.88671875" style="2" customWidth="1"/>
-    <col min="8" max="8" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.33203125" style="7" customWidth="1"/>
-    <col min="10" max="10" width="12.88671875" style="2" customWidth="1"/>
-    <col min="11" max="16384" width="8.88671875" style="6"/>
+    <col min="3" max="3" width="8.6640625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="12.88671875" style="17" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="54.6640625" style="2" customWidth="1"/>
+    <col min="6" max="6" width="15.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.5546875" style="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.88671875" style="16"/>
+    <col min="9" max="9" width="12.88671875" style="17" customWidth="1"/>
+    <col min="10" max="10" width="10.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.33203125" style="7" customWidth="1"/>
+    <col min="12" max="12" width="12.88671875" style="2" customWidth="1"/>
+    <col min="13" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="D1" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C1" s="15" t="s">
+        <v>94</v>
+      </c>
+      <c r="D1" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="G1" s="4" t="s">
+      <c r="H1" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="I1" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="I1" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="J1" s="6"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="H2" s="7"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="6"/>
+      <c r="J1" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="K1" s="6"/>
+      <c r="L1" s="6"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="H2" s="17"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="6"/>
+      <c r="L2" s="6"/>
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J3:J1000 E3:G1000" xr:uid="{B6CB3C84-EE01-4878-B558-650FC19D8248}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L3:L1000 D3:D1000 G3:G1000 I3:I1000" xr:uid="{B6CB3C84-EE01-4878-B558-650FC19D8248}">
       <formula1>"Saw, Hammer, Screwdriver, Wrench, Sockets, Pliers, Measuring, Files, Other"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2" xr:uid="{ACB7A40B-F0EE-4387-88E4-5140AB68313F}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2" xr:uid="{ACB7A40B-F0EE-4387-88E4-5140AB68313F}">
       <formula1>"Fastening/Turning,Measuring/Layout,Striking/Hammering,Gripping/Holding,Cutting/Shaping,Other"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2 I2" xr:uid="{2E543736-2E6D-4F90-9169-21BA7CCD7676}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2 J2" xr:uid="{2E543736-2E6D-4F90-9169-21BA7CCD7676}">
       <formula1>"Operational,Needs Repair,Repair In-Progress,Unusable/Junk"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
typo fix in excel
</commit_message>
<xml_diff>
--- a/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
+++ b/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1a2ae81d67634e6/Desktop/Michanikos Artifex Enterprises/MAE Custom Digital Solutions/MAE Workshop Inventory Management System/GITHUB_MAE_Workshop Inventory App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="183" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4B633391-06E1-4FCF-962D-CCDA56611818}"/>
+  <xr:revisionPtr revIDLastSave="187" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B35E8C10-1828-4F40-A5B8-1C2E59C6C577}"/>
   <bookViews>
-    <workbookView xWindow="2052" yWindow="648" windowWidth="11844" windowHeight="11904" firstSheet="11" activeTab="12" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
+    <workbookView xWindow="2052" yWindow="336" windowWidth="11844" windowHeight="11904" firstSheet="4" activeTab="2" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
   </bookViews>
   <sheets>
     <sheet name="TEST Inventory" sheetId="10" r:id="rId1"/>
@@ -379,7 +379,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -398,6 +398,11 @@
       <color theme="1"/>
       <name val="Aptos"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0A0A0A"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="2">
@@ -420,7 +425,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
       <protection hidden="1"/>
@@ -454,32 +459,230 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
       <protection locked="0" hidden="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
-      <protection locked="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="129">
+  <dxfs count="128">
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -491,13 +694,73 @@
       </extLst>
     </dxf>
     <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="0"/>
     </dxf>
@@ -510,307 +773,22 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
       <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -853,6 +831,14 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="1"/>
     </dxf>
@@ -871,32 +857,6 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
@@ -961,6 +921,44 @@
     <dxf>
       <protection locked="1" hidden="0"/>
     </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -991,15 +989,19 @@
 </FeaturePropertyBags>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}" name="TEST_Inventory" displayName="TEST_Inventory" ref="A1:F5" totalsRowShown="0">
   <autoFilter ref="A1:F5" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="114"/>
-    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="113"/>
-    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="112"/>
-    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="111"/>
-    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="110">
+    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="122"/>
+    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="121"/>
+    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="120"/>
+    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="119"/>
+    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="118">
       <calculatedColumnFormula>TEST_Inventory[[#This Row],[TEST Integer]]*TEST_Inventory[[#This Row],[TEST Currency]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{AB3A5F3C-FCF0-4466-90FD-8ABB6E18DF5C}" name="TEST Dropdown"/>
@@ -1009,56 +1011,56 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:L2" totalsRowShown="0" headerRowDxfId="55" dataDxfId="54">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:L2" totalsRowShown="0" headerRowDxfId="32" dataDxfId="31">
   <autoFilter ref="A1:L2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="53"/>
-    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="22"/>
-    <tableColumn id="12" xr3:uid="{8F0FD29C-682B-41B4-82F2-913D40801887}" name="Tag_ID" dataDxfId="8"/>
-    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="52"/>
-    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="51"/>
-    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="50"/>
-    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="49"/>
-    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="48"/>
-    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="47"/>
-    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="46">
+    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="30"/>
+    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="29"/>
+    <tableColumn id="12" xr3:uid="{8F0FD29C-682B-41B4-82F2-913D40801887}" name="Tag_ID" dataDxfId="28"/>
+    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="27"/>
+    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="26"/>
+    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="25"/>
+    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="24"/>
+    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="23"/>
+    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="22"/>
+    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="21"/>
+    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="20">
       <calculatedColumnFormula>Shop_Consumables[[#This Row],[Current Stock]]*Shop_Consumables[[#This Row],[Unit Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Supplier/Remarks" dataDxfId="45"/>
+    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Supplier/Remarks" dataDxfId="19"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:H2" totalsRowShown="0" headerRowDxfId="44" dataDxfId="43">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:H2" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
   <autoFilter ref="A1:H2" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="42"/>
-    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="41"/>
-    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="40"/>
-    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="39"/>
-    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="38"/>
-    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="37"/>
-    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="36"/>
-    <tableColumn id="8" xr3:uid="{9140C4E8-CB9E-40BF-ABD9-13A971322B09}" name="Remarks" dataDxfId="35"/>
+    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="12"/>
+    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="11"/>
+    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="10"/>
+    <tableColumn id="8" xr3:uid="{9140C4E8-CB9E-40BF-ABD9-13A971322B09}" name="Remarks" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="34" dataDxfId="33">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
   <autoFilter ref="A1:G2" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="32"/>
-    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="31"/>
-    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="30"/>
-    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="29"/>
-    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="28"/>
-    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="27"/>
-    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="26"/>
+    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="6"/>
+    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="4"/>
+    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="2"/>
+    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="1"/>
+    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1068,11 +1070,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}" name="Location" displayName="Location" ref="A1:E2" totalsRowShown="0">
   <autoFilter ref="A1:E2" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="3"/>
-    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Description" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="127"/>
+    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="126"/>
+    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Description" dataDxfId="125"/>
+    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="124"/>
+    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="123"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1082,10 +1084,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}" name="TEST_Dashboard" displayName="TEST_Dashboard" ref="A1:B2" totalsRowShown="0">
   <autoFilter ref="A1:B2" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="109">
+    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="117">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Currency])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="108">
+    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="116">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Integer])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1094,46 +1096,46 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:L2" totalsRowShown="0" headerRowDxfId="128" dataDxfId="127">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:L2" totalsRowShown="0" headerRowDxfId="115" dataDxfId="114">
   <autoFilter ref="A1:L2" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="126"/>
-    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="125">
+    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="113"/>
+    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="112">
       <calculatedColumnFormula>SUM(Resell_Inventory[Total Investment])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="124">
+    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="111">
       <calculatedColumnFormula>SUM(Resell_Inventory[Actual Sale Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="123">
+    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="110">
       <calculatedColumnFormula>SUM(Shop_Machinery[Purchase Cost])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="122">
+    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="109">
       <calculatedColumnFormula>SUM(Shop_Power_Tools[Purchase Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="121">
+    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="108">
       <calculatedColumnFormula>SUM(Shop_Hand_Tools[Purchase Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="120">
+    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="107">
       <calculatedColumnFormula>SUM(Shop_Consumables[Current Inventory Value])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="119">
+    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="106">
       <calculatedColumnFormula>SUM(D2,E2,F2,G2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="118">
+    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="105">
       <calculatedColumnFormula array="1">SUMPRODUCT(--(Shop_Consumables[Current Stock]&lt;=Shop_Consumables[Reorder Point]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="117">
+    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="104">
       <calculatedColumnFormula>SUMIFS(Shop_Overhead[Amount], Shop_Overhead[Due Date], "&lt;="&amp;TODAY()+30, Shop_Overhead[Due Date], "&gt;="&amp;TODAY())</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{E4065760-B1B1-4564-936B-3405D3B80297}" name="Equipment With Operational Issues" dataDxfId="116">
+    <tableColumn id="12" xr3:uid="{E4065760-B1B1-4564-936B-3405D3B80297}" name="Equipment With Operational Issues" dataDxfId="103">
       <calculatedColumnFormula array="1">SUM(
   COUNTIFS(Shop_Machinery[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"}),
   COUNTIFS(Shop_Power_Tools[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"}),
   COUNTIFS(Shop_Hand_Tools[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"})
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{86A5DBCB-1064-4926-8405-405B453A4546}" name="Maintenance Items Due in Next 30 Days" dataDxfId="115">
-      <calculatedColumnFormula>COUNTIFS(Maintenance_Log[Next Service Date], "&lt;="&amp;TODAY()+30, #REF!, FALSE)</calculatedColumnFormula>
+    <tableColumn id="6" xr3:uid="{86A5DBCB-1064-4926-8405-405B453A4546}" name="Maintenance Items Due in Next 30 Days">
+      <calculatedColumnFormula>COUNTIFS(Maintenance_Log[Next Service Date], "&lt;="&amp;TODAY()+30, Maintenance_Log[Complete], FALSE)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1144,8 +1146,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{F579DA07-7AD6-49DA-9B44-D5B1132EDAC6}" name="Overhead_Summary" displayName="Overhead_Summary" ref="A9:B21" totalsRowShown="0">
   <autoFilter ref="A9:B21" xr:uid="{F579DA07-7AD6-49DA-9B44-D5B1132EDAC6}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{7CA4839C-9603-479D-BD1C-8377DFA9603C}" name="Expense Category" dataDxfId="107"/>
-    <tableColumn id="2" xr3:uid="{FE0F7616-EAF3-443D-AC69-DE6541DC10E5}" name="Annual Total" dataDxfId="106">
+    <tableColumn id="1" xr3:uid="{7CA4839C-9603-479D-BD1C-8377DFA9603C}" name="Expense Category" dataDxfId="102"/>
+    <tableColumn id="2" xr3:uid="{FE0F7616-EAF3-443D-AC69-DE6541DC10E5}" name="Annual Total" dataDxfId="101">
       <calculatedColumnFormula>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1154,105 +1156,105 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:O2" totalsRowShown="0" headerRowDxfId="105" dataDxfId="104">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:O2" totalsRowShown="0" headerRowDxfId="100" dataDxfId="99">
   <autoFilter ref="A1:O2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}"/>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="103"/>
-    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="102"/>
-    <tableColumn id="15" xr3:uid="{D25A390C-69B5-4326-A0D4-10EB45DDE5E5}" name="Tag_ID" dataDxfId="25"/>
-    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="19"/>
-    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="101"/>
-    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="100"/>
-    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="99"/>
-    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="98"/>
-    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="97"/>
-    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="96">
+    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="98"/>
+    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="97"/>
+    <tableColumn id="15" xr3:uid="{D25A390C-69B5-4326-A0D4-10EB45DDE5E5}" name="Tag_ID" dataDxfId="96"/>
+    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="95"/>
+    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="94"/>
+    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="93"/>
+    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="92"/>
+    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="91"/>
+    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="90"/>
+    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="89">
       <calculatedColumnFormula>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="95"/>
-    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="94"/>
-    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="93"/>
-    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="92"/>
-    <tableColumn id="16" xr3:uid="{CA8F9851-44B9-4614-9963-24D4EC145034}" name="Sold" dataDxfId="21"/>
+    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="88"/>
+    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="87"/>
+    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="86"/>
+    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="85"/>
+    <tableColumn id="16" xr3:uid="{CA8F9851-44B9-4614-9963-24D4EC145034}" name="Sold" dataDxfId="84"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="91" dataDxfId="90">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="83" dataDxfId="82">
   <autoFilter ref="A1:K2" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="89"/>
-    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="88"/>
-    <tableColumn id="4" xr3:uid="{17EB0B09-11B3-4E08-9442-E3C9AB87A157}" name="Tag_ID" dataDxfId="24"/>
-    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="20"/>
-    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Brand/Model" dataDxfId="87"/>
-    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="86"/>
-    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="85"/>
-    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="84"/>
-    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="83"/>
-    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="82"/>
-    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="81"/>
+    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="81"/>
+    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="80"/>
+    <tableColumn id="4" xr3:uid="{17EB0B09-11B3-4E08-9442-E3C9AB87A157}" name="Tag_ID" dataDxfId="79"/>
+    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="78"/>
+    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Brand/Model" dataDxfId="77"/>
+    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="76"/>
+    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="75"/>
+    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="74"/>
+    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="73"/>
+    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="72"/>
+    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="71"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:K2" totalsRowShown="0" headerRowDxfId="80" dataDxfId="79">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:K2" totalsRowShown="0" headerRowDxfId="70" dataDxfId="69">
   <autoFilter ref="A1:K2" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="78"/>
-    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="77"/>
-    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="76"/>
-    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="75"/>
-    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="74"/>
-    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="6"/>
-    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="73"/>
-    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="72"/>
-    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="71"/>
-    <tableColumn id="11" xr3:uid="{4809319D-ABCA-43DA-A400-5DC91167D78B}" name="Complete" dataDxfId="7"/>
-    <tableColumn id="12" xr3:uid="{920CB592-D743-4B33-A796-C7F3DB32211C}" name="Remarks" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="68"/>
+    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="67"/>
+    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="66"/>
+    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="65"/>
+    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="64"/>
+    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="63"/>
+    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="62"/>
+    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="61"/>
+    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="60"/>
+    <tableColumn id="11" xr3:uid="{4809319D-ABCA-43DA-A400-5DC91167D78B}" name="Complete" dataDxfId="59"/>
+    <tableColumn id="12" xr3:uid="{920CB592-D743-4B33-A796-C7F3DB32211C}" name="Remarks" dataDxfId="58"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:K2" totalsRowShown="0" headerRowDxfId="70" dataDxfId="69">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:K2" totalsRowShown="0" headerRowDxfId="57" dataDxfId="56">
   <autoFilter ref="A1:K2" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="68"/>
-    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="67"/>
-    <tableColumn id="11" xr3:uid="{21951C81-00A4-4344-9E81-B1B1DB06ADEF}" name="Tag_ID" dataDxfId="23"/>
-    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="18"/>
-    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Brand/Model" dataDxfId="66"/>
-    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="65"/>
-    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="64"/>
-    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="63"/>
-    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="62"/>
-    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="61"/>
-    <tableColumn id="10" xr3:uid="{26197E01-2936-4F5F-8081-3AA351C1CD38}" name="Remarks" dataDxfId="60"/>
+    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="55"/>
+    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="54"/>
+    <tableColumn id="11" xr3:uid="{21951C81-00A4-4344-9E81-B1B1DB06ADEF}" name="Tag_ID" dataDxfId="53"/>
+    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="52"/>
+    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Brand/Model" dataDxfId="51"/>
+    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="50"/>
+    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="49"/>
+    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="48"/>
+    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="47"/>
+    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="46"/>
+    <tableColumn id="10" xr3:uid="{26197E01-2936-4F5F-8081-3AA351C1CD38}" name="Remarks" dataDxfId="45"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:J2" totalsRowShown="0" headerRowDxfId="59" dataDxfId="58">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:J2" totalsRowShown="0" headerRowDxfId="44" dataDxfId="43">
   <autoFilter ref="A1:J2" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="57"/>
-    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="56"/>
-    <tableColumn id="10" xr3:uid="{C8BD69AA-9023-4777-9C96-39A81F1E4BE0}" name="Tag_ID" dataDxfId="10"/>
-    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Brand/Model/Description" dataDxfId="12"/>
-    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="13"/>
-    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="14"/>
-    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="15"/>
-    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="17"/>
-    <tableColumn id="9" xr3:uid="{2B57F5E6-66C5-4DBA-8949-836DE0F0791C}" name="Remarks" dataDxfId="16"/>
+    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="42"/>
+    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="41"/>
+    <tableColumn id="10" xr3:uid="{C8BD69AA-9023-4777-9C96-39A81F1E4BE0}" name="Tag_ID" dataDxfId="40"/>
+    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="39"/>
+    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Brand/Model/Description" dataDxfId="38"/>
+    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="37"/>
+    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="36"/>
+    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="35"/>
+    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="34"/>
+    <tableColumn id="9" xr3:uid="{2B57F5E6-66C5-4DBA-8949-836DE0F0791C}" name="Remarks" dataDxfId="33"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1576,7 +1578,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19832549-C5E9-4018-9E8B-E2F74EABCB4B}">
   <dimension ref="A1:F5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
     <col min="2" max="2" width="12" style="4" customWidth="1"/>
@@ -1586,7 +1588,7 @@
     <col min="6" max="6" width="15.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1606,7 +1608,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6">
       <c r="B2" s="4" t="s">
         <v>42</v>
       </c>
@@ -1624,7 +1626,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6">
       <c r="B3" s="4" t="s">
         <v>44</v>
       </c>
@@ -1642,7 +1644,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6">
       <c r="B4" s="4" t="s">
         <v>46</v>
       </c>
@@ -1660,7 +1662,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6">
       <c r="B5" s="4" t="s">
         <v>62</v>
       </c>
@@ -1692,12 +1694,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E1902F1-C59B-4A1A-9D95-2C39AEF944E5}">
   <sheetPr codeName="Sheet7"/>
   <dimension ref="A1:N2"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
     <col min="2" max="2" width="10.33203125" style="14" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.33203125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="22.6640625" style="17" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.6640625" style="6" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="41.6640625" style="2" customWidth="1"/>
     <col min="7" max="7" width="18.44140625" style="2" customWidth="1"/>
     <col min="8" max="8" width="15.5546875" style="2" customWidth="1"/>
@@ -1709,17 +1711,17 @@
     <col min="15" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="C1" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="D1" s="16" t="s">
+      <c r="D1" t="s">
         <v>57</v>
       </c>
       <c r="E1" s="4" t="s">
@@ -1749,7 +1751,7 @@
       <c r="M1" s="6"/>
       <c r="N1" s="6"/>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14">
       <c r="F2" s="2"/>
       <c r="H2" s="7"/>
       <c r="J2" s="3"/>
@@ -1778,7 +1780,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3185D484-1AEA-488F-ADB2-C66611F8B5C9}">
   <sheetPr codeName="Sheet8"/>
   <dimension ref="A1:I2"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
     <col min="2" max="2" width="28.88671875" style="2" customWidth="1"/>
@@ -1791,7 +1793,7 @@
     <col min="10" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1818,7 +1820,7 @@
       </c>
       <c r="I1" s="6"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9">
       <c r="G2" s="2"/>
       <c r="I2" s="6"/>
     </row>
@@ -1848,7 +1850,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6150BED1-88FC-488E-B7E1-4C6CBEB9589C}">
   <sheetPr codeName="Sheet9"/>
   <dimension ref="A1:G1"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
     <col min="2" max="2" width="25.109375" style="1" customWidth="1"/>
@@ -1859,7 +1861,7 @@
     <col min="8" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1893,46 +1895,46 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6A08BCD-5A8C-45EE-A940-2FEFA1E5B102}">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
-    <col min="2" max="2" width="15.6640625" style="16" customWidth="1"/>
+    <col min="2" max="2" width="15.6640625" customWidth="1"/>
     <col min="3" max="3" width="27.44140625" style="4" customWidth="1"/>
-    <col min="4" max="4" width="21.6640625" style="16" customWidth="1"/>
-    <col min="5" max="5" width="30" style="16" customWidth="1"/>
+    <col min="4" max="4" width="21.6640625" customWidth="1"/>
+    <col min="5" max="5" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="B1" t="s">
         <v>57</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D1" s="16" t="s">
+      <c r="D1" t="s">
         <v>58</v>
       </c>
-      <c r="E1" s="16" t="s">
+      <c r="E1" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5">
       <c r="A2" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="B2" s="16" t="s">
+      <c r="B2" t="s">
         <v>95</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="D2" s="16" t="s">
+      <c r="D2" t="s">
         <v>97</v>
       </c>
-      <c r="E2" s="16" t="s">
+      <c r="E2" t="s">
         <v>98</v>
       </c>
     </row>
@@ -1947,13 +1949,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{849BF9A6-CD45-4FD2-AD73-886C99848EAC}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="24.21875" style="5" customWidth="1"/>
     <col min="2" max="2" width="31.5546875" style="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2">
       <c r="A1" s="5" t="s">
         <v>40</v>
       </c>
@@ -1961,7 +1963,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2">
       <c r="A2" s="5">
         <f>SUM(TEST_Inventory[TEST Currency])</f>
         <v>1130</v>
@@ -1983,7 +1985,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2834D935-E140-4D64-A4CD-4A9FB8899FE0}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:L2"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="29.109375" style="3" customWidth="1"/>
@@ -2000,7 +2002,7 @@
     <col min="13" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2038,7 +2040,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12">
       <c r="B2" s="3">
         <f>SUM(Resell_Inventory[Total Investment])</f>
         <v>0</v>
@@ -2083,9 +2085,9 @@
 )</f>
         <v>0</v>
       </c>
-      <c r="L2" s="7" t="e">
-        <f ca="1">COUNTIFS(Maintenance_Log[Next Service Date], "&lt;="&amp;TODAY()+30, #REF!, FALSE)</f>
-        <v>#REF!</v>
+      <c r="L2" s="15">
+        <f ca="1">COUNTIFS(Maintenance_Log[Next Service Date], "&lt;="&amp;TODAY()+30, Maintenance_Log[Complete], FALSE)</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -2101,13 +2103,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E53ED58-AF1A-4384-BD5D-DFB0D7D062C9}">
   <dimension ref="A9:B21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="42.21875" style="4" customWidth="1"/>
     <col min="2" max="2" width="17.5546875" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2">
       <c r="A9" s="4" t="s">
         <v>27</v>
       </c>
@@ -2115,7 +2117,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2">
       <c r="A10" s="2" t="s">
         <v>73</v>
       </c>
@@ -2124,7 +2126,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2">
       <c r="A11" s="2" t="s">
         <v>74</v>
       </c>
@@ -2133,7 +2135,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2">
       <c r="A12" s="2" t="s">
         <v>75</v>
       </c>
@@ -2142,7 +2144,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2">
       <c r="A13" s="2" t="s">
         <v>76</v>
       </c>
@@ -2151,7 +2153,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2">
       <c r="A14" s="2" t="s">
         <v>77</v>
       </c>
@@ -2160,7 +2162,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2">
       <c r="A15" s="2" t="s">
         <v>78</v>
       </c>
@@ -2169,7 +2171,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2">
       <c r="A16" s="2" t="s">
         <v>79</v>
       </c>
@@ -2178,7 +2180,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2">
       <c r="A17" s="2" t="s">
         <v>80</v>
       </c>
@@ -2187,7 +2189,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2">
       <c r="A18" s="2" t="s">
         <v>81</v>
       </c>
@@ -2196,7 +2198,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2">
       <c r="A19" s="2" t="s">
         <v>82</v>
       </c>
@@ -2205,7 +2207,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2">
       <c r="A20" s="2" t="s">
         <v>83</v>
       </c>
@@ -2214,7 +2216,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2">
       <c r="A21" s="2" t="s">
         <v>84</v>
       </c>
@@ -2240,12 +2242,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDE7BF89-A2E7-4A6F-B822-317739E206EC}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:R2"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
     <col min="2" max="2" width="9.5546875" style="14" customWidth="1"/>
     <col min="3" max="3" width="9.5546875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="12.88671875" style="16" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.88671875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="31.44140625" style="2" customWidth="1"/>
     <col min="6" max="6" width="10.5546875" style="2" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="17" style="10" bestFit="1" customWidth="1"/>
@@ -2256,23 +2258,23 @@
     <col min="12" max="12" width="16.6640625" style="3" customWidth="1"/>
     <col min="13" max="13" width="16.88671875" style="3" customWidth="1"/>
     <col min="14" max="14" width="16.88671875" style="14" customWidth="1"/>
-    <col min="16" max="16" width="12.88671875" style="16" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="16.88671875" style="17" customWidth="1"/>
+    <col min="16" max="16" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.88671875" style="6" customWidth="1"/>
     <col min="18" max="18" width="16.88671875" style="2" customWidth="1"/>
     <col min="19" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="C1" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="D1" s="16" t="s">
+      <c r="D1" t="s">
         <v>57</v>
       </c>
       <c r="E1" s="4" t="s">
@@ -2305,22 +2307,20 @@
       <c r="N1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="O1" s="18" t="s">
+      <c r="O1" t="s">
         <v>87</v>
       </c>
       <c r="P1" s="6"/>
-      <c r="Q1" s="6"/>
       <c r="R1" s="6"/>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="D2" s="17"/>
+    <row r="2" spans="1:18">
+      <c r="D2" s="6"/>
       <c r="J2" s="5">
         <f>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</f>
         <v>0</v>
       </c>
-      <c r="O2" s="17"/>
+      <c r="O2" s="6"/>
       <c r="P2" s="6"/>
-      <c r="Q2" s="6"/>
       <c r="R2" s="6"/>
     </row>
   </sheetData>
@@ -2347,12 +2347,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B027EC69-551F-4051-8A71-8B106D207C6D}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:L2"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
     <col min="2" max="2" width="9.5546875" style="14" customWidth="1"/>
     <col min="3" max="3" width="9.5546875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="12.33203125" style="17" customWidth="1"/>
+    <col min="4" max="4" width="12.33203125" style="6" customWidth="1"/>
     <col min="5" max="5" width="28.6640625" style="2" customWidth="1"/>
     <col min="6" max="6" width="14.88671875" style="2" customWidth="1"/>
     <col min="7" max="7" width="14.6640625" style="10" customWidth="1"/>
@@ -2363,17 +2363,17 @@
     <col min="13" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="C1" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="D1" s="16" t="s">
+      <c r="D1" t="s">
         <v>57</v>
       </c>
       <c r="E1" s="4" t="s">
@@ -2399,7 +2399,7 @@
       </c>
       <c r="L1" s="6"/>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12">
       <c r="J2" s="6"/>
       <c r="K2" s="2"/>
       <c r="L2" s="6"/>
@@ -2424,7 +2424,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB7AACC4-9DA2-4A53-AD77-8C5E0C1BF474}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:M2"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.109375" style="14" bestFit="1" customWidth="1"/>
@@ -2435,14 +2435,14 @@
     <col min="7" max="7" width="14.33203125" style="6" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="7" style="3" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="18" style="9" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.44140625" style="16" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.44140625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="18" style="2" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="13.44140625" style="2" customWidth="1"/>
     <col min="13" max="13" width="9.88671875" style="3" customWidth="1"/>
     <col min="14" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2470,7 +2470,7 @@
       <c r="I1" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="J1" s="16" t="s">
+      <c r="J1" t="s">
         <v>89</v>
       </c>
       <c r="K1" s="4" t="s">
@@ -2479,9 +2479,9 @@
       <c r="L1" s="6"/>
       <c r="M1" s="6"/>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13">
       <c r="I2" s="10"/>
-      <c r="J2" s="17"/>
+      <c r="J2" s="6"/>
       <c r="L2" s="6"/>
       <c r="M2" s="6"/>
     </row>
@@ -2508,12 +2508,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEDDDAA7-75C3-4AA5-ABFD-D5FB4C627E4C}">
   <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:M2"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
     <col min="2" max="2" width="8.6640625" style="14" customWidth="1"/>
     <col min="3" max="3" width="8.6640625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="12.88671875" style="17" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.88671875" style="6" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="50.44140625" style="2" customWidth="1"/>
     <col min="6" max="6" width="15.6640625" style="3" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="19.88671875" style="6" bestFit="1" customWidth="1"/>
@@ -2525,17 +2525,17 @@
     <col min="14" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="C1" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="D1" s="16" t="s">
+      <c r="D1" t="s">
         <v>57</v>
       </c>
       <c r="E1" s="4" t="s">
@@ -2561,7 +2561,7 @@
       </c>
       <c r="M1" s="6"/>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13">
       <c r="G2" s="6"/>
       <c r="K2" s="2"/>
       <c r="M2" s="6"/>
@@ -2599,34 +2599,33 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F39ADDA6-CD5F-4655-A9C0-9676DDAC362E}">
   <sheetPr codeName="Sheet6"/>
   <dimension ref="A1:L2"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.6640625" style="14" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.6640625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="12.88671875" style="17" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.88671875" style="6" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="54.6640625" style="2" customWidth="1"/>
     <col min="6" max="6" width="15.6640625" style="3" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.5546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.88671875" style="16"/>
-    <col min="9" max="9" width="12.88671875" style="17" customWidth="1"/>
+    <col min="9" max="9" width="12.88671875" style="6" customWidth="1"/>
     <col min="10" max="10" width="10.33203125" style="4" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="16.33203125" style="7" customWidth="1"/>
     <col min="12" max="12" width="12.88671875" style="2" customWidth="1"/>
     <col min="13" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="C1" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="D1" s="16" t="s">
+      <c r="D1" t="s">
         <v>57</v>
       </c>
       <c r="E1" s="4" t="s">
@@ -2638,10 +2637,10 @@
       <c r="G1" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="16" t="s">
+      <c r="H1" t="s">
         <v>21</v>
       </c>
-      <c r="I1" s="16" t="s">
+      <c r="I1" t="s">
         <v>22</v>
       </c>
       <c r="J1" s="4" t="s">
@@ -2650,8 +2649,8 @@
       <c r="K1" s="6"/>
       <c r="L1" s="6"/>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="H2" s="17"/>
+    <row r="2" spans="1:12">
+      <c r="H2" s="6"/>
       <c r="J2" s="2"/>
       <c r="K2" s="6"/>
       <c r="L2" s="6"/>

</xml_diff>

<commit_message>
added hybrid-inventory feature; ui.js, app.js, config.js, style.css, excel
</commit_message>
<xml_diff>
--- a/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
+++ b/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1a2ae81d67634e6/Desktop/Michanikos Artifex Enterprises/MAE Custom Digital Solutions/MAE Workshop Inventory Management System/GITHUB_MAE_Workshop Inventory App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="188" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9D0DCF16-319A-4A23-AC65-9B406C576162}"/>
+  <xr:revisionPtr revIDLastSave="189" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6DB353D7-7193-4945-BA61-3065EF62EC00}"/>
   <bookViews>
-    <workbookView xWindow="4884" yWindow="1452" windowWidth="20508" windowHeight="11904" firstSheet="11" activeTab="12" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
+    <workbookView xWindow="1452" yWindow="336" windowWidth="20508" windowHeight="11904" firstSheet="6" activeTab="9" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
   </bookViews>
   <sheets>
     <sheet name="TEST Inventory" sheetId="10" r:id="rId1"/>
@@ -471,22 +471,6 @@
   </cellStyles>
   <dxfs count="128">
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="0"/>
     </dxf>
@@ -876,28 +860,6 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
@@ -962,6 +924,44 @@
     <dxf>
       <protection locked="1" hidden="0"/>
     </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1000,11 +1000,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}" name="TEST_Inventory" displayName="TEST_Inventory" ref="A1:F5" totalsRowShown="0">
   <autoFilter ref="A1:F5" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="114"/>
-    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="113"/>
-    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="112"/>
-    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="111"/>
-    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="110">
+    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="122"/>
+    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="121"/>
+    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="120"/>
+    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="119"/>
+    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="118">
       <calculatedColumnFormula>TEST_Inventory[[#This Row],[TEST Integer]]*TEST_Inventory[[#This Row],[TEST Currency]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{AB3A5F3C-FCF0-4466-90FD-8ABB6E18DF5C}" name="TEST Dropdown"/>
@@ -1014,56 +1014,59 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:L2" totalsRowShown="0" headerRowDxfId="37" dataDxfId="36">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:L2" totalsRowShown="0" headerRowDxfId="32" dataDxfId="31">
   <autoFilter ref="A1:L2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="35"/>
-    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="34"/>
-    <tableColumn id="12" xr3:uid="{8F0FD29C-682B-41B4-82F2-913D40801887}" name="Tag_ID" dataDxfId="33"/>
-    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="32"/>
-    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="31"/>
-    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="30"/>
-    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="29"/>
-    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="28"/>
-    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="27"/>
-    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="26"/>
-    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="25">
-      <calculatedColumnFormula>Shop_Consumables[[#This Row],[Current Stock]]*Shop_Consumables[[#This Row],[Unit Cost]]</calculatedColumnFormula>
+    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="30"/>
+    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="29"/>
+    <tableColumn id="12" xr3:uid="{8F0FD29C-682B-41B4-82F2-913D40801887}" name="Tag_ID" dataDxfId="28"/>
+    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="27"/>
+    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="26"/>
+    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="25"/>
+    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="24"/>
+    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="23"/>
+    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="22"/>
+    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="21"/>
+    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="20">
+      <calculatedColumnFormula array="1">IF(ISNUMBER(Shop_Consumables[[#This Row],[Current Stock]]),
+    Shop_Consumables[[#This Row],[Current Stock]] * Shop_Consumables[[#This Row],[Unit Cost]],
+    _xlfn.IFS(Shop_Consumables[[#This Row],[Current Stock]]="Many", 1, Shop_Consumables[[#This Row],[Current Stock]]="Adequate", 0.5, Shop_Consumables[[#This Row],[Current Stock]]="Few", 0.1, TRUE, 0) * Shop_Consumables[[#This Row],[Unit Cost]]
+)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Supplier/Remarks" dataDxfId="24"/>
+    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Supplier/Remarks" dataDxfId="19"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:H2" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:H2" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
   <autoFilter ref="A1:H2" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="20"/>
-    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="16"/>
-    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="15"/>
-    <tableColumn id="8" xr3:uid="{9140C4E8-CB9E-40BF-ABD9-13A971322B09}" name="Remarks" dataDxfId="14"/>
+    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="12"/>
+    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="11"/>
+    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="10"/>
+    <tableColumn id="8" xr3:uid="{9140C4E8-CB9E-40BF-ABD9-13A971322B09}" name="Remarks" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
   <autoFilter ref="A1:G2" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="11"/>
-    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="9"/>
-    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="7"/>
-    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="6"/>
-    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="6"/>
+    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="4"/>
+    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="2"/>
+    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="1"/>
+    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1073,11 +1076,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}" name="Location" displayName="Location" ref="A1:E2" totalsRowShown="0">
   <autoFilter ref="A1:E2" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Description" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="127"/>
+    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="126"/>
+    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Description" dataDxfId="125"/>
+    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="124"/>
+    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="123"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1087,10 +1090,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}" name="TEST_Dashboard" displayName="TEST_Dashboard" ref="A1:B2" totalsRowShown="0">
   <autoFilter ref="A1:B2" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="109">
+    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="117">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Currency])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="108">
+    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="116">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Integer])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1099,38 +1102,38 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:L2" totalsRowShown="0" headerRowDxfId="127" dataDxfId="126">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:L2" totalsRowShown="0" headerRowDxfId="115" dataDxfId="114">
   <autoFilter ref="A1:L2" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="125"/>
-    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="124">
+    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="113"/>
+    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="112">
       <calculatedColumnFormula>SUM(Resell_Inventory[Total Investment])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="123">
+    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="111">
       <calculatedColumnFormula>SUM(Resell_Inventory[Actual Sale Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="122">
+    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="110">
       <calculatedColumnFormula>SUM(Shop_Machinery[Purchase Cost])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="121">
+    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="109">
       <calculatedColumnFormula>SUM(Shop_Power_Tools[Purchase Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="120">
+    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="108">
       <calculatedColumnFormula>SUM(Shop_Hand_Tools[Purchase Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="119">
+    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="107">
       <calculatedColumnFormula>SUM(Shop_Consumables[Current Inventory Value])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="118">
+    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="106">
       <calculatedColumnFormula>SUM(D2,E2,F2,G2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="117">
+    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="105">
       <calculatedColumnFormula array="1">SUMPRODUCT(--(Shop_Consumables[Current Stock]&lt;=Shop_Consumables[Reorder Point]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="116">
+    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="104">
       <calculatedColumnFormula>SUMIFS(Shop_Overhead[Amount], Shop_Overhead[Due Date], "&lt;="&amp;TODAY()+30, Shop_Overhead[Due Date], "&gt;="&amp;TODAY())</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{E4065760-B1B1-4564-936B-3405D3B80297}" name="Equipment With Operational Issues" dataDxfId="115">
+    <tableColumn id="12" xr3:uid="{E4065760-B1B1-4564-936B-3405D3B80297}" name="Equipment With Operational Issues" dataDxfId="103">
       <calculatedColumnFormula array="1">SUM(
   COUNTIFS(Shop_Machinery[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"}),
   COUNTIFS(Shop_Power_Tools[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"}),
@@ -1149,8 +1152,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{F579DA07-7AD6-49DA-9B44-D5B1132EDAC6}" name="Overhead_Summary" displayName="Overhead_Summary" ref="A9:B21" totalsRowShown="0">
   <autoFilter ref="A9:B21" xr:uid="{F579DA07-7AD6-49DA-9B44-D5B1132EDAC6}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{7CA4839C-9603-479D-BD1C-8377DFA9603C}" name="Expense Category" dataDxfId="107"/>
-    <tableColumn id="2" xr3:uid="{FE0F7616-EAF3-443D-AC69-DE6541DC10E5}" name="Annual Total" dataDxfId="106">
+    <tableColumn id="1" xr3:uid="{7CA4839C-9603-479D-BD1C-8377DFA9603C}" name="Expense Category" dataDxfId="102"/>
+    <tableColumn id="2" xr3:uid="{FE0F7616-EAF3-443D-AC69-DE6541DC10E5}" name="Annual Total" dataDxfId="101">
       <calculatedColumnFormula>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1159,105 +1162,105 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:O2" totalsRowShown="0" headerRowDxfId="105" dataDxfId="104">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:O2" totalsRowShown="0" headerRowDxfId="100" dataDxfId="99">
   <autoFilter ref="A1:O2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}"/>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="103"/>
-    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="102"/>
-    <tableColumn id="15" xr3:uid="{D25A390C-69B5-4326-A0D4-10EB45DDE5E5}" name="Tag_ID" dataDxfId="101"/>
-    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="100"/>
-    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="99"/>
-    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="98"/>
-    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="97"/>
-    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="96"/>
-    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="95"/>
-    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="94">
+    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="98"/>
+    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="97"/>
+    <tableColumn id="15" xr3:uid="{D25A390C-69B5-4326-A0D4-10EB45DDE5E5}" name="Tag_ID" dataDxfId="96"/>
+    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="95"/>
+    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="94"/>
+    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="93"/>
+    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="92"/>
+    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="91"/>
+    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="90"/>
+    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="89">
       <calculatedColumnFormula>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="93"/>
-    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="92"/>
-    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="91"/>
-    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="90"/>
-    <tableColumn id="16" xr3:uid="{CA8F9851-44B9-4614-9963-24D4EC145034}" name="Sold" dataDxfId="89"/>
+    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="88"/>
+    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="87"/>
+    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="86"/>
+    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="85"/>
+    <tableColumn id="16" xr3:uid="{CA8F9851-44B9-4614-9963-24D4EC145034}" name="Sold" dataDxfId="84"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="88" dataDxfId="87">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="83" dataDxfId="82">
   <autoFilter ref="A1:K2" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="86"/>
-    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="85"/>
-    <tableColumn id="4" xr3:uid="{17EB0B09-11B3-4E08-9442-E3C9AB87A157}" name="Tag_ID" dataDxfId="84"/>
-    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="83"/>
-    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Brand/Model" dataDxfId="82"/>
-    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="81"/>
-    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="80"/>
-    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="79"/>
-    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="78"/>
-    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="77"/>
-    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="76"/>
+    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="81"/>
+    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="80"/>
+    <tableColumn id="4" xr3:uid="{17EB0B09-11B3-4E08-9442-E3C9AB87A157}" name="Tag_ID" dataDxfId="79"/>
+    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="78"/>
+    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Brand/Model" dataDxfId="77"/>
+    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="76"/>
+    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="75"/>
+    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="74"/>
+    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="73"/>
+    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="72"/>
+    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="71"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:K2" totalsRowShown="0" headerRowDxfId="75" dataDxfId="74">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:K2" totalsRowShown="0" headerRowDxfId="70" dataDxfId="69">
   <autoFilter ref="A1:K2" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="73"/>
-    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="72"/>
-    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="71"/>
-    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="70"/>
-    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="69"/>
-    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="68"/>
-    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="67"/>
-    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="66"/>
-    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="65"/>
-    <tableColumn id="11" xr3:uid="{4809319D-ABCA-43DA-A400-5DC91167D78B}" name="Complete" dataDxfId="64"/>
-    <tableColumn id="12" xr3:uid="{920CB592-D743-4B33-A796-C7F3DB32211C}" name="Remarks" dataDxfId="63"/>
+    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="68"/>
+    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="67"/>
+    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="66"/>
+    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="65"/>
+    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="64"/>
+    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="63"/>
+    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="62"/>
+    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="61"/>
+    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="60"/>
+    <tableColumn id="11" xr3:uid="{4809319D-ABCA-43DA-A400-5DC91167D78B}" name="Complete" dataDxfId="59"/>
+    <tableColumn id="12" xr3:uid="{920CB592-D743-4B33-A796-C7F3DB32211C}" name="Remarks" dataDxfId="58"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:K2" totalsRowShown="0" headerRowDxfId="62" dataDxfId="61">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:K2" totalsRowShown="0" headerRowDxfId="57" dataDxfId="56">
   <autoFilter ref="A1:K2" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="60"/>
-    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="59"/>
-    <tableColumn id="11" xr3:uid="{21951C81-00A4-4344-9E81-B1B1DB06ADEF}" name="Tag_ID" dataDxfId="58"/>
-    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="57"/>
-    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Brand/Model" dataDxfId="56"/>
-    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="55"/>
-    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="54"/>
-    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="53"/>
-    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="52"/>
-    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="51"/>
-    <tableColumn id="10" xr3:uid="{26197E01-2936-4F5F-8081-3AA351C1CD38}" name="Remarks" dataDxfId="50"/>
+    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="55"/>
+    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="54"/>
+    <tableColumn id="11" xr3:uid="{21951C81-00A4-4344-9E81-B1B1DB06ADEF}" name="Tag_ID" dataDxfId="53"/>
+    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="52"/>
+    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Brand/Model" dataDxfId="51"/>
+    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="50"/>
+    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="49"/>
+    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="48"/>
+    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="47"/>
+    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="46"/>
+    <tableColumn id="10" xr3:uid="{26197E01-2936-4F5F-8081-3AA351C1CD38}" name="Remarks" dataDxfId="45"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:J2" totalsRowShown="0" headerRowDxfId="49" dataDxfId="48">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:J2" totalsRowShown="0" headerRowDxfId="44" dataDxfId="43">
   <autoFilter ref="A1:J2" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="47"/>
-    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="46"/>
-    <tableColumn id="10" xr3:uid="{C8BD69AA-9023-4777-9C96-39A81F1E4BE0}" name="Tag_ID" dataDxfId="45"/>
-    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="44"/>
-    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Brand/Model/Description" dataDxfId="43"/>
-    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="42"/>
-    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="41"/>
-    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="40"/>
-    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="39"/>
-    <tableColumn id="9" xr3:uid="{2B57F5E6-66C5-4DBA-8949-836DE0F0791C}" name="Remarks" dataDxfId="38"/>
+    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="42"/>
+    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="41"/>
+    <tableColumn id="10" xr3:uid="{C8BD69AA-9023-4777-9C96-39A81F1E4BE0}" name="Tag_ID" dataDxfId="40"/>
+    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="39"/>
+    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Brand/Model/Description" dataDxfId="38"/>
+    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="37"/>
+    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="36"/>
+    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="35"/>
+    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="34"/>
+    <tableColumn id="9" xr3:uid="{2B57F5E6-66C5-4DBA-8949-836DE0F0791C}" name="Remarks" dataDxfId="33"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1758,8 +1761,11 @@
       <c r="F2" s="2"/>
       <c r="H2" s="7"/>
       <c r="J2" s="3"/>
-      <c r="K2" s="3">
-        <f>Shop_Consumables[[#This Row],[Current Stock]]*Shop_Consumables[[#This Row],[Unit Cost]]</f>
+      <c r="K2" s="3" cm="1">
+        <f t="array" ref="K2">IF(ISNUMBER(Shop_Consumables[[#This Row],[Current Stock]]),
+    Shop_Consumables[[#This Row],[Current Stock]] * Shop_Consumables[[#This Row],[Unit Cost]],
+    _xlfn.IFS(Shop_Consumables[[#This Row],[Current Stock]]="Many", 1, Shop_Consumables[[#This Row],[Current Stock]]="Adequate", 0.5, Shop_Consumables[[#This Row],[Current Stock]]="Few", 0.1, TRUE, 0) * Shop_Consumables[[#This Row],[Unit Cost]]
+)</f>
         <v>0</v>
       </c>
       <c r="L2" s="2"/>
@@ -1767,7 +1773,7 @@
       <c r="N2" s="6"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations disablePrompts="1" count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2" xr:uid="{D2C605E8-D02B-4558-82DE-3169088704E8}">
       <formula1>"Fasteners/Hardware,Abrasives/Cutting,Fluids/Lubricants/Chemicals,Primer/Paint,Safety/PPE,Shop/Janitorial,Welding,Electrical,Other"</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
adding "few" to triggerlow stock alert
</commit_message>
<xml_diff>
--- a/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
+++ b/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1a2ae81d67634e6/Desktop/Michanikos Artifex Enterprises/MAE Custom Digital Solutions/MAE Workshop Inventory Management System/GITHUB_MAE_Workshop Inventory App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="189" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6DB353D7-7193-4945-BA61-3065EF62EC00}"/>
+  <xr:revisionPtr revIDLastSave="203" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{96536185-033E-437F-B042-37811CCC0934}"/>
   <bookViews>
-    <workbookView xWindow="1452" yWindow="336" windowWidth="20508" windowHeight="11904" firstSheet="6" activeTab="9" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="11712" firstSheet="2" activeTab="2" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
   </bookViews>
   <sheets>
     <sheet name="TEST Inventory" sheetId="10" r:id="rId1"/>
@@ -471,24 +471,20 @@
   </cellStyles>
   <dxfs count="128">
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -496,9 +492,33 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -531,60 +551,6 @@
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="1"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -867,10 +833,6 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -947,20 +909,58 @@
       <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1000,11 +1000,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}" name="TEST_Inventory" displayName="TEST_Inventory" ref="A1:F5" totalsRowShown="0">
   <autoFilter ref="A1:F5" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="122"/>
-    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="121"/>
-    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="120"/>
-    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="119"/>
-    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="118">
+    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="113"/>
+    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="112"/>
+    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="111"/>
+    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="110"/>
+    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="109">
       <calculatedColumnFormula>TEST_Inventory[[#This Row],[TEST Integer]]*TEST_Inventory[[#This Row],[TEST Currency]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{AB3A5F3C-FCF0-4466-90FD-8ABB6E18DF5C}" name="TEST Dropdown"/>
@@ -1014,59 +1014,59 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:L2" totalsRowShown="0" headerRowDxfId="32" dataDxfId="31">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:L2" totalsRowShown="0" headerRowDxfId="127" dataDxfId="126">
   <autoFilter ref="A1:L2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="30"/>
-    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="29"/>
-    <tableColumn id="12" xr3:uid="{8F0FD29C-682B-41B4-82F2-913D40801887}" name="Tag_ID" dataDxfId="28"/>
-    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="27"/>
-    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="26"/>
-    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="25"/>
-    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="24"/>
-    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="23"/>
-    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="22"/>
-    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="21"/>
-    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="20">
+    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="125"/>
+    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="124"/>
+    <tableColumn id="12" xr3:uid="{8F0FD29C-682B-41B4-82F2-913D40801887}" name="Tag_ID" dataDxfId="123"/>
+    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="122"/>
+    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="121"/>
+    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="120"/>
+    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="119"/>
+    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="118"/>
+    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="117"/>
+    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="116"/>
+    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="115">
       <calculatedColumnFormula array="1">IF(ISNUMBER(Shop_Consumables[[#This Row],[Current Stock]]),
     Shop_Consumables[[#This Row],[Current Stock]] * Shop_Consumables[[#This Row],[Unit Cost]],
     _xlfn.IFS(Shop_Consumables[[#This Row],[Current Stock]]="Many", 1, Shop_Consumables[[#This Row],[Current Stock]]="Adequate", 0.5, Shop_Consumables[[#This Row],[Current Stock]]="Few", 0.1, TRUE, 0) * Shop_Consumables[[#This Row],[Unit Cost]]
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Supplier/Remarks" dataDxfId="19"/>
+    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Supplier/Remarks" dataDxfId="114"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:H2" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:H2" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23">
   <autoFilter ref="A1:H2" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="16"/>
-    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="15"/>
-    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="14"/>
-    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="13"/>
-    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="12"/>
-    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="11"/>
-    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="10"/>
-    <tableColumn id="8" xr3:uid="{9140C4E8-CB9E-40BF-ABD9-13A971322B09}" name="Remarks" dataDxfId="9"/>
+    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="22"/>
+    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="20"/>
+    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="18"/>
+    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="17"/>
+    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="16"/>
+    <tableColumn id="8" xr3:uid="{9140C4E8-CB9E-40BF-ABD9-13A971322B09}" name="Remarks" dataDxfId="15"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13">
   <autoFilter ref="A1:G2" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="6"/>
-    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="4"/>
-    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="3"/>
-    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="2"/>
-    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="1"/>
-    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="12"/>
+    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="10"/>
+    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="9"/>
+    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="8"/>
+    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="7"/>
+    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1076,11 +1076,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}" name="Location" displayName="Location" ref="A1:E2" totalsRowShown="0">
   <autoFilter ref="A1:E2" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="127"/>
-    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="126"/>
-    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Description" dataDxfId="125"/>
-    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="124"/>
-    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="123"/>
+    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Description" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1090,10 +1090,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}" name="TEST_Dashboard" displayName="TEST_Dashboard" ref="A1:B2" totalsRowShown="0">
   <autoFilter ref="A1:B2" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="117">
+    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="108">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Currency])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="116">
+    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="107">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Integer])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1102,38 +1102,41 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:L2" totalsRowShown="0" headerRowDxfId="115" dataDxfId="114">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:L2" totalsRowShown="0" headerRowDxfId="106" dataDxfId="105">
   <autoFilter ref="A1:L2" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="113"/>
-    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="112">
+    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="104"/>
+    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="103">
       <calculatedColumnFormula>SUM(Resell_Inventory[Total Investment])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="111">
+    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="102">
       <calculatedColumnFormula>SUM(Resell_Inventory[Actual Sale Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="110">
+    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="101">
       <calculatedColumnFormula>SUM(Shop_Machinery[Purchase Cost])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="109">
+    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="100">
       <calculatedColumnFormula>SUM(Shop_Power_Tools[Purchase Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="108">
+    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="99">
       <calculatedColumnFormula>SUM(Shop_Hand_Tools[Purchase Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="107">
+    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="98">
       <calculatedColumnFormula>SUM(Shop_Consumables[Current Inventory Value])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="106">
+    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="97">
       <calculatedColumnFormula>SUM(D2,E2,F2,G2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="105">
-      <calculatedColumnFormula array="1">SUMPRODUCT(--(Shop_Consumables[Current Stock]&lt;=Shop_Consumables[Reorder Point]))</calculatedColumnFormula>
+    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="0">
+      <calculatedColumnFormula array="1">SUMPRODUCT(
+    --( (ISNUMBER(Shop_Consumables[Current Stock])*(Shop_Consumables[Current Stock]&lt;=Shop_Consumables[Reorder Point]))
+    + (Shop_Consumables[Current Stock]="Few") )
+)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="104">
+    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="96">
       <calculatedColumnFormula>SUMIFS(Shop_Overhead[Amount], Shop_Overhead[Due Date], "&lt;="&amp;TODAY()+30, Shop_Overhead[Due Date], "&gt;="&amp;TODAY())</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{E4065760-B1B1-4564-936B-3405D3B80297}" name="Equipment With Operational Issues" dataDxfId="103">
+    <tableColumn id="12" xr3:uid="{E4065760-B1B1-4564-936B-3405D3B80297}" name="Equipment With Operational Issues" dataDxfId="95">
       <calculatedColumnFormula array="1">SUM(
   COUNTIFS(Shop_Machinery[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"}),
   COUNTIFS(Shop_Power_Tools[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"}),
@@ -1152,8 +1155,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{F579DA07-7AD6-49DA-9B44-D5B1132EDAC6}" name="Overhead_Summary" displayName="Overhead_Summary" ref="A9:B21" totalsRowShown="0">
   <autoFilter ref="A9:B21" xr:uid="{F579DA07-7AD6-49DA-9B44-D5B1132EDAC6}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{7CA4839C-9603-479D-BD1C-8377DFA9603C}" name="Expense Category" dataDxfId="102"/>
-    <tableColumn id="2" xr3:uid="{FE0F7616-EAF3-443D-AC69-DE6541DC10E5}" name="Annual Total" dataDxfId="101">
+    <tableColumn id="1" xr3:uid="{7CA4839C-9603-479D-BD1C-8377DFA9603C}" name="Expense Category" dataDxfId="94"/>
+    <tableColumn id="2" xr3:uid="{FE0F7616-EAF3-443D-AC69-DE6541DC10E5}" name="Annual Total" dataDxfId="93">
       <calculatedColumnFormula>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1162,105 +1165,105 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:O2" totalsRowShown="0" headerRowDxfId="100" dataDxfId="99">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:O2" totalsRowShown="0" headerRowDxfId="92" dataDxfId="91">
   <autoFilter ref="A1:O2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}"/>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="98"/>
-    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="97"/>
-    <tableColumn id="15" xr3:uid="{D25A390C-69B5-4326-A0D4-10EB45DDE5E5}" name="Tag_ID" dataDxfId="96"/>
-    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="95"/>
-    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="94"/>
-    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="93"/>
-    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="92"/>
-    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="91"/>
-    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="90"/>
-    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="89">
+    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="90"/>
+    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="89"/>
+    <tableColumn id="15" xr3:uid="{D25A390C-69B5-4326-A0D4-10EB45DDE5E5}" name="Tag_ID" dataDxfId="88"/>
+    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="87"/>
+    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="86"/>
+    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="85"/>
+    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="84"/>
+    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="83"/>
+    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="82"/>
+    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="81">
       <calculatedColumnFormula>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="88"/>
-    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="87"/>
-    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="86"/>
-    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="85"/>
-    <tableColumn id="16" xr3:uid="{CA8F9851-44B9-4614-9963-24D4EC145034}" name="Sold" dataDxfId="84"/>
+    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="80"/>
+    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="79"/>
+    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="78"/>
+    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="77"/>
+    <tableColumn id="16" xr3:uid="{CA8F9851-44B9-4614-9963-24D4EC145034}" name="Sold" dataDxfId="76"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="83" dataDxfId="82">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="75" dataDxfId="74">
   <autoFilter ref="A1:K2" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="81"/>
-    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="80"/>
-    <tableColumn id="4" xr3:uid="{17EB0B09-11B3-4E08-9442-E3C9AB87A157}" name="Tag_ID" dataDxfId="79"/>
-    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="78"/>
-    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Brand/Model" dataDxfId="77"/>
-    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="76"/>
-    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="75"/>
-    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="74"/>
-    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="73"/>
-    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="72"/>
-    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="71"/>
+    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="73"/>
+    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="72"/>
+    <tableColumn id="4" xr3:uid="{17EB0B09-11B3-4E08-9442-E3C9AB87A157}" name="Tag_ID" dataDxfId="71"/>
+    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="70"/>
+    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Brand/Model" dataDxfId="69"/>
+    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="68"/>
+    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="67"/>
+    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="66"/>
+    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="65"/>
+    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="64"/>
+    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="63"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:K2" totalsRowShown="0" headerRowDxfId="70" dataDxfId="69">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:K2" totalsRowShown="0" headerRowDxfId="62" dataDxfId="61">
   <autoFilter ref="A1:K2" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="68"/>
-    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="67"/>
-    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="66"/>
-    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="65"/>
-    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="64"/>
-    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="63"/>
-    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="62"/>
-    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="61"/>
-    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="60"/>
-    <tableColumn id="11" xr3:uid="{4809319D-ABCA-43DA-A400-5DC91167D78B}" name="Complete" dataDxfId="59"/>
-    <tableColumn id="12" xr3:uid="{920CB592-D743-4B33-A796-C7F3DB32211C}" name="Remarks" dataDxfId="58"/>
+    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="60"/>
+    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="59"/>
+    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="58"/>
+    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="57"/>
+    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="56"/>
+    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="55"/>
+    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="54"/>
+    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="53"/>
+    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="52"/>
+    <tableColumn id="11" xr3:uid="{4809319D-ABCA-43DA-A400-5DC91167D78B}" name="Complete" dataDxfId="51"/>
+    <tableColumn id="12" xr3:uid="{920CB592-D743-4B33-A796-C7F3DB32211C}" name="Remarks" dataDxfId="50"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:K2" totalsRowShown="0" headerRowDxfId="57" dataDxfId="56">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:K2" totalsRowShown="0" headerRowDxfId="49" dataDxfId="48">
   <autoFilter ref="A1:K2" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="55"/>
-    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="54"/>
-    <tableColumn id="11" xr3:uid="{21951C81-00A4-4344-9E81-B1B1DB06ADEF}" name="Tag_ID" dataDxfId="53"/>
-    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="52"/>
-    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Brand/Model" dataDxfId="51"/>
-    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="50"/>
-    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="49"/>
-    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="48"/>
-    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="47"/>
-    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="46"/>
-    <tableColumn id="10" xr3:uid="{26197E01-2936-4F5F-8081-3AA351C1CD38}" name="Remarks" dataDxfId="45"/>
+    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="47"/>
+    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="46"/>
+    <tableColumn id="11" xr3:uid="{21951C81-00A4-4344-9E81-B1B1DB06ADEF}" name="Tag_ID" dataDxfId="45"/>
+    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="44"/>
+    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Brand/Model" dataDxfId="43"/>
+    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="42"/>
+    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="41"/>
+    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="40"/>
+    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="39"/>
+    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="38"/>
+    <tableColumn id="10" xr3:uid="{26197E01-2936-4F5F-8081-3AA351C1CD38}" name="Remarks" dataDxfId="37"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:J2" totalsRowShown="0" headerRowDxfId="44" dataDxfId="43">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:J2" totalsRowShown="0" headerRowDxfId="36" dataDxfId="35">
   <autoFilter ref="A1:J2" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="42"/>
-    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="41"/>
-    <tableColumn id="10" xr3:uid="{C8BD69AA-9023-4777-9C96-39A81F1E4BE0}" name="Tag_ID" dataDxfId="40"/>
-    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="39"/>
-    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Brand/Model/Description" dataDxfId="38"/>
-    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="37"/>
-    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="36"/>
-    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="35"/>
-    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="34"/>
-    <tableColumn id="9" xr3:uid="{2B57F5E6-66C5-4DBA-8949-836DE0F0791C}" name="Remarks" dataDxfId="33"/>
+    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="34"/>
+    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="33"/>
+    <tableColumn id="10" xr3:uid="{C8BD69AA-9023-4777-9C96-39A81F1E4BE0}" name="Tag_ID" dataDxfId="32"/>
+    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="31"/>
+    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Brand/Model/Description" dataDxfId="30"/>
+    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="29"/>
+    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="28"/>
+    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="27"/>
+    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="26"/>
+    <tableColumn id="9" xr3:uid="{2B57F5E6-66C5-4DBA-8949-836DE0F0791C}" name="Remarks" dataDxfId="25"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2079,8 +2082,11 @@
         <v>0</v>
       </c>
       <c r="I2" s="12" cm="1">
-        <f t="array" ref="I2">SUMPRODUCT(--(Shop_Consumables[Current Stock]&lt;=Shop_Consumables[Reorder Point]))</f>
-        <v>1</v>
+        <f t="array" ref="I2">SUMPRODUCT(
+    --( (ISNUMBER(Shop_Consumables[Current Stock])*(Shop_Consumables[Current Stock]&lt;=Shop_Consumables[Reorder Point]))
+    + (Shop_Consumables[Current Stock]="Few") )
+)</f>
+        <v>0</v>
       </c>
       <c r="J2" s="3">
         <f ca="1">SUMIFS(Shop_Overhead[Amount], Shop_Overhead[Due Date], "&lt;="&amp;TODAY()+30, Shop_Overhead[Due Date], "&gt;="&amp;TODAY())</f>

</xml_diff>

<commit_message>
Delete hybrid approach to handling text/number; created two columns in Shop_Hand_Tools and Shop_Consumables: one text and one number; refactored
</commit_message>
<xml_diff>
--- a/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
+++ b/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1a2ae81d67634e6/Desktop/Michanikos Artifex Enterprises/MAE Custom Digital Solutions/MAE Workshop Inventory Management System/GITHUB_MAE_Workshop Inventory App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="203" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{96536185-033E-437F-B042-37811CCC0934}"/>
+  <xr:revisionPtr revIDLastSave="218" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5F13A097-AC2E-4DD5-88E5-94DD3903E83C}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="11712" firstSheet="2" activeTab="2" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
+    <workbookView xWindow="72" yWindow="660" windowWidth="20508" windowHeight="11904" firstSheet="6" activeTab="9" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
   </bookViews>
   <sheets>
     <sheet name="TEST Inventory" sheetId="10" r:id="rId1"/>
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="100">
   <si>
     <t>mae_id</t>
   </si>
@@ -141,15 +141,9 @@
     <t>Condition</t>
   </si>
   <si>
-    <t>Quantity</t>
-  </si>
-  <si>
     <t>Unit of Measure</t>
   </si>
   <si>
-    <t>Current Stock</t>
-  </si>
-  <si>
     <t>Reorder Point</t>
   </si>
   <si>
@@ -373,6 +367,12 @@
   </si>
   <si>
     <t>TBD001</t>
+  </si>
+  <si>
+    <t>Stock_Level</t>
+  </si>
+  <si>
+    <t>Stock_Count</t>
   </si>
 </sst>
 </file>
@@ -428,7 +428,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
       <protection hidden="1"/>
@@ -465,26 +465,41 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="128">
-    <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
+  <dxfs count="130">
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -567,7 +582,53 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -829,10 +890,36 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -886,82 +973,6 @@
     <dxf>
       <protection locked="1" hidden="0"/>
     </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1000,11 +1011,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}" name="TEST_Inventory" displayName="TEST_Inventory" ref="A1:F5" totalsRowShown="0">
   <autoFilter ref="A1:F5" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="113"/>
-    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="112"/>
-    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="111"/>
-    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="110"/>
-    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="109">
+    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="116"/>
+    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="115"/>
+    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="114"/>
+    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="113"/>
+    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="112">
       <calculatedColumnFormula>TEST_Inventory[[#This Row],[TEST Integer]]*TEST_Inventory[[#This Row],[TEST Currency]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{AB3A5F3C-FCF0-4466-90FD-8ABB6E18DF5C}" name="TEST Dropdown"/>
@@ -1014,59 +1025,60 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:L2" totalsRowShown="0" headerRowDxfId="127" dataDxfId="126">
-  <autoFilter ref="A1:L2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
-  <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="125"/>
-    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="124"/>
-    <tableColumn id="12" xr3:uid="{8F0FD29C-682B-41B4-82F2-913D40801887}" name="Tag_ID" dataDxfId="123"/>
-    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="122"/>
-    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="121"/>
-    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="120"/>
-    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="119"/>
-    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Current Stock" dataDxfId="118"/>
-    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="117"/>
-    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="116"/>
-    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="115">
-      <calculatedColumnFormula array="1">IF(ISNUMBER(Shop_Consumables[[#This Row],[Current Stock]]),
-    Shop_Consumables[[#This Row],[Current Stock]] * Shop_Consumables[[#This Row],[Unit Cost]],
-    _xlfn.IFS(Shop_Consumables[[#This Row],[Current Stock]]="Many", 1, Shop_Consumables[[#This Row],[Current Stock]]="Adequate", 0.5, Shop_Consumables[[#This Row],[Current Stock]]="Few", 0.1, TRUE, 0) * Shop_Consumables[[#This Row],[Unit Cost]]
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:M2" totalsRowShown="0" headerRowDxfId="40" dataDxfId="39">
+  <autoFilter ref="A1:M2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
+  <tableColumns count="13">
+    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="38"/>
+    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="37"/>
+    <tableColumn id="12" xr3:uid="{8F0FD29C-682B-41B4-82F2-913D40801887}" name="Tag_ID" dataDxfId="36"/>
+    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="35"/>
+    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="34"/>
+    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="33"/>
+    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="32"/>
+    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Stock_Level" dataDxfId="1"/>
+    <tableColumn id="13" xr3:uid="{AA55BCE3-9AC1-4735-8622-15E62CA93E1A}" name="Stock_Count" dataDxfId="0"/>
+    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="31"/>
+    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="30"/>
+    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="29">
+      <calculatedColumnFormula array="1">IF(ISNUMBER(Shop_Consumables[[#This Row],[Stock_Level]]),
+    Shop_Consumables[[#This Row],[Stock_Level]] * Shop_Consumables[[#This Row],[Unit Cost]],
+    _xlfn.IFS(Shop_Consumables[[#This Row],[Stock_Level]]="Many", 1, Shop_Consumables[[#This Row],[Stock_Level]]="Adequate", 0.5, Shop_Consumables[[#This Row],[Stock_Level]]="Few", 0.1, TRUE, 0) * Shop_Consumables[[#This Row],[Unit Cost]]
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Supplier/Remarks" dataDxfId="114"/>
+    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Supplier/Remarks" dataDxfId="28"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:H2" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:H2" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26">
   <autoFilter ref="A1:H2" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="22"/>
-    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="21"/>
-    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="20"/>
-    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="19"/>
-    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="18"/>
-    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="17"/>
-    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="16"/>
-    <tableColumn id="8" xr3:uid="{9140C4E8-CB9E-40BF-ABD9-13A971322B09}" name="Remarks" dataDxfId="15"/>
+    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="25"/>
+    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="24"/>
+    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="23"/>
+    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="22"/>
+    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="21"/>
+    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="20"/>
+    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="19"/>
+    <tableColumn id="8" xr3:uid="{9140C4E8-CB9E-40BF-ABD9-13A971322B09}" name="Remarks" dataDxfId="18"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16">
   <autoFilter ref="A1:G2" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="12"/>
-    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="10"/>
-    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="9"/>
-    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="8"/>
-    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="7"/>
-    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="15"/>
+    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="13"/>
+    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="12"/>
+    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="11"/>
+    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="10"/>
+    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1076,11 +1088,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}" name="Location" displayName="Location" ref="A1:E2" totalsRowShown="0">
   <autoFilter ref="A1:E2" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Description" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Description" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1090,10 +1102,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}" name="TEST_Dashboard" displayName="TEST_Dashboard" ref="A1:B2" totalsRowShown="0">
   <autoFilter ref="A1:B2" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="108">
+    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="111">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Currency])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="107">
+    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="110">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Integer])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1102,41 +1114,41 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:L2" totalsRowShown="0" headerRowDxfId="106" dataDxfId="105">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:L2" totalsRowShown="0" headerRowDxfId="129" dataDxfId="128">
   <autoFilter ref="A1:L2" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="104"/>
-    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="103">
+    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="127"/>
+    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="126">
       <calculatedColumnFormula>SUM(Resell_Inventory[Total Investment])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="102">
+    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="125">
       <calculatedColumnFormula>SUM(Resell_Inventory[Actual Sale Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="101">
+    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="124">
       <calculatedColumnFormula>SUM(Shop_Machinery[Purchase Cost])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="100">
+    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="123">
       <calculatedColumnFormula>SUM(Shop_Power_Tools[Purchase Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="99">
+    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="122">
       <calculatedColumnFormula>SUM(Shop_Hand_Tools[Purchase Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="98">
+    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="121">
       <calculatedColumnFormula>SUM(Shop_Consumables[Current Inventory Value])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="97">
+    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="120">
       <calculatedColumnFormula>SUM(D2,E2,F2,G2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="0">
+    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="119">
       <calculatedColumnFormula array="1">SUMPRODUCT(
-    --( (ISNUMBER(Shop_Consumables[Current Stock])*(Shop_Consumables[Current Stock]&lt;=Shop_Consumables[Reorder Point]))
-    + (Shop_Consumables[Current Stock]="Few") )
+    --( (ISNUMBER(Shop_Consumables[Stock_Level])*(Shop_Consumables[Stock_Level]&lt;=Shop_Consumables[Reorder Point]))
+    + (Shop_Consumables[Stock_Level]="Few") )
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="96">
+    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="118">
       <calculatedColumnFormula>SUMIFS(Shop_Overhead[Amount], Shop_Overhead[Due Date], "&lt;="&amp;TODAY()+30, Shop_Overhead[Due Date], "&gt;="&amp;TODAY())</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{E4065760-B1B1-4564-936B-3405D3B80297}" name="Equipment With Operational Issues" dataDxfId="95">
+    <tableColumn id="12" xr3:uid="{E4065760-B1B1-4564-936B-3405D3B80297}" name="Equipment With Operational Issues" dataDxfId="117">
       <calculatedColumnFormula array="1">SUM(
   COUNTIFS(Shop_Machinery[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"}),
   COUNTIFS(Shop_Power_Tools[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"}),
@@ -1155,8 +1167,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{F579DA07-7AD6-49DA-9B44-D5B1132EDAC6}" name="Overhead_Summary" displayName="Overhead_Summary" ref="A9:B21" totalsRowShown="0">
   <autoFilter ref="A9:B21" xr:uid="{F579DA07-7AD6-49DA-9B44-D5B1132EDAC6}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{7CA4839C-9603-479D-BD1C-8377DFA9603C}" name="Expense Category" dataDxfId="94"/>
-    <tableColumn id="2" xr3:uid="{FE0F7616-EAF3-443D-AC69-DE6541DC10E5}" name="Annual Total" dataDxfId="93">
+    <tableColumn id="1" xr3:uid="{7CA4839C-9603-479D-BD1C-8377DFA9603C}" name="Expense Category" dataDxfId="109"/>
+    <tableColumn id="2" xr3:uid="{FE0F7616-EAF3-443D-AC69-DE6541DC10E5}" name="Annual Total" dataDxfId="108">
       <calculatedColumnFormula>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1165,105 +1177,106 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:O2" totalsRowShown="0" headerRowDxfId="92" dataDxfId="91">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:O2" totalsRowShown="0" headerRowDxfId="107" dataDxfId="106">
   <autoFilter ref="A1:O2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}"/>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="90"/>
-    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="89"/>
-    <tableColumn id="15" xr3:uid="{D25A390C-69B5-4326-A0D4-10EB45DDE5E5}" name="Tag_ID" dataDxfId="88"/>
-    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="87"/>
-    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="86"/>
-    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="85"/>
-    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="84"/>
-    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="83"/>
-    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="82"/>
-    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="81">
+    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="105"/>
+    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="104"/>
+    <tableColumn id="15" xr3:uid="{D25A390C-69B5-4326-A0D4-10EB45DDE5E5}" name="Tag_ID" dataDxfId="103"/>
+    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="102"/>
+    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="101"/>
+    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="100"/>
+    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="99"/>
+    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="98"/>
+    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="97"/>
+    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="96">
       <calculatedColumnFormula>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="80"/>
-    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="79"/>
-    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="78"/>
-    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="77"/>
-    <tableColumn id="16" xr3:uid="{CA8F9851-44B9-4614-9963-24D4EC145034}" name="Sold" dataDxfId="76"/>
+    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="95"/>
+    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="94"/>
+    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="93"/>
+    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="92"/>
+    <tableColumn id="16" xr3:uid="{CA8F9851-44B9-4614-9963-24D4EC145034}" name="Sold" dataDxfId="91"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="75" dataDxfId="74">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="90" dataDxfId="89">
   <autoFilter ref="A1:K2" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="73"/>
-    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="72"/>
-    <tableColumn id="4" xr3:uid="{17EB0B09-11B3-4E08-9442-E3C9AB87A157}" name="Tag_ID" dataDxfId="71"/>
-    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="70"/>
-    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Brand/Model" dataDxfId="69"/>
-    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="68"/>
-    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="67"/>
-    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="66"/>
-    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="65"/>
-    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="64"/>
-    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="63"/>
+    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="88"/>
+    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="87"/>
+    <tableColumn id="4" xr3:uid="{17EB0B09-11B3-4E08-9442-E3C9AB87A157}" name="Tag_ID" dataDxfId="86"/>
+    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="85"/>
+    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Brand/Model" dataDxfId="84"/>
+    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="83"/>
+    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="82"/>
+    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="81"/>
+    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="80"/>
+    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="79"/>
+    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="78"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:K2" totalsRowShown="0" headerRowDxfId="62" dataDxfId="61">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:K2" totalsRowShown="0" headerRowDxfId="77" dataDxfId="76">
   <autoFilter ref="A1:K2" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="60"/>
-    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="59"/>
-    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="58"/>
-    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="57"/>
-    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="56"/>
-    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="55"/>
-    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="54"/>
-    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="53"/>
-    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="52"/>
-    <tableColumn id="11" xr3:uid="{4809319D-ABCA-43DA-A400-5DC91167D78B}" name="Complete" dataDxfId="51"/>
-    <tableColumn id="12" xr3:uid="{920CB592-D743-4B33-A796-C7F3DB32211C}" name="Remarks" dataDxfId="50"/>
+    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="75"/>
+    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="74"/>
+    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="73"/>
+    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="72"/>
+    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="71"/>
+    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="70"/>
+    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="69"/>
+    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="68"/>
+    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="67"/>
+    <tableColumn id="11" xr3:uid="{4809319D-ABCA-43DA-A400-5DC91167D78B}" name="Complete" dataDxfId="66"/>
+    <tableColumn id="12" xr3:uid="{920CB592-D743-4B33-A796-C7F3DB32211C}" name="Remarks" dataDxfId="65"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:K2" totalsRowShown="0" headerRowDxfId="49" dataDxfId="48">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:K2" totalsRowShown="0" headerRowDxfId="64" dataDxfId="63">
   <autoFilter ref="A1:K2" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="47"/>
-    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="46"/>
-    <tableColumn id="11" xr3:uid="{21951C81-00A4-4344-9E81-B1B1DB06ADEF}" name="Tag_ID" dataDxfId="45"/>
-    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="44"/>
-    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Brand/Model" dataDxfId="43"/>
-    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="42"/>
-    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="41"/>
-    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="40"/>
-    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="39"/>
-    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="38"/>
-    <tableColumn id="10" xr3:uid="{26197E01-2936-4F5F-8081-3AA351C1CD38}" name="Remarks" dataDxfId="37"/>
+    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="62"/>
+    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="61"/>
+    <tableColumn id="11" xr3:uid="{21951C81-00A4-4344-9E81-B1B1DB06ADEF}" name="Tag_ID" dataDxfId="60"/>
+    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="59"/>
+    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Brand/Model" dataDxfId="58"/>
+    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="57"/>
+    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="56"/>
+    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="55"/>
+    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="54"/>
+    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="53"/>
+    <tableColumn id="10" xr3:uid="{26197E01-2936-4F5F-8081-3AA351C1CD38}" name="Remarks" dataDxfId="52"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:J2" totalsRowShown="0" headerRowDxfId="36" dataDxfId="35">
-  <autoFilter ref="A1:J2" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}"/>
-  <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="34"/>
-    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="33"/>
-    <tableColumn id="10" xr3:uid="{C8BD69AA-9023-4777-9C96-39A81F1E4BE0}" name="Tag_ID" dataDxfId="32"/>
-    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="31"/>
-    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Brand/Model/Description" dataDxfId="30"/>
-    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="29"/>
-    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="28"/>
-    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="27"/>
-    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Quantity" dataDxfId="26"/>
-    <tableColumn id="9" xr3:uid="{2B57F5E6-66C5-4DBA-8949-836DE0F0791C}" name="Remarks" dataDxfId="25"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:K2" totalsRowShown="0" headerRowDxfId="51" dataDxfId="50">
+  <autoFilter ref="A1:K2" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="49"/>
+    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="48"/>
+    <tableColumn id="10" xr3:uid="{C8BD69AA-9023-4777-9C96-39A81F1E4BE0}" name="Tag_ID" dataDxfId="47"/>
+    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="46"/>
+    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Brand/Model/Description" dataDxfId="45"/>
+    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="44"/>
+    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="43"/>
+    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="42"/>
+    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Stock_Level" dataDxfId="3"/>
+    <tableColumn id="11" xr3:uid="{FD8D2D17-0451-45E0-8688-0BB4F60073DA}" name="Stock_Count" dataDxfId="2"/>
+    <tableColumn id="9" xr3:uid="{2B57F5E6-66C5-4DBA-8949-836DE0F0791C}" name="Remarks" dataDxfId="41"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1602,24 +1615,24 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="E1" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="F1" t="s">
         <v>37</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="F1" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="B2" s="4" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C2" s="8">
         <v>3</v>
@@ -1632,12 +1645,12 @@
         <v>300</v>
       </c>
       <c r="F2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="B3" s="4" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C3" s="8">
         <v>4</v>
@@ -1650,12 +1663,12 @@
         <v>40</v>
       </c>
       <c r="F3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="B4" s="4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C4" s="8">
         <v>5</v>
@@ -1668,12 +1681,12 @@
         <v>100</v>
       </c>
       <c r="F4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="B5" s="4" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C5" s="8">
         <v>1000</v>
@@ -1702,7 +1715,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E1902F1-C59B-4A1A-9D95-2C39AEF944E5}">
   <sheetPr codeName="Sheet7"/>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
@@ -1711,27 +1724,27 @@
     <col min="4" max="4" width="22.6640625" style="6" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="41.6640625" style="2" customWidth="1"/>
     <col min="7" max="7" width="18.44140625" style="2" customWidth="1"/>
-    <col min="8" max="8" width="15.5546875" style="2" customWidth="1"/>
-    <col min="9" max="9" width="14.33203125" style="7" customWidth="1"/>
-    <col min="10" max="10" width="14.109375" style="7" customWidth="1"/>
-    <col min="11" max="11" width="10.44140625" style="3" customWidth="1"/>
-    <col min="13" max="13" width="22.6640625" style="2" customWidth="1"/>
-    <col min="14" max="14" width="46.6640625" style="2" customWidth="1"/>
-    <col min="15" max="16384" width="8.88671875" style="6"/>
+    <col min="8" max="9" width="15.5546875" style="17" customWidth="1"/>
+    <col min="10" max="10" width="14.33203125" style="7" customWidth="1"/>
+    <col min="11" max="11" width="14.109375" style="7" customWidth="1"/>
+    <col min="12" max="12" width="10.44140625" style="3" customWidth="1"/>
+    <col min="14" max="14" width="22.6640625" style="2" customWidth="1"/>
+    <col min="15" max="15" width="46.6640625" style="2" customWidth="1"/>
+    <col min="16" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>2</v>
@@ -1740,40 +1753,42 @@
         <v>3</v>
       </c>
       <c r="G1" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="H1" s="16" t="s">
+        <v>98</v>
+      </c>
+      <c r="I1" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="J1" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="K1" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I1" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="K1" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="L1" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="M1" s="6"/>
+      <c r="L1" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="M1" s="4" t="s">
+        <v>91</v>
+      </c>
       <c r="N1" s="6"/>
-    </row>
-    <row r="2" spans="1:14">
+      <c r="O1" s="6"/>
+    </row>
+    <row r="2" spans="1:15">
       <c r="F2" s="2"/>
-      <c r="H2" s="7"/>
-      <c r="J2" s="3"/>
-      <c r="K2" s="3" cm="1">
-        <f t="array" ref="K2">IF(ISNUMBER(Shop_Consumables[[#This Row],[Current Stock]]),
-    Shop_Consumables[[#This Row],[Current Stock]] * Shop_Consumables[[#This Row],[Unit Cost]],
-    _xlfn.IFS(Shop_Consumables[[#This Row],[Current Stock]]="Many", 1, Shop_Consumables[[#This Row],[Current Stock]]="Adequate", 0.5, Shop_Consumables[[#This Row],[Current Stock]]="Few", 0.1, TRUE, 0) * Shop_Consumables[[#This Row],[Unit Cost]]
+      <c r="K2" s="3"/>
+      <c r="L2" s="3" cm="1">
+        <f t="array" ref="L2">IF(ISNUMBER(Shop_Consumables[[#This Row],[Stock_Level]]),
+    Shop_Consumables[[#This Row],[Stock_Level]] * Shop_Consumables[[#This Row],[Unit Cost]],
+    _xlfn.IFS(Shop_Consumables[[#This Row],[Stock_Level]]="Many", 1, Shop_Consumables[[#This Row],[Stock_Level]]="Adequate", 0.5, Shop_Consumables[[#This Row],[Stock_Level]]="Few", 0.1, TRUE, 0) * Shop_Consumables[[#This Row],[Unit Cost]]
 )</f>
         <v>0</v>
       </c>
-      <c r="L2" s="2"/>
-      <c r="M2" s="6"/>
+      <c r="M2" s="2"/>
       <c r="N2" s="6"/>
+      <c r="O2" s="6"/>
     </row>
   </sheetData>
   <dataValidations disablePrompts="1" count="1">
@@ -1810,25 +1825,25 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="E1" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="G1" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>32</v>
-      </c>
       <c r="H1" s="4" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="I1" s="6"/>
     </row>
@@ -1878,22 +1893,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="G1" s="4" t="s">
         <v>49</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1921,33 +1936,33 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E1" t="s">
         <v>57</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D1" t="s">
-        <v>58</v>
-      </c>
-      <c r="E1" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="1" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="D2" t="s">
         <v>95</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="E2" t="s">
         <v>96</v>
-      </c>
-      <c r="D2" t="s">
-        <v>97</v>
-      </c>
-      <c r="E2" t="s">
-        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -1969,10 +1984,10 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -2019,37 +2034,37 @@
         <v>0</v>
       </c>
       <c r="B1" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="H1" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="I1" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="D1" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="G1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="H1" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="I1" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>71</v>
-      </c>
       <c r="K1" s="8" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L1" s="8" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="2" spans="1:12">
@@ -2083,8 +2098,8 @@
       </c>
       <c r="I2" s="12" cm="1">
         <f t="array" ref="I2">SUMPRODUCT(
-    --( (ISNUMBER(Shop_Consumables[Current Stock])*(Shop_Consumables[Current Stock]&lt;=Shop_Consumables[Reorder Point]))
-    + (Shop_Consumables[Current Stock]="Few") )
+    --( (ISNUMBER(Shop_Consumables[Stock_Level])*(Shop_Consumables[Stock_Level]&lt;=Shop_Consumables[Reorder Point]))
+    + (Shop_Consumables[Stock_Level]="Few") )
 )</f>
         <v>0</v>
       </c>
@@ -2126,15 +2141,15 @@
   <sheetData>
     <row r="9" spans="1:2">
       <c r="A9" s="4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B10" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2143,7 +2158,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B11" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2152,7 +2167,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B12" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2161,7 +2176,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B13" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2170,7 +2185,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B14" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2179,7 +2194,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B15" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2188,7 +2203,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B16" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2197,7 +2212,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B17" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2206,7 +2221,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B18" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2215,7 +2230,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B19" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2224,7 +2239,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B20" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2233,7 +2248,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B21" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2287,10 +2302,10 @@
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>2</v>
@@ -2323,7 +2338,7 @@
         <v>11</v>
       </c>
       <c r="O1" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="P1" s="6"/>
       <c r="R1" s="6"/>
@@ -2386,13 +2401,13 @@
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="F1" s="4" t="s">
         <v>12</v>
@@ -2410,7 +2425,7 @@
         <v>21</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="L1" s="6"/>
     </row>
@@ -2468,7 +2483,7 @@
         <v>1</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E1" s="9" t="s">
         <v>16</v>
@@ -2486,10 +2501,10 @@
         <v>20</v>
       </c>
       <c r="J1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="L1" s="6"/>
       <c r="M1" s="6"/>
@@ -2545,34 +2560,34 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
       <c r="G1" t="s">
+        <v>51</v>
+      </c>
+      <c r="H1" t="s">
+        <v>52</v>
+      </c>
+      <c r="I1" t="s">
         <v>53</v>
-      </c>
-      <c r="H1" t="s">
-        <v>54</v>
-      </c>
-      <c r="I1" t="s">
-        <v>55</v>
       </c>
       <c r="J1" t="s">
         <v>21</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="M1" s="6"/>
     </row>
@@ -2613,7 +2628,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F39ADDA6-CD5F-4655-A9C0-9676DDAC362E}">
   <sheetPr codeName="Sheet6"/>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
@@ -2623,28 +2638,30 @@
     <col min="5" max="5" width="54.6640625" style="2" customWidth="1"/>
     <col min="6" max="6" width="15.6640625" style="3" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.5546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.88671875" style="6" customWidth="1"/>
-    <col min="10" max="10" width="10.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.33203125" style="7" customWidth="1"/>
-    <col min="12" max="12" width="12.88671875" style="2" customWidth="1"/>
-    <col min="13" max="16384" width="8.88671875" style="6"/>
+    <col min="9" max="9" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.6640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.33203125" style="7" customWidth="1"/>
+    <col min="14" max="14" width="12.88671875" style="2" customWidth="1"/>
+    <col min="15" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>5</v>
@@ -2656,29 +2673,35 @@
         <v>21</v>
       </c>
       <c r="I1" t="s">
-        <v>22</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="K1" s="6"/>
+        <v>98</v>
+      </c>
+      <c r="J1" t="s">
+        <v>99</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>88</v>
+      </c>
       <c r="L1" s="6"/>
-    </row>
-    <row r="2" spans="1:12">
+      <c r="M1" s="6"/>
+      <c r="N1" s="6"/>
+    </row>
+    <row r="2" spans="1:14">
       <c r="H2" s="6"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="6"/>
+      <c r="I2" s="6"/>
+      <c r="K2" s="2"/>
       <c r="L2" s="6"/>
+      <c r="M2" s="6"/>
+      <c r="N2" s="6"/>
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L3:L1000 D3:D1000 G3:G1000 I3:I1000" xr:uid="{B6CB3C84-EE01-4878-B558-650FC19D8248}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N3:N1000 D3:D1000 G3:G1000 J3:K1000" xr:uid="{B6CB3C84-EE01-4878-B558-650FC19D8248}">
       <formula1>"Saw, Hammer, Screwdriver, Wrench, Sockets, Pliers, Measuring, Files, Other"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2" xr:uid="{ACB7A40B-F0EE-4387-88E4-5140AB68313F}">
       <formula1>"Fastening/Turning,Measuring/Layout,Striking/Hammering,Gripping/Holding,Cutting/Shaping,Other"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2 J2" xr:uid="{2E543736-2E6D-4F90-9169-21BA7CCD7676}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:K2 H2" xr:uid="{2E543736-2E6D-4F90-9169-21BA7CCD7676}">
       <formula1>"Operational,Needs Repair,Repair In-Progress,Unusable/Junk"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
debug missing dashboard data
</commit_message>
<xml_diff>
--- a/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
+++ b/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1a2ae81d67634e6/Desktop/Michanikos Artifex Enterprises/MAE Custom Digital Solutions/MAE Workshop Inventory Management System/GITHUB_MAE_Workshop Inventory App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="218" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5F13A097-AC2E-4DD5-88E5-94DD3903E83C}"/>
+  <xr:revisionPtr revIDLastSave="221" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D064EFB9-DEE7-42EB-B636-0531BD4D7B14}"/>
   <bookViews>
-    <workbookView xWindow="72" yWindow="660" windowWidth="20508" windowHeight="11904" firstSheet="6" activeTab="9" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
+    <workbookView xWindow="2112" yWindow="924" windowWidth="20508" windowHeight="11904" activeTab="2" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
   </bookViews>
   <sheets>
     <sheet name="TEST Inventory" sheetId="10" r:id="rId1"/>
@@ -428,7 +428,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
       <protection hidden="1"/>
@@ -465,10 +465,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -476,159 +472,101 @@
   <dxfs count="130">
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -887,28 +825,6 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
@@ -973,6 +889,86 @@
     <dxf>
       <protection locked="1" hidden="0"/>
     </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1011,11 +1007,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}" name="TEST_Inventory" displayName="TEST_Inventory" ref="A1:F5" totalsRowShown="0">
   <autoFilter ref="A1:F5" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="116"/>
-    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="115"/>
-    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="114"/>
-    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="113"/>
-    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="112">
+    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="114"/>
+    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="113"/>
+    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="112"/>
+    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="111"/>
+    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="110">
       <calculatedColumnFormula>TEST_Inventory[[#This Row],[TEST Integer]]*TEST_Inventory[[#This Row],[TEST Currency]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{AB3A5F3C-FCF0-4466-90FD-8ABB6E18DF5C}" name="TEST Dropdown"/>
@@ -1025,60 +1021,60 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:M2" totalsRowShown="0" headerRowDxfId="40" dataDxfId="39">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:M2" totalsRowShown="0" headerRowDxfId="129" dataDxfId="128">
   <autoFilter ref="A1:M2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="38"/>
-    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="37"/>
-    <tableColumn id="12" xr3:uid="{8F0FD29C-682B-41B4-82F2-913D40801887}" name="Tag_ID" dataDxfId="36"/>
-    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="35"/>
-    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="34"/>
-    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="33"/>
-    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="32"/>
-    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Stock_Level" dataDxfId="1"/>
-    <tableColumn id="13" xr3:uid="{AA55BCE3-9AC1-4735-8622-15E62CA93E1A}" name="Stock_Count" dataDxfId="0"/>
-    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="31"/>
-    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="30"/>
-    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="29">
+    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="127"/>
+    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="126"/>
+    <tableColumn id="12" xr3:uid="{8F0FD29C-682B-41B4-82F2-913D40801887}" name="Tag_ID" dataDxfId="125"/>
+    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="124"/>
+    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="123"/>
+    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="122"/>
+    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="121"/>
+    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Stock_Level" dataDxfId="120"/>
+    <tableColumn id="13" xr3:uid="{AA55BCE3-9AC1-4735-8622-15E62CA93E1A}" name="Stock_Count" dataDxfId="119"/>
+    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="118"/>
+    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="117"/>
+    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="116">
       <calculatedColumnFormula array="1">IF(ISNUMBER(Shop_Consumables[[#This Row],[Stock_Level]]),
     Shop_Consumables[[#This Row],[Stock_Level]] * Shop_Consumables[[#This Row],[Unit Cost]],
     _xlfn.IFS(Shop_Consumables[[#This Row],[Stock_Level]]="Many", 1, Shop_Consumables[[#This Row],[Stock_Level]]="Adequate", 0.5, Shop_Consumables[[#This Row],[Stock_Level]]="Few", 0.1, TRUE, 0) * Shop_Consumables[[#This Row],[Unit Cost]]
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Supplier/Remarks" dataDxfId="28"/>
+    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Supplier/Remarks" dataDxfId="115"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:H2" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:H2" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
   <autoFilter ref="A1:H2" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="25"/>
-    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="24"/>
-    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="23"/>
-    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="22"/>
-    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="21"/>
-    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="20"/>
-    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="19"/>
-    <tableColumn id="8" xr3:uid="{9140C4E8-CB9E-40BF-ABD9-13A971322B09}" name="Remarks" dataDxfId="18"/>
+    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="20"/>
+    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="19"/>
+    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="18"/>
+    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="17"/>
+    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="16"/>
+    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="15"/>
+    <tableColumn id="8" xr3:uid="{9140C4E8-CB9E-40BF-ABD9-13A971322B09}" name="Remarks" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
   <autoFilter ref="A1:G2" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="15"/>
-    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="13"/>
-    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="12"/>
-    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="11"/>
-    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="10"/>
-    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="9"/>
+    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="11"/>
+    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="9"/>
+    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="7"/>
+    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="6"/>
+    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1088,11 +1084,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}" name="Location" displayName="Location" ref="A1:E2" totalsRowShown="0">
   <autoFilter ref="A1:E2" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Description" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="4"/>
+    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Description" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1102,10 +1098,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}" name="TEST_Dashboard" displayName="TEST_Dashboard" ref="A1:B2" totalsRowShown="0">
   <autoFilter ref="A1:B2" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="111">
+    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="109">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Currency])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="110">
+    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="108">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Integer])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1114,41 +1110,41 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:L2" totalsRowShown="0" headerRowDxfId="129" dataDxfId="128">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:L2" totalsRowShown="0" headerRowDxfId="107" dataDxfId="106">
   <autoFilter ref="A1:L2" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="127"/>
-    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="126">
+    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="105"/>
+    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="104">
       <calculatedColumnFormula>SUM(Resell_Inventory[Total Investment])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="125">
+    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="103">
       <calculatedColumnFormula>SUM(Resell_Inventory[Actual Sale Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="124">
+    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="102">
       <calculatedColumnFormula>SUM(Shop_Machinery[Purchase Cost])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="123">
+    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="101">
       <calculatedColumnFormula>SUM(Shop_Power_Tools[Purchase Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="122">
+    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="100">
       <calculatedColumnFormula>SUM(Shop_Hand_Tools[Purchase Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="121">
+    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="99">
       <calculatedColumnFormula>SUM(Shop_Consumables[Current Inventory Value])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="120">
+    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="98">
       <calculatedColumnFormula>SUM(D2,E2,F2,G2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="119">
+    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="97">
       <calculatedColumnFormula array="1">SUMPRODUCT(
-    --( (ISNUMBER(Shop_Consumables[Stock_Level])*(Shop_Consumables[Stock_Level]&lt;=Shop_Consumables[Reorder Point]))
+    --( (ISNUMBER(Shop_Consumables[Stock_Count])*(Shop_Consumables[Stock_Count]&lt;=Shop_Consumables[Reorder Point]))
     + (Shop_Consumables[Stock_Level]="Few") )
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="118">
+    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="96">
       <calculatedColumnFormula>SUMIFS(Shop_Overhead[Amount], Shop_Overhead[Due Date], "&lt;="&amp;TODAY()+30, Shop_Overhead[Due Date], "&gt;="&amp;TODAY())</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{E4065760-B1B1-4564-936B-3405D3B80297}" name="Equipment With Operational Issues" dataDxfId="117">
+    <tableColumn id="12" xr3:uid="{E4065760-B1B1-4564-936B-3405D3B80297}" name="Equipment With Operational Issues" dataDxfId="95">
       <calculatedColumnFormula array="1">SUM(
   COUNTIFS(Shop_Machinery[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"}),
   COUNTIFS(Shop_Power_Tools[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"}),
@@ -1167,8 +1163,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{F579DA07-7AD6-49DA-9B44-D5B1132EDAC6}" name="Overhead_Summary" displayName="Overhead_Summary" ref="A9:B21" totalsRowShown="0">
   <autoFilter ref="A9:B21" xr:uid="{F579DA07-7AD6-49DA-9B44-D5B1132EDAC6}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{7CA4839C-9603-479D-BD1C-8377DFA9603C}" name="Expense Category" dataDxfId="109"/>
-    <tableColumn id="2" xr3:uid="{FE0F7616-EAF3-443D-AC69-DE6541DC10E5}" name="Annual Total" dataDxfId="108">
+    <tableColumn id="1" xr3:uid="{7CA4839C-9603-479D-BD1C-8377DFA9603C}" name="Expense Category" dataDxfId="94"/>
+    <tableColumn id="2" xr3:uid="{FE0F7616-EAF3-443D-AC69-DE6541DC10E5}" name="Annual Total" dataDxfId="93">
       <calculatedColumnFormula>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1177,106 +1173,106 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:O2" totalsRowShown="0" headerRowDxfId="107" dataDxfId="106">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:O2" totalsRowShown="0" headerRowDxfId="92" dataDxfId="91">
   <autoFilter ref="A1:O2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}"/>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="105"/>
-    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="104"/>
-    <tableColumn id="15" xr3:uid="{D25A390C-69B5-4326-A0D4-10EB45DDE5E5}" name="Tag_ID" dataDxfId="103"/>
-    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="102"/>
-    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="101"/>
-    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="100"/>
-    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="99"/>
-    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="98"/>
-    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="97"/>
-    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="96">
+    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="90"/>
+    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="89"/>
+    <tableColumn id="15" xr3:uid="{D25A390C-69B5-4326-A0D4-10EB45DDE5E5}" name="Tag_ID" dataDxfId="88"/>
+    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="87"/>
+    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="86"/>
+    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="85"/>
+    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="84"/>
+    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="83"/>
+    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="82"/>
+    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="81">
       <calculatedColumnFormula>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="95"/>
-    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="94"/>
-    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="93"/>
-    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="92"/>
-    <tableColumn id="16" xr3:uid="{CA8F9851-44B9-4614-9963-24D4EC145034}" name="Sold" dataDxfId="91"/>
+    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="80"/>
+    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="79"/>
+    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="78"/>
+    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="77"/>
+    <tableColumn id="16" xr3:uid="{CA8F9851-44B9-4614-9963-24D4EC145034}" name="Sold" dataDxfId="76"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="90" dataDxfId="89">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="75" dataDxfId="74">
   <autoFilter ref="A1:K2" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="88"/>
-    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="87"/>
-    <tableColumn id="4" xr3:uid="{17EB0B09-11B3-4E08-9442-E3C9AB87A157}" name="Tag_ID" dataDxfId="86"/>
-    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="85"/>
-    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Brand/Model" dataDxfId="84"/>
-    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="83"/>
-    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="82"/>
-    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="81"/>
-    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="80"/>
-    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="79"/>
-    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="78"/>
+    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="73"/>
+    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="72"/>
+    <tableColumn id="4" xr3:uid="{17EB0B09-11B3-4E08-9442-E3C9AB87A157}" name="Tag_ID" dataDxfId="71"/>
+    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="70"/>
+    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Brand/Model" dataDxfId="69"/>
+    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="68"/>
+    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="67"/>
+    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="66"/>
+    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="65"/>
+    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="64"/>
+    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="63"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:K2" totalsRowShown="0" headerRowDxfId="77" dataDxfId="76">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:K2" totalsRowShown="0" headerRowDxfId="62" dataDxfId="61">
   <autoFilter ref="A1:K2" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="75"/>
-    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="74"/>
-    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="73"/>
-    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="72"/>
-    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="71"/>
-    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="70"/>
-    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="69"/>
-    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="68"/>
-    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="67"/>
-    <tableColumn id="11" xr3:uid="{4809319D-ABCA-43DA-A400-5DC91167D78B}" name="Complete" dataDxfId="66"/>
-    <tableColumn id="12" xr3:uid="{920CB592-D743-4B33-A796-C7F3DB32211C}" name="Remarks" dataDxfId="65"/>
+    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="60"/>
+    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="59"/>
+    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="58"/>
+    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="57"/>
+    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="56"/>
+    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="55"/>
+    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="54"/>
+    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="53"/>
+    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="52"/>
+    <tableColumn id="11" xr3:uid="{4809319D-ABCA-43DA-A400-5DC91167D78B}" name="Complete" dataDxfId="51"/>
+    <tableColumn id="12" xr3:uid="{920CB592-D743-4B33-A796-C7F3DB32211C}" name="Remarks" dataDxfId="50"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:K2" totalsRowShown="0" headerRowDxfId="64" dataDxfId="63">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:K2" totalsRowShown="0" headerRowDxfId="49" dataDxfId="48">
   <autoFilter ref="A1:K2" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="62"/>
-    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="61"/>
-    <tableColumn id="11" xr3:uid="{21951C81-00A4-4344-9E81-B1B1DB06ADEF}" name="Tag_ID" dataDxfId="60"/>
-    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="59"/>
-    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Brand/Model" dataDxfId="58"/>
-    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="57"/>
-    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="56"/>
-    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="55"/>
-    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="54"/>
-    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="53"/>
-    <tableColumn id="10" xr3:uid="{26197E01-2936-4F5F-8081-3AA351C1CD38}" name="Remarks" dataDxfId="52"/>
+    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="47"/>
+    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="46"/>
+    <tableColumn id="11" xr3:uid="{21951C81-00A4-4344-9E81-B1B1DB06ADEF}" name="Tag_ID" dataDxfId="45"/>
+    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="44"/>
+    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Brand/Model" dataDxfId="43"/>
+    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="42"/>
+    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="41"/>
+    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="40"/>
+    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="39"/>
+    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="38"/>
+    <tableColumn id="10" xr3:uid="{26197E01-2936-4F5F-8081-3AA351C1CD38}" name="Remarks" dataDxfId="37"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:K2" totalsRowShown="0" headerRowDxfId="51" dataDxfId="50">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:K2" totalsRowShown="0" headerRowDxfId="36" dataDxfId="35">
   <autoFilter ref="A1:K2" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="49"/>
-    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="48"/>
-    <tableColumn id="10" xr3:uid="{C8BD69AA-9023-4777-9C96-39A81F1E4BE0}" name="Tag_ID" dataDxfId="47"/>
-    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="46"/>
-    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Brand/Model/Description" dataDxfId="45"/>
-    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="44"/>
-    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="43"/>
-    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="42"/>
-    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Stock_Level" dataDxfId="3"/>
-    <tableColumn id="11" xr3:uid="{FD8D2D17-0451-45E0-8688-0BB4F60073DA}" name="Stock_Count" dataDxfId="2"/>
-    <tableColumn id="9" xr3:uid="{2B57F5E6-66C5-4DBA-8949-836DE0F0791C}" name="Remarks" dataDxfId="41"/>
+    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="34"/>
+    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="33"/>
+    <tableColumn id="10" xr3:uid="{C8BD69AA-9023-4777-9C96-39A81F1E4BE0}" name="Tag_ID" dataDxfId="32"/>
+    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="31"/>
+    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Brand/Model/Description" dataDxfId="30"/>
+    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="29"/>
+    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="28"/>
+    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="27"/>
+    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Stock_Level" dataDxfId="26"/>
+    <tableColumn id="11" xr3:uid="{FD8D2D17-0451-45E0-8688-0BB4F60073DA}" name="Stock_Count" dataDxfId="25"/>
+    <tableColumn id="9" xr3:uid="{2B57F5E6-66C5-4DBA-8949-836DE0F0791C}" name="Remarks" dataDxfId="24"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1724,7 +1720,7 @@
     <col min="4" max="4" width="22.6640625" style="6" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="41.6640625" style="2" customWidth="1"/>
     <col min="7" max="7" width="18.44140625" style="2" customWidth="1"/>
-    <col min="8" max="9" width="15.5546875" style="17" customWidth="1"/>
+    <col min="8" max="9" width="15.5546875" style="6" customWidth="1"/>
     <col min="10" max="10" width="14.33203125" style="7" customWidth="1"/>
     <col min="11" max="11" width="14.109375" style="7" customWidth="1"/>
     <col min="12" max="12" width="10.44140625" style="3" customWidth="1"/>
@@ -1755,10 +1751,10 @@
       <c r="G1" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="16" t="s">
+      <c r="H1" t="s">
         <v>98</v>
       </c>
-      <c r="I1" s="16" t="s">
+      <c r="I1" t="s">
         <v>99</v>
       </c>
       <c r="J1" s="8" t="s">
@@ -2098,7 +2094,7 @@
       </c>
       <c r="I2" s="12" cm="1">
         <f t="array" ref="I2">SUMPRODUCT(
-    --( (ISNUMBER(Shop_Consumables[Stock_Level])*(Shop_Consumables[Stock_Level]&lt;=Shop_Consumables[Reorder Point]))
+    --( (ISNUMBER(Shop_Consumables[Stock_Count])*(Shop_Consumables[Stock_Count]&lt;=Shop_Consumables[Reorder Point]))
     + (Shop_Consumables[Stock_Level]="Few") )
 )</f>
         <v>0</v>

</xml_diff>

<commit_message>
removed "Sold" dropdown in Resell Inventory, adjusted Excel adn Config to use dropdown"SOLD" to filter for actual resell sales; changed UI renderTable to only highlight overdue dates (Overhead and Maintenance)
</commit_message>
<xml_diff>
--- a/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
+++ b/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1a2ae81d67634e6/Desktop/Michanikos Artifex Enterprises/MAE Custom Digital Solutions/MAE Workshop Inventory Management System/GITHUB_MAE_Workshop Inventory App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="221" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D064EFB9-DEE7-42EB-B636-0531BD4D7B14}"/>
+  <xr:revisionPtr revIDLastSave="223" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6E8078A7-5E1D-4478-A36F-98DDF835FF7C}"/>
   <bookViews>
-    <workbookView xWindow="2112" yWindow="924" windowWidth="20508" windowHeight="11904" activeTab="2" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
+    <workbookView xWindow="2112" yWindow="336" windowWidth="20508" windowHeight="11904" firstSheet="1" activeTab="4" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
   </bookViews>
   <sheets>
     <sheet name="TEST Inventory" sheetId="10" r:id="rId1"/>
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="99">
   <si>
     <t>mae_id</t>
   </si>
@@ -328,9 +328,6 @@
   </si>
   <si>
     <t>Maintenance Items Due in Next 30 Days</t>
-  </si>
-  <si>
-    <t>Sold</t>
   </si>
   <si>
     <t>Machine Name/Brand/Model</t>
@@ -469,7 +466,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="130">
+  <dxfs count="129">
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -547,6 +544,64 @@
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -755,10 +810,6 @@
       <protection locked="1" hidden="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="1"/>
     </dxf>
@@ -825,6 +876,28 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
@@ -889,86 +962,6 @@
     <dxf>
       <protection locked="1" hidden="0"/>
     </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1007,11 +1000,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}" name="TEST_Inventory" displayName="TEST_Inventory" ref="A1:F5" totalsRowShown="0">
   <autoFilter ref="A1:F5" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="114"/>
-    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="113"/>
-    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="112"/>
-    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="111"/>
-    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="110">
+    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="115"/>
+    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="114"/>
+    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="113"/>
+    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="112"/>
+    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="111">
       <calculatedColumnFormula>TEST_Inventory[[#This Row],[TEST Integer]]*TEST_Inventory[[#This Row],[TEST Currency]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{AB3A5F3C-FCF0-4466-90FD-8ABB6E18DF5C}" name="TEST Dropdown"/>
@@ -1021,27 +1014,27 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:M2" totalsRowShown="0" headerRowDxfId="129" dataDxfId="128">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:M2" totalsRowShown="0" headerRowDxfId="38" dataDxfId="37">
   <autoFilter ref="A1:M2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="127"/>
-    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="126"/>
-    <tableColumn id="12" xr3:uid="{8F0FD29C-682B-41B4-82F2-913D40801887}" name="Tag_ID" dataDxfId="125"/>
-    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="124"/>
-    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="123"/>
-    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="122"/>
-    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="121"/>
-    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Stock_Level" dataDxfId="120"/>
-    <tableColumn id="13" xr3:uid="{AA55BCE3-9AC1-4735-8622-15E62CA93E1A}" name="Stock_Count" dataDxfId="119"/>
-    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="118"/>
-    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="117"/>
-    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="116">
+    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="36"/>
+    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="35"/>
+    <tableColumn id="12" xr3:uid="{8F0FD29C-682B-41B4-82F2-913D40801887}" name="Tag_ID" dataDxfId="34"/>
+    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="33"/>
+    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="32"/>
+    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="31"/>
+    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="30"/>
+    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Stock_Level" dataDxfId="29"/>
+    <tableColumn id="13" xr3:uid="{AA55BCE3-9AC1-4735-8622-15E62CA93E1A}" name="Stock_Count" dataDxfId="28"/>
+    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="27"/>
+    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="26"/>
+    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="25">
       <calculatedColumnFormula array="1">IF(ISNUMBER(Shop_Consumables[[#This Row],[Stock_Level]]),
     Shop_Consumables[[#This Row],[Stock_Level]] * Shop_Consumables[[#This Row],[Unit Cost]],
     _xlfn.IFS(Shop_Consumables[[#This Row],[Stock_Level]]="Many", 1, Shop_Consumables[[#This Row],[Stock_Level]]="Adequate", 0.5, Shop_Consumables[[#This Row],[Stock_Level]]="Few", 0.1, TRUE, 0) * Shop_Consumables[[#This Row],[Unit Cost]]
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Supplier/Remarks" dataDxfId="115"/>
+    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Supplier/Remarks" dataDxfId="24"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1098,10 +1091,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}" name="TEST_Dashboard" displayName="TEST_Dashboard" ref="A1:B2" totalsRowShown="0">
   <autoFilter ref="A1:B2" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="109">
+    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="110">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Currency])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="108">
+    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="109">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Integer])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1110,41 +1103,41 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:L2" totalsRowShown="0" headerRowDxfId="107" dataDxfId="106">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:L2" totalsRowShown="0" headerRowDxfId="128" dataDxfId="127">
   <autoFilter ref="A1:L2" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="105"/>
-    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="104">
-      <calculatedColumnFormula>SUM(Resell_Inventory[Total Investment])</calculatedColumnFormula>
+    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="126"/>
+    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="125">
+      <calculatedColumnFormula>SUMIFS(Resell_Inventory[Actual Sale Price], Resell_Inventory[Current Status], "Sold")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="103">
+    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="124">
       <calculatedColumnFormula>SUM(Resell_Inventory[Actual Sale Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="102">
+    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="123">
       <calculatedColumnFormula>SUM(Shop_Machinery[Purchase Cost])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="101">
+    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="122">
       <calculatedColumnFormula>SUM(Shop_Power_Tools[Purchase Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="100">
+    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="121">
       <calculatedColumnFormula>SUM(Shop_Hand_Tools[Purchase Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="99">
+    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="120">
       <calculatedColumnFormula>SUM(Shop_Consumables[Current Inventory Value])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="98">
+    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="119">
       <calculatedColumnFormula>SUM(D2,E2,F2,G2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="97">
+    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="118">
       <calculatedColumnFormula array="1">SUMPRODUCT(
     --( (ISNUMBER(Shop_Consumables[Stock_Count])*(Shop_Consumables[Stock_Count]&lt;=Shop_Consumables[Reorder Point]))
     + (Shop_Consumables[Stock_Level]="Few") )
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="96">
+    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="117">
       <calculatedColumnFormula>SUMIFS(Shop_Overhead[Amount], Shop_Overhead[Due Date], "&lt;="&amp;TODAY()+30, Shop_Overhead[Due Date], "&gt;="&amp;TODAY())</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{E4065760-B1B1-4564-936B-3405D3B80297}" name="Equipment With Operational Issues" dataDxfId="95">
+    <tableColumn id="12" xr3:uid="{E4065760-B1B1-4564-936B-3405D3B80297}" name="Equipment With Operational Issues" dataDxfId="116">
       <calculatedColumnFormula array="1">SUM(
   COUNTIFS(Shop_Machinery[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"}),
   COUNTIFS(Shop_Power_Tools[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"}),
@@ -1163,8 +1156,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{F579DA07-7AD6-49DA-9B44-D5B1132EDAC6}" name="Overhead_Summary" displayName="Overhead_Summary" ref="A9:B21" totalsRowShown="0">
   <autoFilter ref="A9:B21" xr:uid="{F579DA07-7AD6-49DA-9B44-D5B1132EDAC6}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{7CA4839C-9603-479D-BD1C-8377DFA9603C}" name="Expense Category" dataDxfId="94"/>
-    <tableColumn id="2" xr3:uid="{FE0F7616-EAF3-443D-AC69-DE6541DC10E5}" name="Annual Total" dataDxfId="93">
+    <tableColumn id="1" xr3:uid="{7CA4839C-9603-479D-BD1C-8377DFA9603C}" name="Expense Category" dataDxfId="108"/>
+    <tableColumn id="2" xr3:uid="{FE0F7616-EAF3-443D-AC69-DE6541DC10E5}" name="Annual Total" dataDxfId="107">
       <calculatedColumnFormula>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1173,106 +1166,105 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:O2" totalsRowShown="0" headerRowDxfId="92" dataDxfId="91">
-  <autoFilter ref="A1:O2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}"/>
-  <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="90"/>
-    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="89"/>
-    <tableColumn id="15" xr3:uid="{D25A390C-69B5-4326-A0D4-10EB45DDE5E5}" name="Tag_ID" dataDxfId="88"/>
-    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="87"/>
-    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="86"/>
-    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="85"/>
-    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="84"/>
-    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="83"/>
-    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="82"/>
-    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="81">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:N2" totalsRowShown="0" headerRowDxfId="106" dataDxfId="105">
+  <autoFilter ref="A1:N2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}"/>
+  <tableColumns count="14">
+    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="104"/>
+    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="103"/>
+    <tableColumn id="15" xr3:uid="{D25A390C-69B5-4326-A0D4-10EB45DDE5E5}" name="Tag_ID" dataDxfId="102"/>
+    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="101"/>
+    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="100"/>
+    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="99"/>
+    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="98"/>
+    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="97"/>
+    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="96"/>
+    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="95">
       <calculatedColumnFormula>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="80"/>
-    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="79"/>
-    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="78"/>
-    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="77"/>
-    <tableColumn id="16" xr3:uid="{CA8F9851-44B9-4614-9963-24D4EC145034}" name="Sold" dataDxfId="76"/>
+    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="94"/>
+    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="93"/>
+    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="92"/>
+    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="91"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="75" dataDxfId="74">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="90" dataDxfId="89">
   <autoFilter ref="A1:K2" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="73"/>
-    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="72"/>
-    <tableColumn id="4" xr3:uid="{17EB0B09-11B3-4E08-9442-E3C9AB87A157}" name="Tag_ID" dataDxfId="71"/>
-    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="70"/>
-    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Brand/Model" dataDxfId="69"/>
-    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="68"/>
-    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="67"/>
-    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="66"/>
-    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="65"/>
-    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="64"/>
-    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="63"/>
+    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="88"/>
+    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="87"/>
+    <tableColumn id="4" xr3:uid="{17EB0B09-11B3-4E08-9442-E3C9AB87A157}" name="Tag_ID" dataDxfId="86"/>
+    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="85"/>
+    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Brand/Model" dataDxfId="84"/>
+    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="83"/>
+    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="82"/>
+    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="81"/>
+    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="80"/>
+    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="79"/>
+    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="78"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:K2" totalsRowShown="0" headerRowDxfId="62" dataDxfId="61">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:K2" totalsRowShown="0" headerRowDxfId="77" dataDxfId="76">
   <autoFilter ref="A1:K2" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="60"/>
-    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="59"/>
-    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="58"/>
-    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="57"/>
-    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="56"/>
-    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="55"/>
-    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="54"/>
-    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="53"/>
-    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="52"/>
-    <tableColumn id="11" xr3:uid="{4809319D-ABCA-43DA-A400-5DC91167D78B}" name="Complete" dataDxfId="51"/>
-    <tableColumn id="12" xr3:uid="{920CB592-D743-4B33-A796-C7F3DB32211C}" name="Remarks" dataDxfId="50"/>
+    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="75"/>
+    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="74"/>
+    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="73"/>
+    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="72"/>
+    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="71"/>
+    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="70"/>
+    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="69"/>
+    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="68"/>
+    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="67"/>
+    <tableColumn id="11" xr3:uid="{4809319D-ABCA-43DA-A400-5DC91167D78B}" name="Complete" dataDxfId="66"/>
+    <tableColumn id="12" xr3:uid="{920CB592-D743-4B33-A796-C7F3DB32211C}" name="Remarks" dataDxfId="65"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:K2" totalsRowShown="0" headerRowDxfId="49" dataDxfId="48">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:K2" totalsRowShown="0" headerRowDxfId="64" dataDxfId="63">
   <autoFilter ref="A1:K2" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="47"/>
-    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="46"/>
-    <tableColumn id="11" xr3:uid="{21951C81-00A4-4344-9E81-B1B1DB06ADEF}" name="Tag_ID" dataDxfId="45"/>
-    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="44"/>
-    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Brand/Model" dataDxfId="43"/>
-    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="42"/>
-    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="41"/>
-    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="40"/>
-    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="39"/>
-    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="38"/>
-    <tableColumn id="10" xr3:uid="{26197E01-2936-4F5F-8081-3AA351C1CD38}" name="Remarks" dataDxfId="37"/>
+    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="62"/>
+    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="61"/>
+    <tableColumn id="11" xr3:uid="{21951C81-00A4-4344-9E81-B1B1DB06ADEF}" name="Tag_ID" dataDxfId="60"/>
+    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="59"/>
+    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Brand/Model" dataDxfId="58"/>
+    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="57"/>
+    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="56"/>
+    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="55"/>
+    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="54"/>
+    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="53"/>
+    <tableColumn id="10" xr3:uid="{26197E01-2936-4F5F-8081-3AA351C1CD38}" name="Remarks" dataDxfId="52"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:K2" totalsRowShown="0" headerRowDxfId="36" dataDxfId="35">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:K2" totalsRowShown="0" headerRowDxfId="51" dataDxfId="50">
   <autoFilter ref="A1:K2" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="34"/>
-    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="33"/>
-    <tableColumn id="10" xr3:uid="{C8BD69AA-9023-4777-9C96-39A81F1E4BE0}" name="Tag_ID" dataDxfId="32"/>
-    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="31"/>
-    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Brand/Model/Description" dataDxfId="30"/>
-    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="29"/>
-    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="28"/>
-    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="27"/>
-    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Stock_Level" dataDxfId="26"/>
-    <tableColumn id="11" xr3:uid="{FD8D2D17-0451-45E0-8688-0BB4F60073DA}" name="Stock_Count" dataDxfId="25"/>
-    <tableColumn id="9" xr3:uid="{2B57F5E6-66C5-4DBA-8949-836DE0F0791C}" name="Remarks" dataDxfId="24"/>
+    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="49"/>
+    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="48"/>
+    <tableColumn id="10" xr3:uid="{C8BD69AA-9023-4777-9C96-39A81F1E4BE0}" name="Tag_ID" dataDxfId="47"/>
+    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="46"/>
+    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Brand/Model/Description" dataDxfId="45"/>
+    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="44"/>
+    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="43"/>
+    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="42"/>
+    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Stock_Level" dataDxfId="41"/>
+    <tableColumn id="11" xr3:uid="{FD8D2D17-0451-45E0-8688-0BB4F60073DA}" name="Stock_Count" dataDxfId="40"/>
+    <tableColumn id="9" xr3:uid="{2B57F5E6-66C5-4DBA-8949-836DE0F0791C}" name="Remarks" dataDxfId="39"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1737,7 +1729,7 @@
         <v>59</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D1" t="s">
         <v>55</v>
@@ -1752,10 +1744,10 @@
         <v>22</v>
       </c>
       <c r="H1" t="s">
+        <v>97</v>
+      </c>
+      <c r="I1" t="s">
         <v>98</v>
-      </c>
-      <c r="I1" t="s">
-        <v>99</v>
       </c>
       <c r="J1" s="8" t="s">
         <v>23</v>
@@ -1767,7 +1759,7 @@
         <v>54</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="N1" s="6"/>
       <c r="O1" s="6"/>
@@ -1839,7 +1831,7 @@
         <v>30</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="I1" s="6"/>
     </row>
@@ -1946,19 +1938,19 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="D2" t="s">
         <v>94</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>95</v>
-      </c>
-      <c r="E2" t="s">
-        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -2065,7 +2057,7 @@
     </row>
     <row r="2" spans="1:12">
       <c r="B2" s="3">
-        <f>SUM(Resell_Inventory[Total Investment])</f>
+        <f>SUMIFS(Resell_Inventory[Actual Sale Price], Resell_Inventory[Current Status], "Sold")</f>
         <v>0</v>
       </c>
       <c r="C2" s="3">
@@ -2267,7 +2259,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDE7BF89-A2E7-4A6F-B822-317739E206EC}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:Q2"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
@@ -2284,13 +2276,13 @@
     <col min="12" max="12" width="16.6640625" style="3" customWidth="1"/>
     <col min="13" max="13" width="16.88671875" style="3" customWidth="1"/>
     <col min="14" max="14" width="16.88671875" style="14" customWidth="1"/>
-    <col min="16" max="16" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="16.88671875" style="6" customWidth="1"/>
-    <col min="18" max="18" width="16.88671875" style="2" customWidth="1"/>
-    <col min="19" max="16384" width="8.88671875" style="6"/>
+    <col min="15" max="15" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="16.88671875" style="6" customWidth="1"/>
+    <col min="17" max="17" width="16.88671875" style="2" customWidth="1"/>
+    <col min="18" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18">
+    <row r="1" spans="1:17">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2298,7 +2290,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D1" t="s">
         <v>55</v>
@@ -2333,21 +2325,17 @@
       <c r="N1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="O1" t="s">
-        <v>85</v>
-      </c>
-      <c r="P1" s="6"/>
-      <c r="R1" s="6"/>
-    </row>
-    <row r="2" spans="1:18">
+      <c r="O1" s="6"/>
+      <c r="Q1" s="6"/>
+    </row>
+    <row r="2" spans="1:17">
       <c r="D2" s="6"/>
       <c r="J2" s="5">
         <f>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</f>
         <v>0</v>
       </c>
       <c r="O2" s="6"/>
-      <c r="P2" s="6"/>
-      <c r="R2" s="6"/>
+      <c r="Q2" s="6"/>
     </row>
   </sheetData>
   <dataValidations count="3">
@@ -2397,13 +2385,13 @@
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D1" t="s">
         <v>55</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F1" s="4" t="s">
         <v>12</v>
@@ -2497,10 +2485,10 @@
         <v>20</v>
       </c>
       <c r="J1" t="s">
+        <v>86</v>
+      </c>
+      <c r="K1" s="4" t="s">
         <v>87</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>88</v>
       </c>
       <c r="L1" s="6"/>
       <c r="M1" s="6"/>
@@ -2559,13 +2547,13 @@
         <v>59</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D1" t="s">
         <v>55</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>5</v>
@@ -2583,7 +2571,7 @@
         <v>21</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="M1" s="6"/>
     </row>
@@ -2651,13 +2639,13 @@
         <v>59</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D1" t="s">
         <v>55</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>5</v>
@@ -2669,13 +2657,13 @@
         <v>21</v>
       </c>
       <c r="I1" t="s">
+        <v>97</v>
+      </c>
+      <c r="J1" t="s">
         <v>98</v>
       </c>
-      <c r="J1" t="s">
-        <v>99</v>
-      </c>
       <c r="K1" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="L1" s="6"/>
       <c r="M1" s="6"/>

</xml_diff>

<commit_message>
adding Valuation Governance/Methodology Enforcement for Bulk vs Individual items in Shop Consumables
</commit_message>
<xml_diff>
--- a/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
+++ b/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1a2ae81d67634e6/Desktop/Michanikos Artifex Enterprises/MAE Custom Digital Solutions/MAE Workshop Inventory Management System/GITHUB_MAE_Workshop Inventory App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="223" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6E8078A7-5E1D-4478-A36F-98DDF835FF7C}"/>
+  <xr:revisionPtr revIDLastSave="231" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{007C75AC-1EC2-40BF-B9F4-F7453B5D9ADE}"/>
   <bookViews>
-    <workbookView xWindow="2112" yWindow="336" windowWidth="20508" windowHeight="11904" firstSheet="1" activeTab="4" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="7" activeTab="9" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
   </bookViews>
   <sheets>
     <sheet name="TEST Inventory" sheetId="10" r:id="rId1"/>
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="100">
   <si>
     <t>mae_id</t>
   </si>
@@ -370,6 +370,9 @@
   </si>
   <si>
     <t>Stock_Count</t>
+  </si>
+  <si>
+    <t>Bulk_Value</t>
   </si>
 </sst>
 </file>
@@ -425,7 +428,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
       <protection hidden="1"/>
@@ -462,25 +465,41 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="129">
+  <dxfs count="130">
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
@@ -564,15 +583,7 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -810,94 +821,10 @@
       <protection locked="1" hidden="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="1"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
@@ -962,6 +889,90 @@
     <dxf>
       <protection locked="1" hidden="0"/>
     </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1000,11 +1011,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}" name="TEST_Inventory" displayName="TEST_Inventory" ref="A1:F5" totalsRowShown="0">
   <autoFilter ref="A1:F5" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="115"/>
-    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="114"/>
-    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="113"/>
-    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="112"/>
-    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="111">
+    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="113"/>
+    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="112"/>
+    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="111"/>
+    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="110"/>
+    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="109">
       <calculatedColumnFormula>TEST_Inventory[[#This Row],[TEST Integer]]*TEST_Inventory[[#This Row],[TEST Currency]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{AB3A5F3C-FCF0-4466-90FD-8ABB6E18DF5C}" name="TEST Dropdown"/>
@@ -1014,60 +1025,71 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:M2" totalsRowShown="0" headerRowDxfId="38" dataDxfId="37">
-  <autoFilter ref="A1:M2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
-  <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="36"/>
-    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="35"/>
-    <tableColumn id="12" xr3:uid="{8F0FD29C-682B-41B4-82F2-913D40801887}" name="Tag_ID" dataDxfId="34"/>
-    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="33"/>
-    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="32"/>
-    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="31"/>
-    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="30"/>
-    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Stock_Level" dataDxfId="29"/>
-    <tableColumn id="13" xr3:uid="{AA55BCE3-9AC1-4735-8622-15E62CA93E1A}" name="Stock_Count" dataDxfId="28"/>
-    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="27"/>
-    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="26"/>
-    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="25">
-      <calculatedColumnFormula array="1">IF(ISNUMBER(Shop_Consumables[[#This Row],[Stock_Level]]),
-    Shop_Consumables[[#This Row],[Stock_Level]] * Shop_Consumables[[#This Row],[Unit Cost]],
-    _xlfn.IFS(Shop_Consumables[[#This Row],[Stock_Level]]="Many", 1, Shop_Consumables[[#This Row],[Stock_Level]]="Adequate", 0.5, Shop_Consumables[[#This Row],[Stock_Level]]="Few", 0.1, TRUE, 0) * Shop_Consumables[[#This Row],[Unit Cost]]
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:N2" totalsRowShown="0" headerRowDxfId="39" dataDxfId="38">
+  <autoFilter ref="A1:N2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
+  <tableColumns count="14">
+    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="37"/>
+    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="36"/>
+    <tableColumn id="12" xr3:uid="{8F0FD29C-682B-41B4-82F2-913D40801887}" name="Tag_ID" dataDxfId="35"/>
+    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="34"/>
+    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="33"/>
+    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="32"/>
+    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Stock_Level" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="31"/>
+    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="1"/>
+    <tableColumn id="13" xr3:uid="{AA55BCE3-9AC1-4735-8622-15E62CA93E1A}" name="Stock_Count" dataDxfId="30"/>
+    <tableColumn id="14" xr3:uid="{FA5C79D4-6D25-4E4C-BE9F-4190C63530C2}" name="Bulk_Value" dataDxfId="0"/>
+    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="29"/>
+    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="28">
+      <calculatedColumnFormula array="1">IF(
+    Shop_Consumables[[#This Row],[Stock_Level]]="Counted",
+    Shop_Consumables[[#This Row],[Stock_Count]] * Shop_Consumables[[#This Row],[Unit Cost]],
+    IF(
+        Shop_Consumables[[#This Row],[Stock_Level]]="None",
+        0,
+        Shop_Consumables[[#This Row],[Bulk_Value]] * _xlfn.IFS(
+            Shop_Consumables[[#This Row],[Stock_Level]]="Many", 1,
+            Shop_Consumables[[#This Row],[Stock_Level]]="Adequate", 0.5,
+            Shop_Consumables[[#This Row],[Stock_Level]]="Few", 0.25,
+            TRUE, 0
+        )
+    )
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Supplier/Remarks" dataDxfId="24"/>
+    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Supplier/Remarks" dataDxfId="27"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:H2" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:H2" totalsRowShown="0" headerRowDxfId="26" dataDxfId="25">
   <autoFilter ref="A1:H2" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="20"/>
-    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="16"/>
-    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="15"/>
-    <tableColumn id="8" xr3:uid="{9140C4E8-CB9E-40BF-ABD9-13A971322B09}" name="Remarks" dataDxfId="14"/>
+    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="24"/>
+    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="23"/>
+    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="22"/>
+    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="21"/>
+    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="20"/>
+    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="19"/>
+    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="18"/>
+    <tableColumn id="8" xr3:uid="{9140C4E8-CB9E-40BF-ABD9-13A971322B09}" name="Remarks" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
   <autoFilter ref="A1:G2" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="11"/>
-    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="9"/>
-    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="7"/>
-    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="6"/>
-    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="14"/>
+    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="12"/>
+    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="11"/>
+    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="10"/>
+    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="9"/>
+    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1077,11 +1099,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}" name="Location" displayName="Location" ref="A1:E2" totalsRowShown="0">
   <autoFilter ref="A1:E2" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Description" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Description" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1091,10 +1113,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}" name="TEST_Dashboard" displayName="TEST_Dashboard" ref="A1:B2" totalsRowShown="0">
   <autoFilter ref="A1:B2" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="110">
+    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="108">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Currency])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="109">
+    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="107">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Integer])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1103,41 +1125,41 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:L2" totalsRowShown="0" headerRowDxfId="128" dataDxfId="127">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:L2" totalsRowShown="0" headerRowDxfId="106" dataDxfId="105">
   <autoFilter ref="A1:L2" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="126"/>
-    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="125">
+    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="104"/>
+    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="103">
       <calculatedColumnFormula>SUMIFS(Resell_Inventory[Actual Sale Price], Resell_Inventory[Current Status], "Sold")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="124">
+    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="102">
       <calculatedColumnFormula>SUM(Resell_Inventory[Actual Sale Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="123">
+    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="101">
       <calculatedColumnFormula>SUM(Shop_Machinery[Purchase Cost])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="122">
+    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="100">
       <calculatedColumnFormula>SUM(Shop_Power_Tools[Purchase Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="121">
+    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="99">
       <calculatedColumnFormula>SUM(Shop_Hand_Tools[Purchase Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="120">
+    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="98">
       <calculatedColumnFormula>SUM(Shop_Consumables[Current Inventory Value])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="119">
+    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="97">
       <calculatedColumnFormula>SUM(D2,E2,F2,G2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="118">
+    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="96">
       <calculatedColumnFormula array="1">SUMPRODUCT(
     --( (ISNUMBER(Shop_Consumables[Stock_Count])*(Shop_Consumables[Stock_Count]&lt;=Shop_Consumables[Reorder Point]))
     + (Shop_Consumables[Stock_Level]="Few") )
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="117">
+    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="95">
       <calculatedColumnFormula>SUMIFS(Shop_Overhead[Amount], Shop_Overhead[Due Date], "&lt;="&amp;TODAY()+30, Shop_Overhead[Due Date], "&gt;="&amp;TODAY())</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{E4065760-B1B1-4564-936B-3405D3B80297}" name="Equipment With Operational Issues" dataDxfId="116">
+    <tableColumn id="12" xr3:uid="{E4065760-B1B1-4564-936B-3405D3B80297}" name="Equipment With Operational Issues" dataDxfId="94">
       <calculatedColumnFormula array="1">SUM(
   COUNTIFS(Shop_Machinery[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"}),
   COUNTIFS(Shop_Power_Tools[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"}),
@@ -1156,8 +1178,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{F579DA07-7AD6-49DA-9B44-D5B1132EDAC6}" name="Overhead_Summary" displayName="Overhead_Summary" ref="A9:B21" totalsRowShown="0">
   <autoFilter ref="A9:B21" xr:uid="{F579DA07-7AD6-49DA-9B44-D5B1132EDAC6}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{7CA4839C-9603-479D-BD1C-8377DFA9603C}" name="Expense Category" dataDxfId="108"/>
-    <tableColumn id="2" xr3:uid="{FE0F7616-EAF3-443D-AC69-DE6541DC10E5}" name="Annual Total" dataDxfId="107">
+    <tableColumn id="1" xr3:uid="{7CA4839C-9603-479D-BD1C-8377DFA9603C}" name="Expense Category" dataDxfId="93"/>
+    <tableColumn id="2" xr3:uid="{FE0F7616-EAF3-443D-AC69-DE6541DC10E5}" name="Annual Total" dataDxfId="92">
       <calculatedColumnFormula>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1166,105 +1188,105 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:N2" totalsRowShown="0" headerRowDxfId="106" dataDxfId="105">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:N2" totalsRowShown="0" headerRowDxfId="129" dataDxfId="128">
   <autoFilter ref="A1:N2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}"/>
   <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="104"/>
-    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="103"/>
-    <tableColumn id="15" xr3:uid="{D25A390C-69B5-4326-A0D4-10EB45DDE5E5}" name="Tag_ID" dataDxfId="102"/>
-    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="101"/>
-    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="100"/>
-    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="99"/>
-    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="98"/>
-    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="97"/>
-    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="96"/>
-    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="95">
+    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="127"/>
+    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="126"/>
+    <tableColumn id="15" xr3:uid="{D25A390C-69B5-4326-A0D4-10EB45DDE5E5}" name="Tag_ID" dataDxfId="125"/>
+    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="124"/>
+    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="123"/>
+    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="122"/>
+    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="121"/>
+    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="120"/>
+    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="119"/>
+    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="118">
       <calculatedColumnFormula>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="94"/>
-    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="93"/>
-    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="92"/>
-    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="91"/>
+    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="117"/>
+    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="116"/>
+    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="115"/>
+    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="114"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="90" dataDxfId="89">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="91" dataDxfId="90">
   <autoFilter ref="A1:K2" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="88"/>
-    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="87"/>
-    <tableColumn id="4" xr3:uid="{17EB0B09-11B3-4E08-9442-E3C9AB87A157}" name="Tag_ID" dataDxfId="86"/>
-    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="85"/>
-    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Brand/Model" dataDxfId="84"/>
-    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="83"/>
-    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="82"/>
-    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="81"/>
-    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="80"/>
-    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="79"/>
-    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="78"/>
+    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="89"/>
+    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="88"/>
+    <tableColumn id="4" xr3:uid="{17EB0B09-11B3-4E08-9442-E3C9AB87A157}" name="Tag_ID" dataDxfId="87"/>
+    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="86"/>
+    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Brand/Model" dataDxfId="85"/>
+    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="84"/>
+    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="83"/>
+    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="82"/>
+    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="81"/>
+    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="80"/>
+    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="79"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:K2" totalsRowShown="0" headerRowDxfId="77" dataDxfId="76">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:K2" totalsRowShown="0" headerRowDxfId="78" dataDxfId="77">
   <autoFilter ref="A1:K2" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="75"/>
-    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="74"/>
-    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="73"/>
-    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="72"/>
-    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="71"/>
-    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="70"/>
-    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="69"/>
-    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="68"/>
-    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="67"/>
-    <tableColumn id="11" xr3:uid="{4809319D-ABCA-43DA-A400-5DC91167D78B}" name="Complete" dataDxfId="66"/>
-    <tableColumn id="12" xr3:uid="{920CB592-D743-4B33-A796-C7F3DB32211C}" name="Remarks" dataDxfId="65"/>
+    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="76"/>
+    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="75"/>
+    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="74"/>
+    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="73"/>
+    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="72"/>
+    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="71"/>
+    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="70"/>
+    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="69"/>
+    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="68"/>
+    <tableColumn id="11" xr3:uid="{4809319D-ABCA-43DA-A400-5DC91167D78B}" name="Complete" dataDxfId="67"/>
+    <tableColumn id="12" xr3:uid="{920CB592-D743-4B33-A796-C7F3DB32211C}" name="Remarks" dataDxfId="66"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:K2" totalsRowShown="0" headerRowDxfId="64" dataDxfId="63">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:K2" totalsRowShown="0" headerRowDxfId="65" dataDxfId="64">
   <autoFilter ref="A1:K2" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="62"/>
-    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="61"/>
-    <tableColumn id="11" xr3:uid="{21951C81-00A4-4344-9E81-B1B1DB06ADEF}" name="Tag_ID" dataDxfId="60"/>
-    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="59"/>
-    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Brand/Model" dataDxfId="58"/>
-    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="57"/>
-    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="56"/>
-    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="55"/>
-    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="54"/>
-    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="53"/>
-    <tableColumn id="10" xr3:uid="{26197E01-2936-4F5F-8081-3AA351C1CD38}" name="Remarks" dataDxfId="52"/>
+    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="63"/>
+    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="62"/>
+    <tableColumn id="11" xr3:uid="{21951C81-00A4-4344-9E81-B1B1DB06ADEF}" name="Tag_ID" dataDxfId="61"/>
+    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="60"/>
+    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Brand/Model" dataDxfId="59"/>
+    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="58"/>
+    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="57"/>
+    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="56"/>
+    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="55"/>
+    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="54"/>
+    <tableColumn id="10" xr3:uid="{26197E01-2936-4F5F-8081-3AA351C1CD38}" name="Remarks" dataDxfId="53"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:K2" totalsRowShown="0" headerRowDxfId="51" dataDxfId="50">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:K2" totalsRowShown="0" headerRowDxfId="52" dataDxfId="51">
   <autoFilter ref="A1:K2" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="49"/>
-    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="48"/>
-    <tableColumn id="10" xr3:uid="{C8BD69AA-9023-4777-9C96-39A81F1E4BE0}" name="Tag_ID" dataDxfId="47"/>
-    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="46"/>
-    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Brand/Model/Description" dataDxfId="45"/>
-    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="44"/>
-    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="43"/>
-    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="42"/>
-    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Stock_Level" dataDxfId="41"/>
-    <tableColumn id="11" xr3:uid="{FD8D2D17-0451-45E0-8688-0BB4F60073DA}" name="Stock_Count" dataDxfId="40"/>
-    <tableColumn id="9" xr3:uid="{2B57F5E6-66C5-4DBA-8949-836DE0F0791C}" name="Remarks" dataDxfId="39"/>
+    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="50"/>
+    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="49"/>
+    <tableColumn id="10" xr3:uid="{C8BD69AA-9023-4777-9C96-39A81F1E4BE0}" name="Tag_ID" dataDxfId="48"/>
+    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="47"/>
+    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Brand/Model/Description" dataDxfId="46"/>
+    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="45"/>
+    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="44"/>
+    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="43"/>
+    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Stock_Level" dataDxfId="42"/>
+    <tableColumn id="11" xr3:uid="{FD8D2D17-0451-45E0-8688-0BB4F60073DA}" name="Stock_Count" dataDxfId="41"/>
+    <tableColumn id="9" xr3:uid="{2B57F5E6-66C5-4DBA-8949-836DE0F0791C}" name="Remarks" dataDxfId="40"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1703,7 +1725,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E1902F1-C59B-4A1A-9D95-2C39AEF944E5}">
   <sheetPr codeName="Sheet7"/>
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:R2"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
@@ -1711,17 +1733,21 @@
     <col min="3" max="3" width="10.33203125" style="2" customWidth="1"/>
     <col min="4" max="4" width="22.6640625" style="6" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="41.6640625" style="2" customWidth="1"/>
-    <col min="7" max="7" width="18.44140625" style="2" customWidth="1"/>
-    <col min="8" max="9" width="15.5546875" style="6" customWidth="1"/>
-    <col min="10" max="10" width="14.33203125" style="7" customWidth="1"/>
-    <col min="11" max="11" width="14.109375" style="7" customWidth="1"/>
-    <col min="12" max="12" width="10.44140625" style="3" customWidth="1"/>
-    <col min="14" max="14" width="22.6640625" style="2" customWidth="1"/>
-    <col min="15" max="15" width="46.6640625" style="2" customWidth="1"/>
-    <col min="16" max="16384" width="8.88671875" style="6"/>
+    <col min="7" max="7" width="15.5546875" style="6" customWidth="1"/>
+    <col min="8" max="8" width="18.44140625" style="2" customWidth="1"/>
+    <col min="9" max="9" width="14.33203125" style="7" customWidth="1"/>
+    <col min="10" max="10" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.6640625" style="16" customWidth="1"/>
+    <col min="12" max="12" width="15.5546875" style="6" customWidth="1"/>
+    <col min="13" max="13" width="22.5546875" customWidth="1"/>
+    <col min="14" max="14" width="14.109375" style="7" customWidth="1"/>
+    <col min="15" max="15" width="10.44140625" style="3" customWidth="1"/>
+    <col min="17" max="17" width="22.6640625" style="2" customWidth="1"/>
+    <col min="18" max="18" width="46.6640625" style="2" customWidth="1"/>
+    <col min="19" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15">
+    <row r="1" spans="1:18">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1740,53 +1766,74 @@
       <c r="F1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" t="s">
+        <v>97</v>
+      </c>
+      <c r="H1" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
-        <v>97</v>
-      </c>
-      <c r="I1" t="s">
+      <c r="I1" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="J1" t="s">
         <v>98</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="K1" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="L1" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="K1" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="L1" s="5" t="s">
+      <c r="M1" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="N1" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="N1" s="6"/>
       <c r="O1" s="6"/>
-    </row>
-    <row r="2" spans="1:15">
+      <c r="P1" s="6"/>
+      <c r="Q1" s="6"/>
+      <c r="R1" s="6"/>
+    </row>
+    <row r="2" spans="1:18">
       <c r="F2" s="2"/>
-      <c r="K2" s="3"/>
-      <c r="L2" s="3" cm="1">
-        <f t="array" ref="L2">IF(ISNUMBER(Shop_Consumables[[#This Row],[Stock_Level]]),
-    Shop_Consumables[[#This Row],[Stock_Level]] * Shop_Consumables[[#This Row],[Unit Cost]],
-    _xlfn.IFS(Shop_Consumables[[#This Row],[Stock_Level]]="Many", 1, Shop_Consumables[[#This Row],[Stock_Level]]="Adequate", 0.5, Shop_Consumables[[#This Row],[Stock_Level]]="Few", 0.1, TRUE, 0) * Shop_Consumables[[#This Row],[Unit Cost]]
+      <c r="I2" s="3"/>
+      <c r="J2" s="6"/>
+      <c r="K2" s="17"/>
+      <c r="L2" s="7"/>
+      <c r="M2" s="3" cm="1">
+        <f t="array" ref="M2">IF(
+    Shop_Consumables[[#This Row],[Stock_Level]]="Counted",
+    Shop_Consumables[[#This Row],[Stock_Count]] * Shop_Consumables[[#This Row],[Unit Cost]],
+    IF(
+        Shop_Consumables[[#This Row],[Stock_Level]]="None",
+        0,
+        Shop_Consumables[[#This Row],[Bulk_Value]] * _xlfn.IFS(
+            Shop_Consumables[[#This Row],[Stock_Level]]="Many", 1,
+            Shop_Consumables[[#This Row],[Stock_Level]]="Adequate", 0.5,
+            Shop_Consumables[[#This Row],[Stock_Level]]="Few", 0.25,
+            TRUE, 0
+        )
+    )
 )</f>
         <v>0</v>
       </c>
-      <c r="M2" s="2"/>
-      <c r="N2" s="6"/>
+      <c r="N2" s="2"/>
       <c r="O2" s="6"/>
+      <c r="P2" s="6"/>
+      <c r="Q2" s="6"/>
+      <c r="R2" s="6"/>
     </row>
   </sheetData>
   <dataValidations disablePrompts="1" count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2" xr:uid="{D2C605E8-D02B-4558-82DE-3169088704E8}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:G2" xr:uid="{D2C605E8-D02B-4558-82DE-3169088704E8}">
       <formula1>"Fasteners/Hardware,Abrasives/Cutting,Fluids/Lubricants/Chemicals,Primer/Paint,Safety/PPE,Shop/Janitorial,Welding,Electrical,Other"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
updated formula for low stock alert in excel and config and updated logic in app applyDashboardFilters to account for "none", "few" or counted less than reorder point
</commit_message>
<xml_diff>
--- a/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
+++ b/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1a2ae81d67634e6/Desktop/Michanikos Artifex Enterprises/MAE Custom Digital Solutions/MAE Workshop Inventory Management System/GITHUB_MAE_Workshop Inventory App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="231" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{007C75AC-1EC2-40BF-B9F4-F7453B5D9ADE}"/>
+  <xr:revisionPtr revIDLastSave="232" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D4F35712-2AA5-44A0-8614-3411EAD4A11C}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="7" activeTab="9" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="2" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
   </bookViews>
   <sheets>
     <sheet name="TEST Inventory" sheetId="10" r:id="rId1"/>
@@ -428,7 +428,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
       <protection hidden="1"/>
@@ -465,10 +465,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -476,6 +472,60 @@
   <dxfs count="130">
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -483,72 +533,6 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
       <protection locked="0" hidden="0"/>
     </dxf>
@@ -563,56 +547,6 @@
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="1"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -781,6 +715,68 @@
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
@@ -913,13 +909,25 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="1"/>
+      <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
       <protection locked="0" hidden="0"/>
     </dxf>
@@ -928,19 +936,7 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -1025,22 +1021,22 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:N2" totalsRowShown="0" headerRowDxfId="39" dataDxfId="38">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:N2" totalsRowShown="0" headerRowDxfId="129" dataDxfId="128">
   <autoFilter ref="A1:N2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
   <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="37"/>
-    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="36"/>
-    <tableColumn id="12" xr3:uid="{8F0FD29C-682B-41B4-82F2-913D40801887}" name="Tag_ID" dataDxfId="35"/>
-    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="34"/>
-    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="33"/>
-    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="32"/>
-    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Stock_Level" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="31"/>
-    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="1"/>
-    <tableColumn id="13" xr3:uid="{AA55BCE3-9AC1-4735-8622-15E62CA93E1A}" name="Stock_Count" dataDxfId="30"/>
-    <tableColumn id="14" xr3:uid="{FA5C79D4-6D25-4E4C-BE9F-4190C63530C2}" name="Bulk_Value" dataDxfId="0"/>
-    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="29"/>
-    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="28">
+    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="127"/>
+    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="126"/>
+    <tableColumn id="12" xr3:uid="{8F0FD29C-682B-41B4-82F2-913D40801887}" name="Tag_ID" dataDxfId="125"/>
+    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="124"/>
+    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="123"/>
+    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="122"/>
+    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Stock_Level" dataDxfId="121"/>
+    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="120"/>
+    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="119"/>
+    <tableColumn id="13" xr3:uid="{AA55BCE3-9AC1-4735-8622-15E62CA93E1A}" name="Stock_Count" dataDxfId="118"/>
+    <tableColumn id="14" xr3:uid="{FA5C79D4-6D25-4E4C-BE9F-4190C63530C2}" name="Bulk_Value" dataDxfId="117"/>
+    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="116"/>
+    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="115">
       <calculatedColumnFormula array="1">IF(
     Shop_Consumables[[#This Row],[Stock_Level]]="Counted",
     Shop_Consumables[[#This Row],[Stock_Count]] * Shop_Consumables[[#This Row],[Unit Cost]],
@@ -1056,40 +1052,40 @@
     )
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Supplier/Remarks" dataDxfId="27"/>
+    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Supplier/Remarks" dataDxfId="114"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:H2" totalsRowShown="0" headerRowDxfId="26" dataDxfId="25">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:H2" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
   <autoFilter ref="A1:H2" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="24"/>
-    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="23"/>
-    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="22"/>
-    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="21"/>
-    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="20"/>
-    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="19"/>
-    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="18"/>
-    <tableColumn id="8" xr3:uid="{9140C4E8-CB9E-40BF-ABD9-13A971322B09}" name="Remarks" dataDxfId="17"/>
+    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="20"/>
+    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="19"/>
+    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="18"/>
+    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="17"/>
+    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="16"/>
+    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="15"/>
+    <tableColumn id="8" xr3:uid="{9140C4E8-CB9E-40BF-ABD9-13A971322B09}" name="Remarks" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
   <autoFilter ref="A1:G2" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="14"/>
-    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="12"/>
-    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="11"/>
-    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="10"/>
-    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="9"/>
-    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="11"/>
+    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="9"/>
+    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="7"/>
+    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="6"/>
+    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1099,11 +1095,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}" name="Location" displayName="Location" ref="A1:E2" totalsRowShown="0">
   <autoFilter ref="A1:E2" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Description" dataDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Description" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1152,8 +1148,8 @@
     </tableColumn>
     <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="96">
       <calculatedColumnFormula array="1">SUMPRODUCT(
-    --( (ISNUMBER(Shop_Consumables[Stock_Count])*(Shop_Consumables[Stock_Count]&lt;=Shop_Consumables[Reorder Point]))
-    + (Shop_Consumables[Stock_Level]="Few") )
+    ((Shop_Consumables[Stock_Level]="Counted") * (ISNUMBER(Shop_Consumables[Stock_Count])) * (Shop_Consumables[Stock_Count]&lt;=Shop_Consumables[Reorder Point])) +
+    ((ISNUMBER(MATCH(Shop_Consumables[Stock_Level], {"Few","None"}, 0))))
 )</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="95">
@@ -1188,105 +1184,105 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:N2" totalsRowShown="0" headerRowDxfId="129" dataDxfId="128">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:N2" totalsRowShown="0" headerRowDxfId="91" dataDxfId="90">
   <autoFilter ref="A1:N2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}"/>
   <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="127"/>
-    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="126"/>
-    <tableColumn id="15" xr3:uid="{D25A390C-69B5-4326-A0D4-10EB45DDE5E5}" name="Tag_ID" dataDxfId="125"/>
-    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="124"/>
-    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="123"/>
-    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="122"/>
-    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="121"/>
-    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="120"/>
-    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="119"/>
-    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="118">
+    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="89"/>
+    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="88"/>
+    <tableColumn id="15" xr3:uid="{D25A390C-69B5-4326-A0D4-10EB45DDE5E5}" name="Tag_ID" dataDxfId="87"/>
+    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="86"/>
+    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="85"/>
+    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="84"/>
+    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="83"/>
+    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="82"/>
+    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="81"/>
+    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="80">
       <calculatedColumnFormula>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="117"/>
-    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="116"/>
-    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="115"/>
-    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="114"/>
+    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="79"/>
+    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="78"/>
+    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="77"/>
+    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="76"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="91" dataDxfId="90">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="75" dataDxfId="74">
   <autoFilter ref="A1:K2" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="89"/>
-    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="88"/>
-    <tableColumn id="4" xr3:uid="{17EB0B09-11B3-4E08-9442-E3C9AB87A157}" name="Tag_ID" dataDxfId="87"/>
-    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="86"/>
-    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Brand/Model" dataDxfId="85"/>
-    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="84"/>
-    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="83"/>
-    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="82"/>
-    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="81"/>
-    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="80"/>
-    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="79"/>
+    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="73"/>
+    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="72"/>
+    <tableColumn id="4" xr3:uid="{17EB0B09-11B3-4E08-9442-E3C9AB87A157}" name="Tag_ID" dataDxfId="71"/>
+    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="70"/>
+    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Brand/Model" dataDxfId="69"/>
+    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="68"/>
+    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="67"/>
+    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="66"/>
+    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="65"/>
+    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="64"/>
+    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="63"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:K2" totalsRowShown="0" headerRowDxfId="78" dataDxfId="77">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:K2" totalsRowShown="0" headerRowDxfId="62" dataDxfId="61">
   <autoFilter ref="A1:K2" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="76"/>
-    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="75"/>
-    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="74"/>
-    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="73"/>
-    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="72"/>
-    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="71"/>
-    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="70"/>
-    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="69"/>
-    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="68"/>
-    <tableColumn id="11" xr3:uid="{4809319D-ABCA-43DA-A400-5DC91167D78B}" name="Complete" dataDxfId="67"/>
-    <tableColumn id="12" xr3:uid="{920CB592-D743-4B33-A796-C7F3DB32211C}" name="Remarks" dataDxfId="66"/>
+    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="60"/>
+    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="59"/>
+    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="58"/>
+    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="57"/>
+    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="56"/>
+    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="55"/>
+    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="54"/>
+    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="53"/>
+    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="52"/>
+    <tableColumn id="11" xr3:uid="{4809319D-ABCA-43DA-A400-5DC91167D78B}" name="Complete" dataDxfId="51"/>
+    <tableColumn id="12" xr3:uid="{920CB592-D743-4B33-A796-C7F3DB32211C}" name="Remarks" dataDxfId="50"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:K2" totalsRowShown="0" headerRowDxfId="65" dataDxfId="64">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:K2" totalsRowShown="0" headerRowDxfId="49" dataDxfId="48">
   <autoFilter ref="A1:K2" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="63"/>
-    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="62"/>
-    <tableColumn id="11" xr3:uid="{21951C81-00A4-4344-9E81-B1B1DB06ADEF}" name="Tag_ID" dataDxfId="61"/>
-    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="60"/>
-    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Brand/Model" dataDxfId="59"/>
-    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="58"/>
-    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="57"/>
-    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="56"/>
-    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="55"/>
-    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="54"/>
-    <tableColumn id="10" xr3:uid="{26197E01-2936-4F5F-8081-3AA351C1CD38}" name="Remarks" dataDxfId="53"/>
+    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="47"/>
+    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="46"/>
+    <tableColumn id="11" xr3:uid="{21951C81-00A4-4344-9E81-B1B1DB06ADEF}" name="Tag_ID" dataDxfId="45"/>
+    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="44"/>
+    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Brand/Model" dataDxfId="43"/>
+    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="42"/>
+    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="41"/>
+    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="40"/>
+    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="39"/>
+    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="38"/>
+    <tableColumn id="10" xr3:uid="{26197E01-2936-4F5F-8081-3AA351C1CD38}" name="Remarks" dataDxfId="37"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:K2" totalsRowShown="0" headerRowDxfId="52" dataDxfId="51">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:K2" totalsRowShown="0" headerRowDxfId="36" dataDxfId="35">
   <autoFilter ref="A1:K2" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="50"/>
-    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="49"/>
-    <tableColumn id="10" xr3:uid="{C8BD69AA-9023-4777-9C96-39A81F1E4BE0}" name="Tag_ID" dataDxfId="48"/>
-    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="47"/>
-    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Brand/Model/Description" dataDxfId="46"/>
-    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="45"/>
-    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="44"/>
-    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="43"/>
-    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Stock_Level" dataDxfId="42"/>
-    <tableColumn id="11" xr3:uid="{FD8D2D17-0451-45E0-8688-0BB4F60073DA}" name="Stock_Count" dataDxfId="41"/>
-    <tableColumn id="9" xr3:uid="{2B57F5E6-66C5-4DBA-8949-836DE0F0791C}" name="Remarks" dataDxfId="40"/>
+    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="34"/>
+    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="33"/>
+    <tableColumn id="10" xr3:uid="{C8BD69AA-9023-4777-9C96-39A81F1E4BE0}" name="Tag_ID" dataDxfId="32"/>
+    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="31"/>
+    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Brand/Model/Description" dataDxfId="30"/>
+    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="29"/>
+    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="28"/>
+    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="27"/>
+    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Stock_Level" dataDxfId="26"/>
+    <tableColumn id="11" xr3:uid="{FD8D2D17-0451-45E0-8688-0BB4F60073DA}" name="Stock_Count" dataDxfId="25"/>
+    <tableColumn id="9" xr3:uid="{2B57F5E6-66C5-4DBA-8949-836DE0F0791C}" name="Remarks" dataDxfId="24"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1737,7 +1733,7 @@
     <col min="8" max="8" width="18.44140625" style="2" customWidth="1"/>
     <col min="9" max="9" width="14.33203125" style="7" customWidth="1"/>
     <col min="10" max="10" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.6640625" style="16" customWidth="1"/>
+    <col min="11" max="11" width="13.6640625" customWidth="1"/>
     <col min="12" max="12" width="15.5546875" style="6" customWidth="1"/>
     <col min="13" max="13" width="22.5546875" customWidth="1"/>
     <col min="14" max="14" width="14.109375" style="7" customWidth="1"/>
@@ -1778,7 +1774,7 @@
       <c r="J1" t="s">
         <v>98</v>
       </c>
-      <c r="K1" s="16" t="s">
+      <c r="K1" t="s">
         <v>99</v>
       </c>
       <c r="L1" s="8" t="s">
@@ -1799,7 +1795,7 @@
       <c r="F2" s="2"/>
       <c r="I2" s="3"/>
       <c r="J2" s="6"/>
-      <c r="K2" s="17"/>
+      <c r="K2" s="6"/>
       <c r="L2" s="7"/>
       <c r="M2" s="3" cm="1">
         <f t="array" ref="M2">IF(
@@ -2133,8 +2129,8 @@
       </c>
       <c r="I2" s="12" cm="1">
         <f t="array" ref="I2">SUMPRODUCT(
-    --( (ISNUMBER(Shop_Consumables[Stock_Count])*(Shop_Consumables[Stock_Count]&lt;=Shop_Consumables[Reorder Point]))
-    + (Shop_Consumables[Stock_Level]="Few") )
+    ((Shop_Consumables[Stock_Level]="Counted") * (ISNUMBER(Shop_Consumables[Stock_Count])) * (Shop_Consumables[Stock_Count]&lt;=Shop_Consumables[Reorder Point])) +
+    ((ISNUMBER(MATCH(Shop_Consumables[Stock_Level], {"Few","None"}, 0))))
 )</f>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
updated Config and Excel: Maintenance Log: Service Date to Completion Date and moved it after Complete checkbox
</commit_message>
<xml_diff>
--- a/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
+++ b/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1a2ae81d67634e6/Desktop/Michanikos Artifex Enterprises/MAE Custom Digital Solutions/MAE Workshop Inventory Management System/GITHUB_MAE_Workshop Inventory App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="233" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C7822229-32E1-4812-A8A5-6CC2AFB8B549}"/>
+  <xr:revisionPtr revIDLastSave="238" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3C26E902-4264-46F5-95DC-FA2634EF770C}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="2" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="6" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
   </bookViews>
   <sheets>
     <sheet name="TEST Inventory" sheetId="10" r:id="rId1"/>
@@ -123,9 +123,6 @@
     <t>Log ID</t>
   </si>
   <si>
-    <t>Service Date</t>
-  </si>
-  <si>
     <t>Service Type</t>
   </si>
   <si>
@@ -373,6 +370,9 @@
   </si>
   <si>
     <t>Bulk_Value</t>
+  </si>
+  <si>
+    <t>Completion Date</t>
   </si>
 </sst>
 </file>
@@ -471,6 +471,10 @@
   </cellStyles>
   <dxfs count="130">
     <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
@@ -739,10 +743,6 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -1021,22 +1021,22 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:N2" totalsRowShown="0" headerRowDxfId="39" dataDxfId="38">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:N2" totalsRowShown="0" headerRowDxfId="40" dataDxfId="39">
   <autoFilter ref="A1:N2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
   <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="37"/>
-    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="36"/>
-    <tableColumn id="12" xr3:uid="{8F0FD29C-682B-41B4-82F2-913D40801887}" name="Tag_ID" dataDxfId="35"/>
-    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="34"/>
-    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="33"/>
-    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="32"/>
-    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Stock_Level" dataDxfId="31"/>
-    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="30"/>
-    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="29"/>
-    <tableColumn id="13" xr3:uid="{AA55BCE3-9AC1-4735-8622-15E62CA93E1A}" name="Stock_Count" dataDxfId="28"/>
-    <tableColumn id="14" xr3:uid="{FA5C79D4-6D25-4E4C-BE9F-4190C63530C2}" name="Bulk_Value" dataDxfId="27"/>
-    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="26"/>
-    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="25">
+    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="38"/>
+    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="37"/>
+    <tableColumn id="12" xr3:uid="{8F0FD29C-682B-41B4-82F2-913D40801887}" name="Tag_ID" dataDxfId="36"/>
+    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="35"/>
+    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="34"/>
+    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="33"/>
+    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Stock_Level" dataDxfId="32"/>
+    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="31"/>
+    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="30"/>
+    <tableColumn id="13" xr3:uid="{AA55BCE3-9AC1-4735-8622-15E62CA93E1A}" name="Stock_Count" dataDxfId="29"/>
+    <tableColumn id="14" xr3:uid="{FA5C79D4-6D25-4E4C-BE9F-4190C63530C2}" name="Bulk_Value" dataDxfId="28"/>
+    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="27"/>
+    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="26">
       <calculatedColumnFormula array="1">IF(
     Shop_Consumables[[#This Row],[Stock_Level]]="Counted",
     Shop_Consumables[[#This Row],[Stock_Count]] * Shop_Consumables[[#This Row],[Unit Cost]],
@@ -1052,40 +1052,40 @@
     )
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Supplier/Remarks" dataDxfId="24"/>
+    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Supplier/Remarks" dataDxfId="25"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:H2" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:H2" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23">
   <autoFilter ref="A1:H2" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="20"/>
-    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="16"/>
-    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="15"/>
-    <tableColumn id="8" xr3:uid="{9140C4E8-CB9E-40BF-ABD9-13A971322B09}" name="Remarks" dataDxfId="14"/>
+    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="22"/>
+    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="20"/>
+    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="18"/>
+    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="17"/>
+    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="16"/>
+    <tableColumn id="8" xr3:uid="{9140C4E8-CB9E-40BF-ABD9-13A971322B09}" name="Remarks" dataDxfId="15"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13">
   <autoFilter ref="A1:G2" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="11"/>
-    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="9"/>
-    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="7"/>
-    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="6"/>
-    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="12"/>
+    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="10"/>
+    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="9"/>
+    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="8"/>
+    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="7"/>
+    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1095,11 +1095,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}" name="Location" displayName="Location" ref="A1:E2" totalsRowShown="0">
   <autoFilter ref="A1:E2" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Description" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Description" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1236,53 +1236,53 @@
     <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="75"/>
     <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="74"/>
     <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="73"/>
-    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Service Date" dataDxfId="72"/>
-    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="71"/>
-    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="70"/>
-    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="69"/>
-    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="68"/>
-    <tableColumn id="11" xr3:uid="{4809319D-ABCA-43DA-A400-5DC91167D78B}" name="Complete" dataDxfId="67"/>
-    <tableColumn id="12" xr3:uid="{920CB592-D743-4B33-A796-C7F3DB32211C}" name="Remarks" dataDxfId="66"/>
+    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="72"/>
+    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="71"/>
+    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="70"/>
+    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="69"/>
+    <tableColumn id="11" xr3:uid="{4809319D-ABCA-43DA-A400-5DC91167D78B}" name="Complete" dataDxfId="68"/>
+    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Completion Date" dataDxfId="0"/>
+    <tableColumn id="12" xr3:uid="{920CB592-D743-4B33-A796-C7F3DB32211C}" name="Remarks" dataDxfId="67"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:K2" totalsRowShown="0" headerRowDxfId="65" dataDxfId="64">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:K2" totalsRowShown="0" headerRowDxfId="66" dataDxfId="65">
   <autoFilter ref="A1:K2" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="63"/>
-    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="62"/>
-    <tableColumn id="11" xr3:uid="{21951C81-00A4-4344-9E81-B1B1DB06ADEF}" name="Tag_ID" dataDxfId="61"/>
-    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="60"/>
-    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Brand/Model" dataDxfId="59"/>
-    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="58"/>
-    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="57"/>
-    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="56"/>
-    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="55"/>
-    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="54"/>
-    <tableColumn id="10" xr3:uid="{26197E01-2936-4F5F-8081-3AA351C1CD38}" name="Remarks" dataDxfId="53"/>
+    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="64"/>
+    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="63"/>
+    <tableColumn id="11" xr3:uid="{21951C81-00A4-4344-9E81-B1B1DB06ADEF}" name="Tag_ID" dataDxfId="62"/>
+    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="61"/>
+    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Brand/Model" dataDxfId="60"/>
+    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="59"/>
+    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="58"/>
+    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="57"/>
+    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="56"/>
+    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="55"/>
+    <tableColumn id="10" xr3:uid="{26197E01-2936-4F5F-8081-3AA351C1CD38}" name="Remarks" dataDxfId="54"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:K2" totalsRowShown="0" headerRowDxfId="52" dataDxfId="51">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:K2" totalsRowShown="0" headerRowDxfId="53" dataDxfId="52">
   <autoFilter ref="A1:K2" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="50"/>
-    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="49"/>
-    <tableColumn id="10" xr3:uid="{C8BD69AA-9023-4777-9C96-39A81F1E4BE0}" name="Tag_ID" dataDxfId="48"/>
-    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="47"/>
-    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Brand/Model/Description" dataDxfId="46"/>
-    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="45"/>
-    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="44"/>
-    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="43"/>
-    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Stock_Level" dataDxfId="42"/>
-    <tableColumn id="11" xr3:uid="{FD8D2D17-0451-45E0-8688-0BB4F60073DA}" name="Stock_Count" dataDxfId="41"/>
-    <tableColumn id="9" xr3:uid="{2B57F5E6-66C5-4DBA-8949-836DE0F0791C}" name="Remarks" dataDxfId="40"/>
+    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="51"/>
+    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="50"/>
+    <tableColumn id="10" xr3:uid="{C8BD69AA-9023-4777-9C96-39A81F1E4BE0}" name="Tag_ID" dataDxfId="49"/>
+    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="48"/>
+    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Brand/Model/Description" dataDxfId="47"/>
+    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="46"/>
+    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="45"/>
+    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="44"/>
+    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Stock_Level" dataDxfId="43"/>
+    <tableColumn id="11" xr3:uid="{FD8D2D17-0451-45E0-8688-0BB4F60073DA}" name="Stock_Count" dataDxfId="42"/>
+    <tableColumn id="9" xr3:uid="{2B57F5E6-66C5-4DBA-8949-836DE0F0791C}" name="Remarks" dataDxfId="41"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1621,24 +1621,24 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="D1" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" t="s">
         <v>36</v>
-      </c>
-      <c r="F1" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="B2" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C2" s="8">
         <v>3</v>
@@ -1651,12 +1651,12 @@
         <v>300</v>
       </c>
       <c r="F2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="B3" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C3" s="8">
         <v>4</v>
@@ -1669,12 +1669,12 @@
         <v>40</v>
       </c>
       <c r="F3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="B4" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C4" s="8">
         <v>5</v>
@@ -1687,12 +1687,12 @@
         <v>100</v>
       </c>
       <c r="F4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="B5" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C5" s="8">
         <v>1000</v>
@@ -1748,13 +1748,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>2</v>
@@ -1763,28 +1763,28 @@
         <v>3</v>
       </c>
       <c r="G1" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="J1" t="s">
         <v>97</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="K1" t="s">
+        <v>98</v>
+      </c>
+      <c r="L1" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="I1" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="J1" t="s">
-        <v>98</v>
-      </c>
-      <c r="K1" t="s">
-        <v>99</v>
-      </c>
-      <c r="L1" s="8" t="s">
-        <v>23</v>
-      </c>
       <c r="M1" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="O1" s="6"/>
       <c r="P1" s="6"/>
@@ -1856,25 +1856,25 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="F1" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="4" t="s">
-        <v>30</v>
-      </c>
       <c r="H1" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I1" s="6"/>
     </row>
@@ -1924,22 +1924,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G1" s="4" t="s">
         <v>48</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -1967,33 +1967,33 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" t="s">
         <v>55</v>
       </c>
-      <c r="C1" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>56</v>
-      </c>
-      <c r="E1" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="D2" t="s">
         <v>93</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>94</v>
-      </c>
-      <c r="E2" t="s">
-        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -2015,10 +2015,10 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>38</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -2065,37 +2065,37 @@
         <v>0</v>
       </c>
       <c r="B1" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="D1" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="H1" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="D1" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="F1" s="5" t="s">
+      <c r="I1" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="J1" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="G1" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="I1" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>69</v>
-      </c>
       <c r="K1" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="L1" s="8" t="s">
         <v>83</v>
-      </c>
-      <c r="L1" s="8" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="2" spans="1:12">
@@ -2172,15 +2172,15 @@
   <sheetData>
     <row r="9" spans="1:2">
       <c r="A9" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B10" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2189,7 +2189,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B11" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2198,7 +2198,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B12" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2207,7 +2207,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B13" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2216,7 +2216,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B14" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2225,7 +2225,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B15" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2234,7 +2234,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B16" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2243,7 +2243,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B17" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2252,7 +2252,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B18" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2261,7 +2261,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B19" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2270,7 +2270,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B20" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2279,7 +2279,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B21" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2333,10 +2333,10 @@
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>2</v>
@@ -2428,13 +2428,13 @@
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F1" s="4" t="s">
         <v>12</v>
@@ -2449,10 +2449,10 @@
         <v>11</v>
       </c>
       <c r="J1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="L1" s="6"/>
     </row>
@@ -2480,26 +2480,26 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB7AACC4-9DA2-4A53-AD77-8C5E0C1BF474}">
   <sheetPr codeName="Sheet4"/>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.109375" style="14" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.88671875" style="14" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="28.21875" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.6640625" style="10" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.6640625" style="6" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14.33203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18" style="3" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="18" style="9" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.44140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.44140625" style="2" customWidth="1"/>
-    <col min="13" max="13" width="9.88671875" style="3" customWidth="1"/>
-    <col min="14" max="16384" width="8.88671875" style="6"/>
+    <col min="10" max="10" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.33203125" style="10" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.44140625" style="2" customWidth="1"/>
+    <col min="14" max="14" width="9.88671875" style="3" customWidth="1"/>
+    <col min="15" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2510,48 +2510,54 @@
         <v>1</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="E1" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="E1" t="s">
         <v>16</v>
       </c>
       <c r="F1" t="s">
         <v>17</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="I1" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="J1" t="s">
+      <c r="I1" t="s">
+        <v>85</v>
+      </c>
+      <c r="J1" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="K1" s="4" t="s">
         <v>86</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>87</v>
       </c>
       <c r="L1" s="6"/>
       <c r="M1" s="6"/>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="I2" s="10"/>
-      <c r="J2" s="6"/>
+      <c r="N1" s="6"/>
+    </row>
+    <row r="2" spans="1:14">
+      <c r="E2" s="6"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="10"/>
+      <c r="I2" s="6"/>
+      <c r="J2" s="10"/>
+      <c r="K2" s="2"/>
       <c r="L2" s="6"/>
       <c r="M2" s="6"/>
+      <c r="N2" s="6"/>
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F1000" xr:uid="{E5FFE733-A9D3-430E-8950-CAD58FEAE2C9}">
-      <formula1>"Preventive, Repair"</formula1>
-    </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G3:G1000" xr:uid="{8BC162F1-575A-44E2-AA38-454BF93A8AFF}">
       <formula1>"Self in Shop, Contractor in Shop, Out of Shop"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2" xr:uid="{D78DF6AB-EB66-4EBB-ABC5-55445DBB08E9}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2" xr:uid="{D78DF6AB-EB66-4EBB-ABC5-55445DBB08E9}">
       <formula1>"Self in Shop, Contractor in Shop, Outside Facility"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F3:F1000 E2" xr:uid="{E5FFE733-A9D3-430E-8950-CAD58FEAE2C9}">
+      <formula1>"Preventive, Repair"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2587,34 +2593,34 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
       <c r="G1" t="s">
+        <v>50</v>
+      </c>
+      <c r="H1" t="s">
         <v>51</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>52</v>
       </c>
-      <c r="I1" t="s">
-        <v>53</v>
-      </c>
       <c r="J1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="M1" s="6"/>
     </row>
@@ -2679,16 +2685,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>5</v>
@@ -2697,16 +2703,16 @@
         <v>3</v>
       </c>
       <c r="H1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I1" t="s">
+        <v>96</v>
+      </c>
+      <c r="J1" t="s">
         <v>97</v>
       </c>
-      <c r="J1" t="s">
-        <v>98</v>
-      </c>
       <c r="K1" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="L1" s="6"/>
       <c r="M1" s="6"/>

</xml_diff>

<commit_message>
adjusted config/excel to change and/or hide several columns to reduce unnecessary columns
</commit_message>
<xml_diff>
--- a/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
+++ b/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1a2ae81d67634e6/Desktop/Michanikos Artifex Enterprises/MAE Custom Digital Solutions/MAE Workshop Inventory Management System/GITHUB_MAE_Workshop Inventory App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="238" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3C26E902-4264-46F5-95DC-FA2634EF770C}"/>
+  <xr:revisionPtr revIDLastSave="245" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A23BFEE8-EBF3-46FC-858B-682CAA922A47}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="6" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="6" activeTab="7" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
   </bookViews>
   <sheets>
     <sheet name="TEST Inventory" sheetId="10" r:id="rId1"/>
@@ -111,9 +111,6 @@
     <t>Location</t>
   </si>
   <si>
-    <t>Serial Number</t>
-  </si>
-  <si>
     <t>Purchase Date</t>
   </si>
   <si>
@@ -222,9 +219,6 @@
     <t>Notes/Other Info</t>
   </si>
   <si>
-    <t>Manual Link/Other Info</t>
-  </si>
-  <si>
     <t>Functional Category</t>
   </si>
   <si>
@@ -373,6 +367,12 @@
   </si>
   <si>
     <t>Completion Date</t>
+  </si>
+  <si>
+    <t>Date Sold</t>
+  </si>
+  <si>
+    <t>Serial Number/Other Info</t>
   </si>
 </sst>
 </file>
@@ -721,73 +721,20 @@
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="0"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -883,28 +830,6 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
@@ -958,6 +883,81 @@
     <dxf>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
       <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -1121,41 +1121,41 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:L2" totalsRowShown="0" headerRowDxfId="129" dataDxfId="128">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:L2" totalsRowShown="0" headerRowDxfId="109" dataDxfId="108">
   <autoFilter ref="A1:L2" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="127"/>
-    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="126">
+    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="107"/>
+    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="106">
       <calculatedColumnFormula>SUM(Resell_Inventory[Total Investment])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="125">
+    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="105">
       <calculatedColumnFormula>SUM(Resell_Inventory[Actual Sale Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="124">
+    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="104">
       <calculatedColumnFormula>SUM(Shop_Machinery[Purchase Cost])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="123">
+    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="103">
       <calculatedColumnFormula>SUM(Shop_Power_Tools[Purchase Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="122">
+    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="102">
       <calculatedColumnFormula>SUM(Shop_Hand_Tools[Purchase Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="121">
+    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="101">
       <calculatedColumnFormula>SUM(Shop_Consumables[Current Inventory Value])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="120">
+    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="100">
       <calculatedColumnFormula>SUM(D2,E2,F2,G2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="119">
+    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="99">
       <calculatedColumnFormula array="1">SUMPRODUCT(
     ((Shop_Consumables[Stock_Level]="Counted") * (ISNUMBER(Shop_Consumables[Stock_Count])) * (Shop_Consumables[Stock_Count]&lt;=Shop_Consumables[Reorder Point])) +
     ((ISNUMBER(MATCH(Shop_Consumables[Stock_Level], {"Few","None"}, 0))))
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="118">
+    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="98">
       <calculatedColumnFormula>SUMIFS(Shop_Overhead[Amount], Shop_Overhead[Due Date], "&lt;="&amp;TODAY()+30, Shop_Overhead[Due Date], "&gt;="&amp;TODAY())</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{E4065760-B1B1-4564-936B-3405D3B80297}" name="Equipment With Operational Issues" dataDxfId="117">
+    <tableColumn id="12" xr3:uid="{E4065760-B1B1-4564-936B-3405D3B80297}" name="Equipment With Operational Issues" dataDxfId="97">
       <calculatedColumnFormula array="1">SUM(
   COUNTIFS(Shop_Machinery[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"}),
   COUNTIFS(Shop_Power_Tools[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"}),
@@ -1174,8 +1174,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{F579DA07-7AD6-49DA-9B44-D5B1132EDAC6}" name="Overhead_Summary" displayName="Overhead_Summary" ref="A9:B21" totalsRowShown="0">
   <autoFilter ref="A9:B21" xr:uid="{F579DA07-7AD6-49DA-9B44-D5B1132EDAC6}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{7CA4839C-9603-479D-BD1C-8377DFA9603C}" name="Expense Category" dataDxfId="109"/>
-    <tableColumn id="2" xr3:uid="{FE0F7616-EAF3-443D-AC69-DE6541DC10E5}" name="Annual Total" dataDxfId="108">
+    <tableColumn id="1" xr3:uid="{7CA4839C-9603-479D-BD1C-8377DFA9603C}" name="Expense Category" dataDxfId="96"/>
+    <tableColumn id="2" xr3:uid="{FE0F7616-EAF3-443D-AC69-DE6541DC10E5}" name="Annual Total" dataDxfId="95">
       <calculatedColumnFormula>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1184,65 +1184,65 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:N2" totalsRowShown="0" headerRowDxfId="107" dataDxfId="106">
-  <autoFilter ref="A1:N2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}"/>
-  <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="105"/>
-    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="104"/>
-    <tableColumn id="15" xr3:uid="{D25A390C-69B5-4326-A0D4-10EB45DDE5E5}" name="Tag_ID" dataDxfId="103"/>
-    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="102"/>
-    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="101"/>
-    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="100"/>
-    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="99"/>
-    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="98"/>
-    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="97"/>
-    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="96">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:O2" totalsRowShown="0" headerRowDxfId="94" dataDxfId="93">
+  <autoFilter ref="A1:O2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}"/>
+  <tableColumns count="15">
+    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="92"/>
+    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="91"/>
+    <tableColumn id="15" xr3:uid="{D25A390C-69B5-4326-A0D4-10EB45DDE5E5}" name="Tag_ID" dataDxfId="90"/>
+    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="89"/>
+    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="88"/>
+    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="87"/>
+    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="86"/>
+    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="85"/>
+    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="84"/>
+    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="83">
       <calculatedColumnFormula>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="95"/>
-    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="94"/>
-    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="93"/>
-    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="92"/>
+    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="82"/>
+    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="81"/>
+    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="80"/>
+    <tableColumn id="13" xr3:uid="{71578D4D-1C79-4D4F-9C0F-A2C991F460FD}" name="Date Sold" dataDxfId="0"/>
+    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="79"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="91" dataDxfId="90">
-  <autoFilter ref="A1:K2" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}"/>
-  <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="89"/>
-    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="88"/>
-    <tableColumn id="4" xr3:uid="{17EB0B09-11B3-4E08-9442-E3C9AB87A157}" name="Tag_ID" dataDxfId="87"/>
-    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="86"/>
-    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Brand/Model" dataDxfId="85"/>
-    <tableColumn id="5" xr3:uid="{635BBD6A-77A8-4D20-9604-D9224474672C}" name="Serial Number" dataDxfId="84"/>
-    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="83"/>
-    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="82"/>
-    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="81"/>
-    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="80"/>
-    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Manual Link/Other Info" dataDxfId="79"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:J2" insertRow="1" totalsRowShown="0" headerRowDxfId="78" dataDxfId="77">
+  <autoFilter ref="A1:J2" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}"/>
+  <tableColumns count="10">
+    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="76"/>
+    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="75"/>
+    <tableColumn id="4" xr3:uid="{17EB0B09-11B3-4E08-9442-E3C9AB87A157}" name="Tag_ID" dataDxfId="74"/>
+    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="73"/>
+    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Brand/Model" dataDxfId="72"/>
+    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="71"/>
+    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="70"/>
+    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="69"/>
+    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="68"/>
+    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Serial Number/Other Info" dataDxfId="67"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:K2" totalsRowShown="0" headerRowDxfId="78" dataDxfId="77">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:K2" totalsRowShown="0" headerRowDxfId="129" dataDxfId="128">
   <autoFilter ref="A1:K2" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="76"/>
-    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="75"/>
-    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="74"/>
-    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="73"/>
-    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="72"/>
-    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="71"/>
-    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="70"/>
-    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="69"/>
-    <tableColumn id="11" xr3:uid="{4809319D-ABCA-43DA-A400-5DC91167D78B}" name="Complete" dataDxfId="68"/>
-    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Completion Date" dataDxfId="0"/>
-    <tableColumn id="12" xr3:uid="{920CB592-D743-4B33-A796-C7F3DB32211C}" name="Remarks" dataDxfId="67"/>
+    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="127"/>
+    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="126"/>
+    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="125"/>
+    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="124"/>
+    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="123"/>
+    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="122"/>
+    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="121"/>
+    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="120"/>
+    <tableColumn id="11" xr3:uid="{4809319D-ABCA-43DA-A400-5DC91167D78B}" name="Complete" dataDxfId="119"/>
+    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Completion Date" dataDxfId="118"/>
+    <tableColumn id="12" xr3:uid="{920CB592-D743-4B33-A796-C7F3DB32211C}" name="Remarks" dataDxfId="117"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1621,24 +1621,24 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="D1" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" t="s">
         <v>35</v>
-      </c>
-      <c r="F1" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="B2" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C2" s="8">
         <v>3</v>
@@ -1651,12 +1651,12 @@
         <v>300</v>
       </c>
       <c r="F2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="B3" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C3" s="8">
         <v>4</v>
@@ -1669,12 +1669,12 @@
         <v>40</v>
       </c>
       <c r="F3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="B4" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C4" s="8">
         <v>5</v>
@@ -1687,12 +1687,12 @@
         <v>100</v>
       </c>
       <c r="F4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="B5" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C5" s="8">
         <v>1000</v>
@@ -1748,13 +1748,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>2</v>
@@ -1763,28 +1763,28 @@
         <v>3</v>
       </c>
       <c r="G1" t="s">
+        <v>94</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="J1" t="s">
+        <v>95</v>
+      </c>
+      <c r="K1" t="s">
         <v>96</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="L1" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="I1" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="J1" t="s">
-        <v>97</v>
-      </c>
-      <c r="K1" t="s">
-        <v>98</v>
-      </c>
-      <c r="L1" s="8" t="s">
-        <v>22</v>
-      </c>
       <c r="M1" s="5" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="O1" s="6"/>
       <c r="P1" s="6"/>
@@ -1856,25 +1856,25 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="F1" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="G1" s="4" t="s">
-        <v>29</v>
-      </c>
       <c r="H1" s="4" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="I1" s="6"/>
     </row>
@@ -1924,22 +1924,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="G1" s="4" t="s">
         <v>47</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -1967,33 +1967,33 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E1" t="s">
         <v>54</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D1" t="s">
-        <v>55</v>
-      </c>
-      <c r="E1" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="1" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="D2" t="s">
         <v>91</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="E2" t="s">
         <v>92</v>
-      </c>
-      <c r="D2" t="s">
-        <v>93</v>
-      </c>
-      <c r="E2" t="s">
-        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -2015,10 +2015,10 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>37</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -2065,37 +2065,37 @@
         <v>0</v>
       </c>
       <c r="B1" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="H1" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="I1" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="D1" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="G1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="H1" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="I1" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>68</v>
-      </c>
       <c r="K1" s="8" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="L1" s="8" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:12">
@@ -2172,15 +2172,15 @@
   <sheetData>
     <row r="9" spans="1:2">
       <c r="A9" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B10" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2189,7 +2189,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B11" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2198,7 +2198,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B12" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2207,7 +2207,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B13" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2216,7 +2216,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B14" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2225,7 +2225,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B15" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2234,7 +2234,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B16" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2243,7 +2243,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B17" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2252,7 +2252,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B18" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2261,7 +2261,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B19" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2270,7 +2270,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B20" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2279,7 +2279,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B21" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2302,7 +2302,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDE7BF89-A2E7-4A6F-B822-317739E206EC}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:R2"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
@@ -2318,14 +2318,15 @@
     <col min="11" max="11" width="19.109375" style="2" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="16.6640625" style="3" customWidth="1"/>
     <col min="13" max="13" width="16.88671875" style="3" customWidth="1"/>
-    <col min="14" max="14" width="16.88671875" style="14" customWidth="1"/>
-    <col min="15" max="15" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="16.88671875" style="6" customWidth="1"/>
-    <col min="17" max="17" width="16.88671875" style="2" customWidth="1"/>
-    <col min="18" max="16384" width="8.88671875" style="6"/>
+    <col min="14" max="14" width="16.88671875" style="10" customWidth="1"/>
+    <col min="15" max="15" width="16.88671875" style="14" customWidth="1"/>
+    <col min="16" max="16" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.88671875" style="6" customWidth="1"/>
+    <col min="18" max="18" width="16.88671875" style="2" customWidth="1"/>
+    <col min="19" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17">
+    <row r="1" spans="1:18">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2333,10 +2334,10 @@
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>2</v>
@@ -2365,20 +2366,23 @@
       <c r="M1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="O1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="O1" s="6"/>
-      <c r="Q1" s="6"/>
-    </row>
-    <row r="2" spans="1:17">
+      <c r="P1" s="6"/>
+      <c r="R1" s="6"/>
+    </row>
+    <row r="2" spans="1:18">
       <c r="D2" s="6"/>
       <c r="J2" s="5">
         <f>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</f>
         <v>0</v>
       </c>
-      <c r="O2" s="6"/>
-      <c r="Q2" s="6"/>
+      <c r="P2" s="6"/>
+      <c r="R2" s="6"/>
     </row>
   </sheetData>
   <dataValidations count="3">
@@ -2403,7 +2407,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B027EC69-551F-4051-8A71-8B106D207C6D}">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
@@ -2411,16 +2415,15 @@
     <col min="3" max="3" width="9.5546875" style="2" customWidth="1"/>
     <col min="4" max="4" width="12.33203125" style="6" customWidth="1"/>
     <col min="5" max="5" width="28.6640625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="14.88671875" style="2" customWidth="1"/>
-    <col min="7" max="7" width="14.6640625" style="10" customWidth="1"/>
-    <col min="8" max="8" width="14.6640625" style="3" customWidth="1"/>
-    <col min="9" max="9" width="12.33203125" style="14" customWidth="1"/>
-    <col min="11" max="11" width="11.44140625" style="6" customWidth="1"/>
-    <col min="12" max="12" width="32.6640625" style="2" customWidth="1"/>
-    <col min="13" max="16384" width="8.88671875" style="6"/>
+    <col min="6" max="6" width="14.6640625" style="10" customWidth="1"/>
+    <col min="7" max="7" width="14.6640625" style="3" customWidth="1"/>
+    <col min="8" max="8" width="12.33203125" style="14" customWidth="1"/>
+    <col min="10" max="10" width="40.88671875" style="6" customWidth="1"/>
+    <col min="11" max="11" width="32.6640625" style="2" customWidth="1"/>
+    <col min="12" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:11">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2428,45 +2431,42 @@
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="F1" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="F1" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="G1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="H1" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="I1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="J1" t="s">
-        <v>20</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="L1" s="6"/>
-    </row>
-    <row r="2" spans="1:12">
-      <c r="J2" s="6"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="6"/>
+      <c r="I1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="K1" s="6"/>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="I2" s="6"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="6"/>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K3:K1000" xr:uid="{D25ACF8B-D3DC-4EFD-9C68-FC99372E0DCF}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J3:J1000" xr:uid="{D25ACF8B-D3DC-4EFD-9C68-FC99372E0DCF}">
       <formula1>"Operational, Needs Repair, Unusable"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2" xr:uid="{4B2064CB-79C2-427D-B2C2-7CE85187D094}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2" xr:uid="{4B2064CB-79C2-427D-B2C2-7CE85187D094}">
       <formula1>"Operational, Needs Repair, Repair In-Progress, Unusable/Junk"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2504,34 +2504,34 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" t="s">
         <v>16</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="H1" s="9" t="s">
-        <v>19</v>
-      </c>
       <c r="I1" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="J1" s="9" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="L1" s="6"/>
       <c r="M1" s="6"/>
@@ -2593,34 +2593,34 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
       <c r="G1" t="s">
+        <v>48</v>
+      </c>
+      <c r="H1" t="s">
+        <v>49</v>
+      </c>
+      <c r="I1" t="s">
         <v>50</v>
       </c>
-      <c r="H1" t="s">
-        <v>51</v>
-      </c>
-      <c r="I1" t="s">
-        <v>52</v>
-      </c>
       <c r="J1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="M1" s="6"/>
     </row>
@@ -2685,16 +2685,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>5</v>
@@ -2703,16 +2703,16 @@
         <v>3</v>
       </c>
       <c r="H1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I1" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="J1" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="L1" s="6"/>
       <c r="M1" s="6"/>

</xml_diff>

<commit_message>
Added Tag_Type to support Scannable Label Feature to config and excel
</commit_message>
<xml_diff>
--- a/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
+++ b/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr codeName="ThisWorkbook"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1a2ae81d67634e6/Desktop/Michanikos Artifex Enterprises/MAE Custom Digital Solutions/MAE Workshop Inventory Management System/GITHUB_MAE_Workshop Inventory App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="245" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A23BFEE8-EBF3-46FC-858B-682CAA922A47}"/>
+  <xr:revisionPtr revIDLastSave="264" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{63D4C5E1-46F1-4483-B3A3-EB17702C42F9}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="6" activeTab="7" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="7" activeTab="9" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
   </bookViews>
   <sheets>
     <sheet name="TEST Inventory" sheetId="10" r:id="rId1"/>
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="101">
   <si>
     <t>mae_id</t>
   </si>
@@ -373,6 +373,9 @@
   </si>
   <si>
     <t>Serial Number/Other Info</t>
+  </si>
+  <si>
+    <t>Tag_Type</t>
   </si>
 </sst>
 </file>
@@ -469,52 +472,269 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="130">
+  <dxfs count="135">
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="1" hidden="1"/>
     </dxf>
@@ -529,8 +749,11 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
@@ -545,12 +768,16 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -564,208 +791,11 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="1"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
       <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="1"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
@@ -919,14 +949,25 @@
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="0"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -934,26 +975,8 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="1"/>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -1007,11 +1030,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}" name="TEST_Inventory" displayName="TEST_Inventory" ref="A1:F5" totalsRowShown="0">
   <autoFilter ref="A1:F5" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="116"/>
-    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="115"/>
-    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="114"/>
-    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="113"/>
-    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="112">
+    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="121"/>
+    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="120"/>
+    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="119"/>
+    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="118"/>
+    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="117">
       <calculatedColumnFormula>TEST_Inventory[[#This Row],[TEST Integer]]*TEST_Inventory[[#This Row],[TEST Currency]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{AB3A5F3C-FCF0-4466-90FD-8ABB6E18DF5C}" name="TEST Dropdown"/>
@@ -1021,22 +1044,23 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:N2" totalsRowShown="0" headerRowDxfId="40" dataDxfId="39">
-  <autoFilter ref="A1:N2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
-  <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="38"/>
-    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="37"/>
-    <tableColumn id="12" xr3:uid="{8F0FD29C-682B-41B4-82F2-913D40801887}" name="Tag_ID" dataDxfId="36"/>
-    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="35"/>
-    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="34"/>
-    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="33"/>
-    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Stock_Level" dataDxfId="32"/>
-    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="31"/>
-    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="30"/>
-    <tableColumn id="13" xr3:uid="{AA55BCE3-9AC1-4735-8622-15E62CA93E1A}" name="Stock_Count" dataDxfId="29"/>
-    <tableColumn id="14" xr3:uid="{FA5C79D4-6D25-4E4C-BE9F-4190C63530C2}" name="Bulk_Value" dataDxfId="28"/>
-    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="27"/>
-    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:O2" totalsRowShown="0" headerRowDxfId="45" dataDxfId="44">
+  <autoFilter ref="A1:O2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
+  <tableColumns count="15">
+    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="43"/>
+    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="42"/>
+    <tableColumn id="12" xr3:uid="{8F0FD29C-682B-41B4-82F2-913D40801887}" name="Tag_ID" dataDxfId="41"/>
+    <tableColumn id="15" xr3:uid="{CE0ECF5F-5626-4215-AC71-301755B31D23}" name="Tag_Type" dataDxfId="0"/>
+    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="40"/>
+    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="39"/>
+    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="38"/>
+    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Stock_Level" dataDxfId="37"/>
+    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="36"/>
+    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="35"/>
+    <tableColumn id="13" xr3:uid="{AA55BCE3-9AC1-4735-8622-15E62CA93E1A}" name="Stock_Count" dataDxfId="34"/>
+    <tableColumn id="14" xr3:uid="{FA5C79D4-6D25-4E4C-BE9F-4190C63530C2}" name="Bulk_Value" dataDxfId="33"/>
+    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="32"/>
+    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="31">
       <calculatedColumnFormula array="1">IF(
     Shop_Consumables[[#This Row],[Stock_Level]]="Counted",
     Shop_Consumables[[#This Row],[Stock_Count]] * Shop_Consumables[[#This Row],[Unit Cost]],
@@ -1052,40 +1076,40 @@
     )
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Supplier/Remarks" dataDxfId="25"/>
+    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Supplier/Remarks" dataDxfId="30"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:H2" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:H2" totalsRowShown="0" headerRowDxfId="29" dataDxfId="28">
   <autoFilter ref="A1:H2" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="22"/>
-    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="21"/>
-    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="20"/>
-    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="19"/>
-    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="18"/>
-    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="17"/>
-    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="16"/>
-    <tableColumn id="8" xr3:uid="{9140C4E8-CB9E-40BF-ABD9-13A971322B09}" name="Remarks" dataDxfId="15"/>
+    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="27"/>
+    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="26"/>
+    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="25"/>
+    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="24"/>
+    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="23"/>
+    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="22"/>
+    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="21"/>
+    <tableColumn id="8" xr3:uid="{9140C4E8-CB9E-40BF-ABD9-13A971322B09}" name="Remarks" dataDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
   <autoFilter ref="A1:G2" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="12"/>
-    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="10"/>
-    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="9"/>
-    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="8"/>
-    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="7"/>
-    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="17"/>
+    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="15"/>
+    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="14"/>
+    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="13"/>
+    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="12"/>
+    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="11"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1095,11 +1119,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}" name="Location" displayName="Location" ref="A1:E2" totalsRowShown="0">
   <autoFilter ref="A1:E2" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Description" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Description" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1109,10 +1133,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}" name="TEST_Dashboard" displayName="TEST_Dashboard" ref="A1:B2" totalsRowShown="0">
   <autoFilter ref="A1:B2" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="111">
+    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="116">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Currency])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="110">
+    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="115">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Integer])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1121,41 +1145,41 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:L2" totalsRowShown="0" headerRowDxfId="109" dataDxfId="108">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:L2" totalsRowShown="0" headerRowDxfId="114" dataDxfId="113">
   <autoFilter ref="A1:L2" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="107"/>
-    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="106">
+    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="112"/>
+    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="111">
       <calculatedColumnFormula>SUM(Resell_Inventory[Total Investment])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="105">
+    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="110">
       <calculatedColumnFormula>SUM(Resell_Inventory[Actual Sale Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="104">
+    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="109">
       <calculatedColumnFormula>SUM(Shop_Machinery[Purchase Cost])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="103">
+    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="108">
       <calculatedColumnFormula>SUM(Shop_Power_Tools[Purchase Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="102">
+    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="107">
       <calculatedColumnFormula>SUM(Shop_Hand_Tools[Purchase Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="101">
+    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="106">
       <calculatedColumnFormula>SUM(Shop_Consumables[Current Inventory Value])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="100">
+    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="105">
       <calculatedColumnFormula>SUM(D2,E2,F2,G2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="99">
+    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="104">
       <calculatedColumnFormula array="1">SUMPRODUCT(
     ((Shop_Consumables[Stock_Level]="Counted") * (ISNUMBER(Shop_Consumables[Stock_Count])) * (Shop_Consumables[Stock_Count]&lt;=Shop_Consumables[Reorder Point])) +
     ((ISNUMBER(MATCH(Shop_Consumables[Stock_Level], {"Few","None"}, 0))))
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="98">
+    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="103">
       <calculatedColumnFormula>SUMIFS(Shop_Overhead[Amount], Shop_Overhead[Due Date], "&lt;="&amp;TODAY()+30, Shop_Overhead[Due Date], "&gt;="&amp;TODAY())</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{E4065760-B1B1-4564-936B-3405D3B80297}" name="Equipment With Operational Issues" dataDxfId="97">
+    <tableColumn id="12" xr3:uid="{E4065760-B1B1-4564-936B-3405D3B80297}" name="Equipment With Operational Issues" dataDxfId="102">
       <calculatedColumnFormula array="1">SUM(
   COUNTIFS(Shop_Machinery[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"}),
   COUNTIFS(Shop_Power_Tools[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"}),
@@ -1174,8 +1198,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{F579DA07-7AD6-49DA-9B44-D5B1132EDAC6}" name="Overhead_Summary" displayName="Overhead_Summary" ref="A9:B21" totalsRowShown="0">
   <autoFilter ref="A9:B21" xr:uid="{F579DA07-7AD6-49DA-9B44-D5B1132EDAC6}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{7CA4839C-9603-479D-BD1C-8377DFA9603C}" name="Expense Category" dataDxfId="96"/>
-    <tableColumn id="2" xr3:uid="{FE0F7616-EAF3-443D-AC69-DE6541DC10E5}" name="Annual Total" dataDxfId="95">
+    <tableColumn id="1" xr3:uid="{7CA4839C-9603-479D-BD1C-8377DFA9603C}" name="Expense Category" dataDxfId="101"/>
+    <tableColumn id="2" xr3:uid="{FE0F7616-EAF3-443D-AC69-DE6541DC10E5}" name="Annual Total" dataDxfId="100">
       <calculatedColumnFormula>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1184,105 +1208,109 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:O2" totalsRowShown="0" headerRowDxfId="94" dataDxfId="93">
-  <autoFilter ref="A1:O2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}"/>
-  <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="92"/>
-    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="91"/>
-    <tableColumn id="15" xr3:uid="{D25A390C-69B5-4326-A0D4-10EB45DDE5E5}" name="Tag_ID" dataDxfId="90"/>
-    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="89"/>
-    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="88"/>
-    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="87"/>
-    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="86"/>
-    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="85"/>
-    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="84"/>
-    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="83">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:P2" totalsRowShown="0" headerRowDxfId="99" dataDxfId="98">
+  <autoFilter ref="A1:P2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}"/>
+  <tableColumns count="16">
+    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="97"/>
+    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="96"/>
+    <tableColumn id="15" xr3:uid="{D25A390C-69B5-4326-A0D4-10EB45DDE5E5}" name="Tag_ID" dataDxfId="95"/>
+    <tableColumn id="16" xr3:uid="{57D16231-357C-4C08-B062-20555121C2D6}" name="Tag_Type" dataDxfId="5"/>
+    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="94"/>
+    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="93"/>
+    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="92"/>
+    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="91"/>
+    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="90"/>
+    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="89"/>
+    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="88">
       <calculatedColumnFormula>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="82"/>
-    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="81"/>
-    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="80"/>
-    <tableColumn id="13" xr3:uid="{71578D4D-1C79-4D4F-9C0F-A2C991F460FD}" name="Date Sold" dataDxfId="0"/>
-    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="79"/>
+    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="87"/>
+    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="86"/>
+    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="85"/>
+    <tableColumn id="13" xr3:uid="{71578D4D-1C79-4D4F-9C0F-A2C991F460FD}" name="Date Sold" dataDxfId="84"/>
+    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="83"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:J2" insertRow="1" totalsRowShown="0" headerRowDxfId="78" dataDxfId="77">
-  <autoFilter ref="A1:J2" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}"/>
-  <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="76"/>
-    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="75"/>
-    <tableColumn id="4" xr3:uid="{17EB0B09-11B3-4E08-9442-E3C9AB87A157}" name="Tag_ID" dataDxfId="74"/>
-    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="73"/>
-    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Brand/Model" dataDxfId="72"/>
-    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="71"/>
-    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="70"/>
-    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="69"/>
-    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="68"/>
-    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Serial Number/Other Info" dataDxfId="67"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="82" dataDxfId="81">
+  <autoFilter ref="A1:K2" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="80"/>
+    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="79"/>
+    <tableColumn id="4" xr3:uid="{17EB0B09-11B3-4E08-9442-E3C9AB87A157}" name="Tag_ID" dataDxfId="78"/>
+    <tableColumn id="5" xr3:uid="{72EAA357-95AA-4893-8038-2A77BDD0FB87}" name="Tag_Type" dataDxfId="4"/>
+    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="77"/>
+    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Brand/Model" dataDxfId="76"/>
+    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="75"/>
+    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="74"/>
+    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="73"/>
+    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="72"/>
+    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Serial Number/Other Info" dataDxfId="71"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:K2" totalsRowShown="0" headerRowDxfId="129" dataDxfId="128">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:K2" totalsRowShown="0" headerRowDxfId="70" dataDxfId="69">
   <autoFilter ref="A1:K2" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="127"/>
-    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="126"/>
-    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="125"/>
-    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="124"/>
-    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="123"/>
-    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="122"/>
-    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="121"/>
-    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="120"/>
-    <tableColumn id="11" xr3:uid="{4809319D-ABCA-43DA-A400-5DC91167D78B}" name="Complete" dataDxfId="119"/>
-    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Completion Date" dataDxfId="118"/>
-    <tableColumn id="12" xr3:uid="{920CB592-D743-4B33-A796-C7F3DB32211C}" name="Remarks" dataDxfId="117"/>
+    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="68"/>
+    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="67"/>
+    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="66"/>
+    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="65"/>
+    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="64"/>
+    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="63"/>
+    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="62"/>
+    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="61"/>
+    <tableColumn id="11" xr3:uid="{4809319D-ABCA-43DA-A400-5DC91167D78B}" name="Complete" dataDxfId="60"/>
+    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Completion Date" dataDxfId="59"/>
+    <tableColumn id="12" xr3:uid="{920CB592-D743-4B33-A796-C7F3DB32211C}" name="Remarks" dataDxfId="58"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:K2" totalsRowShown="0" headerRowDxfId="66" dataDxfId="65">
-  <autoFilter ref="A1:K2" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}"/>
-  <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="64"/>
-    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="63"/>
-    <tableColumn id="11" xr3:uid="{21951C81-00A4-4344-9E81-B1B1DB06ADEF}" name="Tag_ID" dataDxfId="62"/>
-    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="61"/>
-    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Brand/Model" dataDxfId="60"/>
-    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="59"/>
-    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="58"/>
-    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="57"/>
-    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="56"/>
-    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="55"/>
-    <tableColumn id="10" xr3:uid="{26197E01-2936-4F5F-8081-3AA351C1CD38}" name="Remarks" dataDxfId="54"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:L2" totalsRowShown="0" headerRowDxfId="134" dataDxfId="133">
+  <autoFilter ref="A1:L2" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}"/>
+  <tableColumns count="12">
+    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="132"/>
+    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="131"/>
+    <tableColumn id="11" xr3:uid="{21951C81-00A4-4344-9E81-B1B1DB06ADEF}" name="Tag_ID" dataDxfId="130"/>
+    <tableColumn id="12" xr3:uid="{7F1AFB3A-34F9-4E3E-A9D3-7E7E1458ECFE}" name="Tag_Type" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="129"/>
+    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Brand/Model" dataDxfId="128"/>
+    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="127"/>
+    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="126"/>
+    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="125"/>
+    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="124"/>
+    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="123"/>
+    <tableColumn id="10" xr3:uid="{26197E01-2936-4F5F-8081-3AA351C1CD38}" name="Remarks" dataDxfId="122"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:K2" totalsRowShown="0" headerRowDxfId="53" dataDxfId="52">
-  <autoFilter ref="A1:K2" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}"/>
-  <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="51"/>
-    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="50"/>
-    <tableColumn id="10" xr3:uid="{C8BD69AA-9023-4777-9C96-39A81F1E4BE0}" name="Tag_ID" dataDxfId="49"/>
-    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="48"/>
-    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Brand/Model/Description" dataDxfId="47"/>
-    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="46"/>
-    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="45"/>
-    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="44"/>
-    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Stock_Level" dataDxfId="43"/>
-    <tableColumn id="11" xr3:uid="{FD8D2D17-0451-45E0-8688-0BB4F60073DA}" name="Stock_Count" dataDxfId="42"/>
-    <tableColumn id="9" xr3:uid="{2B57F5E6-66C5-4DBA-8949-836DE0F0791C}" name="Remarks" dataDxfId="41"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:L2" totalsRowShown="0" headerRowDxfId="57" dataDxfId="56">
+  <autoFilter ref="A1:L2" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}"/>
+  <tableColumns count="12">
+    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="55"/>
+    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="54"/>
+    <tableColumn id="10" xr3:uid="{C8BD69AA-9023-4777-9C96-39A81F1E4BE0}" name="Tag_ID" dataDxfId="53"/>
+    <tableColumn id="12" xr3:uid="{FC4D7CE3-2DF1-465E-A4D1-1D1F02F8B8CA}" name="Tag_Type" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Brand/Model/Description" dataDxfId="52"/>
+    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="51"/>
+    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="50"/>
+    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="49"/>
+    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Stock_Level" dataDxfId="48"/>
+    <tableColumn id="11" xr3:uid="{FD8D2D17-0451-45E0-8688-0BB4F60073DA}" name="Stock_Count" dataDxfId="47"/>
+    <tableColumn id="9" xr3:uid="{2B57F5E6-66C5-4DBA-8949-836DE0F0791C}" name="Remarks" dataDxfId="46"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1721,29 +1749,29 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E1902F1-C59B-4A1A-9D95-2C39AEF944E5}">
   <sheetPr codeName="Sheet7"/>
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:S2"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
     <col min="2" max="2" width="10.33203125" style="14" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.33203125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="22.6640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="41.6640625" style="2" customWidth="1"/>
-    <col min="7" max="7" width="15.5546875" style="6" customWidth="1"/>
-    <col min="8" max="8" width="18.44140625" style="2" customWidth="1"/>
-    <col min="9" max="9" width="14.33203125" style="7" customWidth="1"/>
-    <col min="10" max="10" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.6640625" customWidth="1"/>
-    <col min="12" max="12" width="15.5546875" style="6" customWidth="1"/>
-    <col min="13" max="13" width="22.5546875" customWidth="1"/>
-    <col min="14" max="14" width="14.109375" style="7" customWidth="1"/>
-    <col min="15" max="15" width="10.44140625" style="3" customWidth="1"/>
-    <col min="17" max="17" width="22.6640625" style="2" customWidth="1"/>
-    <col min="18" max="18" width="46.6640625" style="2" customWidth="1"/>
-    <col min="19" max="16384" width="8.88671875" style="6"/>
+    <col min="3" max="4" width="10.33203125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="22.6640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="41.6640625" style="2" customWidth="1"/>
+    <col min="8" max="8" width="15.5546875" style="6" customWidth="1"/>
+    <col min="9" max="9" width="18.44140625" style="2" customWidth="1"/>
+    <col min="10" max="10" width="14.33203125" style="7" customWidth="1"/>
+    <col min="11" max="11" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.6640625" customWidth="1"/>
+    <col min="13" max="13" width="15.5546875" style="6" customWidth="1"/>
+    <col min="14" max="14" width="22.5546875" customWidth="1"/>
+    <col min="15" max="15" width="14.109375" style="7" customWidth="1"/>
+    <col min="16" max="16" width="10.44140625" style="3" customWidth="1"/>
+    <col min="18" max="18" width="22.6640625" style="2" customWidth="1"/>
+    <col min="19" max="19" width="46.6640625" style="2" customWidth="1"/>
+    <col min="20" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18">
+    <row r="1" spans="1:19">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1753,52 +1781,55 @@
       <c r="C1" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="E1" t="s">
         <v>52</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>94</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>95</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>96</v>
       </c>
-      <c r="L1" s="8" t="s">
+      <c r="M1" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="O1" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="O1" s="6"/>
       <c r="P1" s="6"/>
       <c r="Q1" s="6"/>
       <c r="R1" s="6"/>
-    </row>
-    <row r="2" spans="1:18">
-      <c r="F2" s="2"/>
-      <c r="I2" s="3"/>
-      <c r="J2" s="6"/>
+      <c r="S1" s="6"/>
+    </row>
+    <row r="2" spans="1:19">
+      <c r="G2" s="2"/>
+      <c r="J2" s="3"/>
       <c r="K2" s="6"/>
-      <c r="L2" s="7"/>
-      <c r="M2" s="3" cm="1">
-        <f t="array" ref="M2">IF(
+      <c r="L2" s="6"/>
+      <c r="M2" s="7"/>
+      <c r="N2" s="3" cm="1">
+        <f t="array" ref="N2">IF(
     Shop_Consumables[[#This Row],[Stock_Level]]="Counted",
     Shop_Consumables[[#This Row],[Stock_Count]] * Shop_Consumables[[#This Row],[Unit Cost]],
     IF(
@@ -1814,15 +1845,15 @@
 )</f>
         <v>0</v>
       </c>
-      <c r="N2" s="2"/>
-      <c r="O2" s="6"/>
+      <c r="O2" s="2"/>
       <c r="P2" s="6"/>
       <c r="Q2" s="6"/>
       <c r="R2" s="6"/>
+      <c r="S2" s="6"/>
     </row>
   </sheetData>
   <dataValidations disablePrompts="1" count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:G2" xr:uid="{D2C605E8-D02B-4558-82DE-3169088704E8}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:H2" xr:uid="{D2C605E8-D02B-4558-82DE-3169088704E8}">
       <formula1>"Fasteners/Hardware,Abrasives/Cutting,Fluids/Lubricants/Chemicals,Primer/Paint,Safety/PPE,Shop/Janitorial,Welding,Electrical,Other"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2302,31 +2333,31 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDE7BF89-A2E7-4A6F-B822-317739E206EC}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:S2"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
     <col min="2" max="2" width="9.5546875" style="14" customWidth="1"/>
-    <col min="3" max="3" width="9.5546875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="31.44140625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="10.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17" style="10" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.33203125" style="3" customWidth="1"/>
-    <col min="9" max="9" width="16.5546875" style="3" customWidth="1"/>
-    <col min="10" max="10" width="16.6640625" style="5" customWidth="1"/>
-    <col min="11" max="11" width="19.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16.6640625" style="3" customWidth="1"/>
-    <col min="13" max="13" width="16.88671875" style="3" customWidth="1"/>
-    <col min="14" max="14" width="16.88671875" style="10" customWidth="1"/>
-    <col min="15" max="15" width="16.88671875" style="14" customWidth="1"/>
-    <col min="16" max="16" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="16.88671875" style="6" customWidth="1"/>
-    <col min="18" max="18" width="16.88671875" style="2" customWidth="1"/>
-    <col min="19" max="16384" width="8.88671875" style="6"/>
+    <col min="3" max="4" width="9.5546875" style="2" customWidth="1"/>
+    <col min="5" max="5" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="31.44140625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="10.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17" style="10" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.33203125" style="3" customWidth="1"/>
+    <col min="10" max="10" width="16.5546875" style="3" customWidth="1"/>
+    <col min="11" max="11" width="16.6640625" style="5" customWidth="1"/>
+    <col min="12" max="12" width="19.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.6640625" style="3" customWidth="1"/>
+    <col min="14" max="14" width="16.88671875" style="3" customWidth="1"/>
+    <col min="15" max="15" width="16.88671875" style="10" customWidth="1"/>
+    <col min="16" max="16" width="16.88671875" style="14" customWidth="1"/>
+    <col min="17" max="17" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="16.88671875" style="6" customWidth="1"/>
+    <col min="19" max="19" width="16.88671875" style="2" customWidth="1"/>
+    <col min="20" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18">
+    <row r="1" spans="1:19">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2336,63 +2367,66 @@
       <c r="C1" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="E1" t="s">
         <v>52</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="H1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="L1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="M1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="N1" s="9" t="s">
+      <c r="O1" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="P1" s="6"/>
-      <c r="R1" s="6"/>
-    </row>
-    <row r="2" spans="1:18">
-      <c r="D2" s="6"/>
-      <c r="J2" s="5">
+      <c r="Q1" s="6"/>
+      <c r="S1" s="6"/>
+    </row>
+    <row r="2" spans="1:19">
+      <c r="E2" s="6"/>
+      <c r="K2" s="5">
         <f>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</f>
         <v>0</v>
       </c>
-      <c r="P2" s="6"/>
-      <c r="R2" s="6"/>
+      <c r="Q2" s="6"/>
+      <c r="S2" s="6"/>
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K3:K1000" xr:uid="{F45414DD-76C8-4DC4-96E2-15B89FDB5B51}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L3:L1000" xr:uid="{F45414DD-76C8-4DC4-96E2-15B89FDB5B51}">
       <formula1>"work not started, restoration in progress, for sale, sold"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2" xr:uid="{C1AA0387-29B3-4797-A152-88A8C024D825}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2" xr:uid="{C1AA0387-29B3-4797-A152-88A8C024D825}">
       <formula1>"Machinery, Furniture, Electronics, Craft, Auto Related, Other"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2" xr:uid="{3C9AD8AD-AB10-403F-A04B-87B1D7C9B98E}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L2" xr:uid="{3C9AD8AD-AB10-403F-A04B-87B1D7C9B98E}">
       <formula1>"Not Started, In-Progress, Complete, For Sale, Sold"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2407,23 +2441,23 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B027EC69-551F-4051-8A71-8B106D207C6D}">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
     <col min="2" max="2" width="9.5546875" style="14" customWidth="1"/>
-    <col min="3" max="3" width="9.5546875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="12.33203125" style="6" customWidth="1"/>
-    <col min="5" max="5" width="28.6640625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="14.6640625" style="10" customWidth="1"/>
-    <col min="7" max="7" width="14.6640625" style="3" customWidth="1"/>
-    <col min="8" max="8" width="12.33203125" style="14" customWidth="1"/>
-    <col min="10" max="10" width="40.88671875" style="6" customWidth="1"/>
-    <col min="11" max="11" width="32.6640625" style="2" customWidth="1"/>
-    <col min="12" max="16384" width="8.88671875" style="6"/>
+    <col min="3" max="4" width="9.5546875" style="2" customWidth="1"/>
+    <col min="5" max="5" width="12.33203125" style="6" customWidth="1"/>
+    <col min="6" max="6" width="28.6640625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="14.6640625" style="10" customWidth="1"/>
+    <col min="8" max="8" width="14.6640625" style="3" customWidth="1"/>
+    <col min="9" max="9" width="12.33203125" style="14" customWidth="1"/>
+    <col min="11" max="11" width="40.88671875" style="6" customWidth="1"/>
+    <col min="12" max="12" width="32.6640625" style="2" customWidth="1"/>
+    <col min="13" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2433,40 +2467,43 @@
       <c r="C1" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="E1" t="s">
         <v>52</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="G1" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>19</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="K1" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="K1" s="6"/>
-    </row>
-    <row r="2" spans="1:11">
-      <c r="I2" s="6"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="6"/>
+      <c r="L1" s="6"/>
+    </row>
+    <row r="2" spans="1:12">
+      <c r="J2" s="6"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="6"/>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J3:J1000" xr:uid="{D25ACF8B-D3DC-4EFD-9C68-FC99372E0DCF}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K3:K1000" xr:uid="{D25ACF8B-D3DC-4EFD-9C68-FC99372E0DCF}">
       <formula1>"Operational, Needs Repair, Unusable"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2" xr:uid="{4B2064CB-79C2-427D-B2C2-7CE85187D094}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2" xr:uid="{4B2064CB-79C2-427D-B2C2-7CE85187D094}">
       <formula1>"Operational, Needs Repair, Repair In-Progress, Unusable/Junk"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2570,25 +2607,25 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEDDDAA7-75C3-4AA5-ABFD-D5FB4C627E4C}">
   <sheetPr codeName="Sheet5"/>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
     <col min="2" max="2" width="8.6640625" style="14" customWidth="1"/>
-    <col min="3" max="3" width="8.6640625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="12.88671875" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="50.44140625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="15.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.88671875" style="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.88671875" style="6" customWidth="1"/>
-    <col min="10" max="10" width="14.44140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.5546875" style="6" customWidth="1"/>
-    <col min="13" max="13" width="14.44140625" style="2" customWidth="1"/>
-    <col min="14" max="16384" width="8.88671875" style="6"/>
+    <col min="3" max="4" width="8.6640625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="12.88671875" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="50.44140625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="15.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.88671875" style="6" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.88671875" style="6" customWidth="1"/>
+    <col min="11" max="11" width="14.44140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.5546875" style="6" customWidth="1"/>
+    <col min="14" max="14" width="14.44140625" style="2" customWidth="1"/>
+    <col min="15" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2598,56 +2635,59 @@
       <c r="C1" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="E1" t="s">
         <v>52</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>48</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>49</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>50</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>19</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="L1" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="M1" s="6"/>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="G2" s="6"/>
-      <c r="K2" s="2"/>
-      <c r="M2" s="6"/>
+      <c r="N1" s="6"/>
+    </row>
+    <row r="2" spans="1:14">
+      <c r="H2" s="6"/>
+      <c r="L2" s="2"/>
+      <c r="N2" s="6"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <dataValidations count="6">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M3:M1000 H3:J1000" xr:uid="{FF61F80C-5E23-45D6-B39D-7C5635258115}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N3:N1000 I3:K1000" xr:uid="{FF61F80C-5E23-45D6-B39D-7C5635258115}">
       <formula1>"Circular Saw, Drill, Sander, Grinder, Other"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L3:M1000" xr:uid="{DB752B4D-0E75-42D1-B907-2DBC5792F422}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M3:N1000" xr:uid="{DB752B4D-0E75-42D1-B907-2DBC5792F422}">
       <formula1>"New, Operational, Needs Repair, Broken"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2" xr:uid="{05EFC744-2B0C-453D-A1B6-F8391608434D}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2" xr:uid="{05EFC744-2B0C-453D-A1B6-F8391608434D}">
       <formula1>"Drilling, Cutting, Grinding, Sanding, Fastening, Shaping/Routing, Other"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2" xr:uid="{194EFB2B-690A-4D50-8AF6-E8ED45FE2FCA}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2" xr:uid="{194EFB2B-690A-4D50-8AF6-E8ED45FE2FCA}">
       <formula1>"Portable/Handheld, Stationary/Bench Top, Outdoor Power Equipment, "</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:K2" xr:uid="{980AB122-9104-490B-993D-4F2FEF3A4EE6}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2:L2" xr:uid="{980AB122-9104-490B-993D-4F2FEF3A4EE6}">
       <formula1>"Operational, Needs Repair, Repair In-Progress, Unusable/Junk"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2 K2" xr:uid="{47F6EF9A-B127-4EB7-A5E8-0075055489DC}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2 L2" xr:uid="{47F6EF9A-B127-4EB7-A5E8-0075055489DC}">
       <formula1>"Corded(A/C), Cordless/Battery, Pneumatic/Air, Fuel-Powered"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2661,26 +2701,26 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F39ADDA6-CD5F-4655-A9C0-9676DDAC362E}">
   <sheetPr codeName="Sheet6"/>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.6640625" style="14" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.6640625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="12.88671875" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="54.6640625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="15.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.5546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.6640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.33203125" style="7" customWidth="1"/>
-    <col min="14" max="14" width="12.88671875" style="2" customWidth="1"/>
-    <col min="15" max="16384" width="8.88671875" style="6"/>
+    <col min="3" max="4" width="8.6640625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="12.88671875" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="54.6640625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="15.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.5546875" style="6" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.6640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="16.33203125" style="7" customWidth="1"/>
+    <col min="15" max="15" width="12.88671875" style="2" customWidth="1"/>
+    <col min="16" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2690,51 +2730,54 @@
       <c r="C1" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="E1" t="s">
         <v>52</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>3</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>19</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>94</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>95</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="L1" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="L1" s="6"/>
       <c r="M1" s="6"/>
       <c r="N1" s="6"/>
-    </row>
-    <row r="2" spans="1:14">
-      <c r="H2" s="6"/>
+      <c r="O1" s="6"/>
+    </row>
+    <row r="2" spans="1:15">
       <c r="I2" s="6"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="6"/>
+      <c r="J2" s="6"/>
+      <c r="L2" s="2"/>
       <c r="M2" s="6"/>
       <c r="N2" s="6"/>
+      <c r="O2" s="6"/>
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N3:N1000 D3:D1000 G3:G1000 J3:K1000" xr:uid="{B6CB3C84-EE01-4878-B558-650FC19D8248}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O3:O1000 E3:E1000 H3:H1000 K3:L1000" xr:uid="{B6CB3C84-EE01-4878-B558-650FC19D8248}">
       <formula1>"Saw, Hammer, Screwdriver, Wrench, Sockets, Pliers, Measuring, Files, Other"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2" xr:uid="{ACB7A40B-F0EE-4387-88E4-5140AB68313F}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2" xr:uid="{ACB7A40B-F0EE-4387-88E4-5140AB68313F}">
       <formula1>"Fastening/Turning,Measuring/Layout,Striking/Hammering,Gripping/Holding,Cutting/Shaping,Other"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:K2 H2" xr:uid="{2E543736-2E6D-4F90-9169-21BA7CCD7676}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2:L2 I2" xr:uid="{2E543736-2E6D-4F90-9169-21BA7CCD7676}">
       <formula1>"Operational,Needs Repair,Repair In-Progress,Unusable/Junk"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
updated config.js and MASTER excel for inventory tables to have common item name description: Item_Description
</commit_message>
<xml_diff>
--- a/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
+++ b/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1a2ae81d67634e6/Desktop/Michanikos Artifex Enterprises/MAE Custom Digital Solutions/MAE Workshop Inventory Management System/GITHUB_MAE_Workshop Inventory App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="264" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{63D4C5E1-46F1-4483-B3A3-EB17702C42F9}"/>
+  <xr:revisionPtr revIDLastSave="269" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{493A87AF-F71D-4440-9E96-EC13B25D8C66}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="7" activeTab="9" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="4" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
   </bookViews>
   <sheets>
     <sheet name="TEST Inventory" sheetId="10" r:id="rId1"/>
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="98">
   <si>
     <t>mae_id</t>
   </si>
@@ -81,9 +81,6 @@
     <t>Asset ID</t>
   </si>
   <si>
-    <t>Item Name</t>
-  </si>
-  <si>
     <t>Category</t>
   </si>
   <si>
@@ -321,21 +318,12 @@
     <t>Maintenance Items Due in Next 30 Days</t>
   </si>
   <si>
-    <t>Machine Name/Brand/Model</t>
-  </si>
-  <si>
     <t>Complete</t>
   </si>
   <si>
     <t>Remarks</t>
   </si>
   <si>
-    <t>Tool Name/Brand/Model</t>
-  </si>
-  <si>
-    <t>Tool Name/Brand/Model/Description</t>
-  </si>
-  <si>
     <t>Supplier/Remarks</t>
   </si>
   <si>
@@ -376,6 +364,9 @@
   </si>
   <si>
     <t>Tag_Type</t>
+  </si>
+  <si>
+    <t>Item_Description</t>
   </si>
 </sst>
 </file>
@@ -474,74 +465,140 @@
   </cellStyles>
   <dxfs count="135">
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="1"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -552,7 +609,15 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -560,113 +625,11 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
+      <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -777,6 +740,10 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="1"/>
     </dxf>
     <dxf>
@@ -835,6 +802,10 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -951,27 +922,47 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
+      <numFmt numFmtId="1" formatCode="0"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -1030,11 +1021,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}" name="TEST_Inventory" displayName="TEST_Inventory" ref="A1:F5" totalsRowShown="0">
   <autoFilter ref="A1:F5" xr:uid="{8E24649D-B6D3-4E82-B133-E0A5E1711E35}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="121"/>
-    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="120"/>
-    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="119"/>
-    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="118"/>
-    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="117">
+    <tableColumn id="1" xr3:uid="{B0FB5A70-86CF-4587-B50C-E7DDB5961BCE}" name="mae_id" dataDxfId="117"/>
+    <tableColumn id="2" xr3:uid="{1F5221B2-FFA0-40D9-A91A-FC8A4B03C6C2}" name="TEST String" dataDxfId="116"/>
+    <tableColumn id="3" xr3:uid="{2786A104-092C-4BF4-9896-1EB64C071D4A}" name="TEST Integer" dataDxfId="115"/>
+    <tableColumn id="4" xr3:uid="{B1215FF8-A5CC-415A-BE9C-30A04277BFC2}" name="TEST Currency" dataDxfId="114"/>
+    <tableColumn id="5" xr3:uid="{596E6BD2-8E12-473A-9462-5B49301F9318}" name="TEST Formula" dataDxfId="113">
       <calculatedColumnFormula>TEST_Inventory[[#This Row],[TEST Integer]]*TEST_Inventory[[#This Row],[TEST Currency]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{AB3A5F3C-FCF0-4466-90FD-8ABB6E18DF5C}" name="TEST Dropdown"/>
@@ -1044,23 +1035,23 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:O2" totalsRowShown="0" headerRowDxfId="45" dataDxfId="44">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:O2" totalsRowShown="0" headerRowDxfId="134" dataDxfId="133">
   <autoFilter ref="A1:O2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="43"/>
-    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="42"/>
-    <tableColumn id="12" xr3:uid="{8F0FD29C-682B-41B4-82F2-913D40801887}" name="Tag_ID" dataDxfId="41"/>
-    <tableColumn id="15" xr3:uid="{CE0ECF5F-5626-4215-AC71-301755B31D23}" name="Tag_Type" dataDxfId="0"/>
-    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="40"/>
-    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item Name" dataDxfId="39"/>
-    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="38"/>
-    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Stock_Level" dataDxfId="37"/>
-    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="36"/>
-    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="35"/>
-    <tableColumn id="13" xr3:uid="{AA55BCE3-9AC1-4735-8622-15E62CA93E1A}" name="Stock_Count" dataDxfId="34"/>
-    <tableColumn id="14" xr3:uid="{FA5C79D4-6D25-4E4C-BE9F-4190C63530C2}" name="Bulk_Value" dataDxfId="33"/>
-    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="32"/>
-    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="31">
+    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="132"/>
+    <tableColumn id="3" xr3:uid="{93700212-1764-4626-B112-F202F0AA0AAB}" name="Asset_ID" dataDxfId="131"/>
+    <tableColumn id="12" xr3:uid="{8F0FD29C-682B-41B4-82F2-913D40801887}" name="Tag_ID" dataDxfId="130"/>
+    <tableColumn id="15" xr3:uid="{CE0ECF5F-5626-4215-AC71-301755B31D23}" name="Tag_Type" dataDxfId="129"/>
+    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="128"/>
+    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item_Description" dataDxfId="127"/>
+    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="126"/>
+    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Stock_Level" dataDxfId="125"/>
+    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="124"/>
+    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="123"/>
+    <tableColumn id="13" xr3:uid="{AA55BCE3-9AC1-4735-8622-15E62CA93E1A}" name="Stock_Count" dataDxfId="122"/>
+    <tableColumn id="14" xr3:uid="{FA5C79D4-6D25-4E4C-BE9F-4190C63530C2}" name="Bulk_Value" dataDxfId="121"/>
+    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="120"/>
+    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="119">
       <calculatedColumnFormula array="1">IF(
     Shop_Consumables[[#This Row],[Stock_Level]]="Counted",
     Shop_Consumables[[#This Row],[Stock_Count]] * Shop_Consumables[[#This Row],[Unit Cost]],
@@ -1076,40 +1067,40 @@
     )
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Supplier/Remarks" dataDxfId="30"/>
+    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Supplier/Remarks" dataDxfId="118"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:H2" totalsRowShown="0" headerRowDxfId="29" dataDxfId="28">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:H2" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
   <autoFilter ref="A1:H2" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="27"/>
-    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="26"/>
-    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="25"/>
-    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="24"/>
-    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="23"/>
-    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="22"/>
-    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="21"/>
-    <tableColumn id="8" xr3:uid="{9140C4E8-CB9E-40BF-ABD9-13A971322B09}" name="Remarks" dataDxfId="20"/>
+    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="20"/>
+    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="19"/>
+    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="18"/>
+    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="17"/>
+    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="16"/>
+    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="15"/>
+    <tableColumn id="8" xr3:uid="{9140C4E8-CB9E-40BF-ABD9-13A971322B09}" name="Remarks" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
   <autoFilter ref="A1:G2" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="17"/>
-    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="16"/>
-    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="15"/>
-    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="14"/>
-    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="13"/>
-    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="12"/>
-    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="11"/>
+    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="11"/>
+    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="9"/>
+    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="7"/>
+    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="6"/>
+    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1119,11 +1110,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}" name="Location" displayName="Location" ref="A1:E2" totalsRowShown="0">
   <autoFilter ref="A1:E2" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Description" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Description" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{2569BB68-2F34-48DF-B4D9-298E8FFAD0B9}" name="Type" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{C3AEC2FA-3915-4BA0-84FD-35E285F83E09}" name="Parent_Location" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1133,10 +1124,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}" name="TEST_Dashboard" displayName="TEST_Dashboard" ref="A1:B2" totalsRowShown="0">
   <autoFilter ref="A1:B2" xr:uid="{AA6EA604-2DDB-4EBE-8FB2-6DC6B8269D0A}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="116">
+    <tableColumn id="1" xr3:uid="{68FD6298-1F1B-4FCD-AAE1-65AC194B17FD}" name="TEST calc from other table" dataDxfId="112">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Currency])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="115">
+    <tableColumn id="2" xr3:uid="{897E8C99-2561-458C-9F95-86F8CADD8AB6}" name="TEST Number Calc from other table" dataDxfId="111">
       <calculatedColumnFormula>SUM(TEST_Inventory[TEST Integer])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1145,41 +1136,41 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:L2" totalsRowShown="0" headerRowDxfId="114" dataDxfId="113">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:L2" totalsRowShown="0" headerRowDxfId="110" dataDxfId="109">
   <autoFilter ref="A1:L2" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="112"/>
-    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="111">
+    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="108"/>
+    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="107">
       <calculatedColumnFormula>SUM(Resell_Inventory[Total Investment])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="110">
+    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="106">
       <calculatedColumnFormula>SUM(Resell_Inventory[Actual Sale Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="109">
+    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="105">
       <calculatedColumnFormula>SUM(Shop_Machinery[Purchase Cost])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="108">
+    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="104">
       <calculatedColumnFormula>SUM(Shop_Power_Tools[Purchase Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="107">
+    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="103">
       <calculatedColumnFormula>SUM(Shop_Hand_Tools[Purchase Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="106">
+    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="102">
       <calculatedColumnFormula>SUM(Shop_Consumables[Current Inventory Value])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="105">
+    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="101">
       <calculatedColumnFormula>SUM(D2,E2,F2,G2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="104">
+    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="100">
       <calculatedColumnFormula array="1">SUMPRODUCT(
     ((Shop_Consumables[Stock_Level]="Counted") * (ISNUMBER(Shop_Consumables[Stock_Count])) * (Shop_Consumables[Stock_Count]&lt;=Shop_Consumables[Reorder Point])) +
     ((ISNUMBER(MATCH(Shop_Consumables[Stock_Level], {"Few","None"}, 0))))
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="103">
+    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="99">
       <calculatedColumnFormula>SUMIFS(Shop_Overhead[Amount], Shop_Overhead[Due Date], "&lt;="&amp;TODAY()+30, Shop_Overhead[Due Date], "&gt;="&amp;TODAY())</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{E4065760-B1B1-4564-936B-3405D3B80297}" name="Equipment With Operational Issues" dataDxfId="102">
+    <tableColumn id="12" xr3:uid="{E4065760-B1B1-4564-936B-3405D3B80297}" name="Equipment With Operational Issues" dataDxfId="98">
       <calculatedColumnFormula array="1">SUM(
   COUNTIFS(Shop_Machinery[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"}),
   COUNTIFS(Shop_Power_Tools[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"}),
@@ -1198,8 +1189,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{F579DA07-7AD6-49DA-9B44-D5B1132EDAC6}" name="Overhead_Summary" displayName="Overhead_Summary" ref="A9:B21" totalsRowShown="0">
   <autoFilter ref="A9:B21" xr:uid="{F579DA07-7AD6-49DA-9B44-D5B1132EDAC6}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{7CA4839C-9603-479D-BD1C-8377DFA9603C}" name="Expense Category" dataDxfId="101"/>
-    <tableColumn id="2" xr3:uid="{FE0F7616-EAF3-443D-AC69-DE6541DC10E5}" name="Annual Total" dataDxfId="100">
+    <tableColumn id="1" xr3:uid="{7CA4839C-9603-479D-BD1C-8377DFA9603C}" name="Expense Category" dataDxfId="97"/>
+    <tableColumn id="2" xr3:uid="{FE0F7616-EAF3-443D-AC69-DE6541DC10E5}" name="Annual Total" dataDxfId="96">
       <calculatedColumnFormula>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1208,109 +1199,109 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:P2" totalsRowShown="0" headerRowDxfId="99" dataDxfId="98">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:P2" totalsRowShown="0" headerRowDxfId="95" dataDxfId="94">
   <autoFilter ref="A1:P2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}"/>
   <tableColumns count="16">
-    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="97"/>
-    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="96"/>
-    <tableColumn id="15" xr3:uid="{D25A390C-69B5-4326-A0D4-10EB45DDE5E5}" name="Tag_ID" dataDxfId="95"/>
-    <tableColumn id="16" xr3:uid="{57D16231-357C-4C08-B062-20555121C2D6}" name="Tag_Type" dataDxfId="5"/>
-    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="94"/>
-    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item Name" dataDxfId="93"/>
-    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="92"/>
-    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="91"/>
-    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="90"/>
-    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="89"/>
-    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="88">
+    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="93"/>
+    <tableColumn id="2" xr3:uid="{FE11B924-8CA4-4FDB-B876-A0F46F356DAB}" name="Asset ID" dataDxfId="92"/>
+    <tableColumn id="15" xr3:uid="{D25A390C-69B5-4326-A0D4-10EB45DDE5E5}" name="Tag_ID" dataDxfId="91"/>
+    <tableColumn id="16" xr3:uid="{57D16231-357C-4C08-B062-20555121C2D6}" name="Tag_Type" dataDxfId="90"/>
+    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="89"/>
+    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item_Description" dataDxfId="88"/>
+    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="87"/>
+    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="86"/>
+    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="85"/>
+    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="84"/>
+    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="83">
       <calculatedColumnFormula>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="87"/>
-    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="86"/>
-    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="85"/>
-    <tableColumn id="13" xr3:uid="{71578D4D-1C79-4D4F-9C0F-A2C991F460FD}" name="Date Sold" dataDxfId="84"/>
-    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="83"/>
+    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="82"/>
+    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="81"/>
+    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="80"/>
+    <tableColumn id="13" xr3:uid="{71578D4D-1C79-4D4F-9C0F-A2C991F460FD}" name="Date Sold" dataDxfId="79"/>
+    <tableColumn id="14" xr3:uid="{BD7B1CE6-805E-44CC-9E90-B0E0159F46F5}" name="Location" dataDxfId="78"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="82" dataDxfId="81">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:K2" insertRow="1" totalsRowShown="0" headerRowDxfId="77" dataDxfId="76">
   <autoFilter ref="A1:K2" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="80"/>
-    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="79"/>
-    <tableColumn id="4" xr3:uid="{17EB0B09-11B3-4E08-9442-E3C9AB87A157}" name="Tag_ID" dataDxfId="78"/>
-    <tableColumn id="5" xr3:uid="{72EAA357-95AA-4893-8038-2A77BDD0FB87}" name="Tag_Type" dataDxfId="4"/>
-    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="77"/>
-    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Machine Name/Brand/Model" dataDxfId="76"/>
-    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="75"/>
-    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="74"/>
-    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="73"/>
-    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="72"/>
-    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Serial Number/Other Info" dataDxfId="71"/>
+    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="75"/>
+    <tableColumn id="2" xr3:uid="{D22F095D-654C-42BE-A88E-204282C3AC59}" name="Asset ID" dataDxfId="74"/>
+    <tableColumn id="4" xr3:uid="{17EB0B09-11B3-4E08-9442-E3C9AB87A157}" name="Tag_ID" dataDxfId="73"/>
+    <tableColumn id="5" xr3:uid="{72EAA357-95AA-4893-8038-2A77BDD0FB87}" name="Tag_Type" dataDxfId="72"/>
+    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="71"/>
+    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Item_Description" dataDxfId="70"/>
+    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="69"/>
+    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="68"/>
+    <tableColumn id="8" xr3:uid="{F332B8F1-9F04-43B0-BD71-656F6F526EC5}" name="Location" dataDxfId="67"/>
+    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="66"/>
+    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Serial Number/Other Info" dataDxfId="65"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:K2" totalsRowShown="0" headerRowDxfId="70" dataDxfId="69">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:K2" totalsRowShown="0" headerRowDxfId="64" dataDxfId="63">
   <autoFilter ref="A1:K2" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="68"/>
-    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="67"/>
-    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="66"/>
-    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="65"/>
-    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="64"/>
-    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="63"/>
-    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="62"/>
-    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="61"/>
-    <tableColumn id="11" xr3:uid="{4809319D-ABCA-43DA-A400-5DC91167D78B}" name="Complete" dataDxfId="60"/>
-    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Completion Date" dataDxfId="59"/>
-    <tableColumn id="12" xr3:uid="{920CB592-D743-4B33-A796-C7F3DB32211C}" name="Remarks" dataDxfId="58"/>
+    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="62"/>
+    <tableColumn id="2" xr3:uid="{E9B83024-3108-49FE-BABC-CFF148D740E1}" name="Log ID" dataDxfId="61"/>
+    <tableColumn id="3" xr3:uid="{3475773D-2245-4156-9F88-ED7AE0C20402}" name="Asset ID" dataDxfId="60"/>
+    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="59"/>
+    <tableColumn id="5" xr3:uid="{96FAFE7C-F67A-4F71-AD8A-97B41A62C852}" name="Service Type" dataDxfId="58"/>
+    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="57"/>
+    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="56"/>
+    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Next Service Date" dataDxfId="55"/>
+    <tableColumn id="11" xr3:uid="{4809319D-ABCA-43DA-A400-5DC91167D78B}" name="Complete" dataDxfId="54"/>
+    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Completion Date" dataDxfId="53"/>
+    <tableColumn id="12" xr3:uid="{920CB592-D743-4B33-A796-C7F3DB32211C}" name="Remarks" dataDxfId="52"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:L2" totalsRowShown="0" headerRowDxfId="134" dataDxfId="133">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:L2" totalsRowShown="0" headerRowDxfId="51" dataDxfId="50">
   <autoFilter ref="A1:L2" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="132"/>
-    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="131"/>
-    <tableColumn id="11" xr3:uid="{21951C81-00A4-4344-9E81-B1B1DB06ADEF}" name="Tag_ID" dataDxfId="130"/>
-    <tableColumn id="12" xr3:uid="{7F1AFB3A-34F9-4E3E-A9D3-7E7E1458ECFE}" name="Tag_Type" dataDxfId="3"/>
-    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="129"/>
-    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Tool Name/Brand/Model" dataDxfId="128"/>
-    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="127"/>
-    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="126"/>
-    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="125"/>
-    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="124"/>
-    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="123"/>
-    <tableColumn id="10" xr3:uid="{26197E01-2936-4F5F-8081-3AA351C1CD38}" name="Remarks" dataDxfId="122"/>
+    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="49"/>
+    <tableColumn id="2" xr3:uid="{169523C9-3198-448C-A108-CBA0222ED119}" name="Asset_ID" dataDxfId="48"/>
+    <tableColumn id="11" xr3:uid="{21951C81-00A4-4344-9E81-B1B1DB06ADEF}" name="Tag_ID" dataDxfId="47"/>
+    <tableColumn id="12" xr3:uid="{7F1AFB3A-34F9-4E3E-A9D3-7E7E1458ECFE}" name="Tag_Type" dataDxfId="46"/>
+    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="45"/>
+    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Item_Description" dataDxfId="44"/>
+    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="43"/>
+    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="42"/>
+    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="41"/>
+    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="40"/>
+    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="39"/>
+    <tableColumn id="10" xr3:uid="{26197E01-2936-4F5F-8081-3AA351C1CD38}" name="Remarks" dataDxfId="38"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:L2" totalsRowShown="0" headerRowDxfId="57" dataDxfId="56">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:L2" totalsRowShown="0" headerRowDxfId="37" dataDxfId="36">
   <autoFilter ref="A1:L2" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="55"/>
-    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="54"/>
-    <tableColumn id="10" xr3:uid="{C8BD69AA-9023-4777-9C96-39A81F1E4BE0}" name="Tag_ID" dataDxfId="53"/>
-    <tableColumn id="12" xr3:uid="{FC4D7CE3-2DF1-465E-A4D1-1D1F02F8B8CA}" name="Tag_Type" dataDxfId="1"/>
-    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Tool Name/Brand/Model/Description" dataDxfId="52"/>
-    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="51"/>
-    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="50"/>
-    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="49"/>
-    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Stock_Level" dataDxfId="48"/>
-    <tableColumn id="11" xr3:uid="{FD8D2D17-0451-45E0-8688-0BB4F60073DA}" name="Stock_Count" dataDxfId="47"/>
-    <tableColumn id="9" xr3:uid="{2B57F5E6-66C5-4DBA-8949-836DE0F0791C}" name="Remarks" dataDxfId="46"/>
+    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="35"/>
+    <tableColumn id="2" xr3:uid="{679266D2-6F7C-4AA6-A692-6DC107A45D4D}" name="Asset_ID" dataDxfId="34"/>
+    <tableColumn id="10" xr3:uid="{C8BD69AA-9023-4777-9C96-39A81F1E4BE0}" name="Tag_ID" dataDxfId="33"/>
+    <tableColumn id="12" xr3:uid="{FC4D7CE3-2DF1-465E-A4D1-1D1F02F8B8CA}" name="Tag_Type" dataDxfId="32"/>
+    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="31"/>
+    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Item_Description" dataDxfId="30"/>
+    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="29"/>
+    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="28"/>
+    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="27"/>
+    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Stock_Level" dataDxfId="26"/>
+    <tableColumn id="11" xr3:uid="{FD8D2D17-0451-45E0-8688-0BB4F60073DA}" name="Stock_Count" dataDxfId="25"/>
+    <tableColumn id="9" xr3:uid="{2B57F5E6-66C5-4DBA-8949-836DE0F0791C}" name="Remarks" dataDxfId="24"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1649,24 +1640,24 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="D1" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" t="s">
         <v>34</v>
-      </c>
-      <c r="F1" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="B2" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C2" s="8">
         <v>3</v>
@@ -1679,12 +1670,12 @@
         <v>300</v>
       </c>
       <c r="F2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="B3" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C3" s="8">
         <v>4</v>
@@ -1697,12 +1688,12 @@
         <v>40</v>
       </c>
       <c r="F3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="B4" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C4" s="8">
         <v>5</v>
@@ -1715,12 +1706,12 @@
         <v>100</v>
       </c>
       <c r="F4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="B5" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C5" s="8">
         <v>1000</v>
@@ -1776,46 +1767,46 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F1" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="G1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="4" t="s">
-        <v>3</v>
-      </c>
       <c r="H1" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="I1" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="K1" t="s">
+        <v>91</v>
+      </c>
+      <c r="L1" t="s">
+        <v>92</v>
+      </c>
+      <c r="M1" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="J1" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="K1" t="s">
-        <v>95</v>
-      </c>
-      <c r="L1" t="s">
-        <v>96</v>
-      </c>
-      <c r="M1" s="8" t="s">
-        <v>21</v>
-      </c>
       <c r="N1" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="O1" s="4" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="P1" s="6"/>
       <c r="Q1" s="6"/>
@@ -1887,25 +1878,25 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="F1" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="G1" s="4" t="s">
-        <v>28</v>
-      </c>
       <c r="H1" s="4" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="I1" s="6"/>
     </row>
@@ -1955,22 +1946,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="G1" s="4" t="s">
         <v>46</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -1998,33 +1989,33 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D1" t="s">
         <v>52</v>
       </c>
-      <c r="C1" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>53</v>
-      </c>
-      <c r="E1" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="1" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B2" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="D2" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="E2" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
     </row>
   </sheetData>
@@ -2046,10 +2037,10 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>36</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -2096,37 +2087,37 @@
         <v>0</v>
       </c>
       <c r="B1" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="D1" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="H1" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="D1" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="F1" s="5" t="s">
+      <c r="I1" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="J1" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="G1" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="I1" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>66</v>
-      </c>
       <c r="K1" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="L1" s="8" t="s">
         <v>80</v>
-      </c>
-      <c r="L1" s="8" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:12">
@@ -2203,15 +2194,15 @@
   <sheetData>
     <row r="9" spans="1:2">
       <c r="A9" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B10" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2220,7 +2211,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B11" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2229,7 +2220,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B12" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2238,7 +2229,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B13" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2247,7 +2238,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B14" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2256,7 +2247,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B15" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2265,7 +2256,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B16" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2274,7 +2265,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B17" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2283,7 +2274,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B18" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2292,7 +2283,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B19" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2301,7 +2292,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B20" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2310,7 +2301,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B21" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -2365,46 +2356,46 @@
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F1" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="G1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="H1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="I1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="L1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="M1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="O1" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="P1" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="O1" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>11</v>
       </c>
       <c r="Q1" s="6"/>
       <c r="S1" s="6"/>
@@ -2465,31 +2456,31 @@
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>82</v>
+        <v>97</v>
       </c>
       <c r="G1" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="H1" s="5" t="s">
-        <v>13</v>
-      </c>
       <c r="I1" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="L1" s="6"/>
     </row>
@@ -2541,34 +2532,34 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" t="s">
         <v>15</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H1" s="9" t="s">
-        <v>18</v>
-      </c>
       <c r="I1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="J1" s="9" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="L1" s="6"/>
       <c r="M1" s="6"/>
@@ -2630,37 +2621,37 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>85</v>
+        <v>97</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H1" t="s">
+        <v>47</v>
+      </c>
+      <c r="I1" t="s">
         <v>48</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>49</v>
       </c>
-      <c r="J1" t="s">
-        <v>50</v>
-      </c>
       <c r="K1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="N1" s="6"/>
     </row>
@@ -2725,37 +2716,37 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>86</v>
+        <v>97</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J1" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="K1" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="M1" s="6"/>
       <c r="N1" s="6"/>

</xml_diff>

<commit_message>
Added column: "Item_Category" to inventory tables in config.js and excel master
</commit_message>
<xml_diff>
--- a/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
+++ b/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1a2ae81d67634e6/Desktop/Michanikos Artifex Enterprises/MAE Custom Digital Solutions/MAE Workshop Inventory Management System/GITHUB_MAE_Workshop Inventory App/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="300" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F74CF298-3CFE-4507-B918-683E14AF512C}"/>
+  <xr:revisionPtr revIDLastSave="320" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8452EC8A-D701-49FA-9D0C-57212878EA28}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
+    <workbookView xWindow="2472" yWindow="1152" windowWidth="17676" windowHeight="11172" firstSheet="2" activeTab="3" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
   </bookViews>
   <sheets>
     <sheet name="Master Dashboard" sheetId="1" r:id="rId1"/>
@@ -71,7 +71,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="76">
   <si>
     <t>mae_id</t>
   </si>
@@ -296,6 +296,9 @@
   </si>
   <si>
     <t>Scheduled Service Date</t>
+  </si>
+  <si>
+    <t>Item_Category</t>
   </si>
 </sst>
 </file>
@@ -351,7 +354,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
       <protection hidden="1"/>
@@ -385,16 +388,54 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="116">
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
+  <dxfs count="121">
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -402,33 +443,9 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -452,162 +469,6 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -675,13 +536,169 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
       <protection locked="0" hidden="0"/>
     </dxf>
@@ -710,6 +727,78 @@
     </dxf>
     <dxf>
       <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
+    </dxf>
+    <dxf>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <protection locked="1" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="1" hidden="1"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
@@ -780,68 +869,6 @@
     <dxf>
       <protection locked="1" hidden="0"/>
     </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="1" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <protection locked="1" hidden="1"/>
-    </dxf>
-    <dxf>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <protection locked="1" hidden="0"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -877,41 +904,41 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:L2" totalsRowShown="0" headerRowDxfId="99" dataDxfId="98">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}" name="Master_Dashboard" displayName="Master_Dashboard" ref="A1:L2" totalsRowShown="0" headerRowDxfId="120" dataDxfId="119">
   <autoFilter ref="A1:L2" xr:uid="{E23AAC9B-2490-4897-B1B0-35BCA496B1EC}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="97"/>
-    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="96">
+    <tableColumn id="1" xr3:uid="{0FA08005-3EA3-40A4-B1F6-F97329C0333E}" name="mae_id" dataDxfId="118"/>
+    <tableColumn id="2" xr3:uid="{9DC14395-3E47-4AD3-9478-A0A87F06E532}" name="Total Resell Investment" dataDxfId="117">
       <calculatedColumnFormula>SUM(Resell_Inventory[Total Investment])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="95">
+    <tableColumn id="3" xr3:uid="{BD093FBC-8AA5-4D1C-881C-2928F91ADF2E}" name="Total Actual Sales" dataDxfId="116">
       <calculatedColumnFormula>SUM(Resell_Inventory[Actual Sale Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="94">
+    <tableColumn id="8" xr3:uid="{8127FC92-B011-41A5-B229-AFBAD48CACAA}" name="Total Machinery Value" dataDxfId="115">
       <calculatedColumnFormula>SUM(Shop_Machinery[Purchase Cost])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="93">
+    <tableColumn id="9" xr3:uid="{A91267CC-638B-4A12-B7C7-5F4BB2369A54}" name="Total Power Tool Value" dataDxfId="114">
       <calculatedColumnFormula>SUM(Shop_Power_Tools[Purchase Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="92">
+    <tableColumn id="10" xr3:uid="{74988749-A386-4C80-9863-6BDF471B0985}" name="Total Hand Tool Value" dataDxfId="113">
       <calculatedColumnFormula>SUM(Shop_Hand_Tools[Purchase Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="91">
+    <tableColumn id="11" xr3:uid="{45ADA20D-C061-46B8-BB93-1E9FFDB98DBC}" name="Total Consumables Value" dataDxfId="112">
       <calculatedColumnFormula>SUM(Shop_Consumables[Current Inventory Value])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="90">
+    <tableColumn id="4" xr3:uid="{FF13FE4A-758B-454A-B440-546DF0DC594D}" name="Total Shop Asset Value" dataDxfId="111">
       <calculatedColumnFormula>SUM(D2,E2,F2,G2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="89">
+    <tableColumn id="5" xr3:uid="{7A74BF46-8BED-4B91-99D0-B278CC6F7AEC}" name="Low Stock Items Count" dataDxfId="110">
       <calculatedColumnFormula array="1">SUMPRODUCT(
     ((Shop_Consumables[Stock_Level]="Counted") * (ISNUMBER(Shop_Consumables[Stock_Count])) * (Shop_Consumables[Stock_Count]&lt;=Shop_Consumables[Reorder Point])) +
     ((ISNUMBER(MATCH(Shop_Consumables[Stock_Level], {"Few","None"}, 0))))
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="88">
+    <tableColumn id="7" xr3:uid="{F48C34D4-1ECB-427E-9CA9-378ABA1B3979}" name="Total Amount Due Next 30 Days" dataDxfId="109">
       <calculatedColumnFormula>SUMIFS(Shop_Overhead[Amount], Shop_Overhead[Due Date], "&lt;="&amp;TODAY()+30, Shop_Overhead[Due Date], "&gt;="&amp;TODAY())</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{E4065760-B1B1-4564-936B-3405D3B80297}" name="Equipment With Operational Issues" dataDxfId="87">
+    <tableColumn id="12" xr3:uid="{E4065760-B1B1-4564-936B-3405D3B80297}" name="Equipment With Operational Issues" dataDxfId="108">
       <calculatedColumnFormula array="1">SUM(
   COUNTIFS(Shop_Machinery[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"}),
   COUNTIFS(Shop_Power_Tools[Condition], {"Needs Repair","Repair In-Progress","Unusable/Junk"}),
@@ -927,33 +954,33 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:H2" totalsRowShown="0" headerRowDxfId="21" dataDxfId="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:H2" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
   <autoFilter ref="A1:H2" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="19"/>
-    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="18"/>
-    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="17"/>
-    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="16"/>
-    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="15"/>
-    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="14"/>
-    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="13"/>
-    <tableColumn id="8" xr3:uid="{9140C4E8-CB9E-40BF-ABD9-13A971322B09}" name="Remarks" dataDxfId="12"/>
+    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="20"/>
+    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="19"/>
+    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="18"/>
+    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="17"/>
+    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="16"/>
+    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="15"/>
+    <tableColumn id="8" xr3:uid="{9140C4E8-CB9E-40BF-ABD9-13A971322B09}" name="Remarks" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
   <autoFilter ref="A1:G2" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="9"/>
-    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="7"/>
-    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="6"/>
-    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="5"/>
-    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="4"/>
-    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="11"/>
+    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="9"/>
+    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="7"/>
+    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="6"/>
+    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -963,8 +990,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{F579DA07-7AD6-49DA-9B44-D5B1132EDAC6}" name="Overhead_Summary" displayName="Overhead_Summary" ref="A9:B21" totalsRowShown="0">
   <autoFilter ref="A9:B21" xr:uid="{F579DA07-7AD6-49DA-9B44-D5B1132EDAC6}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{7CA4839C-9603-479D-BD1C-8377DFA9603C}" name="Expense Category" dataDxfId="86"/>
-    <tableColumn id="2" xr3:uid="{FE0F7616-EAF3-443D-AC69-DE6541DC10E5}" name="Annual Total" dataDxfId="85">
+    <tableColumn id="1" xr3:uid="{7CA4839C-9603-479D-BD1C-8377DFA9603C}" name="Expense Category" dataDxfId="107"/>
+    <tableColumn id="2" xr3:uid="{FE0F7616-EAF3-443D-AC69-DE6541DC10E5}" name="Annual Total" dataDxfId="106">
       <calculatedColumnFormula>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -976,114 +1003,119 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}" name="Location" displayName="Location" ref="A1:C2" totalsRowShown="0">
   <autoFilter ref="A1:C2" xr:uid="{2ADC87F2-BD10-435C-9D45-DD8DB7DB1902}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Description" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{D3C21C14-3B5F-4EBE-B777-F96EFD0A6C91}" name="mae_id" dataDxfId="105"/>
+    <tableColumn id="2" xr3:uid="{7E953E1D-BE2C-4F7F-AAE5-06F3EDBC1067}" name="Location_ID" dataDxfId="104"/>
+    <tableColumn id="3" xr3:uid="{60368768-3E0A-4CA0-8B3A-F230D9D220C2}" name="Description" dataDxfId="103"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:N2" totalsRowShown="0" headerRowDxfId="115" dataDxfId="114">
-  <autoFilter ref="A1:N2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}"/>
-  <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="113"/>
-    <tableColumn id="15" xr3:uid="{D25A390C-69B5-4326-A0D4-10EB45DDE5E5}" name="Tag_ID" dataDxfId="112"/>
-    <tableColumn id="16" xr3:uid="{57D16231-357C-4C08-B062-20555121C2D6}" name="Tag_Type" dataDxfId="111"/>
-    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="110"/>
-    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item_Description" dataDxfId="109"/>
-    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="108"/>
-    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="107"/>
-    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="106"/>
-    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="105"/>
-    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="104">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}" name="Resell_Inventory" displayName="Resell_Inventory" ref="A1:O2" totalsRowShown="0" headerRowDxfId="102" dataDxfId="101">
+  <autoFilter ref="A1:O2" xr:uid="{C0DAC3A4-C29F-4046-9A11-9992CD804FC2}"/>
+  <tableColumns count="15">
+    <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="100"/>
+    <tableColumn id="15" xr3:uid="{D25A390C-69B5-4326-A0D4-10EB45DDE5E5}" name="Tag_ID" dataDxfId="99"/>
+    <tableColumn id="16" xr3:uid="{57D16231-357C-4C08-B062-20555121C2D6}" name="Tag_Type" dataDxfId="98"/>
+    <tableColumn id="2" xr3:uid="{0EA7C626-291A-4D56-A19A-BC3E098C0307}" name="Item_Category" dataDxfId="4"/>
+    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="97"/>
+    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item_Description" dataDxfId="96"/>
+    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="95"/>
+    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="94"/>
+    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="93"/>
+    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="92"/>
+    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="91">
       <calculatedColumnFormula>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="103"/>
-    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="102"/>
-    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="101"/>
-    <tableColumn id="13" xr3:uid="{71578D4D-1C79-4D4F-9C0F-A2C991F460FD}" name="Date Sold" dataDxfId="100"/>
+    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="90"/>
+    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="89"/>
+    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="88"/>
+    <tableColumn id="13" xr3:uid="{71578D4D-1C79-4D4F-9C0F-A2C991F460FD}" name="Date Sold" dataDxfId="87"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:I2" insertRow="1" totalsRowShown="0" headerRowDxfId="84" dataDxfId="83">
-  <autoFilter ref="A1:I2" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}"/>
-  <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="82"/>
-    <tableColumn id="4" xr3:uid="{17EB0B09-11B3-4E08-9442-E3C9AB87A157}" name="Tag_ID" dataDxfId="81"/>
-    <tableColumn id="5" xr3:uid="{72EAA357-95AA-4893-8038-2A77BDD0FB87}" name="Tag_Type" dataDxfId="80"/>
-    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="79"/>
-    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Item_Description" dataDxfId="78"/>
-    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="77"/>
-    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="76"/>
-    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="75"/>
-    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Serial Number/Other Info" dataDxfId="74"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:J2" insertRow="1" totalsRowShown="0" headerRowDxfId="86" dataDxfId="85">
+  <autoFilter ref="A1:J2" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}"/>
+  <tableColumns count="10">
+    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="84"/>
+    <tableColumn id="4" xr3:uid="{17EB0B09-11B3-4E08-9442-E3C9AB87A157}" name="Tag_ID" dataDxfId="83"/>
+    <tableColumn id="5" xr3:uid="{72EAA357-95AA-4893-8038-2A77BDD0FB87}" name="Tag_Type" dataDxfId="82"/>
+    <tableColumn id="2" xr3:uid="{5F0AA36F-B9A6-466C-A044-4398E5CAD0BF}" name="Item_Category" dataDxfId="3"/>
+    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="81"/>
+    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Item_Description" dataDxfId="80"/>
+    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="79"/>
+    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="78"/>
+    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="77"/>
+    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Serial Number/Other Info" dataDxfId="76"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:K2" totalsRowShown="0" headerRowDxfId="63" dataDxfId="62">
-  <autoFilter ref="A1:K2" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}"/>
-  <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="61"/>
-    <tableColumn id="11" xr3:uid="{21951C81-00A4-4344-9E81-B1B1DB06ADEF}" name="Tag_ID" dataDxfId="60"/>
-    <tableColumn id="12" xr3:uid="{7F1AFB3A-34F9-4E3E-A9D3-7E7E1458ECFE}" name="Tag_Type" dataDxfId="59"/>
-    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="58"/>
-    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Item_Description" dataDxfId="57"/>
-    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="56"/>
-    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="55"/>
-    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="54"/>
-    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="53"/>
-    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="52"/>
-    <tableColumn id="10" xr3:uid="{26197E01-2936-4F5F-8081-3AA351C1CD38}" name="Remarks" dataDxfId="51"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:L2" totalsRowShown="0" headerRowDxfId="75" dataDxfId="74">
+  <autoFilter ref="A1:L2" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}"/>
+  <tableColumns count="12">
+    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="73"/>
+    <tableColumn id="11" xr3:uid="{21951C81-00A4-4344-9E81-B1B1DB06ADEF}" name="Tag_ID" dataDxfId="72"/>
+    <tableColumn id="12" xr3:uid="{7F1AFB3A-34F9-4E3E-A9D3-7E7E1458ECFE}" name="Tag_Type" dataDxfId="71"/>
+    <tableColumn id="2" xr3:uid="{176E61E7-BE6B-42DA-B1B1-AECC0921E70C}" name="Item_Category" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="70"/>
+    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Item_Description" dataDxfId="69"/>
+    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="68"/>
+    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="67"/>
+    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="66"/>
+    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="65"/>
+    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="64"/>
+    <tableColumn id="10" xr3:uid="{26197E01-2936-4F5F-8081-3AA351C1CD38}" name="Remarks" dataDxfId="63"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:K2" totalsRowShown="0" headerRowDxfId="50" dataDxfId="49">
-  <autoFilter ref="A1:K2" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}"/>
-  <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="48"/>
-    <tableColumn id="10" xr3:uid="{C8BD69AA-9023-4777-9C96-39A81F1E4BE0}" name="Tag_ID" dataDxfId="47"/>
-    <tableColumn id="12" xr3:uid="{FC4D7CE3-2DF1-465E-A4D1-1D1F02F8B8CA}" name="Tag_Type" dataDxfId="46"/>
-    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="45"/>
-    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Item_Description" dataDxfId="44"/>
-    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="43"/>
-    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="42"/>
-    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="41"/>
-    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Stock_Level" dataDxfId="40"/>
-    <tableColumn id="11" xr3:uid="{FD8D2D17-0451-45E0-8688-0BB4F60073DA}" name="Stock_Count" dataDxfId="39"/>
-    <tableColumn id="9" xr3:uid="{2B57F5E6-66C5-4DBA-8949-836DE0F0791C}" name="Remarks" dataDxfId="38"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:L2" totalsRowShown="0" headerRowDxfId="62" dataDxfId="61">
+  <autoFilter ref="A1:L2" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}"/>
+  <tableColumns count="12">
+    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="60"/>
+    <tableColumn id="10" xr3:uid="{C8BD69AA-9023-4777-9C96-39A81F1E4BE0}" name="Tag_ID" dataDxfId="59"/>
+    <tableColumn id="12" xr3:uid="{FC4D7CE3-2DF1-465E-A4D1-1D1F02F8B8CA}" name="Tag_Type" dataDxfId="58"/>
+    <tableColumn id="2" xr3:uid="{54155A52-92C4-4BB0-A374-70E75592F98A}" name="Item_Category" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="57"/>
+    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Item_Description" dataDxfId="56"/>
+    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="55"/>
+    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="54"/>
+    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="53"/>
+    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Stock_Level" dataDxfId="52"/>
+    <tableColumn id="11" xr3:uid="{FD8D2D17-0451-45E0-8688-0BB4F60073DA}" name="Stock_Count" dataDxfId="51"/>
+    <tableColumn id="9" xr3:uid="{2B57F5E6-66C5-4DBA-8949-836DE0F0791C}" name="Remarks" dataDxfId="50"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:N2" totalsRowShown="0" headerRowDxfId="37" dataDxfId="36">
-  <autoFilter ref="A1:N2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
-  <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="35"/>
-    <tableColumn id="12" xr3:uid="{8F0FD29C-682B-41B4-82F2-913D40801887}" name="Tag_ID" dataDxfId="34"/>
-    <tableColumn id="15" xr3:uid="{CE0ECF5F-5626-4215-AC71-301755B31D23}" name="Tag_Type" dataDxfId="33"/>
-    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="32"/>
-    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item_Description" dataDxfId="31"/>
-    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="30"/>
-    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Stock_Level" dataDxfId="29"/>
-    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="28"/>
-    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="27"/>
-    <tableColumn id="13" xr3:uid="{AA55BCE3-9AC1-4735-8622-15E62CA93E1A}" name="Stock_Count" dataDxfId="26"/>
-    <tableColumn id="14" xr3:uid="{FA5C79D4-6D25-4E4C-BE9F-4190C63530C2}" name="Bulk_Value" dataDxfId="25"/>
-    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="24"/>
-    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="23">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:O2" totalsRowShown="0" headerRowDxfId="49" dataDxfId="48">
+  <autoFilter ref="A1:O2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
+  <tableColumns count="15">
+    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="47"/>
+    <tableColumn id="12" xr3:uid="{8F0FD29C-682B-41B4-82F2-913D40801887}" name="Tag_ID" dataDxfId="46"/>
+    <tableColumn id="15" xr3:uid="{CE0ECF5F-5626-4215-AC71-301755B31D23}" name="Tag_Type" dataDxfId="45"/>
+    <tableColumn id="3" xr3:uid="{F28BB55E-442A-44A7-9EBB-E9F69B0BE27A}" name="Item_Category" dataDxfId="0"/>
+    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="44"/>
+    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item_Description" dataDxfId="43"/>
+    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="42"/>
+    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Stock_Level" dataDxfId="41"/>
+    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="40"/>
+    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="39"/>
+    <tableColumn id="13" xr3:uid="{AA55BCE3-9AC1-4735-8622-15E62CA93E1A}" name="Stock_Count" dataDxfId="38"/>
+    <tableColumn id="14" xr3:uid="{FA5C79D4-6D25-4E4C-BE9F-4190C63530C2}" name="Bulk_Value" dataDxfId="37"/>
+    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="36"/>
+    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="35">
       <calculatedColumnFormula array="1">IF(
     Shop_Consumables[[#This Row],[Stock_Level]]="Counted",
     Shop_Consumables[[#This Row],[Stock_Count]] * Shop_Consumables[[#This Row],[Unit Cost]],
@@ -1099,24 +1131,24 @@
     )
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Supplier/Remarks" dataDxfId="22"/>
+    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Supplier/Remarks" dataDxfId="34"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:H2" totalsRowShown="0" headerRowDxfId="73" dataDxfId="72">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:H2" totalsRowShown="0" headerRowDxfId="33" dataDxfId="32">
   <autoFilter ref="A1:H2" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="71"/>
-    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="70"/>
-    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="69"/>
-    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="68"/>
-    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Scheduled Service Date" dataDxfId="67"/>
-    <tableColumn id="11" xr3:uid="{4809319D-ABCA-43DA-A400-5DC91167D78B}" name="Complete" dataDxfId="66"/>
-    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Completion Date" dataDxfId="65"/>
-    <tableColumn id="12" xr3:uid="{920CB592-D743-4B33-A796-C7F3DB32211C}" name="Remarks" dataDxfId="64"/>
+    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="31"/>
+    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="30"/>
+    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="29"/>
+    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="28"/>
+    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Scheduled Service Date" dataDxfId="27"/>
+    <tableColumn id="11" xr3:uid="{4809319D-ABCA-43DA-A400-5DC91167D78B}" name="Complete" dataDxfId="26"/>
+    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Completion Date" dataDxfId="25"/>
+    <tableColumn id="12" xr3:uid="{920CB592-D743-4B33-A796-C7F3DB32211C}" name="Remarks" dataDxfId="24"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1856,29 +1888,30 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDE7BF89-A2E7-4A6F-B822-317739E206EC}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:R2"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
     <col min="2" max="3" width="9.5546875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="31.44140625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="10.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17" style="10" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.33203125" style="3" customWidth="1"/>
-    <col min="9" max="9" width="16.5546875" style="3" customWidth="1"/>
-    <col min="10" max="10" width="16.6640625" style="5" customWidth="1"/>
-    <col min="11" max="11" width="19.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16.6640625" style="3" customWidth="1"/>
-    <col min="13" max="13" width="16.88671875" style="3" customWidth="1"/>
-    <col min="14" max="14" width="16.88671875" style="10" customWidth="1"/>
-    <col min="15" max="15" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="16.88671875" style="6" customWidth="1"/>
-    <col min="17" max="17" width="16.88671875" style="2" customWidth="1"/>
-    <col min="18" max="16384" width="8.88671875" style="6"/>
+    <col min="4" max="4" width="15.33203125" style="16" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="31.44140625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="10.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17" style="10" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.33203125" style="3" customWidth="1"/>
+    <col min="10" max="10" width="16.5546875" style="3" customWidth="1"/>
+    <col min="11" max="11" width="16.6640625" style="5" customWidth="1"/>
+    <col min="12" max="12" width="19.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.6640625" style="3" customWidth="1"/>
+    <col min="14" max="14" width="16.88671875" style="3" customWidth="1"/>
+    <col min="15" max="15" width="16.88671875" style="10" customWidth="1"/>
+    <col min="16" max="16" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.88671875" style="6" customWidth="1"/>
+    <col min="18" max="18" width="16.88671875" style="2" customWidth="1"/>
+    <col min="19" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17">
+    <row r="1" spans="1:18">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1888,60 +1921,63 @@
       <c r="C1" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="E1" t="s">
         <v>33</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="H1" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="L1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="M1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="N1" s="9" t="s">
+      <c r="O1" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="O1" s="6"/>
-      <c r="Q1" s="6"/>
-    </row>
-    <row r="2" spans="1:17">
-      <c r="D2" s="6"/>
-      <c r="J2" s="5">
+      <c r="P1" s="6"/>
+      <c r="R1" s="6"/>
+    </row>
+    <row r="2" spans="1:18">
+      <c r="E2" s="6"/>
+      <c r="K2" s="5">
         <f>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</f>
         <v>0</v>
       </c>
-      <c r="O2" s="6"/>
-      <c r="Q2" s="6"/>
+      <c r="P2" s="6"/>
+      <c r="R2" s="6"/>
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K3:K1000" xr:uid="{F45414DD-76C8-4DC4-96E2-15B89FDB5B51}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L3:L1000" xr:uid="{F45414DD-76C8-4DC4-96E2-15B89FDB5B51}">
       <formula1>"work not started, restoration in progress, for sale, sold"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2" xr:uid="{C1AA0387-29B3-4797-A152-88A8C024D825}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2" xr:uid="{C1AA0387-29B3-4797-A152-88A8C024D825}">
       <formula1>"Machinery, Furniture, Electronics, Craft, Auto Related, Other"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2" xr:uid="{3C9AD8AD-AB10-403F-A04B-87B1D7C9B98E}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L2" xr:uid="{3C9AD8AD-AB10-403F-A04B-87B1D7C9B98E}">
       <formula1>"Not Started, In-Progress, Complete, For Sale, Sold"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1956,22 +1992,23 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B027EC69-551F-4051-8A71-8B106D207C6D}">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
     <col min="2" max="3" width="9.5546875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="12.33203125" style="6" customWidth="1"/>
-    <col min="5" max="5" width="28.6640625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="14.6640625" style="10" customWidth="1"/>
-    <col min="7" max="7" width="14.6640625" style="3" customWidth="1"/>
-    <col min="8" max="8" width="12.88671875" customWidth="1"/>
-    <col min="9" max="9" width="40.88671875" style="6" customWidth="1"/>
-    <col min="10" max="10" width="32.6640625" style="2" customWidth="1"/>
-    <col min="11" max="16384" width="8.88671875" style="6"/>
+    <col min="4" max="4" width="15.33203125" style="16" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.33203125" style="6" customWidth="1"/>
+    <col min="6" max="6" width="28.6640625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="14.6640625" style="10" customWidth="1"/>
+    <col min="8" max="8" width="14.6640625" style="3" customWidth="1"/>
+    <col min="9" max="9" width="12.88671875" customWidth="1"/>
+    <col min="10" max="10" width="40.88671875" style="6" customWidth="1"/>
+    <col min="11" max="11" width="32.6640625" style="2" customWidth="1"/>
+    <col min="12" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:11">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1981,37 +2018,40 @@
       <c r="C1" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="E1" t="s">
         <v>33</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="G1" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>13</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="J1" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="J1" s="6"/>
-    </row>
-    <row r="2" spans="1:10">
-      <c r="H2" s="6"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="6"/>
+      <c r="K1" s="6"/>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="I2" s="6"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="6"/>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I3:I1000" xr:uid="{D25ACF8B-D3DC-4EFD-9C68-FC99372E0DCF}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J3:J1000" xr:uid="{D25ACF8B-D3DC-4EFD-9C68-FC99372E0DCF}">
       <formula1>"Operational, Needs Repair, Unusable"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2" xr:uid="{4B2064CB-79C2-427D-B2C2-7CE85187D094}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2" xr:uid="{4B2064CB-79C2-427D-B2C2-7CE85187D094}">
       <formula1>"Operational, Needs Repair, Repair In-Progress, Unusable/Junk"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2025,24 +2065,25 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEDDDAA7-75C3-4AA5-ABFD-D5FB4C627E4C}">
   <sheetPr codeName="Sheet5"/>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
     <col min="2" max="3" width="8.6640625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="12.88671875" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="50.44140625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="15.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.88671875" style="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.88671875" style="6" customWidth="1"/>
-    <col min="10" max="10" width="14.44140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.5546875" style="6" customWidth="1"/>
-    <col min="13" max="13" width="14.44140625" style="2" customWidth="1"/>
-    <col min="14" max="16384" width="8.88671875" style="6"/>
+    <col min="4" max="4" width="15.33203125" style="16" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.88671875" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="50.44140625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="15.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.88671875" style="6" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.88671875" style="6" customWidth="1"/>
+    <col min="11" max="11" width="14.44140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.5546875" style="6" customWidth="1"/>
+    <col min="14" max="14" width="14.44140625" style="2" customWidth="1"/>
+    <col min="15" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2052,56 +2093,59 @@
       <c r="C1" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="E1" t="s">
         <v>33</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>29</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>30</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>31</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>13</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="L1" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="M1" s="6"/>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="G2" s="6"/>
-      <c r="K2" s="2"/>
-      <c r="M2" s="6"/>
+      <c r="N1" s="6"/>
+    </row>
+    <row r="2" spans="1:14">
+      <c r="H2" s="6"/>
+      <c r="L2" s="2"/>
+      <c r="N2" s="6"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <dataValidations count="6">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M3:M1000 H3:J1000" xr:uid="{FF61F80C-5E23-45D6-B39D-7C5635258115}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N3:N1000 I3:K1000" xr:uid="{FF61F80C-5E23-45D6-B39D-7C5635258115}">
       <formula1>"Circular Saw, Drill, Sander, Grinder, Other"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L3:M1000" xr:uid="{DB752B4D-0E75-42D1-B907-2DBC5792F422}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M3:N1000" xr:uid="{DB752B4D-0E75-42D1-B907-2DBC5792F422}">
       <formula1>"New, Operational, Needs Repair, Broken"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2" xr:uid="{05EFC744-2B0C-453D-A1B6-F8391608434D}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2" xr:uid="{05EFC744-2B0C-453D-A1B6-F8391608434D}">
       <formula1>"Drilling, Cutting, Grinding, Sanding, Fastening, Shaping/Routing, Other"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2" xr:uid="{194EFB2B-690A-4D50-8AF6-E8ED45FE2FCA}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2" xr:uid="{194EFB2B-690A-4D50-8AF6-E8ED45FE2FCA}">
       <formula1>"Portable/Handheld, Stationary/Bench Top, Outdoor Power Equipment, "</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:K2" xr:uid="{980AB122-9104-490B-993D-4F2FEF3A4EE6}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2:L2" xr:uid="{980AB122-9104-490B-993D-4F2FEF3A4EE6}">
       <formula1>"Operational, Needs Repair, Repair In-Progress, Unusable/Junk"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2 K2" xr:uid="{47F6EF9A-B127-4EB7-A5E8-0075055489DC}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2 L2" xr:uid="{47F6EF9A-B127-4EB7-A5E8-0075055489DC}">
       <formula1>"Corded(A/C), Cordless/Battery, Pneumatic/Air, Fuel-Powered"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2115,25 +2159,26 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F39ADDA6-CD5F-4655-A9C0-9676DDAC362E}">
   <sheetPr codeName="Sheet6"/>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="8.6640625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="12.88671875" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="54.6640625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="15.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.5546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.6640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.33203125" style="7" customWidth="1"/>
-    <col min="14" max="14" width="12.88671875" style="2" customWidth="1"/>
-    <col min="15" max="16384" width="8.88671875" style="6"/>
+    <col min="4" max="4" width="15.33203125" style="16" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.88671875" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="54.6640625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="15.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.5546875" style="6" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.6640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="16.33203125" style="7" customWidth="1"/>
+    <col min="15" max="15" width="12.88671875" style="2" customWidth="1"/>
+    <col min="16" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2143,51 +2188,54 @@
       <c r="C1" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="E1" t="s">
         <v>33</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>1</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>13</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>66</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>67</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="L1" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="L1" s="6"/>
       <c r="M1" s="6"/>
       <c r="N1" s="6"/>
-    </row>
-    <row r="2" spans="1:14">
-      <c r="H2" s="6"/>
+      <c r="O1" s="6"/>
+    </row>
+    <row r="2" spans="1:15">
       <c r="I2" s="6"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="6"/>
+      <c r="J2" s="6"/>
+      <c r="L2" s="2"/>
       <c r="M2" s="6"/>
       <c r="N2" s="6"/>
+      <c r="O2" s="6"/>
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N3:N1000 D3:D1000 G3:G1000 J3:K1000" xr:uid="{B6CB3C84-EE01-4878-B558-650FC19D8248}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O3:O1000 E3:E1000 H3:H1000 K3:L1000" xr:uid="{B6CB3C84-EE01-4878-B558-650FC19D8248}">
       <formula1>"Saw, Hammer, Screwdriver, Wrench, Sockets, Pliers, Measuring, Files, Other"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2" xr:uid="{ACB7A40B-F0EE-4387-88E4-5140AB68313F}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2" xr:uid="{ACB7A40B-F0EE-4387-88E4-5140AB68313F}">
       <formula1>"Fastening/Turning,Measuring/Layout,Striking/Hammering,Gripping/Holding,Cutting/Shaping,Other"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:K2 H2" xr:uid="{2E543736-2E6D-4F90-9169-21BA7CCD7676}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2:L2 I2" xr:uid="{2E543736-2E6D-4F90-9169-21BA7CCD7676}">
       <formula1>"Operational,Needs Repair,Repair In-Progress,Unusable/Junk"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2201,28 +2249,29 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E1902F1-C59B-4A1A-9D95-2C39AEF944E5}">
   <sheetPr codeName="Sheet7"/>
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:S2"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
     <col min="2" max="3" width="10.33203125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="22.6640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="41.6640625" style="2" customWidth="1"/>
-    <col min="7" max="7" width="15.5546875" style="6" customWidth="1"/>
-    <col min="8" max="8" width="18.44140625" style="2" customWidth="1"/>
-    <col min="9" max="9" width="14.33203125" style="7" customWidth="1"/>
-    <col min="10" max="10" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.6640625" customWidth="1"/>
-    <col min="12" max="12" width="15.5546875" style="6" customWidth="1"/>
-    <col min="13" max="13" width="22.5546875" customWidth="1"/>
-    <col min="14" max="14" width="14.109375" style="7" customWidth="1"/>
-    <col min="15" max="15" width="10.44140625" style="3" customWidth="1"/>
-    <col min="17" max="17" width="22.6640625" style="2" customWidth="1"/>
-    <col min="18" max="18" width="46.6640625" style="2" customWidth="1"/>
-    <col min="19" max="16384" width="8.88671875" style="6"/>
+    <col min="4" max="4" width="15.33203125" style="16" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.6640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="41.6640625" style="2" customWidth="1"/>
+    <col min="8" max="8" width="15.5546875" style="6" customWidth="1"/>
+    <col min="9" max="9" width="18.44140625" style="2" customWidth="1"/>
+    <col min="10" max="10" width="14.33203125" style="7" customWidth="1"/>
+    <col min="11" max="11" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.6640625" customWidth="1"/>
+    <col min="13" max="13" width="15.5546875" style="6" customWidth="1"/>
+    <col min="14" max="14" width="22.5546875" customWidth="1"/>
+    <col min="15" max="15" width="14.109375" style="7" customWidth="1"/>
+    <col min="16" max="16" width="10.44140625" style="3" customWidth="1"/>
+    <col min="18" max="18" width="22.6640625" style="2" customWidth="1"/>
+    <col min="19" max="19" width="46.6640625" style="2" customWidth="1"/>
+    <col min="20" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18">
+    <row r="1" spans="1:19">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2232,52 +2281,55 @@
       <c r="C1" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="E1" t="s">
         <v>33</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>66</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>67</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>68</v>
       </c>
-      <c r="L1" s="8" t="s">
+      <c r="M1" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="O1" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="O1" s="6"/>
       <c r="P1" s="6"/>
       <c r="Q1" s="6"/>
       <c r="R1" s="6"/>
-    </row>
-    <row r="2" spans="1:18">
-      <c r="F2" s="2"/>
-      <c r="I2" s="3"/>
-      <c r="J2" s="6"/>
+      <c r="S1" s="6"/>
+    </row>
+    <row r="2" spans="1:19">
+      <c r="G2" s="2"/>
+      <c r="J2" s="3"/>
       <c r="K2" s="6"/>
-      <c r="L2" s="7"/>
-      <c r="M2" s="3" cm="1">
-        <f t="array" ref="M2">IF(
+      <c r="L2" s="6"/>
+      <c r="M2" s="7"/>
+      <c r="N2" s="3" cm="1">
+        <f t="array" ref="N2">IF(
     Shop_Consumables[[#This Row],[Stock_Level]]="Counted",
     Shop_Consumables[[#This Row],[Stock_Count]] * Shop_Consumables[[#This Row],[Unit Cost]],
     IF(
@@ -2293,15 +2345,15 @@
 )</f>
         <v>0</v>
       </c>
-      <c r="N2" s="2"/>
-      <c r="O2" s="6"/>
+      <c r="O2" s="2"/>
       <c r="P2" s="6"/>
       <c r="Q2" s="6"/>
       <c r="R2" s="6"/>
+      <c r="S2" s="6"/>
     </row>
   </sheetData>
   <dataValidations disablePrompts="1" count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:G2" xr:uid="{D2C605E8-D02B-4558-82DE-3169088704E8}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:H2" xr:uid="{D2C605E8-D02B-4558-82DE-3169088704E8}">
       <formula1>"Fasteners/Hardware,Abrasives/Cutting,Fluids/Lubricants/Chemicals,Primer/Paint,Safety/PPE,Shop/Janitorial,Welding,Electrical,Other"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
refactoring; added src/modules/hid-scanner.js and intake-wizard.js; deleted label.js
</commit_message>
<xml_diff>
--- a/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
+++ b/MAE_Workshop_Inventory_MASTER_TEMPLATE.xlsx
@@ -1,8 +1,8 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30309"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1a2ae81d67634e6/Desktop/Michanikos Artifex Enterprises/MAE Custom Digital Solutions/MAE Workshop Inventory Management System/GITHUB_MAE_Workshop Inventory App/"/>
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="320" documentId="13_ncr:1_{18ABDE8C-9C4E-4F00-B2FF-E4877FFDD8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8452EC8A-D701-49FA-9D0C-57212878EA28}"/>
   <bookViews>
-    <workbookView xWindow="2472" yWindow="1152" windowWidth="17676" windowHeight="11172" firstSheet="2" activeTab="3" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
+    <workbookView xWindow="2472" yWindow="1152" windowWidth="17676" windowHeight="11172" firstSheet="3" activeTab="3" xr2:uid="{BB4209F8-9B83-4E28-9EA3-8709A75F7EFC}"/>
   </bookViews>
   <sheets>
     <sheet name="Master Dashboard" sheetId="1" r:id="rId1"/>
@@ -76,6 +76,108 @@
     <t>mae_id</t>
   </si>
   <si>
+    <t>Total Resell Investment</t>
+  </si>
+  <si>
+    <t>Total Actual Sales</t>
+  </si>
+  <si>
+    <t>Total Machinery Value</t>
+  </si>
+  <si>
+    <t>Total Power Tool Value</t>
+  </si>
+  <si>
+    <t>Total Hand Tool Value</t>
+  </si>
+  <si>
+    <t>Total Consumables Value</t>
+  </si>
+  <si>
+    <t>Total Shop Asset Value</t>
+  </si>
+  <si>
+    <t>Low Stock Items Count</t>
+  </si>
+  <si>
+    <t>Total Amount Due Next 30 Days</t>
+  </si>
+  <si>
+    <t>Equipment With Operational Issues</t>
+  </si>
+  <si>
+    <t>Maintenance Items Due in Next 30 Days</t>
+  </si>
+  <si>
+    <t>Expense Category</t>
+  </si>
+  <si>
+    <t>Annual Total</t>
+  </si>
+  <si>
+    <t>Facility Costs/Rent/Mortgage</t>
+  </si>
+  <si>
+    <t>Insurance</t>
+  </si>
+  <si>
+    <t>Debt/Leases on Equipment/Business Loans</t>
+  </si>
+  <si>
+    <t>Subscriptions</t>
+  </si>
+  <si>
+    <t>Salaries</t>
+  </si>
+  <si>
+    <t>Utilities</t>
+  </si>
+  <si>
+    <t>Maintnance/Repair</t>
+  </si>
+  <si>
+    <t>Marketing/Advertising</t>
+  </si>
+  <si>
+    <t>Professional Fees</t>
+  </si>
+  <si>
+    <t>Travel/Vehicles</t>
+  </si>
+  <si>
+    <t>Depreciation</t>
+  </si>
+  <si>
+    <t>Other/Miscellaneous</t>
+  </si>
+  <si>
+    <t>Location_ID</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>TBD001</t>
+  </si>
+  <si>
+    <t>TBD</t>
+  </si>
+  <si>
+    <t>To Be Determined</t>
+  </si>
+  <si>
+    <t>Tag_ID</t>
+  </si>
+  <si>
+    <t>Tag_Type</t>
+  </si>
+  <si>
+    <t>Item_Category</t>
+  </si>
+  <si>
+    <t>Item_Description</t>
+  </si>
+  <si>
     <t>Category</t>
   </si>
   <si>
@@ -100,34 +202,73 @@
     <t>Actual Sale Price</t>
   </si>
   <si>
+    <t>Date Sold</t>
+  </si>
+  <si>
     <t>Purchase Date</t>
   </si>
   <si>
     <t>Purchase Cost</t>
   </si>
   <si>
+    <t>Condition</t>
+  </si>
+  <si>
+    <t>Serial Number/Other Info</t>
+  </si>
+  <si>
+    <t>Functional Category</t>
+  </si>
+  <si>
+    <t>Operational Category</t>
+  </si>
+  <si>
+    <t>Power Source</t>
+  </si>
+  <si>
+    <t>Remarks</t>
+  </si>
+  <si>
+    <t>Stock_Level</t>
+  </si>
+  <si>
+    <t>Stock_Count</t>
+  </si>
+  <si>
+    <t>Unit of Measure</t>
+  </si>
+  <si>
+    <t>Unit Cost</t>
+  </si>
+  <si>
+    <t>Bulk_Value</t>
+  </si>
+  <si>
+    <t>Reorder Point</t>
+  </si>
+  <si>
+    <t>Current Inventory Value</t>
+  </si>
+  <si>
+    <t>Supplier/Remarks</t>
+  </si>
+  <si>
+    <t>Asset and Service Description</t>
+  </si>
+  <si>
     <t>Performed By</t>
   </si>
   <si>
     <t>Cost</t>
   </si>
   <si>
-    <t>Condition</t>
-  </si>
-  <si>
-    <t>Unit of Measure</t>
-  </si>
-  <si>
-    <t>Reorder Point</t>
-  </si>
-  <si>
-    <t>Unit Cost</t>
-  </si>
-  <si>
-    <t>Expense Category</t>
-  </si>
-  <si>
-    <t>Description</t>
+    <t>Scheduled Service Date</t>
+  </si>
+  <si>
+    <t>Complete</t>
+  </si>
+  <si>
+    <t>Completion Date</t>
   </si>
   <si>
     <t>Payment Frequency</t>
@@ -142,163 +283,22 @@
     <t>Auto-Pay?</t>
   </si>
   <si>
+    <t>Supplier Name</t>
+  </si>
+  <si>
+    <t>Contact Person</t>
+  </si>
+  <si>
+    <t>Phone</t>
+  </si>
+  <si>
     <t>Email</t>
   </si>
   <si>
-    <t>Phone</t>
-  </si>
-  <si>
     <t>Website</t>
   </si>
   <si>
-    <t>Supplier Name</t>
-  </si>
-  <si>
-    <t>Contact Person</t>
-  </si>
-  <si>
     <t>Notes/Other Info</t>
-  </si>
-  <si>
-    <t>Functional Category</t>
-  </si>
-  <si>
-    <t>Operational Category</t>
-  </si>
-  <si>
-    <t>Power Source</t>
-  </si>
-  <si>
-    <t>Current Inventory Value</t>
-  </si>
-  <si>
-    <t>Location_ID</t>
-  </si>
-  <si>
-    <t>Asset and Service Description</t>
-  </si>
-  <si>
-    <t>Total Resell Investment</t>
-  </si>
-  <si>
-    <t>Total Actual Sales</t>
-  </si>
-  <si>
-    <t>Total Shop Asset Value</t>
-  </si>
-  <si>
-    <t>Low Stock Items Count</t>
-  </si>
-  <si>
-    <t>Total Machinery Value</t>
-  </si>
-  <si>
-    <t>Total Power Tool Value</t>
-  </si>
-  <si>
-    <t>Total Consumables Value</t>
-  </si>
-  <si>
-    <t>Total Hand Tool Value</t>
-  </si>
-  <si>
-    <t>Total Amount Due Next 30 Days</t>
-  </si>
-  <si>
-    <t>Annual Total</t>
-  </si>
-  <si>
-    <t>Facility Costs/Rent/Mortgage</t>
-  </si>
-  <si>
-    <t>Insurance</t>
-  </si>
-  <si>
-    <t>Debt/Leases on Equipment/Business Loans</t>
-  </si>
-  <si>
-    <t>Subscriptions</t>
-  </si>
-  <si>
-    <t>Salaries</t>
-  </si>
-  <si>
-    <t>Utilities</t>
-  </si>
-  <si>
-    <t>Maintnance/Repair</t>
-  </si>
-  <si>
-    <t>Marketing/Advertising</t>
-  </si>
-  <si>
-    <t>Professional Fees</t>
-  </si>
-  <si>
-    <t>Travel/Vehicles</t>
-  </si>
-  <si>
-    <t>Depreciation</t>
-  </si>
-  <si>
-    <t>Other/Miscellaneous</t>
-  </si>
-  <si>
-    <t>Equipment With Operational Issues</t>
-  </si>
-  <si>
-    <t>Maintenance Items Due in Next 30 Days</t>
-  </si>
-  <si>
-    <t>Complete</t>
-  </si>
-  <si>
-    <t>Remarks</t>
-  </si>
-  <si>
-    <t>Supplier/Remarks</t>
-  </si>
-  <si>
-    <t>Tag_ID</t>
-  </si>
-  <si>
-    <t>TBD</t>
-  </si>
-  <si>
-    <t>To Be Determined</t>
-  </si>
-  <si>
-    <t>TBD001</t>
-  </si>
-  <si>
-    <t>Stock_Level</t>
-  </si>
-  <si>
-    <t>Stock_Count</t>
-  </si>
-  <si>
-    <t>Bulk_Value</t>
-  </si>
-  <si>
-    <t>Completion Date</t>
-  </si>
-  <si>
-    <t>Date Sold</t>
-  </si>
-  <si>
-    <t>Serial Number/Other Info</t>
-  </si>
-  <si>
-    <t>Tag_Type</t>
-  </si>
-  <si>
-    <t>Item_Description</t>
-  </si>
-  <si>
-    <t>Scheduled Service Date</t>
-  </si>
-  <si>
-    <t>Item_Category</t>
   </si>
 </sst>
 </file>
@@ -398,26 +398,6 @@
   </cellStyles>
   <dxfs count="121">
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="0"/>
     </dxf>
@@ -576,6 +556,10 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="0"/>
     </dxf>
@@ -624,6 +608,10 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="0"/>
     </dxf>
@@ -670,6 +658,10 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <protection locked="0" hidden="0"/>
     </dxf>
@@ -704,6 +696,10 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -766,6 +762,10 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
+      <protection locked="0" hidden="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
@@ -897,10 +897,6 @@
     </a>
   </bag>
 </FeaturePropertyBags>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -954,33 +950,33 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:H2" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}" name="Shop_Overhead" displayName="Shop_Overhead" ref="A1:H2" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
   <autoFilter ref="A1:H2" xr:uid="{D2B78E2D-D1BA-4980-AD28-7371DA7E8BF1}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="20"/>
-    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="16"/>
-    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="15"/>
-    <tableColumn id="8" xr3:uid="{9140C4E8-CB9E-40BF-ABD9-13A971322B09}" name="Remarks" dataDxfId="14"/>
+    <tableColumn id="1" xr3:uid="{D0403366-FF83-43D4-A4A6-53D956BB53D5}" name="mae_id" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{115FC258-36AA-4A2D-895A-FE4B5FFF6B06}" name="Expense Category" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{4B114529-F91B-482E-9657-3D4FA758474D}" name="Description" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{F8FB0744-346B-4B81-82DA-5BADEC284B94}" name="Payment Frequency" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{D172DF65-3EB9-4C6D-9AB1-AF943A035CF4}" name="Due Date" dataDxfId="12"/>
+    <tableColumn id="6" xr3:uid="{B1E060DC-CDE4-40B3-9DE0-440A66FD2817}" name="Amount" dataDxfId="11"/>
+    <tableColumn id="7" xr3:uid="{BE283BC1-242E-4333-BF81-EBC4F9B2483D}" name="Auto-Pay?" dataDxfId="10"/>
+    <tableColumn id="8" xr3:uid="{9140C4E8-CB9E-40BF-ABD9-13A971322B09}" name="Remarks" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}" name="Supplier_Contacts" displayName="Supplier_Contacts" ref="A1:G2" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
   <autoFilter ref="A1:G2" xr:uid="{4D5A2D88-6FFF-49FE-93CF-46B9225A62FF}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="11"/>
-    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="9"/>
-    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="7"/>
-    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="6"/>
-    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{B1057331-F99D-4824-9EC8-9800B5256BF6}" name="mae_id" dataDxfId="6"/>
+    <tableColumn id="11" xr3:uid="{B56AF81F-63CB-4874-A9B8-B76E4D91E239}" name="Supplier Name" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{6D90D0F5-8F28-4725-BF13-0A57A9536E58}" name="Contact Person" dataDxfId="4"/>
+    <tableColumn id="10" xr3:uid="{DBCEF9D0-078A-4536-BA57-A5D99D4510DF}" name="Phone" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{2D53D9C2-51E7-4946-A506-A47B54EDDA21}" name="Email" dataDxfId="2"/>
+    <tableColumn id="12" xr3:uid="{A82FB354-D6D5-4ECA-B820-0C76DC34EF4D}" name="Website" dataDxfId="1"/>
+    <tableColumn id="9" xr3:uid="{48CFB17A-2B61-479C-A6CF-4AC3020D2F09}" name="Notes/Other Info" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1018,104 +1014,104 @@
     <tableColumn id="1" xr3:uid="{31EB6A75-D622-4C6B-8EF2-8277E8A807E0}" name="mae_id" dataDxfId="100"/>
     <tableColumn id="15" xr3:uid="{D25A390C-69B5-4326-A0D4-10EB45DDE5E5}" name="Tag_ID" dataDxfId="99"/>
     <tableColumn id="16" xr3:uid="{57D16231-357C-4C08-B062-20555121C2D6}" name="Tag_Type" dataDxfId="98"/>
-    <tableColumn id="2" xr3:uid="{0EA7C626-291A-4D56-A19A-BC3E098C0307}" name="Item_Category" dataDxfId="4"/>
-    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="97"/>
-    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item_Description" dataDxfId="96"/>
-    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="95"/>
-    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="94"/>
-    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="93"/>
-    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="92"/>
-    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="91">
+    <tableColumn id="2" xr3:uid="{0EA7C626-291A-4D56-A19A-BC3E098C0307}" name="Item_Category" dataDxfId="97"/>
+    <tableColumn id="12" xr3:uid="{0E775026-8B56-4554-BC18-AC94F0BDF20B}" name="Location_ID" dataDxfId="96"/>
+    <tableColumn id="3" xr3:uid="{F0848A0C-E009-47A8-9BE0-A358BFD7AFCB}" name="Item_Description" dataDxfId="95"/>
+    <tableColumn id="4" xr3:uid="{8A489BED-384E-4862-A8F1-BED75945CC4B}" name="Category" dataDxfId="94"/>
+    <tableColumn id="5" xr3:uid="{79CCD507-3486-45B8-B1D7-DE959429BBF9}" name="Acquisition Date" dataDxfId="93"/>
+    <tableColumn id="6" xr3:uid="{563DF2E7-2105-4612-A389-66D5F1AEDDF9}" name="Purchase Price" dataDxfId="92"/>
+    <tableColumn id="7" xr3:uid="{FDBBAA67-6187-4328-A88E-15A2886AD21A}" name="Restoration Cost" dataDxfId="91"/>
+    <tableColumn id="8" xr3:uid="{D8774B66-8C20-45C5-AA6A-345E630152B8}" name="Total Investment" dataDxfId="90">
       <calculatedColumnFormula>Resell_Inventory[[#This Row],[Purchase Price]]+Resell_Inventory[[#This Row],[Restoration Cost]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="90"/>
-    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="89"/>
-    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="88"/>
-    <tableColumn id="13" xr3:uid="{71578D4D-1C79-4D4F-9C0F-A2C991F460FD}" name="Date Sold" dataDxfId="87"/>
+    <tableColumn id="9" xr3:uid="{3664471D-925B-4CA7-9A43-C274BD7CE318}" name="Current Status" dataDxfId="89"/>
+    <tableColumn id="10" xr3:uid="{85695CF1-6906-4EBD-AC4D-EF944B62766A}" name="Target Sale Price" dataDxfId="88"/>
+    <tableColumn id="11" xr3:uid="{F63E0332-DE71-48C1-8BAE-52EDD7B233C7}" name="Actual Sale Price" dataDxfId="87"/>
+    <tableColumn id="13" xr3:uid="{71578D4D-1C79-4D4F-9C0F-A2C991F460FD}" name="Date Sold" dataDxfId="86"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:J2" insertRow="1" totalsRowShown="0" headerRowDxfId="86" dataDxfId="85">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}" name="Shop_Machinery" displayName="Shop_Machinery" ref="A1:J2" insertRow="1" totalsRowShown="0" headerRowDxfId="85" dataDxfId="84">
   <autoFilter ref="A1:J2" xr:uid="{7851396C-069E-4DB6-B1D4-8332D0E308D8}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="84"/>
-    <tableColumn id="4" xr3:uid="{17EB0B09-11B3-4E08-9442-E3C9AB87A157}" name="Tag_ID" dataDxfId="83"/>
-    <tableColumn id="5" xr3:uid="{72EAA357-95AA-4893-8038-2A77BDD0FB87}" name="Tag_Type" dataDxfId="82"/>
-    <tableColumn id="2" xr3:uid="{5F0AA36F-B9A6-466C-A044-4398E5CAD0BF}" name="Item_Category" dataDxfId="3"/>
-    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="81"/>
-    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Item_Description" dataDxfId="80"/>
-    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="79"/>
-    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="78"/>
-    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="77"/>
-    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Serial Number/Other Info" dataDxfId="76"/>
+    <tableColumn id="1" xr3:uid="{4BF4F34A-34E8-41F1-92A8-4DEC12050AE4}" name="mae_id" dataDxfId="83"/>
+    <tableColumn id="4" xr3:uid="{17EB0B09-11B3-4E08-9442-E3C9AB87A157}" name="Tag_ID" dataDxfId="82"/>
+    <tableColumn id="5" xr3:uid="{72EAA357-95AA-4893-8038-2A77BDD0FB87}" name="Tag_Type" dataDxfId="81"/>
+    <tableColumn id="2" xr3:uid="{5F0AA36F-B9A6-466C-A044-4398E5CAD0BF}" name="Item_Category" dataDxfId="80"/>
+    <tableColumn id="11" xr3:uid="{A87C02EA-516D-41DC-8958-0A24FBEA5139}" name="Location_ID" dataDxfId="79"/>
+    <tableColumn id="3" xr3:uid="{16C5F583-C3B4-49E4-BA38-E0F53D0CFD24}" name="Item_Description" dataDxfId="78"/>
+    <tableColumn id="6" xr3:uid="{E313FD7A-F612-42AE-85A6-8693FFF5D72E}" name="Purchase Date" dataDxfId="77"/>
+    <tableColumn id="7" xr3:uid="{5640579F-F227-4CF7-B821-9107014DE941}" name="Purchase Cost" dataDxfId="76"/>
+    <tableColumn id="9" xr3:uid="{4845845F-E747-418E-9E07-D7130AC62B65}" name="Condition" dataDxfId="75"/>
+    <tableColumn id="10" xr3:uid="{5A32000B-4543-43EE-ABB7-FB941F3116BD}" name="Serial Number/Other Info" dataDxfId="74"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:L2" totalsRowShown="0" headerRowDxfId="75" dataDxfId="74">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}" name="Shop_Power_Tools" displayName="Shop_Power_Tools" ref="A1:L2" totalsRowShown="0" headerRowDxfId="73" dataDxfId="72">
   <autoFilter ref="A1:L2" xr:uid="{B256D0AD-5808-43AD-9729-C30859C8E0E2}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="73"/>
-    <tableColumn id="11" xr3:uid="{21951C81-00A4-4344-9E81-B1B1DB06ADEF}" name="Tag_ID" dataDxfId="72"/>
-    <tableColumn id="12" xr3:uid="{7F1AFB3A-34F9-4E3E-A9D3-7E7E1458ECFE}" name="Tag_Type" dataDxfId="71"/>
-    <tableColumn id="2" xr3:uid="{176E61E7-BE6B-42DA-B1B1-AECC0921E70C}" name="Item_Category" dataDxfId="2"/>
-    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="70"/>
-    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Item_Description" dataDxfId="69"/>
-    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="68"/>
-    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="67"/>
-    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="66"/>
-    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="65"/>
-    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="64"/>
-    <tableColumn id="10" xr3:uid="{26197E01-2936-4F5F-8081-3AA351C1CD38}" name="Remarks" dataDxfId="63"/>
+    <tableColumn id="1" xr3:uid="{14D3C0F3-786E-4D59-8EBE-4E8ECDF77355}" name="mae_id" dataDxfId="71"/>
+    <tableColumn id="11" xr3:uid="{21951C81-00A4-4344-9E81-B1B1DB06ADEF}" name="Tag_ID" dataDxfId="70"/>
+    <tableColumn id="12" xr3:uid="{7F1AFB3A-34F9-4E3E-A9D3-7E7E1458ECFE}" name="Tag_Type" dataDxfId="69"/>
+    <tableColumn id="2" xr3:uid="{176E61E7-BE6B-42DA-B1B1-AECC0921E70C}" name="Item_Category" dataDxfId="68"/>
+    <tableColumn id="6" xr3:uid="{713E4785-F162-4507-8CEC-58D1900A8AB6}" name="Location_ID" dataDxfId="67"/>
+    <tableColumn id="3" xr3:uid="{864AFF0F-A6FF-4703-9283-093CABA0AB94}" name="Item_Description" dataDxfId="66"/>
+    <tableColumn id="9" xr3:uid="{DC8BF91E-CE6C-4B37-88B8-9D97E3E9201C}" name="Purchase Price" dataDxfId="65"/>
+    <tableColumn id="4" xr3:uid="{33A9C397-237A-43D3-A581-5DA7BEC5BEAE}" name="Functional Category" dataDxfId="64"/>
+    <tableColumn id="7" xr3:uid="{4343A0FC-A88F-4191-8D18-BC86509BFBFF}" name="Operational Category" dataDxfId="63"/>
+    <tableColumn id="8" xr3:uid="{DE84C9AE-3DAD-4522-AFC2-61396BA01671}" name="Power Source" dataDxfId="62"/>
+    <tableColumn id="5" xr3:uid="{5416B904-9CBE-4604-9D84-C743A1D623A9}" name="Condition" dataDxfId="61"/>
+    <tableColumn id="10" xr3:uid="{26197E01-2936-4F5F-8081-3AA351C1CD38}" name="Remarks" dataDxfId="60"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:L2" totalsRowShown="0" headerRowDxfId="62" dataDxfId="61">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}" name="Shop_Hand_Tools" displayName="Shop_Hand_Tools" ref="A1:L2" totalsRowShown="0" headerRowDxfId="59" dataDxfId="58">
   <autoFilter ref="A1:L2" xr:uid="{FA38DE34-8744-4C90-AB61-00EF0F13B199}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="60"/>
-    <tableColumn id="10" xr3:uid="{C8BD69AA-9023-4777-9C96-39A81F1E4BE0}" name="Tag_ID" dataDxfId="59"/>
-    <tableColumn id="12" xr3:uid="{FC4D7CE3-2DF1-465E-A4D1-1D1F02F8B8CA}" name="Tag_Type" dataDxfId="58"/>
-    <tableColumn id="2" xr3:uid="{54155A52-92C4-4BB0-A374-70E75592F98A}" name="Item_Category" dataDxfId="1"/>
-    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="57"/>
-    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Item_Description" dataDxfId="56"/>
-    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="55"/>
-    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="54"/>
-    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="53"/>
-    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Stock_Level" dataDxfId="52"/>
-    <tableColumn id="11" xr3:uid="{FD8D2D17-0451-45E0-8688-0BB4F60073DA}" name="Stock_Count" dataDxfId="51"/>
-    <tableColumn id="9" xr3:uid="{2B57F5E6-66C5-4DBA-8949-836DE0F0791C}" name="Remarks" dataDxfId="50"/>
+    <tableColumn id="1" xr3:uid="{2B19855D-9BAD-44E0-A316-C1FF95F743CC}" name="mae_id" dataDxfId="57"/>
+    <tableColumn id="10" xr3:uid="{C8BD69AA-9023-4777-9C96-39A81F1E4BE0}" name="Tag_ID" dataDxfId="56"/>
+    <tableColumn id="12" xr3:uid="{FC4D7CE3-2DF1-465E-A4D1-1D1F02F8B8CA}" name="Tag_Type" dataDxfId="55"/>
+    <tableColumn id="2" xr3:uid="{54155A52-92C4-4BB0-A374-70E75592F98A}" name="Item_Category" dataDxfId="54"/>
+    <tableColumn id="7" xr3:uid="{644102FD-D33A-4A70-A829-7ECBDAD17954}" name="Location_ID" dataDxfId="53"/>
+    <tableColumn id="3" xr3:uid="{69442715-C75E-4B47-9564-7C3C4A1F6DAA}" name="Item_Description" dataDxfId="52"/>
+    <tableColumn id="6" xr3:uid="{FEE72CB9-B490-4E03-9BBA-F46847223551}" name="Purchase Price" dataDxfId="51"/>
+    <tableColumn id="4" xr3:uid="{A8D20E4D-22EA-421D-82C7-3A077CDA19E8}" name="Category" dataDxfId="50"/>
+    <tableColumn id="8" xr3:uid="{080EB12A-CA17-4337-B46C-53DEAA3B2327}" name="Condition" dataDxfId="49"/>
+    <tableColumn id="5" xr3:uid="{F2705B4D-CE08-40AB-8854-3954BE8800AA}" name="Stock_Level" dataDxfId="48"/>
+    <tableColumn id="11" xr3:uid="{FD8D2D17-0451-45E0-8688-0BB4F60073DA}" name="Stock_Count" dataDxfId="47"/>
+    <tableColumn id="9" xr3:uid="{2B57F5E6-66C5-4DBA-8949-836DE0F0791C}" name="Remarks" dataDxfId="46"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:O2" totalsRowShown="0" headerRowDxfId="49" dataDxfId="48">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}" name="Shop_Consumables" displayName="Shop_Consumables" ref="A1:O2" totalsRowShown="0" headerRowDxfId="45" dataDxfId="44">
   <autoFilter ref="A1:O2" xr:uid="{212D9CF8-0BB2-4891-BFC6-736775F62E4D}"/>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="47"/>
-    <tableColumn id="12" xr3:uid="{8F0FD29C-682B-41B4-82F2-913D40801887}" name="Tag_ID" dataDxfId="46"/>
-    <tableColumn id="15" xr3:uid="{CE0ECF5F-5626-4215-AC71-301755B31D23}" name="Tag_Type" dataDxfId="45"/>
-    <tableColumn id="3" xr3:uid="{F28BB55E-442A-44A7-9EBB-E9F69B0BE27A}" name="Item_Category" dataDxfId="0"/>
-    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="44"/>
-    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item_Description" dataDxfId="43"/>
-    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="42"/>
-    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Stock_Level" dataDxfId="41"/>
-    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="40"/>
-    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="39"/>
-    <tableColumn id="13" xr3:uid="{AA55BCE3-9AC1-4735-8622-15E62CA93E1A}" name="Stock_Count" dataDxfId="38"/>
-    <tableColumn id="14" xr3:uid="{FA5C79D4-6D25-4E4C-BE9F-4190C63530C2}" name="Bulk_Value" dataDxfId="37"/>
-    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="36"/>
-    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="35">
+    <tableColumn id="1" xr3:uid="{43C4A9D4-2E17-4D62-8C0D-8DEDF0B4423A}" name="mae_id" dataDxfId="43"/>
+    <tableColumn id="12" xr3:uid="{8F0FD29C-682B-41B4-82F2-913D40801887}" name="Tag_ID" dataDxfId="42"/>
+    <tableColumn id="15" xr3:uid="{CE0ECF5F-5626-4215-AC71-301755B31D23}" name="Tag_Type" dataDxfId="41"/>
+    <tableColumn id="3" xr3:uid="{F28BB55E-442A-44A7-9EBB-E9F69B0BE27A}" name="Item_Category" dataDxfId="40"/>
+    <tableColumn id="11" xr3:uid="{511966F0-606F-407D-B09E-02F31902094D}" name="Location_ID" dataDxfId="39"/>
+    <tableColumn id="2" xr3:uid="{89FEB2D0-FBCD-4BE1-84C9-99FC556BBA41}" name="Item_Description" dataDxfId="38"/>
+    <tableColumn id="9" xr3:uid="{3CECC6F9-9090-442B-A1A1-8A7961DEB8AF}" name="Category" dataDxfId="37"/>
+    <tableColumn id="5" xr3:uid="{374E0561-27A0-4254-B830-D7E7F0E1D5AE}" name="Stock_Level" dataDxfId="36"/>
+    <tableColumn id="4" xr3:uid="{BE4BDDA8-E894-4184-B2C5-A998CB44E20F}" name="Unit of Measure" dataDxfId="35"/>
+    <tableColumn id="7" xr3:uid="{EB68210F-A1A5-4B47-B8FB-56CB47C8487E}" name="Unit Cost" dataDxfId="34"/>
+    <tableColumn id="13" xr3:uid="{AA55BCE3-9AC1-4735-8622-15E62CA93E1A}" name="Stock_Count" dataDxfId="33"/>
+    <tableColumn id="14" xr3:uid="{FA5C79D4-6D25-4E4C-BE9F-4190C63530C2}" name="Bulk_Value" dataDxfId="32"/>
+    <tableColumn id="6" xr3:uid="{767749E4-A67C-4AFF-BA8F-5DBF1AF53F43}" name="Reorder Point" dataDxfId="31"/>
+    <tableColumn id="10" xr3:uid="{AD664ABD-E878-4391-A095-B228A1F2A62D}" name="Current Inventory Value" dataDxfId="30">
       <calculatedColumnFormula array="1">IF(
     Shop_Consumables[[#This Row],[Stock_Level]]="Counted",
     Shop_Consumables[[#This Row],[Stock_Count]] * Shop_Consumables[[#This Row],[Unit Cost]],
@@ -1131,24 +1127,24 @@
     )
 )</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Supplier/Remarks" dataDxfId="34"/>
+    <tableColumn id="8" xr3:uid="{E92F90B7-BEB2-4C65-80CE-6243F77F7CC4}" name="Supplier/Remarks" dataDxfId="29"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:H2" totalsRowShown="0" headerRowDxfId="33" dataDxfId="32">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}" name="Maintenance_Log" displayName="Maintenance_Log" ref="A1:H2" totalsRowShown="0" headerRowDxfId="28" dataDxfId="27">
   <autoFilter ref="A1:H2" xr:uid="{4F48D65F-395D-4E16-BB60-D764CB43F7DA}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="31"/>
-    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="30"/>
-    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="29"/>
-    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="28"/>
-    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Scheduled Service Date" dataDxfId="27"/>
-    <tableColumn id="11" xr3:uid="{4809319D-ABCA-43DA-A400-5DC91167D78B}" name="Complete" dataDxfId="26"/>
-    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Completion Date" dataDxfId="25"/>
-    <tableColumn id="12" xr3:uid="{920CB592-D743-4B33-A796-C7F3DB32211C}" name="Remarks" dataDxfId="24"/>
+    <tableColumn id="1" xr3:uid="{89DC1EFB-4874-484F-8A54-71D285209A36}" name="mae_id" dataDxfId="26"/>
+    <tableColumn id="10" xr3:uid="{CE8F9225-208D-4395-B2DF-2A6CBB978A83}" name="Asset and Service Description" dataDxfId="25"/>
+    <tableColumn id="6" xr3:uid="{4C05311A-4D79-4E1B-9C84-A70DDD428604}" name="Performed By" dataDxfId="24"/>
+    <tableColumn id="7" xr3:uid="{42638730-F8E7-4618-B878-1C695760484E}" name="Cost" dataDxfId="23"/>
+    <tableColumn id="8" xr3:uid="{3F292746-268F-4EF2-B0BF-D9E17CC16858}" name="Scheduled Service Date" dataDxfId="22"/>
+    <tableColumn id="11" xr3:uid="{4809319D-ABCA-43DA-A400-5DC91167D78B}" name="Complete" dataDxfId="21"/>
+    <tableColumn id="4" xr3:uid="{2C9C0290-D9A7-42F8-BE3E-7F3F40E5A31F}" name="Completion Date" dataDxfId="20"/>
+    <tableColumn id="12" xr3:uid="{920CB592-D743-4B33-A796-C7F3DB32211C}" name="Remarks" dataDxfId="19"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1473,21 +1469,21 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2834D935-E140-4D64-A4CD-4A9FB8899FE0}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:L2"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="29.109375" style="3" customWidth="1"/>
+    <col min="1" max="1" width="9.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.140625" style="3" customWidth="1"/>
     <col min="3" max="3" width="18" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.44140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.77734375" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="21.44140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="24.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.28515625" style="3" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="22" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="22.109375" style="12" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.140625" style="12" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="29" style="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="32.88671875" style="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="32.88671875" style="7" bestFit="1" customWidth="1"/>
-    <col min="13" max="16384" width="8.88671875" style="6"/>
+    <col min="11" max="11" width="32.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="32.85546875" style="7" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="8.85546875" style="6"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
@@ -1495,37 +1491,37 @@
         <v>0</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>36</v>
+        <v>2</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>39</v>
+        <v>3</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>40</v>
+        <v>4</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>42</v>
+        <v>5</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>41</v>
+        <v>6</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>37</v>
+        <v>7</v>
       </c>
       <c r="I1" s="11" t="s">
-        <v>38</v>
+        <v>8</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>43</v>
+        <v>9</v>
       </c>
       <c r="K1" s="8" t="s">
-        <v>57</v>
+        <v>10</v>
       </c>
       <c r="L1" s="8" t="s">
-        <v>58</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:12">
@@ -1595,17 +1591,17 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3185D484-1AEA-488F-ADB2-C66611F8B5C9}">
   <sheetPr codeName="Sheet8"/>
   <dimension ref="A1:I2"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
-    <col min="2" max="2" width="28.88671875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="60.6640625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="19.33203125" style="2" customWidth="1"/>
-    <col min="5" max="5" width="10.33203125" style="10" customWidth="1"/>
-    <col min="6" max="6" width="9.33203125" style="3" customWidth="1"/>
-    <col min="8" max="8" width="14.33203125" style="2" customWidth="1"/>
-    <col min="9" max="9" width="9.33203125" style="2" customWidth="1"/>
-    <col min="10" max="16384" width="8.88671875" style="6"/>
+    <col min="2" max="2" width="28.85546875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="60.7109375" style="2" customWidth="1"/>
+    <col min="4" max="4" width="19.28515625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="10.28515625" style="10" customWidth="1"/>
+    <col min="6" max="6" width="9.28515625" style="3" customWidth="1"/>
+    <col min="8" max="8" width="14.28515625" style="2" customWidth="1"/>
+    <col min="9" max="9" width="9.28515625" style="2" customWidth="1"/>
+    <col min="10" max="16384" width="8.85546875" style="6"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -1613,25 +1609,25 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>19</v>
+        <v>66</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>20</v>
+        <v>67</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>21</v>
+        <v>68</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>22</v>
+        <v>69</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="I1" s="6"/>
     </row>
@@ -1665,15 +1661,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6150BED1-88FC-488E-B7E1-4C6CBEB9589C}">
   <sheetPr codeName="Sheet9"/>
   <dimension ref="A1:G1"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
-    <col min="2" max="2" width="25.109375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="30.5546875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="25.140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="30.5703125" style="2" customWidth="1"/>
     <col min="4" max="4" width="21" style="2" customWidth="1"/>
-    <col min="5" max="6" width="20.6640625" style="2" customWidth="1"/>
-    <col min="7" max="7" width="32.33203125" style="2" customWidth="1"/>
-    <col min="8" max="16384" width="8.88671875" style="6"/>
+    <col min="5" max="6" width="20.7109375" style="2" customWidth="1"/>
+    <col min="7" max="7" width="32.28515625" style="2" customWidth="1"/>
+    <col min="8" max="16384" width="8.85546875" style="6"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -1681,22 +1677,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>26</v>
+        <v>70</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>27</v>
+        <v>71</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>24</v>
+        <v>72</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>23</v>
+        <v>73</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>25</v>
+        <v>74</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>28</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -1710,23 +1706,23 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E53ED58-AF1A-4384-BD5D-DFB0D7D062C9}">
   <dimension ref="A9:B21"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="42.21875" style="4" customWidth="1"/>
-    <col min="2" max="2" width="17.5546875" style="5" customWidth="1"/>
+    <col min="1" max="1" width="42.28515625" style="4" customWidth="1"/>
+    <col min="2" max="2" width="17.5703125" style="5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="9" spans="1:2">
       <c r="A9" s="4" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>44</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2" t="s">
-        <v>45</v>
+        <v>14</v>
       </c>
       <c r="B10" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -1735,7 +1731,7 @@
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="2" t="s">
-        <v>46</v>
+        <v>15</v>
       </c>
       <c r="B11" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -1744,7 +1740,7 @@
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2" t="s">
-        <v>47</v>
+        <v>16</v>
       </c>
       <c r="B12" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -1753,7 +1749,7 @@
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="2" t="s">
-        <v>48</v>
+        <v>17</v>
       </c>
       <c r="B13" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -1762,7 +1758,7 @@
     </row>
     <row r="14" spans="1:2">
       <c r="A14" s="2" t="s">
-        <v>49</v>
+        <v>18</v>
       </c>
       <c r="B14" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -1771,7 +1767,7 @@
     </row>
     <row r="15" spans="1:2">
       <c r="A15" s="2" t="s">
-        <v>50</v>
+        <v>19</v>
       </c>
       <c r="B15" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -1780,7 +1776,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" s="2" t="s">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="B16" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -1789,7 +1785,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" s="2" t="s">
-        <v>52</v>
+        <v>21</v>
       </c>
       <c r="B17" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -1798,7 +1794,7 @@
     </row>
     <row r="18" spans="1:2">
       <c r="A18" s="2" t="s">
-        <v>53</v>
+        <v>22</v>
       </c>
       <c r="B18" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -1807,7 +1803,7 @@
     </row>
     <row r="19" spans="1:2">
       <c r="A19" s="2" t="s">
-        <v>54</v>
+        <v>23</v>
       </c>
       <c r="B19" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -1816,7 +1812,7 @@
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="2" t="s">
-        <v>55</v>
+        <v>24</v>
       </c>
       <c r="B20" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -1825,7 +1821,7 @@
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="2" t="s">
-        <v>56</v>
+        <v>25</v>
       </c>
       <c r="B21" s="5">
         <f>SUMIF(Shop_Overhead[Expense Category], Overhead_Summary[[#This Row],[Expense Category]], Shop_Overhead[Amount])</f>
@@ -1848,11 +1844,11 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6A08BCD-5A8C-45EE-A940-2FEFA1E5B102}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
-    <col min="2" max="2" width="96.88671875" customWidth="1"/>
-    <col min="3" max="3" width="95.77734375" style="4" customWidth="1"/>
+    <col min="2" max="2" width="96.85546875" customWidth="1"/>
+    <col min="3" max="3" width="95.7109375" style="4" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1860,21 +1856,21 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="1" t="s">
-        <v>65</v>
+        <v>28</v>
       </c>
       <c r="B2" t="s">
-        <v>63</v>
+        <v>29</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>64</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -1889,26 +1885,26 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDE7BF89-A2E7-4A6F-B822-317739E206EC}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:R2"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
-    <col min="2" max="3" width="9.5546875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="15.33203125" style="16" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="31.44140625" style="2" customWidth="1"/>
-    <col min="7" max="7" width="10.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="9.5703125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="15.28515625" style="16" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="31.42578125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="10.5703125" style="2" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="17" style="10" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.33203125" style="3" customWidth="1"/>
-    <col min="10" max="10" width="16.5546875" style="3" customWidth="1"/>
-    <col min="11" max="11" width="16.6640625" style="5" customWidth="1"/>
-    <col min="12" max="12" width="19.109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.6640625" style="3" customWidth="1"/>
-    <col min="14" max="14" width="16.88671875" style="3" customWidth="1"/>
-    <col min="15" max="15" width="16.88671875" style="10" customWidth="1"/>
-    <col min="16" max="16" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="16.88671875" style="6" customWidth="1"/>
-    <col min="18" max="18" width="16.88671875" style="2" customWidth="1"/>
-    <col min="19" max="16384" width="8.88671875" style="6"/>
+    <col min="9" max="9" width="15.28515625" style="3" customWidth="1"/>
+    <col min="10" max="10" width="16.5703125" style="3" customWidth="1"/>
+    <col min="11" max="11" width="16.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="19.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.7109375" style="3" customWidth="1"/>
+    <col min="14" max="14" width="16.85546875" style="3" customWidth="1"/>
+    <col min="15" max="15" width="16.85546875" style="10" customWidth="1"/>
+    <col min="16" max="16" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.85546875" style="6" customWidth="1"/>
+    <col min="18" max="18" width="16.85546875" style="2" customWidth="1"/>
+    <col min="19" max="16384" width="8.85546875" style="6"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
@@ -1916,46 +1912,46 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>62</v>
+        <v>31</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>72</v>
+        <v>32</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="E1" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>73</v>
+        <v>34</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="H1" s="9" t="s">
-        <v>2</v>
+        <v>36</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>3</v>
+        <v>37</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>4</v>
+        <v>38</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>5</v>
+        <v>39</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>6</v>
+        <v>40</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>7</v>
+        <v>41</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>8</v>
+        <v>42</v>
       </c>
       <c r="O1" s="9" t="s">
-        <v>70</v>
+        <v>43</v>
       </c>
       <c r="P1" s="6"/>
       <c r="R1" s="6"/>
@@ -1993,19 +1989,19 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B027EC69-551F-4051-8A71-8B106D207C6D}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:K2"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
-    <col min="2" max="3" width="9.5546875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="15.33203125" style="16" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.33203125" style="6" customWidth="1"/>
-    <col min="6" max="6" width="28.6640625" style="2" customWidth="1"/>
-    <col min="7" max="7" width="14.6640625" style="10" customWidth="1"/>
-    <col min="8" max="8" width="14.6640625" style="3" customWidth="1"/>
-    <col min="9" max="9" width="12.88671875" customWidth="1"/>
-    <col min="10" max="10" width="40.88671875" style="6" customWidth="1"/>
-    <col min="11" max="11" width="32.6640625" style="2" customWidth="1"/>
-    <col min="12" max="16384" width="8.88671875" style="6"/>
+    <col min="2" max="3" width="9.5703125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="15.28515625" style="16" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.28515625" style="6" customWidth="1"/>
+    <col min="6" max="6" width="28.7109375" style="2" customWidth="1"/>
+    <col min="7" max="7" width="14.7109375" style="10" customWidth="1"/>
+    <col min="8" max="8" width="14.7109375" style="3" customWidth="1"/>
+    <col min="9" max="9" width="12.85546875" customWidth="1"/>
+    <col min="10" max="10" width="40.85546875" style="6" customWidth="1"/>
+    <col min="11" max="11" width="32.7109375" style="2" customWidth="1"/>
+    <col min="12" max="16384" width="8.85546875" style="6"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
@@ -2013,31 +2009,31 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>62</v>
+        <v>31</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>72</v>
+        <v>32</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="E1" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>73</v>
+        <v>34</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>9</v>
+        <v>44</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="I1" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>71</v>
+        <v>47</v>
       </c>
       <c r="K1" s="6"/>
     </row>
@@ -2066,21 +2062,21 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEDDDAA7-75C3-4AA5-ABFD-D5FB4C627E4C}">
   <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:N2"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
-    <col min="2" max="3" width="8.6640625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="15.33203125" style="16" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.88671875" style="6" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="50.44140625" style="2" customWidth="1"/>
-    <col min="7" max="7" width="15.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.88671875" style="6" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="19.88671875" style="6" customWidth="1"/>
-    <col min="11" max="11" width="14.44140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.5546875" style="6" customWidth="1"/>
-    <col min="14" max="14" width="14.44140625" style="2" customWidth="1"/>
-    <col min="15" max="16384" width="8.88671875" style="6"/>
+    <col min="2" max="3" width="8.7109375" style="2" customWidth="1"/>
+    <col min="4" max="4" width="15.28515625" style="16" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="50.42578125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="15.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.85546875" style="6" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.85546875" style="6" customWidth="1"/>
+    <col min="11" max="11" width="14.42578125" style="6" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.5703125" style="6" customWidth="1"/>
+    <col min="14" max="14" width="14.42578125" style="2" customWidth="1"/>
+    <col min="15" max="16384" width="8.85546875" style="6"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -2088,37 +2084,37 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>62</v>
+        <v>31</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>72</v>
+        <v>32</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="E1" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>73</v>
+        <v>34</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>3</v>
+        <v>37</v>
       </c>
       <c r="H1" t="s">
-        <v>29</v>
+        <v>48</v>
       </c>
       <c r="I1" t="s">
-        <v>30</v>
+        <v>49</v>
       </c>
       <c r="J1" t="s">
-        <v>31</v>
+        <v>50</v>
       </c>
       <c r="K1" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="N1" s="6"/>
     </row>
@@ -2160,22 +2156,22 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F39ADDA6-CD5F-4655-A9C0-9676DDAC362E}">
   <sheetPr codeName="Sheet6"/>
   <dimension ref="A1:O2"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="8.6640625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="15.33203125" style="16" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.88671875" style="6" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="54.6640625" style="2" customWidth="1"/>
-    <col min="7" max="7" width="15.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.5546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.6640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="16.33203125" style="7" customWidth="1"/>
-    <col min="15" max="15" width="12.88671875" style="2" customWidth="1"/>
-    <col min="16" max="16384" width="8.88671875" style="6"/>
+    <col min="1" max="1" width="9.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="8.7109375" style="2" customWidth="1"/>
+    <col min="4" max="4" width="15.28515625" style="16" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="54.7109375" style="2" customWidth="1"/>
+    <col min="7" max="7" width="15.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.5703125" style="6" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="16.28515625" style="7" customWidth="1"/>
+    <col min="15" max="15" width="12.85546875" style="2" customWidth="1"/>
+    <col min="16" max="16384" width="8.85546875" style="6"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
@@ -2183,37 +2179,37 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>62</v>
+        <v>31</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>72</v>
+        <v>32</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="E1" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>73</v>
+        <v>34</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>3</v>
+        <v>37</v>
       </c>
       <c r="H1" t="s">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="I1" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="J1" t="s">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="K1" t="s">
-        <v>67</v>
+        <v>53</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="M1" s="6"/>
       <c r="N1" s="6"/>
@@ -2250,25 +2246,25 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E1902F1-C59B-4A1A-9D95-2C39AEF944E5}">
   <sheetPr codeName="Sheet7"/>
   <dimension ref="A1:S2"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="9" style="1" customWidth="1"/>
-    <col min="2" max="3" width="10.33203125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="15.33203125" style="16" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.6640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="41.6640625" style="2" customWidth="1"/>
-    <col min="8" max="8" width="15.5546875" style="6" customWidth="1"/>
-    <col min="9" max="9" width="18.44140625" style="2" customWidth="1"/>
-    <col min="10" max="10" width="14.33203125" style="7" customWidth="1"/>
-    <col min="11" max="11" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.6640625" customWidth="1"/>
-    <col min="13" max="13" width="15.5546875" style="6" customWidth="1"/>
-    <col min="14" max="14" width="22.5546875" customWidth="1"/>
-    <col min="15" max="15" width="14.109375" style="7" customWidth="1"/>
-    <col min="16" max="16" width="10.44140625" style="3" customWidth="1"/>
-    <col min="18" max="18" width="22.6640625" style="2" customWidth="1"/>
-    <col min="19" max="19" width="46.6640625" style="2" customWidth="1"/>
-    <col min="20" max="16384" width="8.88671875" style="6"/>
+    <col min="2" max="3" width="10.28515625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="15.28515625" style="16" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="41.7109375" style="2" customWidth="1"/>
+    <col min="8" max="8" width="15.5703125" style="6" customWidth="1"/>
+    <col min="9" max="9" width="18.42578125" style="2" customWidth="1"/>
+    <col min="10" max="10" width="14.28515625" style="7" customWidth="1"/>
+    <col min="11" max="11" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.7109375" customWidth="1"/>
+    <col min="13" max="13" width="15.5703125" style="6" customWidth="1"/>
+    <col min="14" max="14" width="22.5703125" customWidth="1"/>
+    <col min="15" max="15" width="14.140625" style="7" customWidth="1"/>
+    <col min="16" max="16" width="10.42578125" style="3" customWidth="1"/>
+    <col min="18" max="18" width="22.7109375" style="2" customWidth="1"/>
+    <col min="19" max="19" width="46.7109375" style="2" customWidth="1"/>
+    <col min="20" max="16384" width="8.85546875" style="6"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">
@@ -2276,46 +2272,46 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>62</v>
+        <v>31</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>72</v>
+        <v>32</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="E1" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>73</v>
+        <v>34</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="H1" t="s">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>14</v>
+        <v>54</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>16</v>
+        <v>55</v>
       </c>
       <c r="K1" t="s">
-        <v>67</v>
+        <v>53</v>
       </c>
       <c r="L1" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="M1" s="8" t="s">
-        <v>15</v>
+        <v>57</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>32</v>
+        <v>58</v>
       </c>
       <c r="O1" s="4" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="P1" s="6"/>
       <c r="Q1" s="6"/>
@@ -2369,20 +2365,20 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB7AACC4-9DA2-4A53-AD77-8C5E0C1BF474}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:K2"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.21875" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.6640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.33203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.44140625" style="9" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.33203125" style="10" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.28515625" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.42578125" style="9" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.28515625" style="10" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="18" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.44140625" style="2" customWidth="1"/>
-    <col min="11" max="11" width="9.88671875" style="3" customWidth="1"/>
-    <col min="12" max="16384" width="8.88671875" style="6"/>
+    <col min="10" max="10" width="13.42578125" style="2" customWidth="1"/>
+    <col min="11" max="11" width="9.85546875" style="3" customWidth="1"/>
+    <col min="12" max="16384" width="8.85546875" style="6"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
@@ -2390,25 +2386,25 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>34</v>
+        <v>60</v>
       </c>
       <c r="C1" t="s">
-        <v>11</v>
+        <v>61</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>12</v>
+        <v>62</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="F1" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="I1" s="6"/>
       <c r="J1" s="6"/>

</xml_diff>